<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-14 22:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -29775,7 +29775,7 @@
     </row>
     <row r="620" spans="1:12">
       <c r="A620" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="B620" t="s">
         <v>656</v>
@@ -29799,7 +29799,7 @@
         <v>1571</v>
       </c>
       <c r="I620" t="s">
-        <v>1645</v>
+        <v>1587</v>
       </c>
       <c r="J620" t="s">
         <v>2315</v>
@@ -29808,7 +29808,7 @@
         <v>2410</v>
       </c>
       <c r="L620" t="s">
-        <v>2528</v>
+        <v>2540</v>
       </c>
     </row>
     <row r="621" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-16 02:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -103,6 +103,9 @@
     <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>ADMISSIBILIDADE DA SECRETARIA DO GATE</t>
   </si>
   <si>
@@ -124,9 +127,6 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ECONOMIA</t>
   </si>
   <si>
-    <t>SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>NÚCLEO TÉCNICO DE ENGENHARIA, SECRETARIA GERAL DO GATE</t>
   </si>
   <si>
@@ -4966,106 +4966,106 @@
     <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
   </si>
   <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>SUZAN NIGRI</t>
+  </si>
+  <si>
+    <t>PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
+    <t>THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES,JULIANA MARTINS BAHIENSE,RODRIGO VALENTE SERRA</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>REINALDO DE SOUZA MACHADO</t>
+  </si>
+  <si>
+    <t>RODRIGO VENTURA MARRA,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>CHRISTIANA ROSA FERREIRA</t>
+  </si>
+  <si>
+    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
+  </si>
+  <si>
+    <t>JULIANA MARTINS BAHIENSE,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>CAROLINE OLIVEIRA DE MENEZES</t>
+  </si>
+  <si>
+    <t>PATRICIA PASSARO DA SILVA TOLEDO,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>EDUARDO COUTO SOLEDADE</t>
+  </si>
+  <si>
+    <t>HELENA FERREIRA DE LIMA</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>DIANA DELGADO DA COSTA DA SILVA</t>
+  </si>
+  <si>
+    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT</t>
+  </si>
+  <si>
+    <t>MARCELO KOLBLINGER DE GODOY</t>
+  </si>
+  <si>
+    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,SEZISNANDO JOSE PRIMO PAES</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA,ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
+  </si>
+  <si>
+    <t>FERNANDA ZUCOLOTTO</t>
+  </si>
+  <si>
+    <t>RAQUEL SILVA FERNANDES LYRA</t>
+  </si>
+  <si>
+    <t>RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>FERNANDA ZUCOLOTTO,MARINA DE AQUINO PARREIRA XAVIER</t>
+  </si>
+  <si>
+    <t>DAYSE BARBOSA DE ARAÚJO GÓIS</t>
+  </si>
+  <si>
+    <t>FLAVIA REIS RIBEIRO BASTOS, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>SEZISNANDO JOSE PRIMO PAES</t>
+  </si>
+  <si>
+    <t>LEONARDO ARAÚJO DE SOUZA</t>
+  </si>
+  <si>
+    <t>RODRIGO VALENTE SERRA,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
     <t>GLAUCO CASTILHO DE ALMEIDA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>SUZAN NIGRI</t>
-  </si>
-  <si>
-    <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES,JULIANA MARTINS BAHIENSE,RODRIGO VALENTE SERRA</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>REINALDO DE SOUZA MACHADO</t>
-  </si>
-  <si>
-    <t>RODRIGO VENTURA MARRA,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>CHRISTIANA ROSA FERREIRA</t>
-  </si>
-  <si>
-    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>JULIANA MARTINS BAHIENSE,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>CAROLINE OLIVEIRA DE MENEZES</t>
-  </si>
-  <si>
-    <t>PATRICIA PASSARO DA SILVA TOLEDO,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>EDUARDO COUTO SOLEDADE</t>
-  </si>
-  <si>
-    <t>HELENA FERREIRA DE LIMA</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>DIANA DELGADO DA COSTA DA SILVA</t>
-  </si>
-  <si>
-    <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT</t>
-  </si>
-  <si>
-    <t>MARCELO KOLBLINGER DE GODOY</t>
-  </si>
-  <si>
-    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,SEZISNANDO JOSE PRIMO PAES</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA,ELIANA MIRANDA ARAUJO DA SILVA SOARES</t>
-  </si>
-  <si>
-    <t>FERNANDA ZUCOLOTTO</t>
-  </si>
-  <si>
-    <t>RAQUEL SILVA FERNANDES LYRA</t>
-  </si>
-  <si>
-    <t>RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>FERNANDA ZUCOLOTTO,MARINA DE AQUINO PARREIRA XAVIER</t>
-  </si>
-  <si>
-    <t>DAYSE BARBOSA DE ARAÚJO GÓIS</t>
-  </si>
-  <si>
-    <t>FLAVIA REIS RIBEIRO BASTOS, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>SEZISNANDO JOSE PRIMO PAES</t>
-  </si>
-  <si>
-    <t>LEONARDO ARAÚJO DE SOUZA</t>
-  </si>
-  <si>
-    <t>RODRIGO VALENTE SERRA,VANESSA FERNANDES LEÃO</t>
   </si>
   <si>
     <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
@@ -9833,7 +9833,7 @@
         <v>1740</v>
       </c>
       <c r="K51" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="L51" t="s">
         <v>2477</v>
@@ -14884,7 +14884,7 @@
     </row>
     <row r="196" spans="1:12">
       <c r="A196" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="B196" t="s">
         <v>234</v>
@@ -14905,7 +14905,7 @@
         <v>1563</v>
       </c>
       <c r="I196" t="s">
-        <v>1650</v>
+        <v>1596</v>
       </c>
       <c r="J196" t="s">
         <v>1906</v>
@@ -15150,7 +15150,7 @@
         <v>1563</v>
       </c>
       <c r="I203" t="s">
-        <v>1651</v>
+        <v>1650</v>
       </c>
       <c r="J203" t="s">
         <v>1913</v>
@@ -15185,7 +15185,7 @@
         <v>1563</v>
       </c>
       <c r="I204" t="s">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="J204" t="s">
         <v>1914</v>
@@ -15339,7 +15339,7 @@
     </row>
     <row r="209" spans="1:12">
       <c r="A209" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B209" t="s">
         <v>247</v>
@@ -15360,7 +15360,7 @@
         <v>1563</v>
       </c>
       <c r="I209" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J209" t="s">
         <v>1919</v>
@@ -15395,7 +15395,7 @@
         <v>1563</v>
       </c>
       <c r="I210" t="s">
-        <v>1654</v>
+        <v>1653</v>
       </c>
       <c r="J210" t="s">
         <v>1920</v>
@@ -15514,7 +15514,7 @@
     </row>
     <row r="214" spans="1:12">
       <c r="A214" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B214" t="s">
         <v>252</v>
@@ -15535,7 +15535,7 @@
         <v>1563</v>
       </c>
       <c r="I214" t="s">
-        <v>1655</v>
+        <v>1654</v>
       </c>
       <c r="J214" t="s">
         <v>1924</v>
@@ -15584,7 +15584,7 @@
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B216" t="s">
         <v>254</v>
@@ -15605,7 +15605,7 @@
         <v>1563</v>
       </c>
       <c r="I216" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J216" t="s">
         <v>1926</v>
@@ -15640,7 +15640,7 @@
         <v>1563</v>
       </c>
       <c r="I217" t="s">
-        <v>1657</v>
+        <v>1656</v>
       </c>
       <c r="J217" t="s">
         <v>1927</v>
@@ -15675,7 +15675,7 @@
         <v>1563</v>
       </c>
       <c r="I218" t="s">
-        <v>1658</v>
+        <v>1657</v>
       </c>
       <c r="J218" t="s">
         <v>1928</v>
@@ -15853,7 +15853,7 @@
         <v>1563</v>
       </c>
       <c r="I223" t="s">
-        <v>1659</v>
+        <v>1658</v>
       </c>
       <c r="J223" t="s">
         <v>1933</v>
@@ -15888,7 +15888,7 @@
         <v>1563</v>
       </c>
       <c r="I224" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="J224" t="s">
         <v>1934</v>
@@ -15923,7 +15923,7 @@
         <v>1563</v>
       </c>
       <c r="I225" t="s">
-        <v>1661</v>
+        <v>1660</v>
       </c>
       <c r="J225" t="s">
         <v>1935</v>
@@ -16042,7 +16042,7 @@
     </row>
     <row r="229" spans="1:12">
       <c r="A229" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B229" t="s">
         <v>267</v>
@@ -16063,7 +16063,7 @@
         <v>1563</v>
       </c>
       <c r="I229" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J229" t="s">
         <v>1939</v>
@@ -16133,7 +16133,7 @@
         <v>1563</v>
       </c>
       <c r="I231" t="s">
-        <v>1663</v>
+        <v>1662</v>
       </c>
       <c r="J231" t="s">
         <v>1941</v>
@@ -16168,7 +16168,7 @@
         <v>1563</v>
       </c>
       <c r="I232" t="s">
-        <v>1664</v>
+        <v>1663</v>
       </c>
       <c r="J232" t="s">
         <v>1942</v>
@@ -16217,7 +16217,7 @@
     </row>
     <row r="234" spans="1:12">
       <c r="A234" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B234" t="s">
         <v>272</v>
@@ -16238,7 +16238,7 @@
         <v>1563</v>
       </c>
       <c r="I234" t="s">
-        <v>1665</v>
+        <v>1664</v>
       </c>
       <c r="J234" t="s">
         <v>1944</v>
@@ -16287,7 +16287,7 @@
     </row>
     <row r="236" spans="1:12">
       <c r="A236" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B236" t="s">
         <v>274</v>
@@ -16308,7 +16308,7 @@
         <v>1563</v>
       </c>
       <c r="I236" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J236" t="s">
         <v>1946</v>
@@ -16343,7 +16343,7 @@
         <v>1563</v>
       </c>
       <c r="I237" t="s">
-        <v>1666</v>
+        <v>1665</v>
       </c>
       <c r="J237" t="s">
         <v>1947</v>
@@ -16497,7 +16497,7 @@
     </row>
     <row r="242" spans="1:12">
       <c r="A242" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B242" t="s">
         <v>280</v>
@@ -16518,7 +16518,7 @@
         <v>1563</v>
       </c>
       <c r="I242" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J242" t="s">
         <v>1952</v>
@@ -16623,7 +16623,7 @@
         <v>1563</v>
       </c>
       <c r="I245" t="s">
-        <v>1667</v>
+        <v>1666</v>
       </c>
       <c r="J245" t="s">
         <v>1955</v>
@@ -16672,7 +16672,7 @@
     </row>
     <row r="247" spans="1:12">
       <c r="A247" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B247" t="s">
         <v>285</v>
@@ -16693,7 +16693,7 @@
         <v>1563</v>
       </c>
       <c r="I247" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J247" t="s">
         <v>1957</v>
@@ -16707,7 +16707,7 @@
     </row>
     <row r="248" spans="1:12">
       <c r="A248" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B248" t="s">
         <v>286</v>
@@ -16728,7 +16728,7 @@
         <v>1563</v>
       </c>
       <c r="I248" t="s">
-        <v>1668</v>
+        <v>1667</v>
       </c>
       <c r="J248" t="s">
         <v>1958</v>
@@ -16882,7 +16882,7 @@
     </row>
     <row r="253" spans="1:12">
       <c r="A253" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B253" t="s">
         <v>291</v>
@@ -16903,7 +16903,7 @@
         <v>1563</v>
       </c>
       <c r="I253" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J253" t="s">
         <v>1963</v>
@@ -17060,7 +17060,7 @@
     </row>
     <row r="258" spans="1:12">
       <c r="A258" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B258" t="s">
         <v>296</v>
@@ -17084,7 +17084,7 @@
         <v>1568</v>
       </c>
       <c r="I258" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J258" t="s">
         <v>1968</v>
@@ -17203,7 +17203,7 @@
     </row>
     <row r="262" spans="1:12">
       <c r="A262" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B262" t="s">
         <v>300</v>
@@ -17224,7 +17224,7 @@
         <v>1563</v>
       </c>
       <c r="I262" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J262" t="s">
         <v>1972</v>
@@ -17238,7 +17238,7 @@
     </row>
     <row r="263" spans="1:12">
       <c r="A263" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B263" t="s">
         <v>301</v>
@@ -17259,7 +17259,7 @@
         <v>1563</v>
       </c>
       <c r="I263" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J263" t="s">
         <v>1973</v>
@@ -17399,7 +17399,7 @@
         <v>1563</v>
       </c>
       <c r="I267" t="s">
-        <v>1669</v>
+        <v>1668</v>
       </c>
       <c r="J267" t="s">
         <v>1977</v>
@@ -17434,7 +17434,7 @@
         <v>1563</v>
       </c>
       <c r="I268" t="s">
-        <v>1670</v>
+        <v>1669</v>
       </c>
       <c r="J268" t="s">
         <v>1978</v>
@@ -17448,7 +17448,7 @@
     </row>
     <row r="269" spans="1:12">
       <c r="A269" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B269" t="s">
         <v>307</v>
@@ -17469,7 +17469,7 @@
         <v>1563</v>
       </c>
       <c r="I269" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J269" t="s">
         <v>1979</v>
@@ -17504,7 +17504,7 @@
         <v>1563</v>
       </c>
       <c r="I270" t="s">
-        <v>1671</v>
+        <v>1670</v>
       </c>
       <c r="J270" t="s">
         <v>1980</v>
@@ -17798,7 +17798,7 @@
     </row>
     <row r="279" spans="1:12">
       <c r="A279" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B279" t="s">
         <v>317</v>
@@ -17819,7 +17819,7 @@
         <v>1563</v>
       </c>
       <c r="I279" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J279" t="s">
         <v>1989</v>
@@ -17903,7 +17903,7 @@
     </row>
     <row r="282" spans="1:12">
       <c r="A282" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B282" t="s">
         <v>320</v>
@@ -17924,7 +17924,7 @@
         <v>1563</v>
       </c>
       <c r="I282" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J282" t="s">
         <v>1992</v>
@@ -17973,7 +17973,7 @@
     </row>
     <row r="284" spans="1:12">
       <c r="A284" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B284" t="s">
         <v>322</v>
@@ -17994,7 +17994,7 @@
         <v>1563</v>
       </c>
       <c r="I284" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J284" t="s">
         <v>1994</v>
@@ -18148,7 +18148,7 @@
     </row>
     <row r="289" spans="1:12">
       <c r="A289" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B289" t="s">
         <v>327</v>
@@ -18169,7 +18169,7 @@
         <v>1563</v>
       </c>
       <c r="I289" t="s">
-        <v>1673</v>
+        <v>1672</v>
       </c>
       <c r="J289" t="s">
         <v>1999</v>
@@ -18239,7 +18239,7 @@
         <v>1563</v>
       </c>
       <c r="I291" t="s">
-        <v>1674</v>
+        <v>1673</v>
       </c>
       <c r="J291" t="s">
         <v>2001</v>
@@ -18323,7 +18323,7 @@
     </row>
     <row r="294" spans="1:12">
       <c r="A294" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B294" t="s">
         <v>332</v>
@@ -18344,7 +18344,7 @@
         <v>1563</v>
       </c>
       <c r="I294" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J294" t="s">
         <v>2004</v>
@@ -18428,7 +18428,7 @@
     </row>
     <row r="297" spans="1:12">
       <c r="A297" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B297" t="s">
         <v>335</v>
@@ -18449,7 +18449,7 @@
         <v>1563</v>
       </c>
       <c r="I297" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J297" t="s">
         <v>2007</v>
@@ -18554,7 +18554,7 @@
         <v>1563</v>
       </c>
       <c r="I300" t="s">
-        <v>1669</v>
+        <v>1668</v>
       </c>
       <c r="J300" t="s">
         <v>2010</v>
@@ -18883,7 +18883,7 @@
     </row>
     <row r="310" spans="1:12">
       <c r="A310" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B310" t="s">
         <v>348</v>
@@ -18904,7 +18904,7 @@
         <v>1563</v>
       </c>
       <c r="I310" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J310" t="s">
         <v>2020</v>
@@ -19303,7 +19303,7 @@
     </row>
     <row r="322" spans="1:12">
       <c r="A322" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B322" t="s">
         <v>360</v>
@@ -19324,7 +19324,7 @@
         <v>1563</v>
       </c>
       <c r="I322" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J322" t="s">
         <v>2032</v>
@@ -19397,7 +19397,7 @@
         <v>1514</v>
       </c>
       <c r="I324" t="s">
-        <v>1675</v>
+        <v>1674</v>
       </c>
       <c r="J324" t="s">
         <v>2034</v>
@@ -19481,7 +19481,7 @@
     </row>
     <row r="327" spans="1:12">
       <c r="A327" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B327" t="s">
         <v>365</v>
@@ -19502,7 +19502,7 @@
         <v>1563</v>
       </c>
       <c r="I327" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J327" t="s">
         <v>2037</v>
@@ -19516,7 +19516,7 @@
     </row>
     <row r="328" spans="1:12">
       <c r="A328" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B328" t="s">
         <v>366</v>
@@ -19537,7 +19537,7 @@
         <v>1563</v>
       </c>
       <c r="I328" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J328" t="s">
         <v>2038</v>
@@ -19869,7 +19869,7 @@
     </row>
     <row r="338" spans="1:12">
       <c r="A338" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B338" t="s">
         <v>376</v>
@@ -19890,7 +19890,7 @@
         <v>1563</v>
       </c>
       <c r="I338" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J338" t="s">
         <v>2048</v>
@@ -20044,7 +20044,7 @@
     </row>
     <row r="343" spans="1:12">
       <c r="A343" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B343" t="s">
         <v>381</v>
@@ -20065,7 +20065,7 @@
         <v>1563</v>
       </c>
       <c r="I343" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J343" t="s">
         <v>2053</v>
@@ -20149,7 +20149,7 @@
     </row>
     <row r="346" spans="1:12">
       <c r="A346" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B346" t="s">
         <v>384</v>
@@ -20170,7 +20170,7 @@
         <v>1563</v>
       </c>
       <c r="I346" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J346" t="s">
         <v>2056</v>
@@ -20184,7 +20184,7 @@
     </row>
     <row r="347" spans="1:12">
       <c r="A347" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B347" t="s">
         <v>385</v>
@@ -20205,7 +20205,7 @@
         <v>1563</v>
       </c>
       <c r="I347" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J347" t="s">
         <v>2057</v>
@@ -20219,7 +20219,7 @@
     </row>
     <row r="348" spans="1:12">
       <c r="A348" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B348" t="s">
         <v>386</v>
@@ -20240,7 +20240,7 @@
         <v>1563</v>
       </c>
       <c r="I348" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J348" t="s">
         <v>2058</v>
@@ -20289,7 +20289,7 @@
     </row>
     <row r="350" spans="1:12">
       <c r="A350" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B350" t="s">
         <v>388</v>
@@ -20310,7 +20310,7 @@
         <v>1563</v>
       </c>
       <c r="I350" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J350" t="s">
         <v>2060</v>
@@ -20324,7 +20324,7 @@
     </row>
     <row r="351" spans="1:12">
       <c r="A351" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B351" t="s">
         <v>389</v>
@@ -20345,7 +20345,7 @@
         <v>1563</v>
       </c>
       <c r="I351" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J351" t="s">
         <v>2061</v>
@@ -20394,7 +20394,7 @@
     </row>
     <row r="353" spans="1:12">
       <c r="A353" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B353" t="s">
         <v>391</v>
@@ -20418,7 +20418,7 @@
         <v>1570</v>
       </c>
       <c r="I353" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J353" t="s">
         <v>2063</v>
@@ -20453,7 +20453,7 @@
         <v>1563</v>
       </c>
       <c r="I354" t="s">
-        <v>1677</v>
+        <v>1676</v>
       </c>
       <c r="J354" t="s">
         <v>2064</v>
@@ -20467,7 +20467,7 @@
     </row>
     <row r="355" spans="1:12">
       <c r="A355" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B355" t="s">
         <v>393</v>
@@ -20488,7 +20488,7 @@
         <v>1563</v>
       </c>
       <c r="I355" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J355" t="s">
         <v>2065</v>
@@ -20502,7 +20502,7 @@
     </row>
     <row r="356" spans="1:12">
       <c r="A356" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B356" t="s">
         <v>394</v>
@@ -20523,7 +20523,7 @@
         <v>1563</v>
       </c>
       <c r="I356" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J356" t="s">
         <v>2066</v>
@@ -20537,7 +20537,7 @@
     </row>
     <row r="357" spans="1:12">
       <c r="A357" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B357" t="s">
         <v>395</v>
@@ -20558,7 +20558,7 @@
         <v>1563</v>
       </c>
       <c r="I357" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J357" t="s">
         <v>2067</v>
@@ -20607,7 +20607,7 @@
     </row>
     <row r="359" spans="1:12">
       <c r="A359" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B359" t="s">
         <v>397</v>
@@ -20628,7 +20628,7 @@
         <v>1563</v>
       </c>
       <c r="I359" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J359" t="s">
         <v>2069</v>
@@ -20642,7 +20642,7 @@
     </row>
     <row r="360" spans="1:12">
       <c r="A360" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B360" t="s">
         <v>398</v>
@@ -20663,7 +20663,7 @@
         <v>1563</v>
       </c>
       <c r="I360" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J360" t="s">
         <v>2070</v>
@@ -20677,7 +20677,7 @@
     </row>
     <row r="361" spans="1:12">
       <c r="A361" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B361" t="s">
         <v>399</v>
@@ -20698,7 +20698,7 @@
         <v>1563</v>
       </c>
       <c r="I361" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J361" t="s">
         <v>2071</v>
@@ -20782,7 +20782,7 @@
     </row>
     <row r="364" spans="1:12">
       <c r="A364" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B364" t="s">
         <v>402</v>
@@ -20803,7 +20803,7 @@
         <v>1563</v>
       </c>
       <c r="I364" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J364" t="s">
         <v>2074</v>
@@ -20887,7 +20887,7 @@
     </row>
     <row r="367" spans="1:12">
       <c r="A367" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B367" t="s">
         <v>405</v>
@@ -20908,7 +20908,7 @@
         <v>1563</v>
       </c>
       <c r="I367" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J367" t="s">
         <v>2077</v>
@@ -20957,7 +20957,7 @@
     </row>
     <row r="369" spans="1:12">
       <c r="A369" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B369" t="s">
         <v>407</v>
@@ -20978,7 +20978,7 @@
         <v>1563</v>
       </c>
       <c r="I369" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J369" t="s">
         <v>2079</v>
@@ -21118,7 +21118,7 @@
         <v>1563</v>
       </c>
       <c r="I373" t="s">
-        <v>1678</v>
+        <v>1677</v>
       </c>
       <c r="J373" t="s">
         <v>2083</v>
@@ -21167,7 +21167,7 @@
     </row>
     <row r="375" spans="1:12">
       <c r="A375" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B375" t="s">
         <v>413</v>
@@ -21188,7 +21188,7 @@
         <v>1565</v>
       </c>
       <c r="I375" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J375" t="s">
         <v>2085</v>
@@ -21223,7 +21223,7 @@
         <v>1563</v>
       </c>
       <c r="I376" t="s">
-        <v>1679</v>
+        <v>1678</v>
       </c>
       <c r="J376" t="s">
         <v>2086</v>
@@ -21412,7 +21412,7 @@
     </row>
     <row r="382" spans="1:12">
       <c r="A382" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B382" t="s">
         <v>420</v>
@@ -21433,7 +21433,7 @@
         <v>1563</v>
       </c>
       <c r="I382" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="J382" t="s">
         <v>2092</v>
@@ -21447,7 +21447,7 @@
     </row>
     <row r="383" spans="1:12">
       <c r="A383" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B383" t="s">
         <v>421</v>
@@ -21468,7 +21468,7 @@
         <v>1563</v>
       </c>
       <c r="I383" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J383" t="s">
         <v>2093</v>
@@ -21517,7 +21517,7 @@
     </row>
     <row r="385" spans="1:12">
       <c r="A385" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B385" t="s">
         <v>423</v>
@@ -21538,7 +21538,7 @@
         <v>1563</v>
       </c>
       <c r="I385" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="J385" t="s">
         <v>2095</v>
@@ -21622,7 +21622,7 @@
     </row>
     <row r="388" spans="1:12">
       <c r="A388" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B388" t="s">
         <v>426</v>
@@ -21643,7 +21643,7 @@
         <v>1563</v>
       </c>
       <c r="I388" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J388" t="s">
         <v>2098</v>
@@ -21657,7 +21657,7 @@
     </row>
     <row r="389" spans="1:12">
       <c r="A389" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B389" t="s">
         <v>427</v>
@@ -21678,7 +21678,7 @@
         <v>1563</v>
       </c>
       <c r="I389" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J389" t="s">
         <v>2099</v>
@@ -21727,7 +21727,7 @@
     </row>
     <row r="391" spans="1:12">
       <c r="A391" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B391" t="s">
         <v>429</v>
@@ -21748,7 +21748,7 @@
         <v>1563</v>
       </c>
       <c r="I391" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J391" t="s">
         <v>2101</v>
@@ -21853,7 +21853,7 @@
         <v>1563</v>
       </c>
       <c r="I394" t="s">
-        <v>1671</v>
+        <v>1670</v>
       </c>
       <c r="J394" t="s">
         <v>2104</v>
@@ -21937,7 +21937,7 @@
     </row>
     <row r="397" spans="1:12">
       <c r="A397" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B397" t="s">
         <v>435</v>
@@ -21958,7 +21958,7 @@
         <v>1563</v>
       </c>
       <c r="I397" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J397" t="s">
         <v>2107</v>
@@ -22063,7 +22063,7 @@
         <v>1563</v>
       </c>
       <c r="I400" t="s">
-        <v>1681</v>
+        <v>1680</v>
       </c>
       <c r="J400" t="s">
         <v>2110</v>
@@ -22112,7 +22112,7 @@
     </row>
     <row r="402" spans="1:12">
       <c r="A402" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B402" t="s">
         <v>440</v>
@@ -22133,7 +22133,7 @@
         <v>1563</v>
       </c>
       <c r="I402" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J402" t="s">
         <v>2112</v>
@@ -22168,7 +22168,7 @@
         <v>1563</v>
       </c>
       <c r="I403" t="s">
-        <v>1654</v>
+        <v>1653</v>
       </c>
       <c r="J403" t="s">
         <v>2113</v>
@@ -22238,7 +22238,7 @@
         <v>1563</v>
       </c>
       <c r="I405" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="J405" t="s">
         <v>2115</v>
@@ -22308,7 +22308,7 @@
         <v>1563</v>
       </c>
       <c r="I407" t="s">
-        <v>1681</v>
+        <v>1680</v>
       </c>
       <c r="J407" t="s">
         <v>2117</v>
@@ -22535,7 +22535,7 @@
     </row>
     <row r="414" spans="1:12">
       <c r="A414" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B414" t="s">
         <v>452</v>
@@ -22556,7 +22556,7 @@
         <v>1563</v>
       </c>
       <c r="I414" t="s">
-        <v>1683</v>
+        <v>1682</v>
       </c>
       <c r="J414" t="s">
         <v>2124</v>
@@ -22605,7 +22605,7 @@
     </row>
     <row r="416" spans="1:12">
       <c r="A416" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B416" t="s">
         <v>454</v>
@@ -22626,7 +22626,7 @@
         <v>1563</v>
       </c>
       <c r="I416" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J416" t="s">
         <v>2126</v>
@@ -22675,7 +22675,7 @@
     </row>
     <row r="418" spans="1:12">
       <c r="A418" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B418" t="s">
         <v>456</v>
@@ -22696,7 +22696,7 @@
         <v>1563</v>
       </c>
       <c r="I418" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J418" t="s">
         <v>2128</v>
@@ -22710,7 +22710,7 @@
     </row>
     <row r="419" spans="1:12">
       <c r="A419" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B419" t="s">
         <v>457</v>
@@ -22731,7 +22731,7 @@
         <v>1563</v>
       </c>
       <c r="I419" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J419" t="s">
         <v>2129</v>
@@ -22769,7 +22769,7 @@
         <v>1538</v>
       </c>
       <c r="I420" t="s">
-        <v>1650</v>
+        <v>1683</v>
       </c>
       <c r="J420" t="s">
         <v>2130</v>
@@ -22783,7 +22783,7 @@
     </row>
     <row r="421" spans="1:12">
       <c r="A421" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B421" t="s">
         <v>459</v>
@@ -22923,7 +22923,7 @@
     </row>
     <row r="425" spans="1:12">
       <c r="A425" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B425" t="s">
         <v>463</v>
@@ -22958,7 +22958,7 @@
     </row>
     <row r="426" spans="1:12">
       <c r="A426" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B426" t="s">
         <v>464</v>
@@ -22979,7 +22979,7 @@
         <v>1563</v>
       </c>
       <c r="I426" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J426" t="s">
         <v>2136</v>
@@ -23028,7 +23028,7 @@
     </row>
     <row r="428" spans="1:12">
       <c r="A428" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B428" t="s">
         <v>466</v>
@@ -23049,7 +23049,7 @@
         <v>1563</v>
       </c>
       <c r="I428" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J428" t="s">
         <v>2138</v>
@@ -23098,7 +23098,7 @@
     </row>
     <row r="430" spans="1:12">
       <c r="A430" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B430" t="s">
         <v>468</v>
@@ -23119,7 +23119,7 @@
         <v>1563</v>
       </c>
       <c r="I430" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J430" t="s">
         <v>2140</v>
@@ -23133,7 +23133,7 @@
     </row>
     <row r="431" spans="1:12">
       <c r="A431" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B431" t="s">
         <v>469</v>
@@ -23154,7 +23154,7 @@
         <v>1563</v>
       </c>
       <c r="I431" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J431" t="s">
         <v>2141</v>
@@ -23189,7 +23189,7 @@
         <v>1563</v>
       </c>
       <c r="I432" t="s">
-        <v>1667</v>
+        <v>1666</v>
       </c>
       <c r="J432" t="s">
         <v>2142</v>
@@ -23203,7 +23203,7 @@
     </row>
     <row r="433" spans="1:12">
       <c r="A433" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B433" t="s">
         <v>471</v>
@@ -23224,7 +23224,7 @@
         <v>1563</v>
       </c>
       <c r="I433" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J433" t="s">
         <v>2143</v>
@@ -23238,7 +23238,7 @@
     </row>
     <row r="434" spans="1:12">
       <c r="A434" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B434" t="s">
         <v>472</v>
@@ -23259,7 +23259,7 @@
         <v>1563</v>
       </c>
       <c r="I434" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J434" t="s">
         <v>2144</v>
@@ -23273,7 +23273,7 @@
     </row>
     <row r="435" spans="1:12">
       <c r="A435" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B435" t="s">
         <v>473</v>
@@ -23294,7 +23294,7 @@
         <v>1563</v>
       </c>
       <c r="I435" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J435" t="s">
         <v>2145</v>
@@ -23308,7 +23308,7 @@
     </row>
     <row r="436" spans="1:12">
       <c r="A436" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B436" t="s">
         <v>474</v>
@@ -23329,7 +23329,7 @@
         <v>1563</v>
       </c>
       <c r="I436" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J436" t="s">
         <v>2112</v>
@@ -23591,7 +23591,7 @@
     </row>
     <row r="444" spans="1:12">
       <c r="A444" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B444" t="s">
         <v>482</v>
@@ -23612,7 +23612,7 @@
         <v>1563</v>
       </c>
       <c r="I444" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J444" t="s">
         <v>2153</v>
@@ -23626,7 +23626,7 @@
     </row>
     <row r="445" spans="1:12">
       <c r="A445" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B445" t="s">
         <v>483</v>
@@ -23647,7 +23647,7 @@
         <v>1563</v>
       </c>
       <c r="I445" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J445" t="s">
         <v>2154</v>
@@ -23661,7 +23661,7 @@
     </row>
     <row r="446" spans="1:12">
       <c r="A446" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B446" t="s">
         <v>484</v>
@@ -23682,7 +23682,7 @@
         <v>1563</v>
       </c>
       <c r="I446" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J446" t="s">
         <v>2155</v>
@@ -23766,7 +23766,7 @@
     </row>
     <row r="449" spans="1:12">
       <c r="A449" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B449" t="s">
         <v>487</v>
@@ -23787,7 +23787,7 @@
         <v>1563</v>
       </c>
       <c r="I449" t="s">
-        <v>1680</v>
+        <v>1679</v>
       </c>
       <c r="J449" t="s">
         <v>2158</v>
@@ -23801,7 +23801,7 @@
     </row>
     <row r="450" spans="1:12">
       <c r="A450" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B450" t="s">
         <v>488</v>
@@ -23822,7 +23822,7 @@
         <v>1563</v>
       </c>
       <c r="I450" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J450" t="s">
         <v>2159</v>
@@ -23836,7 +23836,7 @@
     </row>
     <row r="451" spans="1:12">
       <c r="A451" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B451" t="s">
         <v>489</v>
@@ -23857,7 +23857,7 @@
         <v>1563</v>
       </c>
       <c r="I451" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J451" t="s">
         <v>2160</v>
@@ -23871,7 +23871,7 @@
     </row>
     <row r="452" spans="1:12">
       <c r="A452" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B452" t="s">
         <v>490</v>
@@ -23892,7 +23892,7 @@
         <v>1563</v>
       </c>
       <c r="I452" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J452" t="s">
         <v>2161</v>
@@ -23906,7 +23906,7 @@
     </row>
     <row r="453" spans="1:12">
       <c r="A453" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B453" t="s">
         <v>491</v>
@@ -23927,7 +23927,7 @@
         <v>1563</v>
       </c>
       <c r="I453" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J453" t="s">
         <v>2162</v>
@@ -23976,7 +23976,7 @@
     </row>
     <row r="455" spans="1:12">
       <c r="A455" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B455" t="s">
         <v>493</v>
@@ -23997,7 +23997,7 @@
         <v>1563</v>
       </c>
       <c r="I455" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J455" t="s">
         <v>2164</v>
@@ -24081,7 +24081,7 @@
     </row>
     <row r="458" spans="1:12">
       <c r="A458" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B458" t="s">
         <v>496</v>
@@ -24102,7 +24102,7 @@
         <v>1563</v>
       </c>
       <c r="I458" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J458" t="s">
         <v>2167</v>
@@ -24116,7 +24116,7 @@
     </row>
     <row r="459" spans="1:12">
       <c r="A459" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B459" t="s">
         <v>497</v>
@@ -24137,7 +24137,7 @@
         <v>1563</v>
       </c>
       <c r="I459" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J459" t="s">
         <v>2168</v>
@@ -24186,7 +24186,7 @@
     </row>
     <row r="461" spans="1:12">
       <c r="A461" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B461" t="s">
         <v>499</v>
@@ -24207,7 +24207,7 @@
         <v>1563</v>
       </c>
       <c r="I461" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J461" t="s">
         <v>2170</v>
@@ -24312,7 +24312,7 @@
         <v>1563</v>
       </c>
       <c r="I464" t="s">
-        <v>1667</v>
+        <v>1666</v>
       </c>
       <c r="J464" t="s">
         <v>2173</v>
@@ -24326,7 +24326,7 @@
     </row>
     <row r="465" spans="1:12">
       <c r="A465" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B465" t="s">
         <v>503</v>
@@ -24347,7 +24347,7 @@
         <v>1563</v>
       </c>
       <c r="I465" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J465" t="s">
         <v>2174</v>
@@ -24361,7 +24361,7 @@
     </row>
     <row r="466" spans="1:12">
       <c r="A466" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B466" t="s">
         <v>504</v>
@@ -24396,7 +24396,7 @@
     </row>
     <row r="467" spans="1:12">
       <c r="A467" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B467" t="s">
         <v>505</v>
@@ -24431,7 +24431,7 @@
     </row>
     <row r="468" spans="1:12">
       <c r="A468" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B468" t="s">
         <v>506</v>
@@ -24466,7 +24466,7 @@
     </row>
     <row r="469" spans="1:12">
       <c r="A469" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B469" t="s">
         <v>507</v>
@@ -24501,7 +24501,7 @@
     </row>
     <row r="470" spans="1:12">
       <c r="A470" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B470" t="s">
         <v>508</v>
@@ -24536,7 +24536,7 @@
     </row>
     <row r="471" spans="1:12">
       <c r="A471" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B471" t="s">
         <v>509</v>
@@ -24571,7 +24571,7 @@
     </row>
     <row r="472" spans="1:12">
       <c r="A472" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B472" t="s">
         <v>510</v>
@@ -24606,7 +24606,7 @@
     </row>
     <row r="473" spans="1:12">
       <c r="A473" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B473" t="s">
         <v>511</v>
@@ -24641,7 +24641,7 @@
     </row>
     <row r="474" spans="1:12">
       <c r="A474" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B474" t="s">
         <v>512</v>
@@ -24676,7 +24676,7 @@
     </row>
     <row r="475" spans="1:12">
       <c r="A475" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B475" t="s">
         <v>513</v>
@@ -24711,7 +24711,7 @@
     </row>
     <row r="476" spans="1:12">
       <c r="A476" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B476" t="s">
         <v>514</v>
@@ -24746,7 +24746,7 @@
     </row>
     <row r="477" spans="1:12">
       <c r="A477" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B477" t="s">
         <v>515</v>
@@ -24781,7 +24781,7 @@
     </row>
     <row r="478" spans="1:12">
       <c r="A478" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B478" t="s">
         <v>516</v>
@@ -24816,7 +24816,7 @@
     </row>
     <row r="479" spans="1:12">
       <c r="A479" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B479" t="s">
         <v>517</v>
@@ -24851,7 +24851,7 @@
     </row>
     <row r="480" spans="1:12">
       <c r="A480" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B480" t="s">
         <v>518</v>
@@ -24886,7 +24886,7 @@
     </row>
     <row r="481" spans="1:12">
       <c r="A481" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B481" t="s">
         <v>519</v>
@@ -24921,7 +24921,7 @@
     </row>
     <row r="482" spans="1:12">
       <c r="A482" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B482" t="s">
         <v>520</v>
@@ -24956,7 +24956,7 @@
     </row>
     <row r="483" spans="1:12">
       <c r="A483" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B483" t="s">
         <v>521</v>
@@ -24991,7 +24991,7 @@
     </row>
     <row r="484" spans="1:12">
       <c r="A484" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B484" t="s">
         <v>522</v>
@@ -25026,7 +25026,7 @@
     </row>
     <row r="485" spans="1:12">
       <c r="A485" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B485" t="s">
         <v>523</v>
@@ -25047,7 +25047,7 @@
         <v>1563</v>
       </c>
       <c r="I485" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J485" t="s">
         <v>2194</v>
@@ -25096,7 +25096,7 @@
     </row>
     <row r="487" spans="1:12">
       <c r="A487" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B487" t="s">
         <v>525</v>
@@ -25117,7 +25117,7 @@
         <v>1563</v>
       </c>
       <c r="I487" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J487" t="s">
         <v>2196</v>
@@ -25131,7 +25131,7 @@
     </row>
     <row r="488" spans="1:12">
       <c r="A488" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B488" t="s">
         <v>526</v>
@@ -25152,7 +25152,7 @@
         <v>1563</v>
       </c>
       <c r="I488" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J488" t="s">
         <v>2196</v>
@@ -25166,7 +25166,7 @@
     </row>
     <row r="489" spans="1:12">
       <c r="A489" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B489" t="s">
         <v>527</v>
@@ -25187,7 +25187,7 @@
         <v>1563</v>
       </c>
       <c r="I489" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J489" t="s">
         <v>2196</v>
@@ -25271,7 +25271,7 @@
     </row>
     <row r="492" spans="1:12">
       <c r="A492" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B492" t="s">
         <v>529</v>
@@ -25292,7 +25292,7 @@
         <v>1563</v>
       </c>
       <c r="I492" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J492" t="s">
         <v>2198</v>
@@ -25379,7 +25379,7 @@
     </row>
     <row r="495" spans="1:12">
       <c r="A495" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B495" t="s">
         <v>532</v>
@@ -25414,7 +25414,7 @@
     </row>
     <row r="496" spans="1:12">
       <c r="A496" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B496" t="s">
         <v>533</v>
@@ -25484,7 +25484,7 @@
     </row>
     <row r="498" spans="1:12">
       <c r="A498" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B498" t="s">
         <v>535</v>
@@ -25519,7 +25519,7 @@
     </row>
     <row r="499" spans="1:12">
       <c r="A499" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B499" t="s">
         <v>536</v>
@@ -25540,7 +25540,7 @@
         <v>1563</v>
       </c>
       <c r="I499" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J499" t="s">
         <v>2205</v>
@@ -25648,7 +25648,7 @@
         <v>1563</v>
       </c>
       <c r="I502" t="s">
-        <v>1670</v>
+        <v>1669</v>
       </c>
       <c r="J502" t="s">
         <v>2208</v>
@@ -25697,7 +25697,7 @@
     </row>
     <row r="504" spans="1:12">
       <c r="A504" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B504" t="s">
         <v>541</v>
@@ -25718,7 +25718,7 @@
         <v>1563</v>
       </c>
       <c r="I504" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J504" t="s">
         <v>2210</v>
@@ -25802,7 +25802,7 @@
     </row>
     <row r="507" spans="1:12">
       <c r="A507" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B507" t="s">
         <v>544</v>
@@ -25823,7 +25823,7 @@
         <v>1563</v>
       </c>
       <c r="I507" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J507" t="s">
         <v>2213</v>
@@ -25837,7 +25837,7 @@
     </row>
     <row r="508" spans="1:12">
       <c r="A508" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B508" t="s">
         <v>545</v>
@@ -25896,7 +25896,7 @@
         <v>1572</v>
       </c>
       <c r="I509" t="s">
-        <v>1660</v>
+        <v>1659</v>
       </c>
       <c r="J509" t="s">
         <v>2215</v>
@@ -25910,7 +25910,7 @@
     </row>
     <row r="510" spans="1:12">
       <c r="A510" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B510" t="s">
         <v>547</v>
@@ -25931,7 +25931,7 @@
         <v>1563</v>
       </c>
       <c r="I510" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J510" t="s">
         <v>2216</v>
@@ -25945,7 +25945,7 @@
     </row>
     <row r="511" spans="1:12">
       <c r="A511" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B511" t="s">
         <v>548</v>
@@ -25966,7 +25966,7 @@
         <v>1563</v>
       </c>
       <c r="I511" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J511" t="s">
         <v>2217</v>
@@ -26015,7 +26015,7 @@
     </row>
     <row r="513" spans="1:12">
       <c r="A513" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B513" t="s">
         <v>550</v>
@@ -26085,7 +26085,7 @@
     </row>
     <row r="515" spans="1:12">
       <c r="A515" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B515" t="s">
         <v>552</v>
@@ -26120,7 +26120,7 @@
     </row>
     <row r="516" spans="1:12">
       <c r="A516" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B516" t="s">
         <v>553</v>
@@ -26225,7 +26225,7 @@
     </row>
     <row r="519" spans="1:12">
       <c r="A519" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B519" t="s">
         <v>556</v>
@@ -26260,7 +26260,7 @@
     </row>
     <row r="520" spans="1:12">
       <c r="A520" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B520" t="s">
         <v>557</v>
@@ -26295,7 +26295,7 @@
     </row>
     <row r="521" spans="1:12">
       <c r="A521" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B521" t="s">
         <v>558</v>
@@ -26470,7 +26470,7 @@
     </row>
     <row r="526" spans="1:12">
       <c r="A526" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B526" t="s">
         <v>563</v>
@@ -26491,7 +26491,7 @@
         <v>1563</v>
       </c>
       <c r="I526" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J526" t="s">
         <v>2232</v>
@@ -26505,7 +26505,7 @@
     </row>
     <row r="527" spans="1:12">
       <c r="A527" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B527" t="s">
         <v>564</v>
@@ -26526,7 +26526,7 @@
         <v>1563</v>
       </c>
       <c r="I527" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J527" t="s">
         <v>2233</v>
@@ -26610,7 +26610,7 @@
     </row>
     <row r="530" spans="1:12">
       <c r="A530" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B530" t="s">
         <v>567</v>
@@ -26631,7 +26631,7 @@
         <v>1563</v>
       </c>
       <c r="I530" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J530" t="s">
         <v>2236</v>
@@ -26645,7 +26645,7 @@
     </row>
     <row r="531" spans="1:12">
       <c r="A531" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B531" t="s">
         <v>568</v>
@@ -26666,7 +26666,7 @@
         <v>1563</v>
       </c>
       <c r="I531" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J531" t="s">
         <v>2237</v>
@@ -26680,7 +26680,7 @@
     </row>
     <row r="532" spans="1:12">
       <c r="A532" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B532" t="s">
         <v>569</v>
@@ -26701,7 +26701,7 @@
         <v>1563</v>
       </c>
       <c r="I532" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J532" t="s">
         <v>2238</v>
@@ -26736,7 +26736,7 @@
         <v>1563</v>
       </c>
       <c r="I533" t="s">
-        <v>1674</v>
+        <v>1673</v>
       </c>
       <c r="J533" t="s">
         <v>2239</v>
@@ -26861,7 +26861,7 @@
     </row>
     <row r="537" spans="1:12">
       <c r="A537" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B537" t="s">
         <v>573</v>
@@ -26896,7 +26896,7 @@
     </row>
     <row r="538" spans="1:12">
       <c r="A538" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B538" t="s">
         <v>574</v>
@@ -26917,7 +26917,7 @@
         <v>1563</v>
       </c>
       <c r="I538" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J538" t="s">
         <v>2243</v>
@@ -26966,7 +26966,7 @@
     </row>
     <row r="540" spans="1:12">
       <c r="A540" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B540" t="s">
         <v>576</v>
@@ -26987,7 +26987,7 @@
         <v>1563</v>
       </c>
       <c r="I540" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J540" t="s">
         <v>2245</v>
@@ -27001,7 +27001,7 @@
     </row>
     <row r="541" spans="1:12">
       <c r="A541" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B541" t="s">
         <v>577</v>
@@ -27022,7 +27022,7 @@
         <v>1563</v>
       </c>
       <c r="I541" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J541" t="s">
         <v>2246</v>
@@ -27071,7 +27071,7 @@
     </row>
     <row r="543" spans="1:12">
       <c r="A543" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B543" t="s">
         <v>579</v>
@@ -27092,7 +27092,7 @@
         <v>1563</v>
       </c>
       <c r="I543" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J543" t="s">
         <v>2248</v>
@@ -27141,7 +27141,7 @@
     </row>
     <row r="545" spans="1:12">
       <c r="A545" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B545" t="s">
         <v>581</v>
@@ -27162,7 +27162,7 @@
         <v>1563</v>
       </c>
       <c r="I545" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J545" t="s">
         <v>2250</v>
@@ -27211,7 +27211,7 @@
     </row>
     <row r="547" spans="1:12">
       <c r="A547" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B547" t="s">
         <v>583</v>
@@ -27235,7 +27235,7 @@
         <v>1575</v>
       </c>
       <c r="I547" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J547" t="s">
         <v>2252</v>
@@ -27395,7 +27395,7 @@
     </row>
     <row r="552" spans="1:12">
       <c r="A552" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B552" t="s">
         <v>588</v>
@@ -27416,7 +27416,7 @@
         <v>1563</v>
       </c>
       <c r="I552" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J552" t="s">
         <v>2257</v>
@@ -27465,7 +27465,7 @@
     </row>
     <row r="554" spans="1:12">
       <c r="A554" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B554" t="s">
         <v>590</v>
@@ -27486,7 +27486,7 @@
         <v>1563</v>
       </c>
       <c r="I554" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J554" t="s">
         <v>2259</v>
@@ -27500,7 +27500,7 @@
     </row>
     <row r="555" spans="1:12">
       <c r="A555" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B555" t="s">
         <v>591</v>
@@ -27535,7 +27535,7 @@
     </row>
     <row r="556" spans="1:12">
       <c r="A556" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B556" t="s">
         <v>592</v>
@@ -27556,7 +27556,7 @@
         <v>1563</v>
       </c>
       <c r="I556" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J556" t="s">
         <v>2261</v>
@@ -27570,7 +27570,7 @@
     </row>
     <row r="557" spans="1:12">
       <c r="A557" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B557" t="s">
         <v>593</v>
@@ -27605,7 +27605,7 @@
     </row>
     <row r="558" spans="1:12">
       <c r="A558" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B558" t="s">
         <v>594</v>
@@ -27626,7 +27626,7 @@
         <v>1563</v>
       </c>
       <c r="I558" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J558" t="s">
         <v>2263</v>
@@ -27640,7 +27640,7 @@
     </row>
     <row r="559" spans="1:12">
       <c r="A559" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B559" t="s">
         <v>595</v>
@@ -27661,7 +27661,7 @@
         <v>1563</v>
       </c>
       <c r="I559" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J559" t="s">
         <v>2264</v>
@@ -27675,7 +27675,7 @@
     </row>
     <row r="560" spans="1:12">
       <c r="A560" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B560" t="s">
         <v>596</v>
@@ -27696,7 +27696,7 @@
         <v>1563</v>
       </c>
       <c r="I560" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J560" t="s">
         <v>2265</v>
@@ -27745,7 +27745,7 @@
     </row>
     <row r="562" spans="1:12">
       <c r="A562" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B562" t="s">
         <v>598</v>
@@ -27766,7 +27766,7 @@
         <v>1563</v>
       </c>
       <c r="I562" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J562" t="s">
         <v>2149</v>
@@ -27780,7 +27780,7 @@
     </row>
     <row r="563" spans="1:12">
       <c r="A563" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B563" t="s">
         <v>599</v>
@@ -27853,7 +27853,7 @@
     </row>
     <row r="565" spans="1:12">
       <c r="A565" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B565" t="s">
         <v>601</v>
@@ -27996,7 +27996,7 @@
     </row>
     <row r="569" spans="1:12">
       <c r="A569" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B569" t="s">
         <v>605</v>
@@ -28017,7 +28017,7 @@
         <v>1563</v>
       </c>
       <c r="I569" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J569" t="s">
         <v>2273</v>
@@ -28101,7 +28101,7 @@
     </row>
     <row r="572" spans="1:12">
       <c r="A572" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B572" t="s">
         <v>608</v>
@@ -28122,7 +28122,7 @@
         <v>1563</v>
       </c>
       <c r="I572" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J572" t="s">
         <v>2276</v>
@@ -28195,7 +28195,7 @@
         <v>1563</v>
       </c>
       <c r="I574" t="s">
-        <v>1682</v>
+        <v>1681</v>
       </c>
       <c r="J574" t="s">
         <v>2278</v>
@@ -28244,7 +28244,7 @@
     </row>
     <row r="576" spans="1:12">
       <c r="A576" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B576" t="s">
         <v>612</v>
@@ -28279,7 +28279,7 @@
     </row>
     <row r="577" spans="1:12">
       <c r="A577" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B577" t="s">
         <v>613</v>
@@ -28314,7 +28314,7 @@
     </row>
     <row r="578" spans="1:12">
       <c r="A578" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B578" t="s">
         <v>614</v>
@@ -28349,7 +28349,7 @@
     </row>
     <row r="579" spans="1:12">
       <c r="A579" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B579" t="s">
         <v>615</v>
@@ -28370,7 +28370,7 @@
         <v>1563</v>
       </c>
       <c r="I579" t="s">
-        <v>1662</v>
+        <v>1661</v>
       </c>
       <c r="J579" t="s">
         <v>2283</v>
@@ -28384,7 +28384,7 @@
     </row>
     <row r="580" spans="1:12">
       <c r="A580" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B580" t="s">
         <v>616</v>
@@ -28405,7 +28405,7 @@
         <v>1563</v>
       </c>
       <c r="I580" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J580" t="s">
         <v>2284</v>
@@ -28524,7 +28524,7 @@
     </row>
     <row r="584" spans="1:12">
       <c r="A584" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B584" t="s">
         <v>620</v>
@@ -28594,7 +28594,7 @@
     </row>
     <row r="586" spans="1:12">
       <c r="A586" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B586" t="s">
         <v>622</v>
@@ -28985,7 +28985,7 @@
     </row>
     <row r="597" spans="1:12">
       <c r="A597" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B597" t="s">
         <v>633</v>
@@ -29041,7 +29041,7 @@
         <v>1563</v>
       </c>
       <c r="I598" t="s">
-        <v>1666</v>
+        <v>1665</v>
       </c>
       <c r="J598" t="s">
         <v>2302</v>
@@ -29111,7 +29111,7 @@
         <v>1563</v>
       </c>
       <c r="I600" t="s">
-        <v>1670</v>
+        <v>1669</v>
       </c>
       <c r="J600" t="s">
         <v>2304</v>
@@ -29146,7 +29146,7 @@
         <v>1563</v>
       </c>
       <c r="I601" t="s">
-        <v>1667</v>
+        <v>1666</v>
       </c>
       <c r="J601" t="s">
         <v>2305</v>
@@ -29198,7 +29198,7 @@
     </row>
     <row r="603" spans="1:12">
       <c r="A603" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B603" t="s">
         <v>639</v>
@@ -29233,7 +29233,7 @@
     </row>
     <row r="604" spans="1:12">
       <c r="A604" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B604" t="s">
         <v>640</v>
@@ -29268,7 +29268,7 @@
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B605" t="s">
         <v>641</v>
@@ -29303,7 +29303,7 @@
     </row>
     <row r="606" spans="1:12">
       <c r="A606" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B606" t="s">
         <v>642</v>
@@ -29446,7 +29446,7 @@
     </row>
     <row r="610" spans="1:12">
       <c r="A610" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B610" t="s">
         <v>646</v>
@@ -29467,7 +29467,7 @@
         <v>1563</v>
       </c>
       <c r="I610" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J610" t="s">
         <v>2314</v>
@@ -29557,7 +29557,7 @@
     </row>
     <row r="613" spans="1:12">
       <c r="A613" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B613" t="s">
         <v>649</v>
@@ -29578,7 +29578,7 @@
         <v>1563</v>
       </c>
       <c r="I613" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J613" t="s">
         <v>2317</v>
@@ -29627,7 +29627,7 @@
     </row>
     <row r="615" spans="1:12">
       <c r="A615" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B615" t="s">
         <v>651</v>
@@ -29648,7 +29648,7 @@
         <v>1563</v>
       </c>
       <c r="I615" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J615" t="s">
         <v>2319</v>
@@ -29697,7 +29697,7 @@
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B617" t="s">
         <v>653</v>
@@ -29732,7 +29732,7 @@
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B618" t="s">
         <v>654</v>
@@ -29767,7 +29767,7 @@
     </row>
     <row r="619" spans="1:12">
       <c r="A619" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B619" t="s">
         <v>655</v>
@@ -29802,7 +29802,7 @@
     </row>
     <row r="620" spans="1:12">
       <c r="A620" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B620" t="s">
         <v>656</v>
@@ -29837,7 +29837,7 @@
     </row>
     <row r="621" spans="1:12">
       <c r="A621" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B621" t="s">
         <v>657</v>
@@ -29907,7 +29907,7 @@
     </row>
     <row r="623" spans="1:12">
       <c r="A623" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B623" t="s">
         <v>659</v>
@@ -29928,7 +29928,7 @@
         <v>1563</v>
       </c>
       <c r="I623" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J623" t="s">
         <v>2326</v>
@@ -29942,7 +29942,7 @@
     </row>
     <row r="624" spans="1:12">
       <c r="A624" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B624" t="s">
         <v>660</v>
@@ -29977,7 +29977,7 @@
     </row>
     <row r="625" spans="1:12">
       <c r="A625" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B625" t="s">
         <v>661</v>
@@ -30036,7 +30036,7 @@
         <v>1551</v>
       </c>
       <c r="I626" t="s">
-        <v>1679</v>
+        <v>1678</v>
       </c>
       <c r="J626" t="s">
         <v>2329</v>
@@ -30050,7 +30050,7 @@
     </row>
     <row r="627" spans="1:12">
       <c r="A627" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B627" t="s">
         <v>663</v>
@@ -30071,7 +30071,7 @@
         <v>1563</v>
       </c>
       <c r="I627" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J627" t="s">
         <v>2330</v>
@@ -30120,7 +30120,7 @@
     </row>
     <row r="629" spans="1:12">
       <c r="A629" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B629" t="s">
         <v>665</v>
@@ -30141,7 +30141,7 @@
         <v>1563</v>
       </c>
       <c r="I629" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J629" t="s">
         <v>2332</v>
@@ -30266,7 +30266,7 @@
     </row>
     <row r="633" spans="1:12">
       <c r="A633" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B633" t="s">
         <v>669</v>
@@ -30287,7 +30287,7 @@
         <v>1563</v>
       </c>
       <c r="I633" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J633" t="s">
         <v>2336</v>
@@ -30339,7 +30339,7 @@
     </row>
     <row r="635" spans="1:12">
       <c r="A635" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B635" t="s">
         <v>671</v>
@@ -30374,7 +30374,7 @@
     </row>
     <row r="636" spans="1:12">
       <c r="A636" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B636" t="s">
         <v>672</v>
@@ -30409,7 +30409,7 @@
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B637" t="s">
         <v>673</v>
@@ -30444,7 +30444,7 @@
     </row>
     <row r="638" spans="1:12">
       <c r="A638" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B638" t="s">
         <v>674</v>
@@ -30465,7 +30465,7 @@
         <v>1563</v>
       </c>
       <c r="I638" t="s">
-        <v>1653</v>
+        <v>1652</v>
       </c>
       <c r="J638" t="s">
         <v>2340</v>
@@ -30479,7 +30479,7 @@
     </row>
     <row r="639" spans="1:12">
       <c r="A639" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B639" t="s">
         <v>675</v>
@@ -30555,7 +30555,7 @@
     </row>
     <row r="641" spans="1:12">
       <c r="A641" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B641" t="s">
         <v>677</v>
@@ -30576,7 +30576,7 @@
         <v>1563</v>
       </c>
       <c r="I641" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J641" t="s">
         <v>2343</v>
@@ -30628,7 +30628,7 @@
     </row>
     <row r="643" spans="1:12">
       <c r="A643" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B643" t="s">
         <v>679</v>
@@ -30701,7 +30701,7 @@
     </row>
     <row r="645" spans="1:12">
       <c r="A645" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B645" t="s">
         <v>681</v>
@@ -30736,7 +30736,7 @@
     </row>
     <row r="646" spans="1:12">
       <c r="A646" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B646" t="s">
         <v>682</v>
@@ -30771,7 +30771,7 @@
     </row>
     <row r="647" spans="1:12">
       <c r="A647" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B647" t="s">
         <v>683</v>
@@ -30806,7 +30806,7 @@
     </row>
     <row r="648" spans="1:12">
       <c r="A648" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B648" t="s">
         <v>684</v>
@@ -30827,7 +30827,7 @@
         <v>1563</v>
       </c>
       <c r="I648" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J648" t="s">
         <v>2350</v>
@@ -30841,7 +30841,7 @@
     </row>
     <row r="649" spans="1:12">
       <c r="A649" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B649" t="s">
         <v>685</v>
@@ -30862,7 +30862,7 @@
         <v>1563</v>
       </c>
       <c r="I649" t="s">
-        <v>1656</v>
+        <v>1655</v>
       </c>
       <c r="J649" t="s">
         <v>2351</v>
@@ -30876,7 +30876,7 @@
     </row>
     <row r="650" spans="1:12">
       <c r="A650" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B650" t="s">
         <v>686</v>
@@ -30911,7 +30911,7 @@
     </row>
     <row r="651" spans="1:12">
       <c r="A651" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B651" t="s">
         <v>687</v>
@@ -30946,7 +30946,7 @@
     </row>
     <row r="652" spans="1:12">
       <c r="A652" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B652" t="s">
         <v>688</v>
@@ -30984,7 +30984,7 @@
     </row>
     <row r="653" spans="1:12">
       <c r="A653" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B653" t="s">
         <v>689</v>
@@ -31008,7 +31008,7 @@
         <v>1587</v>
       </c>
       <c r="I653" t="s">
-        <v>1676</v>
+        <v>1675</v>
       </c>
       <c r="J653" t="s">
         <v>2355</v>
@@ -31022,7 +31022,7 @@
     </row>
     <row r="654" spans="1:12">
       <c r="A654" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B654" t="s">
         <v>690</v>
@@ -31046,7 +31046,7 @@
         <v>1591</v>
       </c>
       <c r="I654" t="s">
-        <v>1672</v>
+        <v>1671</v>
       </c>
       <c r="J654" t="s">
         <v>2356</v>
@@ -31060,7 +31060,7 @@
     </row>
     <row r="655" spans="1:12">
       <c r="A655" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B655" t="s">
         <v>691</v>
@@ -31092,7 +31092,7 @@
     </row>
     <row r="656" spans="1:12">
       <c r="A656" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B656" t="s">
         <v>692</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-16 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -29732,7 +29732,7 @@
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="B618" t="s">
         <v>654</v>
@@ -29753,7 +29753,7 @@
         <v>1563</v>
       </c>
       <c r="I618" t="s">
-        <v>1707</v>
+        <v>1596</v>
       </c>
       <c r="J618" t="s">
         <v>2322</v>
@@ -30479,7 +30479,7 @@
     </row>
     <row r="639" spans="1:12">
       <c r="A639" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="B639" t="s">
         <v>675</v>
@@ -30494,7 +30494,7 @@
         <v>5</v>
       </c>
       <c r="F639" t="s">
-        <v>1558</v>
+        <v>1560</v>
       </c>
       <c r="G639" t="s">
         <v>1565</v>
@@ -30503,7 +30503,7 @@
         <v>1586</v>
       </c>
       <c r="I639" t="s">
-        <v>1707</v>
+        <v>1669</v>
       </c>
       <c r="J639" t="s">
         <v>2341</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-18 20:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -64,6 +64,9 @@
     <t>NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
   </si>
   <si>
@@ -97,9 +100,6 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIA DE DADOS,NÚCLEO TÉCNICO DE CONTABILIDADE</t>
   </si>
   <si>
-    <t>SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>GRUPO EXECUTIVO DE FISCALIZAÇÃO DE UNIDADES POLICIAIS E PRISIONAIS 18 - DES</t>
   </si>
   <si>
@@ -3973,15 +3973,18 @@
     <t>ITAMAR COSTA KALIL</t>
   </si>
   <si>
+    <t>_SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>LILIAN ALVES DE ARAUJO</t>
+  </si>
+  <si>
+    <t>VANESSA TRINDADE CAMPOS DA SILVA</t>
+  </si>
+  <si>
     <t>MARCELO TEIXEIRA SANTANA</t>
   </si>
   <si>
-    <t>LILIAN ALVES DE ARAUJO</t>
-  </si>
-  <si>
-    <t>VANESSA TRINDADE CAMPOS DA SILVA</t>
-  </si>
-  <si>
     <t>VANESSA FERNANDES LEÃO</t>
   </si>
   <si>
@@ -4103,9 +4106,6 @@
   </si>
   <si>
     <t>ALESSANDRA ALMEIDA DIAS DA SILVA,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>_SEM USUARIO ATRIBUIDO</t>
   </si>
   <si>
     <t>NIVANA DANIELLE SILVA COSTA</t>
@@ -8330,7 +8330,7 @@
     </row>
     <row r="45" spans="1:12">
       <c r="A45" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B45" t="s">
         <v>78</v>
@@ -8351,7 +8351,7 @@
         <v>1284</v>
       </c>
       <c r="I45" t="s">
-        <v>1319</v>
+        <v>1322</v>
       </c>
       <c r="J45" t="s">
         <v>1469</v>
@@ -8427,7 +8427,7 @@
         <v>1450</v>
       </c>
       <c r="K47" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="L47" t="s">
         <v>2057</v>
@@ -8435,7 +8435,7 @@
     </row>
     <row r="48" spans="1:12">
       <c r="A48" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B48" t="s">
         <v>81</v>
@@ -8456,7 +8456,7 @@
         <v>1284</v>
       </c>
       <c r="I48" t="s">
-        <v>1322</v>
+        <v>1323</v>
       </c>
       <c r="J48" t="s">
         <v>1471</v>
@@ -8491,7 +8491,7 @@
         <v>1284</v>
       </c>
       <c r="I49" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="J49" t="s">
         <v>1472</v>
@@ -8505,7 +8505,7 @@
     </row>
     <row r="50" spans="1:12">
       <c r="A50" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B50" t="s">
         <v>83</v>
@@ -8526,7 +8526,7 @@
         <v>1284</v>
       </c>
       <c r="I50" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
       <c r="J50" t="s">
         <v>1473</v>
@@ -8750,7 +8750,7 @@
     </row>
     <row r="57" spans="1:12">
       <c r="A57" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B57" t="s">
         <v>90</v>
@@ -8771,7 +8771,7 @@
         <v>1284</v>
       </c>
       <c r="I57" t="s">
-        <v>1325</v>
+        <v>1326</v>
       </c>
       <c r="J57" t="s">
         <v>1480</v>
@@ -8841,7 +8841,7 @@
         <v>1284</v>
       </c>
       <c r="I59" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="J59" t="s">
         <v>1482</v>
@@ -8855,7 +8855,7 @@
     </row>
     <row r="60" spans="1:12">
       <c r="A60" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B60" t="s">
         <v>93</v>
@@ -8876,7 +8876,7 @@
         <v>1284</v>
       </c>
       <c r="I60" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
       <c r="J60" t="s">
         <v>1483</v>
@@ -8890,7 +8890,7 @@
     </row>
     <row r="61" spans="1:12">
       <c r="A61" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B61" t="s">
         <v>94</v>
@@ -8911,7 +8911,7 @@
         <v>1284</v>
       </c>
       <c r="I61" t="s">
-        <v>1327</v>
+        <v>1328</v>
       </c>
       <c r="J61" t="s">
         <v>1484</v>
@@ -9030,7 +9030,7 @@
     </row>
     <row r="65" spans="1:12">
       <c r="A65" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B65" t="s">
         <v>98</v>
@@ -9051,7 +9051,7 @@
         <v>1284</v>
       </c>
       <c r="I65" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="J65" t="s">
         <v>1488</v>
@@ -9135,7 +9135,7 @@
     </row>
     <row r="68" spans="1:12">
       <c r="A68" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B68" t="s">
         <v>101</v>
@@ -9275,7 +9275,7 @@
     </row>
     <row r="72" spans="1:12">
       <c r="A72" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B72" t="s">
         <v>105</v>
@@ -9380,7 +9380,7 @@
     </row>
     <row r="75" spans="1:12">
       <c r="A75" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B75" t="s">
         <v>108</v>
@@ -9401,7 +9401,7 @@
         <v>1284</v>
       </c>
       <c r="I75" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="J75" t="s">
         <v>1498</v>
@@ -9450,7 +9450,7 @@
     </row>
     <row r="77" spans="1:12">
       <c r="A77" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B77" t="s">
         <v>110</v>
@@ -9471,7 +9471,7 @@
         <v>1284</v>
       </c>
       <c r="I77" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="J77" t="s">
         <v>1500</v>
@@ -9520,7 +9520,7 @@
     </row>
     <row r="79" spans="1:12">
       <c r="A79" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B79" t="s">
         <v>112</v>
@@ -9576,7 +9576,7 @@
         <v>1284</v>
       </c>
       <c r="I80" t="s">
-        <v>1331</v>
+        <v>1332</v>
       </c>
       <c r="J80" t="s">
         <v>1503</v>
@@ -9590,7 +9590,7 @@
     </row>
     <row r="81" spans="1:12">
       <c r="A81" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B81" t="s">
         <v>114</v>
@@ -9660,7 +9660,7 @@
     </row>
     <row r="83" spans="1:12">
       <c r="A83" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B83" t="s">
         <v>116</v>
@@ -9681,7 +9681,7 @@
         <v>1284</v>
       </c>
       <c r="I83" t="s">
-        <v>1332</v>
+        <v>1333</v>
       </c>
       <c r="J83" t="s">
         <v>1506</v>
@@ -9730,7 +9730,7 @@
     </row>
     <row r="85" spans="1:12">
       <c r="A85" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B85" t="s">
         <v>118</v>
@@ -9751,7 +9751,7 @@
         <v>1284</v>
       </c>
       <c r="I85" t="s">
-        <v>1333</v>
+        <v>1334</v>
       </c>
       <c r="J85" t="s">
         <v>1508</v>
@@ -9800,7 +9800,7 @@
     </row>
     <row r="87" spans="1:12">
       <c r="A87" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B87" t="s">
         <v>120</v>
@@ -9821,7 +9821,7 @@
         <v>1284</v>
       </c>
       <c r="I87" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="J87" t="s">
         <v>1510</v>
@@ -9856,7 +9856,7 @@
         <v>1284</v>
       </c>
       <c r="I88" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="J88" t="s">
         <v>1511</v>
@@ -9870,7 +9870,7 @@
     </row>
     <row r="89" spans="1:12">
       <c r="A89" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B89" t="s">
         <v>122</v>
@@ -9891,7 +9891,7 @@
         <v>1284</v>
       </c>
       <c r="I89" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="J89" t="s">
         <v>1512</v>
@@ -9905,7 +9905,7 @@
     </row>
     <row r="90" spans="1:12">
       <c r="A90" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B90" t="s">
         <v>123</v>
@@ -9926,7 +9926,7 @@
         <v>1284</v>
       </c>
       <c r="I90" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="J90" t="s">
         <v>1513</v>
@@ -9940,7 +9940,7 @@
     </row>
     <row r="91" spans="1:12">
       <c r="A91" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B91" t="s">
         <v>124</v>
@@ -10031,7 +10031,7 @@
         <v>1284</v>
       </c>
       <c r="I93" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="J93" t="s">
         <v>1516</v>
@@ -10045,7 +10045,7 @@
     </row>
     <row r="94" spans="1:12">
       <c r="A94" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B94" t="s">
         <v>127</v>
@@ -10066,7 +10066,7 @@
         <v>1284</v>
       </c>
       <c r="I94" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
       <c r="J94" t="s">
         <v>1517</v>
@@ -10150,7 +10150,7 @@
     </row>
     <row r="97" spans="1:12">
       <c r="A97" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B97" t="s">
         <v>130</v>
@@ -10185,7 +10185,7 @@
     </row>
     <row r="98" spans="1:12">
       <c r="A98" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B98" t="s">
         <v>131</v>
@@ -10360,7 +10360,7 @@
     </row>
     <row r="103" spans="1:12">
       <c r="A103" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B103" t="s">
         <v>136</v>
@@ -10395,7 +10395,7 @@
     </row>
     <row r="104" spans="1:12">
       <c r="A104" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B104" t="s">
         <v>137</v>
@@ -10416,7 +10416,7 @@
         <v>1284</v>
       </c>
       <c r="I104" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="J104" t="s">
         <v>1527</v>
@@ -10451,7 +10451,7 @@
         <v>1284</v>
       </c>
       <c r="I105" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="J105" t="s">
         <v>1528</v>
@@ -10465,7 +10465,7 @@
     </row>
     <row r="106" spans="1:12">
       <c r="A106" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B106" t="s">
         <v>139</v>
@@ -10486,7 +10486,7 @@
         <v>1284</v>
       </c>
       <c r="I106" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="J106" t="s">
         <v>1529</v>
@@ -10521,7 +10521,7 @@
         <v>1284</v>
       </c>
       <c r="I107" t="s">
-        <v>1343</v>
+        <v>1344</v>
       </c>
       <c r="J107" t="s">
         <v>1530</v>
@@ -10535,7 +10535,7 @@
     </row>
     <row r="108" spans="1:12">
       <c r="A108" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B108" t="s">
         <v>141</v>
@@ -10556,7 +10556,7 @@
         <v>1284</v>
       </c>
       <c r="I108" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="J108" t="s">
         <v>1531</v>
@@ -10605,7 +10605,7 @@
     </row>
     <row r="110" spans="1:12">
       <c r="A110" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B110" t="s">
         <v>143</v>
@@ -10766,7 +10766,7 @@
         <v>1284</v>
       </c>
       <c r="I114" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="J114" t="s">
         <v>1537</v>
@@ -10780,7 +10780,7 @@
     </row>
     <row r="115" spans="1:12">
       <c r="A115" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B115" t="s">
         <v>148</v>
@@ -10804,7 +10804,7 @@
         <v>1287</v>
       </c>
       <c r="I115" t="s">
-        <v>1346</v>
+        <v>1347</v>
       </c>
       <c r="J115" t="s">
         <v>1538</v>
@@ -10839,7 +10839,7 @@
         <v>1284</v>
       </c>
       <c r="I116" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="J116" t="s">
         <v>1539</v>
@@ -10853,7 +10853,7 @@
     </row>
     <row r="117" spans="1:12">
       <c r="A117" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B117" t="s">
         <v>150</v>
@@ -10888,7 +10888,7 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B118" t="s">
         <v>151</v>
@@ -10958,7 +10958,7 @@
     </row>
     <row r="120" spans="1:12">
       <c r="A120" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B120" t="s">
         <v>153</v>
@@ -10979,7 +10979,7 @@
         <v>1284</v>
       </c>
       <c r="I120" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
       <c r="J120" t="s">
         <v>1543</v>
@@ -10993,7 +10993,7 @@
     </row>
     <row r="121" spans="1:12">
       <c r="A121" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B121" t="s">
         <v>154</v>
@@ -11014,7 +11014,7 @@
         <v>1284</v>
       </c>
       <c r="I121" t="s">
-        <v>1349</v>
+        <v>1350</v>
       </c>
       <c r="J121" t="s">
         <v>1544</v>
@@ -11028,7 +11028,7 @@
     </row>
     <row r="122" spans="1:12">
       <c r="A122" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B122" t="s">
         <v>155</v>
@@ -11049,7 +11049,7 @@
         <v>1284</v>
       </c>
       <c r="I122" t="s">
-        <v>1350</v>
+        <v>1351</v>
       </c>
       <c r="J122" t="s">
         <v>1545</v>
@@ -11063,7 +11063,7 @@
     </row>
     <row r="123" spans="1:12">
       <c r="A123" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B123" t="s">
         <v>156</v>
@@ -11098,7 +11098,7 @@
     </row>
     <row r="124" spans="1:12">
       <c r="A124" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B124" t="s">
         <v>157</v>
@@ -11119,7 +11119,7 @@
         <v>1284</v>
       </c>
       <c r="I124" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="J124" t="s">
         <v>1547</v>
@@ -11133,7 +11133,7 @@
     </row>
     <row r="125" spans="1:12">
       <c r="A125" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B125" t="s">
         <v>158</v>
@@ -11168,7 +11168,7 @@
     </row>
     <row r="126" spans="1:12">
       <c r="A126" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B126" t="s">
         <v>159</v>
@@ -11189,7 +11189,7 @@
         <v>1284</v>
       </c>
       <c r="I126" t="s">
-        <v>1351</v>
+        <v>1352</v>
       </c>
       <c r="J126" t="s">
         <v>1549</v>
@@ -11203,7 +11203,7 @@
     </row>
     <row r="127" spans="1:12">
       <c r="A127" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B127" t="s">
         <v>160</v>
@@ -11224,7 +11224,7 @@
         <v>1284</v>
       </c>
       <c r="I127" t="s">
-        <v>1352</v>
+        <v>1353</v>
       </c>
       <c r="J127" t="s">
         <v>1550</v>
@@ -11273,7 +11273,7 @@
     </row>
     <row r="129" spans="1:12">
       <c r="A129" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B129" t="s">
         <v>162</v>
@@ -11294,7 +11294,7 @@
         <v>1284</v>
       </c>
       <c r="I129" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
       <c r="J129" t="s">
         <v>1552</v>
@@ -11308,7 +11308,7 @@
     </row>
     <row r="130" spans="1:12">
       <c r="A130" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B130" t="s">
         <v>163</v>
@@ -11329,7 +11329,7 @@
         <v>1284</v>
       </c>
       <c r="I130" t="s">
-        <v>1353</v>
+        <v>1354</v>
       </c>
       <c r="J130" t="s">
         <v>1553</v>
@@ -11343,7 +11343,7 @@
     </row>
     <row r="131" spans="1:12">
       <c r="A131" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B131" t="s">
         <v>164</v>
@@ -11364,7 +11364,7 @@
         <v>1284</v>
       </c>
       <c r="I131" t="s">
-        <v>1344</v>
+        <v>1345</v>
       </c>
       <c r="J131" t="s">
         <v>1554</v>
@@ -11378,7 +11378,7 @@
     </row>
     <row r="132" spans="1:12">
       <c r="A132" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B132" t="s">
         <v>165</v>
@@ -11399,7 +11399,7 @@
         <v>1284</v>
       </c>
       <c r="I132" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="J132" t="s">
         <v>1555</v>
@@ -11469,7 +11469,7 @@
         <v>1284</v>
       </c>
       <c r="I134" t="s">
-        <v>1341</v>
+        <v>1342</v>
       </c>
       <c r="J134" t="s">
         <v>1557</v>
@@ -11553,7 +11553,7 @@
     </row>
     <row r="137" spans="1:12">
       <c r="A137" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B137" t="s">
         <v>170</v>
@@ -11609,7 +11609,7 @@
         <v>1284</v>
       </c>
       <c r="I138" t="s">
-        <v>1347</v>
+        <v>1348</v>
       </c>
       <c r="J138" t="s">
         <v>1560</v>
@@ -11658,7 +11658,7 @@
     </row>
     <row r="140" spans="1:12">
       <c r="A140" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B140" t="s">
         <v>173</v>
@@ -11693,7 +11693,7 @@
     </row>
     <row r="141" spans="1:12">
       <c r="A141" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B141" t="s">
         <v>174</v>
@@ -11728,7 +11728,7 @@
     </row>
     <row r="142" spans="1:12">
       <c r="A142" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B142" t="s">
         <v>175</v>
@@ -11763,7 +11763,7 @@
     </row>
     <row r="143" spans="1:12">
       <c r="A143" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B143" t="s">
         <v>176</v>
@@ -11798,7 +11798,7 @@
     </row>
     <row r="144" spans="1:12">
       <c r="A144" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B144" t="s">
         <v>177</v>
@@ -11819,7 +11819,7 @@
         <v>1284</v>
       </c>
       <c r="I144" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="J144" t="s">
         <v>1566</v>
@@ -11868,7 +11868,7 @@
     </row>
     <row r="146" spans="1:12">
       <c r="A146" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B146" t="s">
         <v>179</v>
@@ -11889,7 +11889,7 @@
         <v>1284</v>
       </c>
       <c r="I146" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
       <c r="J146" t="s">
         <v>1568</v>
@@ -11903,7 +11903,7 @@
     </row>
     <row r="147" spans="1:12">
       <c r="A147" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B147" t="s">
         <v>180</v>
@@ -11938,7 +11938,7 @@
     </row>
     <row r="148" spans="1:12">
       <c r="A148" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B148" t="s">
         <v>181</v>
@@ -11973,7 +11973,7 @@
     </row>
     <row r="149" spans="1:12">
       <c r="A149" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B149" t="s">
         <v>182</v>
@@ -12029,7 +12029,7 @@
         <v>1284</v>
       </c>
       <c r="I150" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="J150" t="s">
         <v>1572</v>
@@ -12134,7 +12134,7 @@
         <v>1284</v>
       </c>
       <c r="I153" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="J153" t="s">
         <v>1575</v>
@@ -12148,7 +12148,7 @@
     </row>
     <row r="154" spans="1:12">
       <c r="A154" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B154" t="s">
         <v>187</v>
@@ -12218,7 +12218,7 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B156" t="s">
         <v>189</v>
@@ -12288,7 +12288,7 @@
     </row>
     <row r="158" spans="1:12">
       <c r="A158" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B158" t="s">
         <v>191</v>
@@ -12344,7 +12344,7 @@
         <v>1284</v>
       </c>
       <c r="I159" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="J159" t="s">
         <v>1581</v>
@@ -12358,7 +12358,7 @@
     </row>
     <row r="160" spans="1:12">
       <c r="A160" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B160" t="s">
         <v>193</v>
@@ -12449,7 +12449,7 @@
         <v>1284</v>
       </c>
       <c r="I162" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="J162" t="s">
         <v>1584</v>
@@ -12463,7 +12463,7 @@
     </row>
     <row r="163" spans="1:12">
       <c r="A163" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B163" t="s">
         <v>196</v>
@@ -12484,7 +12484,7 @@
         <v>1284</v>
       </c>
       <c r="I163" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="J163" t="s">
         <v>1585</v>
@@ -12498,7 +12498,7 @@
     </row>
     <row r="164" spans="1:12">
       <c r="A164" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B164" t="s">
         <v>197</v>
@@ -12533,7 +12533,7 @@
     </row>
     <row r="165" spans="1:12">
       <c r="A165" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B165" t="s">
         <v>198</v>
@@ -12638,7 +12638,7 @@
     </row>
     <row r="168" spans="1:12">
       <c r="A168" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B168" t="s">
         <v>201</v>
@@ -12708,7 +12708,7 @@
     </row>
     <row r="170" spans="1:12">
       <c r="A170" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B170" t="s">
         <v>203</v>
@@ -12764,7 +12764,7 @@
         <v>1284</v>
       </c>
       <c r="I171" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="J171" t="s">
         <v>1593</v>
@@ -12848,7 +12848,7 @@
     </row>
     <row r="174" spans="1:12">
       <c r="A174" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B174" t="s">
         <v>207</v>
@@ -12953,7 +12953,7 @@
     </row>
     <row r="177" spans="1:12">
       <c r="A177" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B177" t="s">
         <v>210</v>
@@ -12974,7 +12974,7 @@
         <v>1284</v>
       </c>
       <c r="I177" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="J177" t="s">
         <v>1599</v>
@@ -13009,7 +13009,7 @@
         <v>1284</v>
       </c>
       <c r="I178" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="J178" t="s">
         <v>1600</v>
@@ -13058,7 +13058,7 @@
     </row>
     <row r="180" spans="1:12">
       <c r="A180" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B180" t="s">
         <v>213</v>
@@ -13079,7 +13079,7 @@
         <v>1284</v>
       </c>
       <c r="I180" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="J180" t="s">
         <v>1602</v>
@@ -13128,7 +13128,7 @@
     </row>
     <row r="182" spans="1:12">
       <c r="A182" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B182" t="s">
         <v>215</v>
@@ -13149,7 +13149,7 @@
         <v>1284</v>
       </c>
       <c r="I182" t="s">
-        <v>1363</v>
+        <v>1319</v>
       </c>
       <c r="J182" t="s">
         <v>1604</v>
@@ -13198,7 +13198,7 @@
     </row>
     <row r="184" spans="1:12">
       <c r="A184" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B184" t="s">
         <v>217</v>
@@ -13233,7 +13233,7 @@
     </row>
     <row r="185" spans="1:12">
       <c r="A185" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B185" t="s">
         <v>218</v>
@@ -13338,7 +13338,7 @@
     </row>
     <row r="188" spans="1:12">
       <c r="A188" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B188" t="s">
         <v>221</v>
@@ -13408,7 +13408,7 @@
     </row>
     <row r="190" spans="1:12">
       <c r="A190" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B190" t="s">
         <v>223</v>
@@ -13443,7 +13443,7 @@
     </row>
     <row r="191" spans="1:12">
       <c r="A191" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B191" t="s">
         <v>224</v>
@@ -13513,7 +13513,7 @@
     </row>
     <row r="193" spans="1:12">
       <c r="A193" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B193" t="s">
         <v>226</v>
@@ -13653,7 +13653,7 @@
     </row>
     <row r="197" spans="1:12">
       <c r="A197" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B197" t="s">
         <v>230</v>
@@ -14003,7 +14003,7 @@
     </row>
     <row r="207" spans="1:12">
       <c r="A207" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B207" t="s">
         <v>240</v>
@@ -14038,7 +14038,7 @@
     </row>
     <row r="208" spans="1:12">
       <c r="A208" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B208" t="s">
         <v>241</v>
@@ -14073,7 +14073,7 @@
     </row>
     <row r="209" spans="1:12">
       <c r="A209" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B209" t="s">
         <v>242</v>
@@ -14108,7 +14108,7 @@
     </row>
     <row r="210" spans="1:12">
       <c r="A210" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B210" t="s">
         <v>243</v>
@@ -14146,7 +14146,7 @@
     </row>
     <row r="211" spans="1:12">
       <c r="A211" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B211" t="s">
         <v>244</v>
@@ -14181,7 +14181,7 @@
     </row>
     <row r="212" spans="1:12">
       <c r="A212" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B212" t="s">
         <v>245</v>
@@ -14286,7 +14286,7 @@
     </row>
     <row r="215" spans="1:12">
       <c r="A215" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B215" t="s">
         <v>248</v>
@@ -14321,7 +14321,7 @@
     </row>
     <row r="216" spans="1:12">
       <c r="A216" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B216" t="s">
         <v>249</v>
@@ -14356,7 +14356,7 @@
     </row>
     <row r="217" spans="1:12">
       <c r="A217" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B217" t="s">
         <v>250</v>
@@ -14461,7 +14461,7 @@
     </row>
     <row r="220" spans="1:12">
       <c r="A220" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B220" t="s">
         <v>253</v>
@@ -14531,7 +14531,7 @@
     </row>
     <row r="222" spans="1:12">
       <c r="A222" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B222" t="s">
         <v>255</v>
@@ -14566,7 +14566,7 @@
     </row>
     <row r="223" spans="1:12">
       <c r="A223" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B223" t="s">
         <v>256</v>
@@ -14916,7 +14916,7 @@
     </row>
     <row r="233" spans="1:12">
       <c r="A233" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B233" t="s">
         <v>266</v>
@@ -14951,7 +14951,7 @@
     </row>
     <row r="234" spans="1:12">
       <c r="A234" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B234" t="s">
         <v>267</v>
@@ -15091,7 +15091,7 @@
     </row>
     <row r="238" spans="1:12">
       <c r="A238" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B238" t="s">
         <v>271</v>
@@ -15126,7 +15126,7 @@
     </row>
     <row r="239" spans="1:12">
       <c r="A239" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B239" t="s">
         <v>272</v>
@@ -15517,7 +15517,7 @@
     </row>
     <row r="250" spans="1:12">
       <c r="A250" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B250" t="s">
         <v>283</v>
@@ -15552,7 +15552,7 @@
     </row>
     <row r="251" spans="1:12">
       <c r="A251" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B251" t="s">
         <v>284</v>
@@ -15587,7 +15587,7 @@
     </row>
     <row r="252" spans="1:12">
       <c r="A252" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B252" t="s">
         <v>285</v>
@@ -15622,7 +15622,7 @@
     </row>
     <row r="253" spans="1:12">
       <c r="A253" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B253" t="s">
         <v>286</v>
@@ -15832,7 +15832,7 @@
     </row>
     <row r="259" spans="1:12">
       <c r="A259" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B259" t="s">
         <v>292</v>
@@ -15972,7 +15972,7 @@
     </row>
     <row r="263" spans="1:12">
       <c r="A263" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B263" t="s">
         <v>296</v>
@@ -16063,7 +16063,7 @@
         <v>1284</v>
       </c>
       <c r="I265" t="s">
-        <v>1323</v>
+        <v>1324</v>
       </c>
       <c r="J265" t="s">
         <v>1687</v>
@@ -16182,7 +16182,7 @@
     </row>
     <row r="269" spans="1:12">
       <c r="A269" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B269" t="s">
         <v>302</v>
@@ -16287,7 +16287,7 @@
     </row>
     <row r="272" spans="1:12">
       <c r="A272" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B272" t="s">
         <v>305</v>
@@ -16553,7 +16553,7 @@
         <v>1284</v>
       </c>
       <c r="I279" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="J279" t="s">
         <v>1701</v>
@@ -16567,7 +16567,7 @@
     </row>
     <row r="280" spans="1:12">
       <c r="A280" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B280" t="s">
         <v>313</v>
@@ -16672,7 +16672,7 @@
     </row>
     <row r="283" spans="1:12">
       <c r="A283" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B283" t="s">
         <v>316</v>
@@ -16917,7 +16917,7 @@
     </row>
     <row r="290" spans="1:12">
       <c r="A290" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B290" t="s">
         <v>323</v>
@@ -16952,7 +16952,7 @@
     </row>
     <row r="291" spans="1:12">
       <c r="A291" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B291" t="s">
         <v>324</v>
@@ -16987,7 +16987,7 @@
     </row>
     <row r="292" spans="1:12">
       <c r="A292" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B292" t="s">
         <v>325</v>
@@ -17057,7 +17057,7 @@
     </row>
     <row r="294" spans="1:12">
       <c r="A294" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B294" t="s">
         <v>327</v>
@@ -17078,7 +17078,7 @@
         <v>1284</v>
       </c>
       <c r="I294" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="J294" t="s">
         <v>1716</v>
@@ -17340,7 +17340,7 @@
     </row>
     <row r="302" spans="1:12">
       <c r="A302" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B302" t="s">
         <v>335</v>
@@ -17361,7 +17361,7 @@
         <v>1284</v>
       </c>
       <c r="I302" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="J302" t="s">
         <v>1724</v>
@@ -17483,7 +17483,7 @@
     </row>
     <row r="306" spans="1:12">
       <c r="A306" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B306" t="s">
         <v>339</v>
@@ -17658,7 +17658,7 @@
     </row>
     <row r="311" spans="1:12">
       <c r="A311" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B311" t="s">
         <v>344</v>
@@ -17693,7 +17693,7 @@
     </row>
     <row r="312" spans="1:12">
       <c r="A312" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B312" t="s">
         <v>345</v>
@@ -18113,7 +18113,7 @@
     </row>
     <row r="324" spans="1:12">
       <c r="A324" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B324" t="s">
         <v>357</v>
@@ -18484,7 +18484,7 @@
         <v>1284</v>
       </c>
       <c r="I334" t="s">
-        <v>1345</v>
+        <v>1346</v>
       </c>
       <c r="J334" t="s">
         <v>1756</v>
@@ -18603,7 +18603,7 @@
     </row>
     <row r="338" spans="1:12">
       <c r="A338" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B338" t="s">
         <v>371</v>
@@ -18638,7 +18638,7 @@
     </row>
     <row r="339" spans="1:12">
       <c r="A339" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B339" t="s">
         <v>372</v>
@@ -18708,7 +18708,7 @@
     </row>
     <row r="341" spans="1:12">
       <c r="A341" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B341" t="s">
         <v>374</v>
@@ -18778,7 +18778,7 @@
     </row>
     <row r="343" spans="1:12">
       <c r="A343" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B343" t="s">
         <v>376</v>
@@ -18834,7 +18834,7 @@
         <v>1284</v>
       </c>
       <c r="I344" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="J344" t="s">
         <v>1766</v>
@@ -18883,7 +18883,7 @@
     </row>
     <row r="346" spans="1:12">
       <c r="A346" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B346" t="s">
         <v>379</v>
@@ -18953,7 +18953,7 @@
     </row>
     <row r="348" spans="1:12">
       <c r="A348" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B348" t="s">
         <v>381</v>
@@ -18974,7 +18974,7 @@
         <v>1284</v>
       </c>
       <c r="I348" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="J348" t="s">
         <v>1770</v>
@@ -19023,7 +19023,7 @@
     </row>
     <row r="350" spans="1:12">
       <c r="A350" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B350" t="s">
         <v>383</v>
@@ -19058,7 +19058,7 @@
     </row>
     <row r="351" spans="1:12">
       <c r="A351" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B351" t="s">
         <v>384</v>
@@ -19093,7 +19093,7 @@
     </row>
     <row r="352" spans="1:12">
       <c r="A352" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B352" t="s">
         <v>385</v>
@@ -19114,7 +19114,7 @@
         <v>1284</v>
       </c>
       <c r="I352" t="s">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="J352" t="s">
         <v>1774</v>
@@ -19198,7 +19198,7 @@
     </row>
     <row r="355" spans="1:12">
       <c r="A355" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B355" t="s">
         <v>388</v>
@@ -19233,7 +19233,7 @@
     </row>
     <row r="356" spans="1:12">
       <c r="A356" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B356" t="s">
         <v>389</v>
@@ -19268,7 +19268,7 @@
     </row>
     <row r="357" spans="1:12">
       <c r="A357" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B357" t="s">
         <v>390</v>
@@ -19376,7 +19376,7 @@
     </row>
     <row r="360" spans="1:12">
       <c r="A360" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B360" t="s">
         <v>393</v>
@@ -19446,7 +19446,7 @@
     </row>
     <row r="362" spans="1:12">
       <c r="A362" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B362" t="s">
         <v>395</v>
@@ -19586,7 +19586,7 @@
     </row>
     <row r="366" spans="1:12">
       <c r="A366" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B366" t="s">
         <v>399</v>
@@ -19659,7 +19659,7 @@
     </row>
     <row r="368" spans="1:12">
       <c r="A368" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B368" t="s">
         <v>401</v>
@@ -19694,7 +19694,7 @@
     </row>
     <row r="369" spans="1:12">
       <c r="A369" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B369" t="s">
         <v>402</v>
@@ -19764,7 +19764,7 @@
     </row>
     <row r="371" spans="1:12">
       <c r="A371" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B371" t="s">
         <v>404</v>
@@ -19799,7 +19799,7 @@
     </row>
     <row r="372" spans="1:12">
       <c r="A372" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B372" t="s">
         <v>405</v>
@@ -19869,7 +19869,7 @@
     </row>
     <row r="374" spans="1:12">
       <c r="A374" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B374" t="s">
         <v>407</v>
@@ -19893,7 +19893,7 @@
         <v>1292</v>
       </c>
       <c r="I374" t="s">
-        <v>1342</v>
+        <v>1343</v>
       </c>
       <c r="J374" t="s">
         <v>1796</v>
@@ -19977,7 +19977,7 @@
     </row>
     <row r="377" spans="1:12">
       <c r="A377" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B377" t="s">
         <v>410</v>
@@ -20012,7 +20012,7 @@
     </row>
     <row r="378" spans="1:12">
       <c r="A378" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B378" t="s">
         <v>411</v>
@@ -20047,7 +20047,7 @@
     </row>
     <row r="379" spans="1:12">
       <c r="A379" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B379" t="s">
         <v>412</v>
@@ -20327,7 +20327,7 @@
     </row>
     <row r="387" spans="1:12">
       <c r="A387" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B387" t="s">
         <v>420</v>
@@ -20467,7 +20467,7 @@
     </row>
     <row r="391" spans="1:12">
       <c r="A391" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B391" t="s">
         <v>424</v>
@@ -20502,7 +20502,7 @@
     </row>
     <row r="392" spans="1:12">
       <c r="A392" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B392" t="s">
         <v>425</v>
@@ -20537,7 +20537,7 @@
     </row>
     <row r="393" spans="1:12">
       <c r="A393" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B393" t="s">
         <v>426</v>
@@ -20572,7 +20572,7 @@
     </row>
     <row r="394" spans="1:12">
       <c r="A394" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B394" t="s">
         <v>427</v>
@@ -20607,7 +20607,7 @@
     </row>
     <row r="395" spans="1:12">
       <c r="A395" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B395" t="s">
         <v>428</v>
@@ -20642,7 +20642,7 @@
     </row>
     <row r="396" spans="1:12">
       <c r="A396" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B396" t="s">
         <v>429</v>
@@ -20677,7 +20677,7 @@
     </row>
     <row r="397" spans="1:12">
       <c r="A397" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B397" t="s">
         <v>430</v>
@@ -20712,7 +20712,7 @@
     </row>
     <row r="398" spans="1:12">
       <c r="A398" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B398" t="s">
         <v>431</v>
@@ -20747,7 +20747,7 @@
     </row>
     <row r="399" spans="1:12">
       <c r="A399" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B399" t="s">
         <v>432</v>
@@ -20782,7 +20782,7 @@
     </row>
     <row r="400" spans="1:12">
       <c r="A400" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B400" t="s">
         <v>433</v>
@@ -20817,7 +20817,7 @@
     </row>
     <row r="401" spans="1:12">
       <c r="A401" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B401" t="s">
         <v>434</v>
@@ -20852,7 +20852,7 @@
     </row>
     <row r="402" spans="1:12">
       <c r="A402" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B402" t="s">
         <v>435</v>
@@ -20887,7 +20887,7 @@
     </row>
     <row r="403" spans="1:12">
       <c r="A403" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B403" t="s">
         <v>436</v>
@@ -20922,7 +20922,7 @@
     </row>
     <row r="404" spans="1:12">
       <c r="A404" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B404" t="s">
         <v>437</v>
@@ -20957,7 +20957,7 @@
     </row>
     <row r="405" spans="1:12">
       <c r="A405" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B405" t="s">
         <v>438</v>
@@ -20992,7 +20992,7 @@
     </row>
     <row r="406" spans="1:12">
       <c r="A406" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B406" t="s">
         <v>439</v>
@@ -21027,7 +21027,7 @@
     </row>
     <row r="407" spans="1:12">
       <c r="A407" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B407" t="s">
         <v>440</v>
@@ -21062,7 +21062,7 @@
     </row>
     <row r="408" spans="1:12">
       <c r="A408" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B408" t="s">
         <v>441</v>
@@ -21097,7 +21097,7 @@
     </row>
     <row r="409" spans="1:12">
       <c r="A409" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B409" t="s">
         <v>442</v>
@@ -21132,7 +21132,7 @@
     </row>
     <row r="410" spans="1:12">
       <c r="A410" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B410" t="s">
         <v>443</v>
@@ -21167,7 +21167,7 @@
     </row>
     <row r="411" spans="1:12">
       <c r="A411" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B411" t="s">
         <v>444</v>
@@ -21202,7 +21202,7 @@
     </row>
     <row r="412" spans="1:12">
       <c r="A412" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B412" t="s">
         <v>444</v>
@@ -21272,7 +21272,7 @@
     </row>
     <row r="414" spans="1:12">
       <c r="A414" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B414" t="s">
         <v>446</v>
@@ -21380,7 +21380,7 @@
     </row>
     <row r="417" spans="1:12">
       <c r="A417" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B417" t="s">
         <v>449</v>
@@ -21415,7 +21415,7 @@
     </row>
     <row r="418" spans="1:12">
       <c r="A418" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B418" t="s">
         <v>450</v>
@@ -21488,7 +21488,7 @@
     </row>
     <row r="420" spans="1:12">
       <c r="A420" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B420" t="s">
         <v>452</v>
@@ -21523,7 +21523,7 @@
     </row>
     <row r="421" spans="1:12">
       <c r="A421" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B421" t="s">
         <v>453</v>
@@ -21701,7 +21701,7 @@
     </row>
     <row r="426" spans="1:12">
       <c r="A426" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B426" t="s">
         <v>458</v>
@@ -21806,7 +21806,7 @@
     </row>
     <row r="429" spans="1:12">
       <c r="A429" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B429" t="s">
         <v>461</v>
@@ -21981,7 +21981,7 @@
     </row>
     <row r="434" spans="1:12">
       <c r="A434" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B434" t="s">
         <v>466</v>
@@ -22016,7 +22016,7 @@
     </row>
     <row r="435" spans="1:12">
       <c r="A435" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B435" t="s">
         <v>467</v>
@@ -22051,7 +22051,7 @@
     </row>
     <row r="436" spans="1:12">
       <c r="A436" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B436" t="s">
         <v>468</v>
@@ -22121,7 +22121,7 @@
     </row>
     <row r="438" spans="1:12">
       <c r="A438" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B438" t="s">
         <v>470</v>
@@ -22159,7 +22159,7 @@
     </row>
     <row r="439" spans="1:12">
       <c r="A439" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B439" t="s">
         <v>470</v>
@@ -22197,7 +22197,7 @@
     </row>
     <row r="440" spans="1:12">
       <c r="A440" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B440" t="s">
         <v>471</v>
@@ -22267,7 +22267,7 @@
     </row>
     <row r="442" spans="1:12">
       <c r="A442" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B442" t="s">
         <v>473</v>
@@ -22302,7 +22302,7 @@
     </row>
     <row r="443" spans="1:12">
       <c r="A443" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B443" t="s">
         <v>474</v>
@@ -22372,7 +22372,7 @@
     </row>
     <row r="445" spans="1:12">
       <c r="A445" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B445" t="s">
         <v>476</v>
@@ -22407,7 +22407,7 @@
     </row>
     <row r="446" spans="1:12">
       <c r="A446" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B446" t="s">
         <v>477</v>
@@ -22480,7 +22480,7 @@
     </row>
     <row r="448" spans="1:12">
       <c r="A448" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B448" t="s">
         <v>479</v>
@@ -22588,7 +22588,7 @@
     </row>
     <row r="451" spans="1:12">
       <c r="A451" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B451" t="s">
         <v>482</v>
@@ -22623,7 +22623,7 @@
     </row>
     <row r="452" spans="1:12">
       <c r="A452" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B452" t="s">
         <v>483</v>
@@ -22658,7 +22658,7 @@
     </row>
     <row r="453" spans="1:12">
       <c r="A453" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B453" t="s">
         <v>484</v>
@@ -22766,7 +22766,7 @@
     </row>
     <row r="456" spans="1:12">
       <c r="A456" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B456" t="s">
         <v>487</v>
@@ -22801,7 +22801,7 @@
     </row>
     <row r="457" spans="1:12">
       <c r="A457" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B457" t="s">
         <v>488</v>
@@ -22906,7 +22906,7 @@
     </row>
     <row r="460" spans="1:12">
       <c r="A460" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B460" t="s">
         <v>491</v>
@@ -23122,7 +23122,7 @@
     </row>
     <row r="466" spans="1:12">
       <c r="A466" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B466" t="s">
         <v>497</v>
@@ -23297,7 +23297,7 @@
     </row>
     <row r="471" spans="1:12">
       <c r="A471" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B471" t="s">
         <v>502</v>
@@ -23461,7 +23461,7 @@
         <v>1284</v>
       </c>
       <c r="I475" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="J475" t="s">
         <v>1895</v>
@@ -23475,7 +23475,7 @@
     </row>
     <row r="476" spans="1:12">
       <c r="A476" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B476" t="s">
         <v>507</v>
@@ -23513,7 +23513,7 @@
     </row>
     <row r="477" spans="1:12">
       <c r="A477" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B477" t="s">
         <v>508</v>
@@ -23817,7 +23817,7 @@
         <v>1284</v>
       </c>
       <c r="I485" t="s">
-        <v>1363</v>
+        <v>1319</v>
       </c>
       <c r="J485" t="s">
         <v>1904</v>
@@ -23831,7 +23831,7 @@
     </row>
     <row r="486" spans="1:12">
       <c r="A486" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B486" t="s">
         <v>517</v>
@@ -23866,7 +23866,7 @@
     </row>
     <row r="487" spans="1:12">
       <c r="A487" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B487" t="s">
         <v>518</v>
@@ -24144,7 +24144,7 @@
         <v>1301</v>
       </c>
       <c r="I494" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="J494" t="s">
         <v>1913</v>
@@ -24158,7 +24158,7 @@
     </row>
     <row r="495" spans="1:12">
       <c r="A495" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B495" t="s">
         <v>526</v>
@@ -24193,7 +24193,7 @@
     </row>
     <row r="496" spans="1:12">
       <c r="A496" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B496" t="s">
         <v>527</v>
@@ -24269,7 +24269,7 @@
     </row>
     <row r="498" spans="1:12">
       <c r="A498" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B498" t="s">
         <v>529</v>
@@ -24293,7 +24293,7 @@
         <v>1304</v>
       </c>
       <c r="I498" t="s">
-        <v>1348</v>
+        <v>1349</v>
       </c>
       <c r="J498" t="s">
         <v>1917</v>
@@ -24307,7 +24307,7 @@
     </row>
     <row r="499" spans="1:12">
       <c r="A499" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B499" t="s">
         <v>530</v>
@@ -24377,7 +24377,7 @@
     </row>
     <row r="501" spans="1:12">
       <c r="A501" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B501" t="s">
         <v>532</v>
@@ -24415,7 +24415,7 @@
     </row>
     <row r="502" spans="1:12">
       <c r="A502" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B502" t="s">
         <v>533</v>
@@ -24453,7 +24453,7 @@
     </row>
     <row r="503" spans="1:12">
       <c r="A503" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B503" t="s">
         <v>534</v>
@@ -24526,7 +24526,7 @@
     </row>
     <row r="505" spans="1:12">
       <c r="A505" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B505" t="s">
         <v>536</v>
@@ -24561,7 +24561,7 @@
     </row>
     <row r="506" spans="1:12">
       <c r="A506" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B506" t="s">
         <v>537</v>
@@ -24704,7 +24704,7 @@
     </row>
     <row r="510" spans="1:12">
       <c r="A510" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B510" t="s">
         <v>541</v>
@@ -24739,7 +24739,7 @@
     </row>
     <row r="511" spans="1:12">
       <c r="A511" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B511" t="s">
         <v>542</v>
@@ -24809,7 +24809,7 @@
     </row>
     <row r="513" spans="1:12">
       <c r="A513" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B513" t="s">
         <v>544</v>
@@ -24844,7 +24844,7 @@
     </row>
     <row r="514" spans="1:12">
       <c r="A514" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B514" t="s">
         <v>545</v>
@@ -24879,7 +24879,7 @@
     </row>
     <row r="515" spans="1:12">
       <c r="A515" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B515" t="s">
         <v>546</v>
@@ -24917,7 +24917,7 @@
     </row>
     <row r="516" spans="1:12">
       <c r="A516" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B516" t="s">
         <v>547</v>
@@ -24952,7 +24952,7 @@
     </row>
     <row r="517" spans="1:12">
       <c r="A517" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B517" t="s">
         <v>548</v>
@@ -25060,7 +25060,7 @@
     </row>
     <row r="520" spans="1:12">
       <c r="A520" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B520" t="s">
         <v>551</v>
@@ -25095,7 +25095,7 @@
     </row>
     <row r="521" spans="1:12">
       <c r="A521" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B521" t="s">
         <v>552</v>
@@ -25127,7 +25127,7 @@
     </row>
     <row r="522" spans="1:12">
       <c r="A522" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B522" t="s">
         <v>553</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-19 00:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -6834,7 +6834,7 @@
         <v>1073</v>
       </c>
       <c r="E2">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F2" t="s">
         <v>1279</v>
@@ -6869,7 +6869,7 @@
         <v>1074</v>
       </c>
       <c r="E3">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F3" t="s">
         <v>1279</v>
@@ -6904,7 +6904,7 @@
         <v>1075</v>
       </c>
       <c r="E4">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="F4" t="s">
         <v>1279</v>
@@ -6939,7 +6939,7 @@
         <v>1076</v>
       </c>
       <c r="E5">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F5" t="s">
         <v>1279</v>
@@ -6974,7 +6974,7 @@
         <v>1077</v>
       </c>
       <c r="E6">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="F6" t="s">
         <v>1279</v>
@@ -7009,7 +7009,7 @@
         <v>1078</v>
       </c>
       <c r="E7">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="F7" t="s">
         <v>1279</v>
@@ -7044,7 +7044,7 @@
         <v>1079</v>
       </c>
       <c r="E8">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F8" t="s">
         <v>1279</v>
@@ -7079,7 +7079,7 @@
         <v>1080</v>
       </c>
       <c r="E9">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F9" t="s">
         <v>1279</v>
@@ -7114,7 +7114,7 @@
         <v>1081</v>
       </c>
       <c r="E10">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F10" t="s">
         <v>1279</v>
@@ -7149,7 +7149,7 @@
         <v>1081</v>
       </c>
       <c r="E11">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="F11" t="s">
         <v>1279</v>
@@ -7184,7 +7184,7 @@
         <v>1082</v>
       </c>
       <c r="E12">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F12" t="s">
         <v>1279</v>
@@ -7219,7 +7219,7 @@
         <v>1083</v>
       </c>
       <c r="E13">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F13" t="s">
         <v>1279</v>
@@ -7254,7 +7254,7 @@
         <v>1084</v>
       </c>
       <c r="E14">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F14" t="s">
         <v>1279</v>
@@ -7289,7 +7289,7 @@
         <v>1084</v>
       </c>
       <c r="E15">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F15" t="s">
         <v>1279</v>
@@ -7324,7 +7324,7 @@
         <v>1085</v>
       </c>
       <c r="E16">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F16" t="s">
         <v>1279</v>
@@ -7359,7 +7359,7 @@
         <v>1085</v>
       </c>
       <c r="E17">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F17" t="s">
         <v>1279</v>
@@ -7394,7 +7394,7 @@
         <v>1086</v>
       </c>
       <c r="E18">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F18" t="s">
         <v>1279</v>
@@ -7429,7 +7429,7 @@
         <v>1087</v>
       </c>
       <c r="E19">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F19" t="s">
         <v>1279</v>
@@ -7464,7 +7464,7 @@
         <v>1088</v>
       </c>
       <c r="E20">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F20" t="s">
         <v>1279</v>
@@ -7499,7 +7499,7 @@
         <v>1089</v>
       </c>
       <c r="E21">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F21" t="s">
         <v>1279</v>
@@ -7534,7 +7534,7 @@
         <v>1090</v>
       </c>
       <c r="E22">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F22" t="s">
         <v>1279</v>
@@ -7572,7 +7572,7 @@
         <v>1091</v>
       </c>
       <c r="E23">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F23" t="s">
         <v>1279</v>
@@ -7607,7 +7607,7 @@
         <v>1092</v>
       </c>
       <c r="E24">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F24" t="s">
         <v>1279</v>
@@ -7642,7 +7642,7 @@
         <v>1093</v>
       </c>
       <c r="E25">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F25" t="s">
         <v>1279</v>
@@ -7677,7 +7677,7 @@
         <v>1094</v>
       </c>
       <c r="E26">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F26" t="s">
         <v>1279</v>
@@ -7712,7 +7712,7 @@
         <v>1095</v>
       </c>
       <c r="E27">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F27" t="s">
         <v>1279</v>
@@ -7747,7 +7747,7 @@
         <v>1096</v>
       </c>
       <c r="E28">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F28" t="s">
         <v>1279</v>
@@ -7782,7 +7782,7 @@
         <v>1097</v>
       </c>
       <c r="E29">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F29" t="s">
         <v>1279</v>
@@ -7817,7 +7817,7 @@
         <v>1098</v>
       </c>
       <c r="E30">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F30" t="s">
         <v>1279</v>
@@ -7852,7 +7852,7 @@
         <v>1099</v>
       </c>
       <c r="E31">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F31" t="s">
         <v>1279</v>
@@ -7887,7 +7887,7 @@
         <v>1100</v>
       </c>
       <c r="E32">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F32" t="s">
         <v>1279</v>
@@ -7922,7 +7922,7 @@
         <v>1101</v>
       </c>
       <c r="E33">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F33" t="s">
         <v>1279</v>
@@ -7957,7 +7957,7 @@
         <v>1102</v>
       </c>
       <c r="E34">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F34" t="s">
         <v>1279</v>
@@ -7992,7 +7992,7 @@
         <v>1103</v>
       </c>
       <c r="E35">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F35" t="s">
         <v>1279</v>
@@ -8027,7 +8027,7 @@
         <v>1104</v>
       </c>
       <c r="E36">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F36" t="s">
         <v>1279</v>
@@ -8062,7 +8062,7 @@
         <v>1104</v>
       </c>
       <c r="E37">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F37" t="s">
         <v>1279</v>
@@ -8097,7 +8097,7 @@
         <v>1105</v>
       </c>
       <c r="E38">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="F38" t="s">
         <v>1279</v>
@@ -8132,7 +8132,7 @@
         <v>1106</v>
       </c>
       <c r="E39">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F39" t="s">
         <v>1279</v>
@@ -8167,7 +8167,7 @@
         <v>1107</v>
       </c>
       <c r="E40">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F40" t="s">
         <v>1279</v>
@@ -8202,7 +8202,7 @@
         <v>1107</v>
       </c>
       <c r="E41">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F41" t="s">
         <v>1279</v>
@@ -8237,7 +8237,7 @@
         <v>1108</v>
       </c>
       <c r="E42">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F42" t="s">
         <v>1279</v>
@@ -8272,7 +8272,7 @@
         <v>1108</v>
       </c>
       <c r="E43">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F43" t="s">
         <v>1279</v>
@@ -8307,7 +8307,7 @@
         <v>1109</v>
       </c>
       <c r="E44">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F44" t="s">
         <v>1279</v>
@@ -8342,7 +8342,7 @@
         <v>1110</v>
       </c>
       <c r="E45">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F45" t="s">
         <v>1279</v>
@@ -8377,7 +8377,7 @@
         <v>1111</v>
       </c>
       <c r="E46">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F46" t="s">
         <v>1279</v>
@@ -8412,7 +8412,7 @@
         <v>1112</v>
       </c>
       <c r="E47">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F47" t="s">
         <v>1279</v>
@@ -8447,7 +8447,7 @@
         <v>1112</v>
       </c>
       <c r="E48">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F48" t="s">
         <v>1279</v>
@@ -8482,7 +8482,7 @@
         <v>1113</v>
       </c>
       <c r="E49">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F49" t="s">
         <v>1279</v>
@@ -8517,7 +8517,7 @@
         <v>1114</v>
       </c>
       <c r="E50">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="F50" t="s">
         <v>1279</v>
@@ -8552,7 +8552,7 @@
         <v>1115</v>
       </c>
       <c r="E51">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F51" t="s">
         <v>1279</v>
@@ -8587,7 +8587,7 @@
         <v>1116</v>
       </c>
       <c r="E52">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F52" t="s">
         <v>1279</v>
@@ -8622,7 +8622,7 @@
         <v>1117</v>
       </c>
       <c r="E53">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F53" t="s">
         <v>1279</v>
@@ -8657,7 +8657,7 @@
         <v>1118</v>
       </c>
       <c r="E54">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F54" t="s">
         <v>1279</v>
@@ -8692,7 +8692,7 @@
         <v>1119</v>
       </c>
       <c r="E55">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F55" t="s">
         <v>1279</v>
@@ -8727,7 +8727,7 @@
         <v>1119</v>
       </c>
       <c r="E56">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F56" t="s">
         <v>1279</v>
@@ -8762,7 +8762,7 @@
         <v>1119</v>
       </c>
       <c r="E57">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F57" t="s">
         <v>1279</v>
@@ -8797,7 +8797,7 @@
         <v>1120</v>
       </c>
       <c r="E58">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F58" t="s">
         <v>1279</v>
@@ -8832,7 +8832,7 @@
         <v>1121</v>
       </c>
       <c r="E59">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F59" t="s">
         <v>1279</v>
@@ -8867,7 +8867,7 @@
         <v>1122</v>
       </c>
       <c r="E60">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F60" t="s">
         <v>1279</v>
@@ -8902,7 +8902,7 @@
         <v>1122</v>
       </c>
       <c r="E61">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F61" t="s">
         <v>1279</v>
@@ -8937,7 +8937,7 @@
         <v>1123</v>
       </c>
       <c r="E62">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F62" t="s">
         <v>1279</v>
@@ -8972,7 +8972,7 @@
         <v>1124</v>
       </c>
       <c r="E63">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F63" t="s">
         <v>1279</v>
@@ -9007,7 +9007,7 @@
         <v>1124</v>
       </c>
       <c r="E64">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F64" t="s">
         <v>1279</v>
@@ -9042,7 +9042,7 @@
         <v>1124</v>
       </c>
       <c r="E65">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F65" t="s">
         <v>1279</v>
@@ -9077,7 +9077,7 @@
         <v>1125</v>
       </c>
       <c r="E66">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F66" t="s">
         <v>1279</v>
@@ -9112,7 +9112,7 @@
         <v>1126</v>
       </c>
       <c r="E67">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F67" t="s">
         <v>1279</v>
@@ -9147,7 +9147,7 @@
         <v>1126</v>
       </c>
       <c r="E68">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F68" t="s">
         <v>1279</v>
@@ -9182,7 +9182,7 @@
         <v>1126</v>
       </c>
       <c r="E69">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F69" t="s">
         <v>1280</v>
@@ -9217,7 +9217,7 @@
         <v>1126</v>
       </c>
       <c r="E70">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F70" t="s">
         <v>1279</v>
@@ -9252,7 +9252,7 @@
         <v>1127</v>
       </c>
       <c r="E71">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F71" t="s">
         <v>1279</v>
@@ -9287,7 +9287,7 @@
         <v>1128</v>
       </c>
       <c r="E72">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F72" t="s">
         <v>1279</v>
@@ -9322,7 +9322,7 @@
         <v>1128</v>
       </c>
       <c r="E73">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F73" t="s">
         <v>1279</v>
@@ -9357,7 +9357,7 @@
         <v>1129</v>
       </c>
       <c r="E74">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F74" t="s">
         <v>1279</v>
@@ -9392,7 +9392,7 @@
         <v>1130</v>
       </c>
       <c r="E75">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F75" t="s">
         <v>1279</v>
@@ -9427,7 +9427,7 @@
         <v>1131</v>
       </c>
       <c r="E76">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F76" t="s">
         <v>1279</v>
@@ -9462,7 +9462,7 @@
         <v>1132</v>
       </c>
       <c r="E77">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F77" t="s">
         <v>1279</v>
@@ -9497,7 +9497,7 @@
         <v>1132</v>
       </c>
       <c r="E78">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F78" t="s">
         <v>1279</v>
@@ -9532,7 +9532,7 @@
         <v>1132</v>
       </c>
       <c r="E79">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F79" t="s">
         <v>1279</v>
@@ -9567,7 +9567,7 @@
         <v>1132</v>
       </c>
       <c r="E80">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F80" t="s">
         <v>1279</v>
@@ -9602,7 +9602,7 @@
         <v>1132</v>
       </c>
       <c r="E81">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F81" t="s">
         <v>1279</v>
@@ -9637,7 +9637,7 @@
         <v>1132</v>
       </c>
       <c r="E82">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F82" t="s">
         <v>1279</v>
@@ -9672,7 +9672,7 @@
         <v>1133</v>
       </c>
       <c r="E83">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F83" t="s">
         <v>1279</v>
@@ -9707,7 +9707,7 @@
         <v>1134</v>
       </c>
       <c r="E84">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F84" t="s">
         <v>1279</v>
@@ -9742,7 +9742,7 @@
         <v>1135</v>
       </c>
       <c r="E85">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F85" t="s">
         <v>1279</v>
@@ -9777,7 +9777,7 @@
         <v>1135</v>
       </c>
       <c r="E86">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F86" t="s">
         <v>1279</v>
@@ -9812,7 +9812,7 @@
         <v>1136</v>
       </c>
       <c r="E87">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F87" t="s">
         <v>1281</v>
@@ -9847,7 +9847,7 @@
         <v>1137</v>
       </c>
       <c r="E88">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F88" t="s">
         <v>1279</v>
@@ -9882,7 +9882,7 @@
         <v>1138</v>
       </c>
       <c r="E89">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F89" t="s">
         <v>1279</v>
@@ -9917,7 +9917,7 @@
         <v>1138</v>
       </c>
       <c r="E90">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F90" t="s">
         <v>1279</v>
@@ -9952,7 +9952,7 @@
         <v>1139</v>
       </c>
       <c r="E91">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F91" t="s">
         <v>1279</v>
@@ -9987,7 +9987,7 @@
         <v>1140</v>
       </c>
       <c r="E92">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F92" t="s">
         <v>1279</v>
@@ -10022,7 +10022,7 @@
         <v>1141</v>
       </c>
       <c r="E93">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F93" t="s">
         <v>1279</v>
@@ -10057,7 +10057,7 @@
         <v>1142</v>
       </c>
       <c r="E94">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F94" t="s">
         <v>1279</v>
@@ -10092,7 +10092,7 @@
         <v>1143</v>
       </c>
       <c r="E95">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F95" t="s">
         <v>1279</v>
@@ -10127,7 +10127,7 @@
         <v>1143</v>
       </c>
       <c r="E96">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F96" t="s">
         <v>1279</v>
@@ -10162,7 +10162,7 @@
         <v>1144</v>
       </c>
       <c r="E97">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F97" t="s">
         <v>1279</v>
@@ -10197,7 +10197,7 @@
         <v>1144</v>
       </c>
       <c r="E98">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F98" t="s">
         <v>1279</v>
@@ -10232,7 +10232,7 @@
         <v>1144</v>
       </c>
       <c r="E99">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F99" t="s">
         <v>1279</v>
@@ -10267,7 +10267,7 @@
         <v>1145</v>
       </c>
       <c r="E100">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F100" t="s">
         <v>1279</v>
@@ -10302,7 +10302,7 @@
         <v>1145</v>
       </c>
       <c r="E101">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F101" t="s">
         <v>1279</v>
@@ -10337,7 +10337,7 @@
         <v>1146</v>
       </c>
       <c r="E102">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F102" t="s">
         <v>1279</v>
@@ -10372,7 +10372,7 @@
         <v>1147</v>
       </c>
       <c r="E103">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F103" t="s">
         <v>1279</v>
@@ -10407,7 +10407,7 @@
         <v>1148</v>
       </c>
       <c r="E104">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F104" t="s">
         <v>1279</v>
@@ -10442,7 +10442,7 @@
         <v>1148</v>
       </c>
       <c r="E105">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F105" t="s">
         <v>1279</v>
@@ -10477,7 +10477,7 @@
         <v>1149</v>
       </c>
       <c r="E106">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F106" t="s">
         <v>1279</v>
@@ -10512,7 +10512,7 @@
         <v>1149</v>
       </c>
       <c r="E107">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F107" t="s">
         <v>1279</v>
@@ -10547,7 +10547,7 @@
         <v>1150</v>
       </c>
       <c r="E108">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F108" t="s">
         <v>1279</v>
@@ -10582,7 +10582,7 @@
         <v>1151</v>
       </c>
       <c r="E109">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F109" t="s">
         <v>1279</v>
@@ -10617,7 +10617,7 @@
         <v>1151</v>
       </c>
       <c r="E110">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F110" t="s">
         <v>1279</v>
@@ -10652,7 +10652,7 @@
         <v>1152</v>
       </c>
       <c r="E111">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F111" t="s">
         <v>1279</v>
@@ -10687,7 +10687,7 @@
         <v>1153</v>
       </c>
       <c r="E112">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F112" t="s">
         <v>1279</v>
@@ -10722,7 +10722,7 @@
         <v>1153</v>
       </c>
       <c r="E113">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F113" t="s">
         <v>1279</v>
@@ -10757,7 +10757,7 @@
         <v>1154</v>
       </c>
       <c r="E114">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F114" t="s">
         <v>1279</v>
@@ -10792,7 +10792,7 @@
         <v>1155</v>
       </c>
       <c r="E115">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F115" t="s">
         <v>1279</v>
@@ -10830,7 +10830,7 @@
         <v>1155</v>
       </c>
       <c r="E116">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F116" t="s">
         <v>1279</v>
@@ -10865,7 +10865,7 @@
         <v>1155</v>
       </c>
       <c r="E117">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F117" t="s">
         <v>1279</v>
@@ -10900,7 +10900,7 @@
         <v>1155</v>
       </c>
       <c r="E118">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F118" t="s">
         <v>1279</v>
@@ -10935,7 +10935,7 @@
         <v>1156</v>
       </c>
       <c r="E119">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F119" t="s">
         <v>1280</v>
@@ -10970,7 +10970,7 @@
         <v>1157</v>
       </c>
       <c r="E120">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F120" t="s">
         <v>1279</v>
@@ -11005,7 +11005,7 @@
         <v>1157</v>
       </c>
       <c r="E121">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F121" t="s">
         <v>1279</v>
@@ -11040,7 +11040,7 @@
         <v>1157</v>
       </c>
       <c r="E122">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F122" t="s">
         <v>1279</v>
@@ -11075,7 +11075,7 @@
         <v>1157</v>
       </c>
       <c r="E123">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F123" t="s">
         <v>1279</v>
@@ -11110,7 +11110,7 @@
         <v>1158</v>
       </c>
       <c r="E124">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F124" t="s">
         <v>1279</v>
@@ -11145,7 +11145,7 @@
         <v>1158</v>
       </c>
       <c r="E125">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F125" t="s">
         <v>1279</v>
@@ -11180,7 +11180,7 @@
         <v>1158</v>
       </c>
       <c r="E126">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F126" t="s">
         <v>1279</v>
@@ -11215,7 +11215,7 @@
         <v>1158</v>
       </c>
       <c r="E127">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F127" t="s">
         <v>1279</v>
@@ -11250,7 +11250,7 @@
         <v>1158</v>
       </c>
       <c r="E128">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F128" t="s">
         <v>1279</v>
@@ -11285,7 +11285,7 @@
         <v>1158</v>
       </c>
       <c r="E129">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F129" t="s">
         <v>1279</v>
@@ -11320,7 +11320,7 @@
         <v>1158</v>
       </c>
       <c r="E130">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F130" t="s">
         <v>1279</v>
@@ -11355,7 +11355,7 @@
         <v>1159</v>
       </c>
       <c r="E131">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F131" t="s">
         <v>1279</v>
@@ -11390,7 +11390,7 @@
         <v>1159</v>
       </c>
       <c r="E132">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F132" t="s">
         <v>1279</v>
@@ -11425,7 +11425,7 @@
         <v>1160</v>
       </c>
       <c r="E133">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F133" t="s">
         <v>1279</v>
@@ -11460,7 +11460,7 @@
         <v>1161</v>
       </c>
       <c r="E134">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F134" t="s">
         <v>1279</v>
@@ -11495,7 +11495,7 @@
         <v>1161</v>
       </c>
       <c r="E135">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F135" t="s">
         <v>1279</v>
@@ -11530,7 +11530,7 @@
         <v>1161</v>
       </c>
       <c r="E136">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F136" t="s">
         <v>1279</v>
@@ -11565,7 +11565,7 @@
         <v>1162</v>
       </c>
       <c r="E137">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F137" t="s">
         <v>1279</v>
@@ -11600,7 +11600,7 @@
         <v>1162</v>
       </c>
       <c r="E138">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F138" t="s">
         <v>1279</v>
@@ -11635,7 +11635,7 @@
         <v>1162</v>
       </c>
       <c r="E139">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F139" t="s">
         <v>1279</v>
@@ -11670,7 +11670,7 @@
         <v>1162</v>
       </c>
       <c r="E140">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F140" t="s">
         <v>1279</v>
@@ -11705,7 +11705,7 @@
         <v>1162</v>
       </c>
       <c r="E141">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F141" t="s">
         <v>1279</v>
@@ -11740,7 +11740,7 @@
         <v>1162</v>
       </c>
       <c r="E142">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F142" t="s">
         <v>1279</v>
@@ -11775,7 +11775,7 @@
         <v>1162</v>
       </c>
       <c r="E143">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F143" t="s">
         <v>1279</v>
@@ -11810,7 +11810,7 @@
         <v>1162</v>
       </c>
       <c r="E144">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F144" t="s">
         <v>1279</v>
@@ -11845,7 +11845,7 @@
         <v>1162</v>
       </c>
       <c r="E145">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F145" t="s">
         <v>1279</v>
@@ -11880,7 +11880,7 @@
         <v>1163</v>
       </c>
       <c r="E146">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F146" t="s">
         <v>1279</v>
@@ -11915,7 +11915,7 @@
         <v>1163</v>
       </c>
       <c r="E147">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F147" t="s">
         <v>1279</v>
@@ -11950,7 +11950,7 @@
         <v>1163</v>
       </c>
       <c r="E148">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F148" t="s">
         <v>1279</v>
@@ -11985,7 +11985,7 @@
         <v>1164</v>
       </c>
       <c r="E149">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F149" t="s">
         <v>1279</v>
@@ -12020,7 +12020,7 @@
         <v>1164</v>
       </c>
       <c r="E150">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F150" t="s">
         <v>1280</v>
@@ -12055,7 +12055,7 @@
         <v>1164</v>
       </c>
       <c r="E151">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F151" t="s">
         <v>1279</v>
@@ -12090,7 +12090,7 @@
         <v>1165</v>
       </c>
       <c r="E152">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F152" t="s">
         <v>1279</v>
@@ -12125,7 +12125,7 @@
         <v>1165</v>
       </c>
       <c r="E153">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F153" t="s">
         <v>1279</v>
@@ -12160,7 +12160,7 @@
         <v>1166</v>
       </c>
       <c r="E154">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F154" t="s">
         <v>1279</v>
@@ -12195,7 +12195,7 @@
         <v>1166</v>
       </c>
       <c r="E155">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F155" t="s">
         <v>1279</v>
@@ -12230,7 +12230,7 @@
         <v>1167</v>
       </c>
       <c r="E156">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F156" t="s">
         <v>1279</v>
@@ -12265,7 +12265,7 @@
         <v>1167</v>
       </c>
       <c r="E157">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F157" t="s">
         <v>1279</v>
@@ -12300,7 +12300,7 @@
         <v>1168</v>
       </c>
       <c r="E158">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F158" t="s">
         <v>1279</v>
@@ -12335,7 +12335,7 @@
         <v>1168</v>
       </c>
       <c r="E159">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F159" t="s">
         <v>1279</v>
@@ -12370,7 +12370,7 @@
         <v>1168</v>
       </c>
       <c r="E160">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F160" t="s">
         <v>1279</v>
@@ -12405,7 +12405,7 @@
         <v>1169</v>
       </c>
       <c r="E161">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F161" t="s">
         <v>1279</v>
@@ -12440,7 +12440,7 @@
         <v>1169</v>
       </c>
       <c r="E162">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F162" t="s">
         <v>1279</v>
@@ -12475,7 +12475,7 @@
         <v>1170</v>
       </c>
       <c r="E163">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F163" t="s">
         <v>1279</v>
@@ -12510,7 +12510,7 @@
         <v>1171</v>
       </c>
       <c r="E164">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F164" t="s">
         <v>1279</v>
@@ -12545,7 +12545,7 @@
         <v>1171</v>
       </c>
       <c r="E165">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F165" t="s">
         <v>1279</v>
@@ -12580,7 +12580,7 @@
         <v>1171</v>
       </c>
       <c r="E166">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F166" t="s">
         <v>1279</v>
@@ -12615,7 +12615,7 @@
         <v>1171</v>
       </c>
       <c r="E167">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F167" t="s">
         <v>1279</v>
@@ -12650,7 +12650,7 @@
         <v>1172</v>
       </c>
       <c r="E168">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F168" t="s">
         <v>1279</v>
@@ -12685,7 +12685,7 @@
         <v>1173</v>
       </c>
       <c r="E169">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F169" t="s">
         <v>1279</v>
@@ -12720,7 +12720,7 @@
         <v>1173</v>
       </c>
       <c r="E170">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F170" t="s">
         <v>1279</v>
@@ -12755,7 +12755,7 @@
         <v>1173</v>
       </c>
       <c r="E171">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F171" t="s">
         <v>1279</v>
@@ -12790,7 +12790,7 @@
         <v>1173</v>
       </c>
       <c r="E172">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F172" t="s">
         <v>1279</v>
@@ -12825,7 +12825,7 @@
         <v>1173</v>
       </c>
       <c r="E173">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F173" t="s">
         <v>1279</v>
@@ -12860,7 +12860,7 @@
         <v>1174</v>
       </c>
       <c r="E174">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F174" t="s">
         <v>1279</v>
@@ -12895,7 +12895,7 @@
         <v>1174</v>
       </c>
       <c r="E175">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F175" t="s">
         <v>1279</v>
@@ -12930,7 +12930,7 @@
         <v>1174</v>
       </c>
       <c r="E176">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F176" t="s">
         <v>1279</v>
@@ -12965,7 +12965,7 @@
         <v>1174</v>
       </c>
       <c r="E177">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F177" t="s">
         <v>1279</v>
@@ -13000,7 +13000,7 @@
         <v>1174</v>
       </c>
       <c r="E178">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F178" t="s">
         <v>1279</v>
@@ -13035,7 +13035,7 @@
         <v>1174</v>
       </c>
       <c r="E179">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F179" t="s">
         <v>1279</v>
@@ -13070,7 +13070,7 @@
         <v>1175</v>
       </c>
       <c r="E180">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F180" t="s">
         <v>1279</v>
@@ -13105,7 +13105,7 @@
         <v>1175</v>
       </c>
       <c r="E181">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F181" t="s">
         <v>1279</v>
@@ -13140,7 +13140,7 @@
         <v>1175</v>
       </c>
       <c r="E182">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F182" t="s">
         <v>1279</v>
@@ -13175,7 +13175,7 @@
         <v>1175</v>
       </c>
       <c r="E183">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F183" t="s">
         <v>1279</v>
@@ -13210,7 +13210,7 @@
         <v>1176</v>
       </c>
       <c r="E184">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F184" t="s">
         <v>1279</v>
@@ -13245,7 +13245,7 @@
         <v>1176</v>
       </c>
       <c r="E185">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F185" t="s">
         <v>1279</v>
@@ -13280,7 +13280,7 @@
         <v>1177</v>
       </c>
       <c r="E186">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F186" t="s">
         <v>1279</v>
@@ -13315,7 +13315,7 @@
         <v>1178</v>
       </c>
       <c r="E187">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F187" t="s">
         <v>1279</v>
@@ -13350,7 +13350,7 @@
         <v>1178</v>
       </c>
       <c r="E188">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F188" t="s">
         <v>1279</v>
@@ -13385,7 +13385,7 @@
         <v>1179</v>
       </c>
       <c r="E189">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F189" t="s">
         <v>1279</v>
@@ -13420,7 +13420,7 @@
         <v>1180</v>
       </c>
       <c r="E190">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F190" t="s">
         <v>1279</v>
@@ -13455,7 +13455,7 @@
         <v>1180</v>
       </c>
       <c r="E191">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F191" t="s">
         <v>1279</v>
@@ -13490,7 +13490,7 @@
         <v>1181</v>
       </c>
       <c r="E192">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F192" t="s">
         <v>1279</v>
@@ -13525,7 +13525,7 @@
         <v>1181</v>
       </c>
       <c r="E193">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F193" t="s">
         <v>1279</v>
@@ -13560,7 +13560,7 @@
         <v>1182</v>
       </c>
       <c r="E194">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="F194" t="s">
         <v>1279</v>
@@ -13595,7 +13595,7 @@
         <v>1183</v>
       </c>
       <c r="E195">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F195" t="s">
         <v>1279</v>
@@ -13630,7 +13630,7 @@
         <v>1183</v>
       </c>
       <c r="E196">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F196" t="s">
         <v>1279</v>
@@ -13665,7 +13665,7 @@
         <v>1183</v>
       </c>
       <c r="E197">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F197" t="s">
         <v>1279</v>
@@ -13700,7 +13700,7 @@
         <v>1184</v>
       </c>
       <c r="E198">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F198" t="s">
         <v>1279</v>
@@ -13735,7 +13735,7 @@
         <v>1184</v>
       </c>
       <c r="E199">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F199" t="s">
         <v>1279</v>
@@ -13770,7 +13770,7 @@
         <v>1185</v>
       </c>
       <c r="E200">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F200" t="s">
         <v>1279</v>
@@ -13805,7 +13805,7 @@
         <v>1186</v>
       </c>
       <c r="E201">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F201" t="s">
         <v>1279</v>
@@ -13840,7 +13840,7 @@
         <v>1186</v>
       </c>
       <c r="E202">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F202" t="s">
         <v>1279</v>
@@ -13875,7 +13875,7 @@
         <v>1186</v>
       </c>
       <c r="E203">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F203" t="s">
         <v>1279</v>
@@ -13910,7 +13910,7 @@
         <v>1187</v>
       </c>
       <c r="E204">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F204" t="s">
         <v>1279</v>
@@ -13945,7 +13945,7 @@
         <v>1187</v>
       </c>
       <c r="E205">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F205" t="s">
         <v>1279</v>
@@ -13980,7 +13980,7 @@
         <v>1188</v>
       </c>
       <c r="E206">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F206" t="s">
         <v>1279</v>
@@ -14015,7 +14015,7 @@
         <v>1188</v>
       </c>
       <c r="E207">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F207" t="s">
         <v>1281</v>
@@ -14050,7 +14050,7 @@
         <v>1188</v>
       </c>
       <c r="E208">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F208" t="s">
         <v>1279</v>
@@ -14085,7 +14085,7 @@
         <v>1189</v>
       </c>
       <c r="E209">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F209" t="s">
         <v>1279</v>
@@ -14120,7 +14120,7 @@
         <v>1189</v>
       </c>
       <c r="E210">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F210" t="s">
         <v>1279</v>
@@ -14158,7 +14158,7 @@
         <v>1189</v>
       </c>
       <c r="E211">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F211" t="s">
         <v>1279</v>
@@ -14193,7 +14193,7 @@
         <v>1189</v>
       </c>
       <c r="E212">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F212" t="s">
         <v>1279</v>
@@ -14228,7 +14228,7 @@
         <v>1189</v>
       </c>
       <c r="E213">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F213" t="s">
         <v>1279</v>
@@ -14263,7 +14263,7 @@
         <v>1189</v>
       </c>
       <c r="E214">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F214" t="s">
         <v>1279</v>
@@ -14298,7 +14298,7 @@
         <v>1190</v>
       </c>
       <c r="E215">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F215" t="s">
         <v>1279</v>
@@ -14333,7 +14333,7 @@
         <v>1190</v>
       </c>
       <c r="E216">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F216" t="s">
         <v>1279</v>
@@ -14368,7 +14368,7 @@
         <v>1190</v>
       </c>
       <c r="E217">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F217" t="s">
         <v>1279</v>
@@ -14403,7 +14403,7 @@
         <v>1191</v>
       </c>
       <c r="E218">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F218" t="s">
         <v>1279</v>
@@ -14438,7 +14438,7 @@
         <v>1191</v>
       </c>
       <c r="E219">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F219" t="s">
         <v>1279</v>
@@ -14473,7 +14473,7 @@
         <v>1191</v>
       </c>
       <c r="E220">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F220" t="s">
         <v>1279</v>
@@ -14508,7 +14508,7 @@
         <v>1192</v>
       </c>
       <c r="E221">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F221" t="s">
         <v>1279</v>
@@ -14543,7 +14543,7 @@
         <v>1192</v>
       </c>
       <c r="E222">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F222" t="s">
         <v>1279</v>
@@ -14578,7 +14578,7 @@
         <v>1192</v>
       </c>
       <c r="E223">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F223" t="s">
         <v>1279</v>
@@ -14613,7 +14613,7 @@
         <v>1193</v>
       </c>
       <c r="E224">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F224" t="s">
         <v>1279</v>
@@ -14648,7 +14648,7 @@
         <v>1193</v>
       </c>
       <c r="E225">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F225" t="s">
         <v>1279</v>
@@ -14683,7 +14683,7 @@
         <v>1193</v>
       </c>
       <c r="E226">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F226" t="s">
         <v>1279</v>
@@ -14718,7 +14718,7 @@
         <v>1193</v>
       </c>
       <c r="E227">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F227" t="s">
         <v>1279</v>
@@ -14753,7 +14753,7 @@
         <v>1193</v>
       </c>
       <c r="E228">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F228" t="s">
         <v>1279</v>
@@ -14788,7 +14788,7 @@
         <v>1193</v>
       </c>
       <c r="E229">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F229" t="s">
         <v>1279</v>
@@ -14823,7 +14823,7 @@
         <v>1194</v>
       </c>
       <c r="E230">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F230" t="s">
         <v>1279</v>
@@ -14858,7 +14858,7 @@
         <v>1195</v>
       </c>
       <c r="E231">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F231" t="s">
         <v>1279</v>
@@ -14893,7 +14893,7 @@
         <v>1195</v>
       </c>
       <c r="E232">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F232" t="s">
         <v>1282</v>
@@ -14928,7 +14928,7 @@
         <v>1195</v>
       </c>
       <c r="E233">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F233" t="s">
         <v>1279</v>
@@ -14963,7 +14963,7 @@
         <v>1195</v>
       </c>
       <c r="E234">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F234" t="s">
         <v>1279</v>
@@ -14998,7 +14998,7 @@
         <v>1196</v>
       </c>
       <c r="E235">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F235" t="s">
         <v>1279</v>
@@ -15033,7 +15033,7 @@
         <v>1196</v>
       </c>
       <c r="E236">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F236" t="s">
         <v>1279</v>
@@ -15068,7 +15068,7 @@
         <v>1196</v>
       </c>
       <c r="E237">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F237" t="s">
         <v>1279</v>
@@ -15103,7 +15103,7 @@
         <v>1196</v>
       </c>
       <c r="E238">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F238" t="s">
         <v>1279</v>
@@ -15138,7 +15138,7 @@
         <v>1197</v>
       </c>
       <c r="E239">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F239" t="s">
         <v>1279</v>
@@ -15176,7 +15176,7 @@
         <v>1198</v>
       </c>
       <c r="E240">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F240" t="s">
         <v>1279</v>
@@ -15211,7 +15211,7 @@
         <v>1198</v>
       </c>
       <c r="E241">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F241" t="s">
         <v>1279</v>
@@ -15246,7 +15246,7 @@
         <v>1198</v>
       </c>
       <c r="E242">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F242" t="s">
         <v>1279</v>
@@ -15281,7 +15281,7 @@
         <v>1198</v>
       </c>
       <c r="E243">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F243" t="s">
         <v>1279</v>
@@ -15319,7 +15319,7 @@
         <v>1198</v>
       </c>
       <c r="E244">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F244" t="s">
         <v>1279</v>
@@ -15354,7 +15354,7 @@
         <v>1199</v>
       </c>
       <c r="E245">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F245" t="s">
         <v>1279</v>
@@ -15389,7 +15389,7 @@
         <v>1199</v>
       </c>
       <c r="E246">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F246" t="s">
         <v>1279</v>
@@ -15424,7 +15424,7 @@
         <v>1200</v>
       </c>
       <c r="E247">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F247" t="s">
         <v>1279</v>
@@ -15459,7 +15459,7 @@
         <v>1200</v>
       </c>
       <c r="E248">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F248" t="s">
         <v>1279</v>
@@ -15494,7 +15494,7 @@
         <v>1200</v>
       </c>
       <c r="E249">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F249" t="s">
         <v>1279</v>
@@ -15529,7 +15529,7 @@
         <v>1201</v>
       </c>
       <c r="E250">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F250" t="s">
         <v>1279</v>
@@ -15564,7 +15564,7 @@
         <v>1201</v>
       </c>
       <c r="E251">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F251" t="s">
         <v>1279</v>
@@ -15599,7 +15599,7 @@
         <v>1202</v>
       </c>
       <c r="E252">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F252" t="s">
         <v>1279</v>
@@ -15634,7 +15634,7 @@
         <v>1203</v>
       </c>
       <c r="E253">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F253" t="s">
         <v>1279</v>
@@ -15669,7 +15669,7 @@
         <v>1203</v>
       </c>
       <c r="E254">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F254" t="s">
         <v>1279</v>
@@ -15704,7 +15704,7 @@
         <v>1203</v>
       </c>
       <c r="E255">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F255" t="s">
         <v>1279</v>
@@ -15739,7 +15739,7 @@
         <v>1203</v>
       </c>
       <c r="E256">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F256" t="s">
         <v>1279</v>
@@ -15774,7 +15774,7 @@
         <v>1204</v>
       </c>
       <c r="E257">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F257" t="s">
         <v>1279</v>
@@ -15809,7 +15809,7 @@
         <v>1204</v>
       </c>
       <c r="E258">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F258" t="s">
         <v>1279</v>
@@ -15844,7 +15844,7 @@
         <v>1204</v>
       </c>
       <c r="E259">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F259" t="s">
         <v>1279</v>
@@ -15879,7 +15879,7 @@
         <v>1205</v>
       </c>
       <c r="E260">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F260" t="s">
         <v>1279</v>
@@ -15914,7 +15914,7 @@
         <v>1206</v>
       </c>
       <c r="E261">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F261" t="s">
         <v>1279</v>
@@ -15949,7 +15949,7 @@
         <v>1206</v>
       </c>
       <c r="E262">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F262" t="s">
         <v>1279</v>
@@ -15984,7 +15984,7 @@
         <v>1206</v>
       </c>
       <c r="E263">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F263" t="s">
         <v>1279</v>
@@ -16019,7 +16019,7 @@
         <v>1207</v>
       </c>
       <c r="E264">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F264" t="s">
         <v>1279</v>
@@ -16054,7 +16054,7 @@
         <v>1207</v>
       </c>
       <c r="E265">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F265" t="s">
         <v>1279</v>
@@ -16089,7 +16089,7 @@
         <v>1207</v>
       </c>
       <c r="E266">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F266" t="s">
         <v>1279</v>
@@ -16124,7 +16124,7 @@
         <v>1208</v>
       </c>
       <c r="E267">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F267" t="s">
         <v>1279</v>
@@ -16159,7 +16159,7 @@
         <v>1209</v>
       </c>
       <c r="E268">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F268" t="s">
         <v>1279</v>
@@ -16194,7 +16194,7 @@
         <v>1210</v>
       </c>
       <c r="E269">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F269" t="s">
         <v>1279</v>
@@ -16229,7 +16229,7 @@
         <v>1210</v>
       </c>
       <c r="E270">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F270" t="s">
         <v>1279</v>
@@ -16264,7 +16264,7 @@
         <v>1210</v>
       </c>
       <c r="E271">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F271" t="s">
         <v>1279</v>
@@ -16299,7 +16299,7 @@
         <v>1210</v>
       </c>
       <c r="E272">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F272" t="s">
         <v>1279</v>
@@ -16334,7 +16334,7 @@
         <v>1211</v>
       </c>
       <c r="E273">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F273" t="s">
         <v>1279</v>
@@ -16369,7 +16369,7 @@
         <v>1212</v>
       </c>
       <c r="E274">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F274" t="s">
         <v>1279</v>
@@ -16404,7 +16404,7 @@
         <v>1212</v>
       </c>
       <c r="E275">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F275" t="s">
         <v>1279</v>
@@ -16439,7 +16439,7 @@
         <v>1213</v>
       </c>
       <c r="E276">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F276" t="s">
         <v>1279</v>
@@ -16474,7 +16474,7 @@
         <v>1214</v>
       </c>
       <c r="E277">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F277" t="s">
         <v>1279</v>
@@ -16509,7 +16509,7 @@
         <v>1215</v>
       </c>
       <c r="E278">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F278" t="s">
         <v>1279</v>
@@ -16544,7 +16544,7 @@
         <v>1215</v>
       </c>
       <c r="E279">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F279" t="s">
         <v>1279</v>
@@ -16579,7 +16579,7 @@
         <v>1216</v>
       </c>
       <c r="E280">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F280" t="s">
         <v>1279</v>
@@ -16614,7 +16614,7 @@
         <v>1216</v>
       </c>
       <c r="E281">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F281" t="s">
         <v>1279</v>
@@ -16649,7 +16649,7 @@
         <v>1216</v>
       </c>
       <c r="E282">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F282" t="s">
         <v>1279</v>
@@ -16684,7 +16684,7 @@
         <v>1217</v>
       </c>
       <c r="E283">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F283" t="s">
         <v>1279</v>
@@ -16719,7 +16719,7 @@
         <v>1217</v>
       </c>
       <c r="E284">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F284" t="s">
         <v>1279</v>
@@ -16754,7 +16754,7 @@
         <v>1217</v>
       </c>
       <c r="E285">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F285" t="s">
         <v>1279</v>
@@ -16789,7 +16789,7 @@
         <v>1217</v>
       </c>
       <c r="E286">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F286" t="s">
         <v>1279</v>
@@ -16824,7 +16824,7 @@
         <v>1217</v>
       </c>
       <c r="E287">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F287" t="s">
         <v>1279</v>
@@ -16859,7 +16859,7 @@
         <v>1217</v>
       </c>
       <c r="E288">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F288" t="s">
         <v>1279</v>
@@ -16894,7 +16894,7 @@
         <v>1217</v>
       </c>
       <c r="E289">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F289" t="s">
         <v>1279</v>
@@ -16929,7 +16929,7 @@
         <v>1217</v>
       </c>
       <c r="E290">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F290" t="s">
         <v>1279</v>
@@ -16964,7 +16964,7 @@
         <v>1218</v>
       </c>
       <c r="E291">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F291" t="s">
         <v>1279</v>
@@ -16999,7 +16999,7 @@
         <v>1218</v>
       </c>
       <c r="E292">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F292" t="s">
         <v>1279</v>
@@ -17034,7 +17034,7 @@
         <v>1218</v>
       </c>
       <c r="E293">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F293" t="s">
         <v>1279</v>
@@ -17069,7 +17069,7 @@
         <v>1219</v>
       </c>
       <c r="E294">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F294" t="s">
         <v>1279</v>
@@ -17104,7 +17104,7 @@
         <v>1220</v>
       </c>
       <c r="E295">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F295" t="s">
         <v>1279</v>
@@ -17139,7 +17139,7 @@
         <v>1220</v>
       </c>
       <c r="E296">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F296" t="s">
         <v>1279</v>
@@ -17174,7 +17174,7 @@
         <v>1220</v>
       </c>
       <c r="E297">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F297" t="s">
         <v>1279</v>
@@ -17209,7 +17209,7 @@
         <v>1220</v>
       </c>
       <c r="E298">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F298" t="s">
         <v>1283</v>
@@ -17247,7 +17247,7 @@
         <v>1220</v>
       </c>
       <c r="E299">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F299" t="s">
         <v>1279</v>
@@ -17282,7 +17282,7 @@
         <v>1220</v>
       </c>
       <c r="E300">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F300" t="s">
         <v>1279</v>
@@ -17317,7 +17317,7 @@
         <v>1221</v>
       </c>
       <c r="E301">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F301" t="s">
         <v>1279</v>
@@ -17352,7 +17352,7 @@
         <v>1221</v>
       </c>
       <c r="E302">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F302" t="s">
         <v>1279</v>
@@ -17387,7 +17387,7 @@
         <v>1221</v>
       </c>
       <c r="E303">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F303" t="s">
         <v>1279</v>
@@ -17425,7 +17425,7 @@
         <v>1221</v>
       </c>
       <c r="E304">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F304" t="s">
         <v>1279</v>
@@ -17460,7 +17460,7 @@
         <v>1221</v>
       </c>
       <c r="E305">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F305" t="s">
         <v>1279</v>
@@ -17495,7 +17495,7 @@
         <v>1221</v>
       </c>
       <c r="E306">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F306" t="s">
         <v>1279</v>
@@ -17530,7 +17530,7 @@
         <v>1221</v>
       </c>
       <c r="E307">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F307" t="s">
         <v>1279</v>
@@ -17565,7 +17565,7 @@
         <v>1221</v>
       </c>
       <c r="E308">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F308" t="s">
         <v>1279</v>
@@ -17600,7 +17600,7 @@
         <v>1222</v>
       </c>
       <c r="E309">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F309" t="s">
         <v>1280</v>
@@ -17635,7 +17635,7 @@
         <v>1223</v>
       </c>
       <c r="E310">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F310" t="s">
         <v>1283</v>
@@ -17670,7 +17670,7 @@
         <v>1224</v>
       </c>
       <c r="E311">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F311" t="s">
         <v>1279</v>
@@ -17705,7 +17705,7 @@
         <v>1224</v>
       </c>
       <c r="E312">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F312" t="s">
         <v>1279</v>
@@ -17740,7 +17740,7 @@
         <v>1225</v>
       </c>
       <c r="E313">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F313" t="s">
         <v>1279</v>
@@ -17775,7 +17775,7 @@
         <v>1226</v>
       </c>
       <c r="E314">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F314" t="s">
         <v>1282</v>
@@ -17810,7 +17810,7 @@
         <v>1226</v>
       </c>
       <c r="E315">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F315" t="s">
         <v>1279</v>
@@ -17845,7 +17845,7 @@
         <v>1226</v>
       </c>
       <c r="E316">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F316" t="s">
         <v>1279</v>
@@ -17880,7 +17880,7 @@
         <v>1226</v>
       </c>
       <c r="E317">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F317" t="s">
         <v>1279</v>
@@ -17915,7 +17915,7 @@
         <v>1227</v>
       </c>
       <c r="E318">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F318" t="s">
         <v>1279</v>
@@ -17950,7 +17950,7 @@
         <v>1228</v>
       </c>
       <c r="E319">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F319" t="s">
         <v>1279</v>
@@ -17985,7 +17985,7 @@
         <v>1228</v>
       </c>
       <c r="E320">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F320" t="s">
         <v>1279</v>
@@ -18020,7 +18020,7 @@
         <v>1229</v>
       </c>
       <c r="E321">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F321" t="s">
         <v>1279</v>
@@ -18055,7 +18055,7 @@
         <v>1230</v>
       </c>
       <c r="E322">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F322" t="s">
         <v>1279</v>
@@ -18090,7 +18090,7 @@
         <v>1230</v>
       </c>
       <c r="E323">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F323" t="s">
         <v>1279</v>
@@ -18125,7 +18125,7 @@
         <v>1230</v>
       </c>
       <c r="E324">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F324" t="s">
         <v>1279</v>
@@ -18160,7 +18160,7 @@
         <v>1230</v>
       </c>
       <c r="E325">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F325" t="s">
         <v>1279</v>
@@ -18195,7 +18195,7 @@
         <v>1230</v>
       </c>
       <c r="E326">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F326" t="s">
         <v>1279</v>
@@ -18230,7 +18230,7 @@
         <v>1230</v>
       </c>
       <c r="E327">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F327" t="s">
         <v>1279</v>
@@ -18265,7 +18265,7 @@
         <v>1230</v>
       </c>
       <c r="E328">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F328" t="s">
         <v>1279</v>
@@ -18300,7 +18300,7 @@
         <v>1231</v>
       </c>
       <c r="E329">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F329" t="s">
         <v>1279</v>
@@ -18335,7 +18335,7 @@
         <v>1231</v>
       </c>
       <c r="E330">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F330" t="s">
         <v>1279</v>
@@ -18370,7 +18370,7 @@
         <v>1231</v>
       </c>
       <c r="E331">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F331" t="s">
         <v>1280</v>
@@ -18405,7 +18405,7 @@
         <v>1232</v>
       </c>
       <c r="E332">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F332" t="s">
         <v>1279</v>
@@ -18440,7 +18440,7 @@
         <v>1232</v>
       </c>
       <c r="E333">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F333" t="s">
         <v>1279</v>
@@ -18475,7 +18475,7 @@
         <v>1232</v>
       </c>
       <c r="E334">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F334" t="s">
         <v>1279</v>
@@ -18510,7 +18510,7 @@
         <v>1232</v>
       </c>
       <c r="E335">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F335" t="s">
         <v>1279</v>
@@ -18545,7 +18545,7 @@
         <v>1232</v>
       </c>
       <c r="E336">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F336" t="s">
         <v>1279</v>
@@ -18580,7 +18580,7 @@
         <v>1232</v>
       </c>
       <c r="E337">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F337" t="s">
         <v>1282</v>
@@ -18615,7 +18615,7 @@
         <v>1233</v>
       </c>
       <c r="E338">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F338" t="s">
         <v>1279</v>
@@ -18650,7 +18650,7 @@
         <v>1233</v>
       </c>
       <c r="E339">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F339" t="s">
         <v>1279</v>
@@ -18685,7 +18685,7 @@
         <v>1233</v>
       </c>
       <c r="E340">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F340" t="s">
         <v>1279</v>
@@ -18720,7 +18720,7 @@
         <v>1234</v>
       </c>
       <c r="E341">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F341" t="s">
         <v>1282</v>
@@ -18755,7 +18755,7 @@
         <v>1234</v>
       </c>
       <c r="E342">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F342" t="s">
         <v>1279</v>
@@ -18790,7 +18790,7 @@
         <v>1234</v>
       </c>
       <c r="E343">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F343" t="s">
         <v>1279</v>
@@ -18825,7 +18825,7 @@
         <v>1235</v>
       </c>
       <c r="E344">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F344" t="s">
         <v>1279</v>
@@ -18860,7 +18860,7 @@
         <v>1235</v>
       </c>
       <c r="E345">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F345" t="s">
         <v>1279</v>
@@ -18895,7 +18895,7 @@
         <v>1235</v>
       </c>
       <c r="E346">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F346" t="s">
         <v>1279</v>
@@ -18930,7 +18930,7 @@
         <v>1235</v>
       </c>
       <c r="E347">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F347" t="s">
         <v>1279</v>
@@ -18965,7 +18965,7 @@
         <v>1235</v>
       </c>
       <c r="E348">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F348" t="s">
         <v>1281</v>
@@ -19000,7 +19000,7 @@
         <v>1235</v>
       </c>
       <c r="E349">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F349" t="s">
         <v>1279</v>
@@ -19035,7 +19035,7 @@
         <v>1236</v>
       </c>
       <c r="E350">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F350" t="s">
         <v>1279</v>
@@ -19070,7 +19070,7 @@
         <v>1236</v>
       </c>
       <c r="E351">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F351" t="s">
         <v>1279</v>
@@ -19105,7 +19105,7 @@
         <v>1236</v>
       </c>
       <c r="E352">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F352" t="s">
         <v>1279</v>
@@ -19140,7 +19140,7 @@
         <v>1236</v>
       </c>
       <c r="E353">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F353" t="s">
         <v>1279</v>
@@ -19175,7 +19175,7 @@
         <v>1237</v>
       </c>
       <c r="E354">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F354" t="s">
         <v>1279</v>
@@ -19210,7 +19210,7 @@
         <v>1237</v>
       </c>
       <c r="E355">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F355" t="s">
         <v>1279</v>
@@ -19245,7 +19245,7 @@
         <v>1237</v>
       </c>
       <c r="E356">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F356" t="s">
         <v>1279</v>
@@ -19280,7 +19280,7 @@
         <v>1237</v>
       </c>
       <c r="E357">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F357" t="s">
         <v>1279</v>
@@ -19315,7 +19315,7 @@
         <v>1237</v>
       </c>
       <c r="E358">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F358" t="s">
         <v>1279</v>
@@ -19353,7 +19353,7 @@
         <v>1238</v>
       </c>
       <c r="E359">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F359" t="s">
         <v>1279</v>
@@ -19388,7 +19388,7 @@
         <v>1238</v>
       </c>
       <c r="E360">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F360" t="s">
         <v>1279</v>
@@ -19423,7 +19423,7 @@
         <v>1238</v>
       </c>
       <c r="E361">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F361" t="s">
         <v>1279</v>
@@ -19458,7 +19458,7 @@
         <v>1238</v>
       </c>
       <c r="E362">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F362" t="s">
         <v>1279</v>
@@ -19493,7 +19493,7 @@
         <v>1238</v>
       </c>
       <c r="E363">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F363" t="s">
         <v>1279</v>
@@ -19528,7 +19528,7 @@
         <v>1238</v>
       </c>
       <c r="E364">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F364" t="s">
         <v>1279</v>
@@ -19563,7 +19563,7 @@
         <v>1239</v>
       </c>
       <c r="E365">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F365" t="s">
         <v>1280</v>
@@ -19598,7 +19598,7 @@
         <v>1240</v>
       </c>
       <c r="E366">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F366" t="s">
         <v>1279</v>
@@ -19633,7 +19633,7 @@
         <v>1241</v>
       </c>
       <c r="E367">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F367" t="s">
         <v>1281</v>
@@ -19671,7 +19671,7 @@
         <v>1242</v>
       </c>
       <c r="E368">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F368" t="s">
         <v>1279</v>
@@ -19706,7 +19706,7 @@
         <v>1242</v>
       </c>
       <c r="E369">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F369" t="s">
         <v>1279</v>
@@ -19741,7 +19741,7 @@
         <v>1242</v>
       </c>
       <c r="E370">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F370" t="s">
         <v>1279</v>
@@ -19776,7 +19776,7 @@
         <v>1243</v>
       </c>
       <c r="E371">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F371" t="s">
         <v>1279</v>
@@ -19811,7 +19811,7 @@
         <v>1243</v>
       </c>
       <c r="E372">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F372" t="s">
         <v>1279</v>
@@ -19846,7 +19846,7 @@
         <v>1244</v>
       </c>
       <c r="E373">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F373" t="s">
         <v>1279</v>
@@ -19881,7 +19881,7 @@
         <v>1244</v>
       </c>
       <c r="E374">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F374" t="s">
         <v>1283</v>
@@ -19919,7 +19919,7 @@
         <v>1244</v>
       </c>
       <c r="E375">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F375" t="s">
         <v>1279</v>
@@ -19954,7 +19954,7 @@
         <v>1244</v>
       </c>
       <c r="E376">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F376" t="s">
         <v>1283</v>
@@ -19989,7 +19989,7 @@
         <v>1245</v>
       </c>
       <c r="E377">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F377" t="s">
         <v>1279</v>
@@ -20024,7 +20024,7 @@
         <v>1246</v>
       </c>
       <c r="E378">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F378" t="s">
         <v>1279</v>
@@ -20059,7 +20059,7 @@
         <v>1246</v>
       </c>
       <c r="E379">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F379" t="s">
         <v>1279</v>
@@ -20094,7 +20094,7 @@
         <v>1246</v>
       </c>
       <c r="E380">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F380" t="s">
         <v>1279</v>
@@ -20129,7 +20129,7 @@
         <v>1246</v>
       </c>
       <c r="E381">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F381" t="s">
         <v>1279</v>
@@ -20164,7 +20164,7 @@
         <v>1247</v>
       </c>
       <c r="E382">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F382" t="s">
         <v>1283</v>
@@ -20199,7 +20199,7 @@
         <v>1247</v>
       </c>
       <c r="E383">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F383" t="s">
         <v>1279</v>
@@ -20234,7 +20234,7 @@
         <v>1247</v>
       </c>
       <c r="E384">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F384" t="s">
         <v>1279</v>
@@ -20269,7 +20269,7 @@
         <v>1248</v>
       </c>
       <c r="E385">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F385" t="s">
         <v>1279</v>
@@ -20304,7 +20304,7 @@
         <v>1249</v>
       </c>
       <c r="E386">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F386" t="s">
         <v>1279</v>
@@ -20339,7 +20339,7 @@
         <v>1249</v>
       </c>
       <c r="E387">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F387" t="s">
         <v>1279</v>
@@ -20374,7 +20374,7 @@
         <v>1250</v>
       </c>
       <c r="E388">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F388" t="s">
         <v>1279</v>
@@ -20409,7 +20409,7 @@
         <v>1250</v>
       </c>
       <c r="E389">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F389" t="s">
         <v>1279</v>
@@ -20444,7 +20444,7 @@
         <v>1250</v>
       </c>
       <c r="E390">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F390" t="s">
         <v>1279</v>
@@ -20479,7 +20479,7 @@
         <v>1250</v>
       </c>
       <c r="E391">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F391" t="s">
         <v>1279</v>
@@ -20514,7 +20514,7 @@
         <v>1250</v>
       </c>
       <c r="E392">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F392" t="s">
         <v>1279</v>
@@ -20549,7 +20549,7 @@
         <v>1250</v>
       </c>
       <c r="E393">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F393" t="s">
         <v>1279</v>
@@ -20584,7 +20584,7 @@
         <v>1250</v>
       </c>
       <c r="E394">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F394" t="s">
         <v>1279</v>
@@ -20619,7 +20619,7 @@
         <v>1250</v>
       </c>
       <c r="E395">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F395" t="s">
         <v>1279</v>
@@ -20654,7 +20654,7 @@
         <v>1250</v>
       </c>
       <c r="E396">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F396" t="s">
         <v>1279</v>
@@ -20689,7 +20689,7 @@
         <v>1250</v>
       </c>
       <c r="E397">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F397" t="s">
         <v>1279</v>
@@ -20724,7 +20724,7 @@
         <v>1250</v>
       </c>
       <c r="E398">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F398" t="s">
         <v>1279</v>
@@ -20759,7 +20759,7 @@
         <v>1250</v>
       </c>
       <c r="E399">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F399" t="s">
         <v>1279</v>
@@ -20794,7 +20794,7 @@
         <v>1250</v>
       </c>
       <c r="E400">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F400" t="s">
         <v>1279</v>
@@ -20829,7 +20829,7 @@
         <v>1250</v>
       </c>
       <c r="E401">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F401" t="s">
         <v>1279</v>
@@ -20864,7 +20864,7 @@
         <v>1250</v>
       </c>
       <c r="E402">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F402" t="s">
         <v>1279</v>
@@ -20899,7 +20899,7 @@
         <v>1250</v>
       </c>
       <c r="E403">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F403" t="s">
         <v>1279</v>
@@ -20934,7 +20934,7 @@
         <v>1250</v>
       </c>
       <c r="E404">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F404" t="s">
         <v>1279</v>
@@ -20969,7 +20969,7 @@
         <v>1250</v>
       </c>
       <c r="E405">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F405" t="s">
         <v>1279</v>
@@ -21004,7 +21004,7 @@
         <v>1250</v>
       </c>
       <c r="E406">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F406" t="s">
         <v>1279</v>
@@ -21039,7 +21039,7 @@
         <v>1250</v>
       </c>
       <c r="E407">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F407" t="s">
         <v>1279</v>
@@ -21074,7 +21074,7 @@
         <v>1250</v>
       </c>
       <c r="E408">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F408" t="s">
         <v>1279</v>
@@ -21109,7 +21109,7 @@
         <v>1250</v>
       </c>
       <c r="E409">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F409" t="s">
         <v>1279</v>
@@ -21144,7 +21144,7 @@
         <v>1251</v>
       </c>
       <c r="E410">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F410" t="s">
         <v>1279</v>
@@ -21179,7 +21179,7 @@
         <v>1251</v>
       </c>
       <c r="E411">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F411" t="s">
         <v>1279</v>
@@ -21214,7 +21214,7 @@
         <v>1251</v>
       </c>
       <c r="E412">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F412" t="s">
         <v>1283</v>
@@ -21249,7 +21249,7 @@
         <v>1252</v>
       </c>
       <c r="E413">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F413" t="s">
         <v>1279</v>
@@ -21284,7 +21284,7 @@
         <v>1253</v>
       </c>
       <c r="E414">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F414" t="s">
         <v>1281</v>
@@ -21322,7 +21322,7 @@
         <v>1253</v>
       </c>
       <c r="E415">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F415" t="s">
         <v>1279</v>
@@ -21357,7 +21357,7 @@
         <v>1253</v>
       </c>
       <c r="E416">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F416" t="s">
         <v>1279</v>
@@ -21392,7 +21392,7 @@
         <v>1253</v>
       </c>
       <c r="E417">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F417" t="s">
         <v>1279</v>
@@ -21427,7 +21427,7 @@
         <v>1254</v>
       </c>
       <c r="E418">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F418" t="s">
         <v>1279</v>
@@ -21465,7 +21465,7 @@
         <v>1254</v>
       </c>
       <c r="E419">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F419" t="s">
         <v>1283</v>
@@ -21500,7 +21500,7 @@
         <v>1254</v>
       </c>
       <c r="E420">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F420" t="s">
         <v>1281</v>
@@ -21535,7 +21535,7 @@
         <v>1254</v>
       </c>
       <c r="E421">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F421" t="s">
         <v>1279</v>
@@ -21570,7 +21570,7 @@
         <v>1254</v>
       </c>
       <c r="E422">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F422" t="s">
         <v>1279</v>
@@ -21605,7 +21605,7 @@
         <v>1254</v>
       </c>
       <c r="E423">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F423" t="s">
         <v>1279</v>
@@ -21640,7 +21640,7 @@
         <v>1254</v>
       </c>
       <c r="E424">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F424" t="s">
         <v>1279</v>
@@ -21675,7 +21675,7 @@
         <v>1255</v>
       </c>
       <c r="E425">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F425" t="s">
         <v>1283</v>
@@ -21713,7 +21713,7 @@
         <v>1256</v>
       </c>
       <c r="E426">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F426" t="s">
         <v>1279</v>
@@ -21748,7 +21748,7 @@
         <v>1256</v>
       </c>
       <c r="E427">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F427" t="s">
         <v>1279</v>
@@ -21783,7 +21783,7 @@
         <v>1256</v>
       </c>
       <c r="E428">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F428" t="s">
         <v>1279</v>
@@ -21818,7 +21818,7 @@
         <v>1257</v>
       </c>
       <c r="E429">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F429" t="s">
         <v>1279</v>
@@ -21853,7 +21853,7 @@
         <v>1257</v>
       </c>
       <c r="E430">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F430" t="s">
         <v>1279</v>
@@ -21888,7 +21888,7 @@
         <v>1257</v>
       </c>
       <c r="E431">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F431" t="s">
         <v>1279</v>
@@ -21923,7 +21923,7 @@
         <v>1257</v>
       </c>
       <c r="E432">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F432" t="s">
         <v>1281</v>
@@ -21958,7 +21958,7 @@
         <v>1257</v>
       </c>
       <c r="E433">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F433" t="s">
         <v>1279</v>
@@ -21993,7 +21993,7 @@
         <v>1258</v>
       </c>
       <c r="E434">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F434" t="s">
         <v>1279</v>
@@ -22028,7 +22028,7 @@
         <v>1258</v>
       </c>
       <c r="E435">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F435" t="s">
         <v>1279</v>
@@ -22063,7 +22063,7 @@
         <v>1258</v>
       </c>
       <c r="E436">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F436" t="s">
         <v>1279</v>
@@ -22098,7 +22098,7 @@
         <v>1258</v>
       </c>
       <c r="E437">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F437" t="s">
         <v>1279</v>
@@ -22133,7 +22133,7 @@
         <v>1258</v>
       </c>
       <c r="E438">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F438" t="s">
         <v>1279</v>
@@ -22171,7 +22171,7 @@
         <v>1258</v>
       </c>
       <c r="E439">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F439" t="s">
         <v>1281</v>
@@ -22209,7 +22209,7 @@
         <v>1258</v>
       </c>
       <c r="E440">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F440" t="s">
         <v>1281</v>
@@ -22244,7 +22244,7 @@
         <v>1259</v>
       </c>
       <c r="E441">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F441" t="s">
         <v>1279</v>
@@ -22279,7 +22279,7 @@
         <v>1259</v>
       </c>
       <c r="E442">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F442" t="s">
         <v>1279</v>
@@ -22314,7 +22314,7 @@
         <v>1259</v>
       </c>
       <c r="E443">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F443" t="s">
         <v>1279</v>
@@ -22349,7 +22349,7 @@
         <v>1260</v>
       </c>
       <c r="E444">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F444" t="s">
         <v>1279</v>
@@ -22384,7 +22384,7 @@
         <v>1260</v>
       </c>
       <c r="E445">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F445" t="s">
         <v>1279</v>
@@ -22419,7 +22419,7 @@
         <v>1260</v>
       </c>
       <c r="E446">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F446" t="s">
         <v>1281</v>
@@ -22457,7 +22457,7 @@
         <v>1260</v>
       </c>
       <c r="E447">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F447" t="s">
         <v>1279</v>
@@ -22492,7 +22492,7 @@
         <v>1261</v>
       </c>
       <c r="E448">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F448" t="s">
         <v>1279</v>
@@ -22527,7 +22527,7 @@
         <v>1261</v>
       </c>
       <c r="E449">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F449" t="s">
         <v>1279</v>
@@ -22562,7 +22562,7 @@
         <v>1262</v>
       </c>
       <c r="E450">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F450" t="s">
         <v>1281</v>
@@ -22600,7 +22600,7 @@
         <v>1262</v>
       </c>
       <c r="E451">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F451" t="s">
         <v>1279</v>
@@ -22635,7 +22635,7 @@
         <v>1262</v>
       </c>
       <c r="E452">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F452" t="s">
         <v>1279</v>
@@ -22670,7 +22670,7 @@
         <v>1263</v>
       </c>
       <c r="E453">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F453" t="s">
         <v>1281</v>
@@ -22705,7 +22705,7 @@
         <v>1263</v>
       </c>
       <c r="E454">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F454" t="s">
         <v>1279</v>
@@ -22740,7 +22740,7 @@
         <v>1263</v>
       </c>
       <c r="E455">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F455" t="s">
         <v>1281</v>
@@ -22778,7 +22778,7 @@
         <v>1263</v>
       </c>
       <c r="E456">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F456" t="s">
         <v>1279</v>
@@ -22813,7 +22813,7 @@
         <v>1263</v>
       </c>
       <c r="E457">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F457" t="s">
         <v>1279</v>
@@ -22848,7 +22848,7 @@
         <v>1264</v>
       </c>
       <c r="E458">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F458" t="s">
         <v>1279</v>
@@ -22883,7 +22883,7 @@
         <v>1264</v>
       </c>
       <c r="E459">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F459" t="s">
         <v>1279</v>
@@ -22918,7 +22918,7 @@
         <v>1265</v>
       </c>
       <c r="E460">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F460" t="s">
         <v>1279</v>
@@ -22953,7 +22953,7 @@
         <v>1265</v>
       </c>
       <c r="E461">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F461" t="s">
         <v>1279</v>
@@ -22988,7 +22988,7 @@
         <v>1265</v>
       </c>
       <c r="E462">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F462" t="s">
         <v>1279</v>
@@ -23023,7 +23023,7 @@
         <v>1265</v>
       </c>
       <c r="E463">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F463" t="s">
         <v>1281</v>
@@ -23061,7 +23061,7 @@
         <v>1266</v>
       </c>
       <c r="E464">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F464" t="s">
         <v>1279</v>
@@ -23096,7 +23096,7 @@
         <v>1266</v>
       </c>
       <c r="E465">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F465" t="s">
         <v>1283</v>
@@ -23134,7 +23134,7 @@
         <v>1266</v>
       </c>
       <c r="E466">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F466" t="s">
         <v>1279</v>
@@ -23169,7 +23169,7 @@
         <v>1266</v>
       </c>
       <c r="E467">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F467" t="s">
         <v>1279</v>
@@ -23204,7 +23204,7 @@
         <v>1267</v>
       </c>
       <c r="E468">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F468" t="s">
         <v>1279</v>
@@ -23239,7 +23239,7 @@
         <v>1267</v>
       </c>
       <c r="E469">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F469" t="s">
         <v>1279</v>
@@ -23274,7 +23274,7 @@
         <v>1267</v>
       </c>
       <c r="E470">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F470" t="s">
         <v>1279</v>
@@ -23309,7 +23309,7 @@
         <v>1267</v>
       </c>
       <c r="E471">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F471" t="s">
         <v>1279</v>
@@ -23344,7 +23344,7 @@
         <v>1267</v>
       </c>
       <c r="E472">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F472" t="s">
         <v>1279</v>
@@ -23379,7 +23379,7 @@
         <v>1267</v>
       </c>
       <c r="E473">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F473" t="s">
         <v>1281</v>
@@ -23417,7 +23417,7 @@
         <v>1268</v>
       </c>
       <c r="E474">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F474" t="s">
         <v>1279</v>
@@ -23452,7 +23452,7 @@
         <v>1268</v>
       </c>
       <c r="E475">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F475" t="s">
         <v>1281</v>
@@ -23487,7 +23487,7 @@
         <v>1269</v>
       </c>
       <c r="E476">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F476" t="s">
         <v>1281</v>
@@ -23525,7 +23525,7 @@
         <v>1269</v>
       </c>
       <c r="E477">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F477" t="s">
         <v>1281</v>
@@ -23563,7 +23563,7 @@
         <v>1269</v>
       </c>
       <c r="E478">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F478" t="s">
         <v>1279</v>
@@ -23598,7 +23598,7 @@
         <v>1269</v>
       </c>
       <c r="E479">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F479" t="s">
         <v>1279</v>
@@ -23633,7 +23633,7 @@
         <v>1270</v>
       </c>
       <c r="E480">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F480" t="s">
         <v>1279</v>
@@ -23668,7 +23668,7 @@
         <v>1271</v>
       </c>
       <c r="E481">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F481" t="s">
         <v>1279</v>
@@ -23703,7 +23703,7 @@
         <v>1271</v>
       </c>
       <c r="E482">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F482" t="s">
         <v>1279</v>
@@ -23738,7 +23738,7 @@
         <v>1271</v>
       </c>
       <c r="E483">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F483" t="s">
         <v>1279</v>
@@ -23773,7 +23773,7 @@
         <v>1271</v>
       </c>
       <c r="E484">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F484" t="s">
         <v>1279</v>
@@ -23808,7 +23808,7 @@
         <v>1271</v>
       </c>
       <c r="E485">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F485" t="s">
         <v>1279</v>
@@ -23843,7 +23843,7 @@
         <v>1271</v>
       </c>
       <c r="E486">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F486" t="s">
         <v>1279</v>
@@ -23878,7 +23878,7 @@
         <v>1271</v>
       </c>
       <c r="E487">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F487" t="s">
         <v>1279</v>
@@ -23913,7 +23913,7 @@
         <v>1271</v>
       </c>
       <c r="E488">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F488" t="s">
         <v>1281</v>
@@ -23951,7 +23951,7 @@
         <v>1272</v>
       </c>
       <c r="E489">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F489" t="s">
         <v>1279</v>
@@ -23986,7 +23986,7 @@
         <v>1272</v>
       </c>
       <c r="E490">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F490" t="s">
         <v>1279</v>
@@ -24021,7 +24021,7 @@
         <v>1272</v>
       </c>
       <c r="E491">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F491" t="s">
         <v>1279</v>
@@ -24056,7 +24056,7 @@
         <v>1272</v>
       </c>
       <c r="E492">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F492" t="s">
         <v>1281</v>
@@ -24094,7 +24094,7 @@
         <v>1272</v>
       </c>
       <c r="E493">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F493" t="s">
         <v>1281</v>
@@ -24132,7 +24132,7 @@
         <v>1272</v>
       </c>
       <c r="E494">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F494" t="s">
         <v>1281</v>
@@ -24170,7 +24170,7 @@
         <v>1272</v>
       </c>
       <c r="E495">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F495" t="s">
         <v>1279</v>
@@ -24205,7 +24205,7 @@
         <v>1273</v>
       </c>
       <c r="E496">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F496" t="s">
         <v>1281</v>
@@ -24243,7 +24243,7 @@
         <v>1273</v>
       </c>
       <c r="E497">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F497" t="s">
         <v>1281</v>
@@ -24281,7 +24281,7 @@
         <v>1274</v>
       </c>
       <c r="E498">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F498" t="s">
         <v>1281</v>
@@ -24319,7 +24319,7 @@
         <v>1274</v>
       </c>
       <c r="E499">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F499" t="s">
         <v>1279</v>
@@ -24354,7 +24354,7 @@
         <v>1275</v>
       </c>
       <c r="E500">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F500" t="s">
         <v>1279</v>
@@ -24389,7 +24389,7 @@
         <v>1275</v>
       </c>
       <c r="E501">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F501" t="s">
         <v>1279</v>
@@ -24427,7 +24427,7 @@
         <v>1275</v>
       </c>
       <c r="E502">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F502" t="s">
         <v>1281</v>
@@ -24465,7 +24465,7 @@
         <v>1276</v>
       </c>
       <c r="E503">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F503" t="s">
         <v>1279</v>
@@ -24503,7 +24503,7 @@
         <v>1276</v>
       </c>
       <c r="E504">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F504" t="s">
         <v>1279</v>
@@ -24538,7 +24538,7 @@
         <v>1276</v>
       </c>
       <c r="E505">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F505" t="s">
         <v>1279</v>
@@ -24573,7 +24573,7 @@
         <v>1276</v>
       </c>
       <c r="E506">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F506" t="s">
         <v>1279</v>
@@ -24608,7 +24608,7 @@
         <v>1276</v>
       </c>
       <c r="E507">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F507" t="s">
         <v>1279</v>
@@ -24643,7 +24643,7 @@
         <v>1276</v>
       </c>
       <c r="E508">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F508" t="s">
         <v>1281</v>
@@ -24681,7 +24681,7 @@
         <v>1277</v>
       </c>
       <c r="E509">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F509" t="s">
         <v>1279</v>
@@ -24716,7 +24716,7 @@
         <v>1277</v>
       </c>
       <c r="E510">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F510" t="s">
         <v>1279</v>
@@ -24751,7 +24751,7 @@
         <v>1277</v>
       </c>
       <c r="E511">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F511" t="s">
         <v>1279</v>
@@ -24786,7 +24786,7 @@
         <v>1277</v>
       </c>
       <c r="E512">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F512" t="s">
         <v>1279</v>
@@ -24821,7 +24821,7 @@
         <v>1277</v>
       </c>
       <c r="E513">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F513" t="s">
         <v>1279</v>
@@ -24856,7 +24856,7 @@
         <v>1277</v>
       </c>
       <c r="E514">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F514" t="s">
         <v>1279</v>
@@ -24891,7 +24891,7 @@
         <v>1278</v>
       </c>
       <c r="E515">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F515" t="s">
         <v>1279</v>
@@ -24929,7 +24929,7 @@
         <v>1278</v>
       </c>
       <c r="E516">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F516" t="s">
         <v>1279</v>
@@ -24964,7 +24964,7 @@
         <v>1278</v>
       </c>
       <c r="E517">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F517" t="s">
         <v>1279</v>
@@ -24999,7 +24999,7 @@
         <v>1278</v>
       </c>
       <c r="E518">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F518" t="s">
         <v>1279</v>
@@ -25037,7 +25037,7 @@
         <v>1278</v>
       </c>
       <c r="E519">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F519" t="s">
         <v>1279</v>
@@ -25072,7 +25072,7 @@
         <v>1278</v>
       </c>
       <c r="E520">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F520" t="s">
         <v>1281</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-20 00:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -6834,7 +6834,7 @@
         <v>1073</v>
       </c>
       <c r="E2">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="F2" t="s">
         <v>1279</v>
@@ -6869,7 +6869,7 @@
         <v>1074</v>
       </c>
       <c r="E3">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F3" t="s">
         <v>1279</v>
@@ -6904,7 +6904,7 @@
         <v>1075</v>
       </c>
       <c r="E4">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F4" t="s">
         <v>1279</v>
@@ -6939,7 +6939,7 @@
         <v>1076</v>
       </c>
       <c r="E5">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F5" t="s">
         <v>1279</v>
@@ -6974,7 +6974,7 @@
         <v>1077</v>
       </c>
       <c r="E6">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F6" t="s">
         <v>1279</v>
@@ -7009,7 +7009,7 @@
         <v>1078</v>
       </c>
       <c r="E7">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F7" t="s">
         <v>1279</v>
@@ -7044,7 +7044,7 @@
         <v>1079</v>
       </c>
       <c r="E8">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F8" t="s">
         <v>1279</v>
@@ -7079,7 +7079,7 @@
         <v>1080</v>
       </c>
       <c r="E9">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F9" t="s">
         <v>1279</v>
@@ -7114,7 +7114,7 @@
         <v>1081</v>
       </c>
       <c r="E10">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F10" t="s">
         <v>1279</v>
@@ -7149,7 +7149,7 @@
         <v>1081</v>
       </c>
       <c r="E11">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F11" t="s">
         <v>1279</v>
@@ -7184,7 +7184,7 @@
         <v>1082</v>
       </c>
       <c r="E12">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F12" t="s">
         <v>1279</v>
@@ -7219,7 +7219,7 @@
         <v>1083</v>
       </c>
       <c r="E13">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F13" t="s">
         <v>1279</v>
@@ -7254,7 +7254,7 @@
         <v>1084</v>
       </c>
       <c r="E14">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F14" t="s">
         <v>1279</v>
@@ -7289,7 +7289,7 @@
         <v>1084</v>
       </c>
       <c r="E15">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F15" t="s">
         <v>1279</v>
@@ -7324,7 +7324,7 @@
         <v>1085</v>
       </c>
       <c r="E16">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F16" t="s">
         <v>1279</v>
@@ -7359,7 +7359,7 @@
         <v>1085</v>
       </c>
       <c r="E17">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="F17" t="s">
         <v>1279</v>
@@ -7394,7 +7394,7 @@
         <v>1086</v>
       </c>
       <c r="E18">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F18" t="s">
         <v>1279</v>
@@ -7429,7 +7429,7 @@
         <v>1087</v>
       </c>
       <c r="E19">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F19" t="s">
         <v>1279</v>
@@ -7464,7 +7464,7 @@
         <v>1088</v>
       </c>
       <c r="E20">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F20" t="s">
         <v>1279</v>
@@ -7499,7 +7499,7 @@
         <v>1089</v>
       </c>
       <c r="E21">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F21" t="s">
         <v>1279</v>
@@ -7534,7 +7534,7 @@
         <v>1090</v>
       </c>
       <c r="E22">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F22" t="s">
         <v>1279</v>
@@ -7572,7 +7572,7 @@
         <v>1091</v>
       </c>
       <c r="E23">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F23" t="s">
         <v>1279</v>
@@ -7607,7 +7607,7 @@
         <v>1092</v>
       </c>
       <c r="E24">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F24" t="s">
         <v>1279</v>
@@ -7642,7 +7642,7 @@
         <v>1093</v>
       </c>
       <c r="E25">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F25" t="s">
         <v>1279</v>
@@ -7677,7 +7677,7 @@
         <v>1094</v>
       </c>
       <c r="E26">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F26" t="s">
         <v>1279</v>
@@ -7712,7 +7712,7 @@
         <v>1095</v>
       </c>
       <c r="E27">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F27" t="s">
         <v>1279</v>
@@ -7747,7 +7747,7 @@
         <v>1096</v>
       </c>
       <c r="E28">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F28" t="s">
         <v>1279</v>
@@ -7782,7 +7782,7 @@
         <v>1097</v>
       </c>
       <c r="E29">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F29" t="s">
         <v>1279</v>
@@ -7817,7 +7817,7 @@
         <v>1098</v>
       </c>
       <c r="E30">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F30" t="s">
         <v>1279</v>
@@ -7852,7 +7852,7 @@
         <v>1099</v>
       </c>
       <c r="E31">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F31" t="s">
         <v>1279</v>
@@ -7887,7 +7887,7 @@
         <v>1100</v>
       </c>
       <c r="E32">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F32" t="s">
         <v>1279</v>
@@ -7922,7 +7922,7 @@
         <v>1101</v>
       </c>
       <c r="E33">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="F33" t="s">
         <v>1279</v>
@@ -7957,7 +7957,7 @@
         <v>1102</v>
       </c>
       <c r="E34">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F34" t="s">
         <v>1279</v>
@@ -7992,7 +7992,7 @@
         <v>1103</v>
       </c>
       <c r="E35">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F35" t="s">
         <v>1279</v>
@@ -8027,7 +8027,7 @@
         <v>1104</v>
       </c>
       <c r="E36">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F36" t="s">
         <v>1279</v>
@@ -8062,7 +8062,7 @@
         <v>1104</v>
       </c>
       <c r="E37">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F37" t="s">
         <v>1279</v>
@@ -8097,7 +8097,7 @@
         <v>1105</v>
       </c>
       <c r="E38">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F38" t="s">
         <v>1279</v>
@@ -8132,7 +8132,7 @@
         <v>1106</v>
       </c>
       <c r="E39">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F39" t="s">
         <v>1279</v>
@@ -8167,7 +8167,7 @@
         <v>1107</v>
       </c>
       <c r="E40">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F40" t="s">
         <v>1279</v>
@@ -8202,7 +8202,7 @@
         <v>1107</v>
       </c>
       <c r="E41">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F41" t="s">
         <v>1279</v>
@@ -8237,7 +8237,7 @@
         <v>1108</v>
       </c>
       <c r="E42">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F42" t="s">
         <v>1279</v>
@@ -8272,7 +8272,7 @@
         <v>1108</v>
       </c>
       <c r="E43">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F43" t="s">
         <v>1279</v>
@@ -8307,7 +8307,7 @@
         <v>1109</v>
       </c>
       <c r="E44">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F44" t="s">
         <v>1279</v>
@@ -8342,7 +8342,7 @@
         <v>1110</v>
       </c>
       <c r="E45">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F45" t="s">
         <v>1279</v>
@@ -8377,7 +8377,7 @@
         <v>1111</v>
       </c>
       <c r="E46">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F46" t="s">
         <v>1279</v>
@@ -8412,7 +8412,7 @@
         <v>1112</v>
       </c>
       <c r="E47">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F47" t="s">
         <v>1279</v>
@@ -8447,7 +8447,7 @@
         <v>1112</v>
       </c>
       <c r="E48">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F48" t="s">
         <v>1279</v>
@@ -8482,7 +8482,7 @@
         <v>1113</v>
       </c>
       <c r="E49">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="F49" t="s">
         <v>1279</v>
@@ -8517,7 +8517,7 @@
         <v>1114</v>
       </c>
       <c r="E50">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F50" t="s">
         <v>1279</v>
@@ -8552,7 +8552,7 @@
         <v>1115</v>
       </c>
       <c r="E51">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F51" t="s">
         <v>1279</v>
@@ -8587,7 +8587,7 @@
         <v>1116</v>
       </c>
       <c r="E52">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F52" t="s">
         <v>1279</v>
@@ -8622,7 +8622,7 @@
         <v>1117</v>
       </c>
       <c r="E53">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F53" t="s">
         <v>1279</v>
@@ -8657,7 +8657,7 @@
         <v>1118</v>
       </c>
       <c r="E54">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F54" t="s">
         <v>1279</v>
@@ -8692,7 +8692,7 @@
         <v>1119</v>
       </c>
       <c r="E55">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F55" t="s">
         <v>1279</v>
@@ -8727,7 +8727,7 @@
         <v>1119</v>
       </c>
       <c r="E56">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F56" t="s">
         <v>1279</v>
@@ -8762,7 +8762,7 @@
         <v>1119</v>
       </c>
       <c r="E57">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F57" t="s">
         <v>1279</v>
@@ -8797,7 +8797,7 @@
         <v>1120</v>
       </c>
       <c r="E58">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F58" t="s">
         <v>1279</v>
@@ -8832,7 +8832,7 @@
         <v>1121</v>
       </c>
       <c r="E59">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F59" t="s">
         <v>1279</v>
@@ -8867,7 +8867,7 @@
         <v>1122</v>
       </c>
       <c r="E60">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F60" t="s">
         <v>1279</v>
@@ -8902,7 +8902,7 @@
         <v>1122</v>
       </c>
       <c r="E61">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F61" t="s">
         <v>1279</v>
@@ -8937,7 +8937,7 @@
         <v>1123</v>
       </c>
       <c r="E62">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F62" t="s">
         <v>1279</v>
@@ -8972,7 +8972,7 @@
         <v>1124</v>
       </c>
       <c r="E63">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F63" t="s">
         <v>1279</v>
@@ -9007,7 +9007,7 @@
         <v>1124</v>
       </c>
       <c r="E64">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F64" t="s">
         <v>1279</v>
@@ -9042,7 +9042,7 @@
         <v>1124</v>
       </c>
       <c r="E65">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F65" t="s">
         <v>1279</v>
@@ -9077,7 +9077,7 @@
         <v>1125</v>
       </c>
       <c r="E66">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F66" t="s">
         <v>1279</v>
@@ -9112,7 +9112,7 @@
         <v>1126</v>
       </c>
       <c r="E67">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F67" t="s">
         <v>1279</v>
@@ -9147,7 +9147,7 @@
         <v>1126</v>
       </c>
       <c r="E68">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F68" t="s">
         <v>1279</v>
@@ -9182,7 +9182,7 @@
         <v>1126</v>
       </c>
       <c r="E69">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F69" t="s">
         <v>1280</v>
@@ -9217,7 +9217,7 @@
         <v>1126</v>
       </c>
       <c r="E70">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F70" t="s">
         <v>1279</v>
@@ -9252,7 +9252,7 @@
         <v>1127</v>
       </c>
       <c r="E71">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F71" t="s">
         <v>1279</v>
@@ -9287,7 +9287,7 @@
         <v>1128</v>
       </c>
       <c r="E72">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F72" t="s">
         <v>1279</v>
@@ -9322,7 +9322,7 @@
         <v>1128</v>
       </c>
       <c r="E73">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F73" t="s">
         <v>1279</v>
@@ -9357,7 +9357,7 @@
         <v>1129</v>
       </c>
       <c r="E74">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F74" t="s">
         <v>1279</v>
@@ -9392,7 +9392,7 @@
         <v>1130</v>
       </c>
       <c r="E75">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F75" t="s">
         <v>1279</v>
@@ -9427,7 +9427,7 @@
         <v>1131</v>
       </c>
       <c r="E76">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F76" t="s">
         <v>1279</v>
@@ -9462,7 +9462,7 @@
         <v>1132</v>
       </c>
       <c r="E77">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F77" t="s">
         <v>1279</v>
@@ -9497,7 +9497,7 @@
         <v>1132</v>
       </c>
       <c r="E78">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F78" t="s">
         <v>1279</v>
@@ -9532,7 +9532,7 @@
         <v>1132</v>
       </c>
       <c r="E79">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F79" t="s">
         <v>1279</v>
@@ -9567,7 +9567,7 @@
         <v>1132</v>
       </c>
       <c r="E80">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F80" t="s">
         <v>1279</v>
@@ -9602,7 +9602,7 @@
         <v>1132</v>
       </c>
       <c r="E81">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F81" t="s">
         <v>1279</v>
@@ -9637,7 +9637,7 @@
         <v>1132</v>
       </c>
       <c r="E82">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F82" t="s">
         <v>1279</v>
@@ -9672,7 +9672,7 @@
         <v>1133</v>
       </c>
       <c r="E83">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F83" t="s">
         <v>1279</v>
@@ -9707,7 +9707,7 @@
         <v>1134</v>
       </c>
       <c r="E84">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F84" t="s">
         <v>1279</v>
@@ -9742,7 +9742,7 @@
         <v>1135</v>
       </c>
       <c r="E85">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F85" t="s">
         <v>1279</v>
@@ -9777,7 +9777,7 @@
         <v>1135</v>
       </c>
       <c r="E86">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F86" t="s">
         <v>1279</v>
@@ -9812,7 +9812,7 @@
         <v>1136</v>
       </c>
       <c r="E87">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F87" t="s">
         <v>1281</v>
@@ -9847,7 +9847,7 @@
         <v>1137</v>
       </c>
       <c r="E88">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F88" t="s">
         <v>1279</v>
@@ -9882,7 +9882,7 @@
         <v>1138</v>
       </c>
       <c r="E89">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F89" t="s">
         <v>1279</v>
@@ -9917,7 +9917,7 @@
         <v>1138</v>
       </c>
       <c r="E90">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F90" t="s">
         <v>1279</v>
@@ -9952,7 +9952,7 @@
         <v>1139</v>
       </c>
       <c r="E91">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F91" t="s">
         <v>1279</v>
@@ -9987,7 +9987,7 @@
         <v>1140</v>
       </c>
       <c r="E92">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F92" t="s">
         <v>1279</v>
@@ -10022,7 +10022,7 @@
         <v>1141</v>
       </c>
       <c r="E93">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F93" t="s">
         <v>1279</v>
@@ -10057,7 +10057,7 @@
         <v>1142</v>
       </c>
       <c r="E94">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F94" t="s">
         <v>1279</v>
@@ -10092,7 +10092,7 @@
         <v>1143</v>
       </c>
       <c r="E95">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F95" t="s">
         <v>1279</v>
@@ -10127,7 +10127,7 @@
         <v>1143</v>
       </c>
       <c r="E96">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F96" t="s">
         <v>1279</v>
@@ -10162,7 +10162,7 @@
         <v>1144</v>
       </c>
       <c r="E97">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F97" t="s">
         <v>1279</v>
@@ -10197,7 +10197,7 @@
         <v>1144</v>
       </c>
       <c r="E98">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F98" t="s">
         <v>1279</v>
@@ -10232,7 +10232,7 @@
         <v>1144</v>
       </c>
       <c r="E99">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F99" t="s">
         <v>1279</v>
@@ -10267,7 +10267,7 @@
         <v>1145</v>
       </c>
       <c r="E100">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F100" t="s">
         <v>1279</v>
@@ -10302,7 +10302,7 @@
         <v>1145</v>
       </c>
       <c r="E101">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F101" t="s">
         <v>1279</v>
@@ -10337,7 +10337,7 @@
         <v>1146</v>
       </c>
       <c r="E102">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F102" t="s">
         <v>1279</v>
@@ -10372,7 +10372,7 @@
         <v>1147</v>
       </c>
       <c r="E103">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F103" t="s">
         <v>1279</v>
@@ -10407,7 +10407,7 @@
         <v>1148</v>
       </c>
       <c r="E104">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F104" t="s">
         <v>1279</v>
@@ -10442,7 +10442,7 @@
         <v>1148</v>
       </c>
       <c r="E105">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F105" t="s">
         <v>1279</v>
@@ -10477,7 +10477,7 @@
         <v>1149</v>
       </c>
       <c r="E106">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F106" t="s">
         <v>1279</v>
@@ -10512,7 +10512,7 @@
         <v>1149</v>
       </c>
       <c r="E107">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F107" t="s">
         <v>1279</v>
@@ -10547,7 +10547,7 @@
         <v>1150</v>
       </c>
       <c r="E108">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F108" t="s">
         <v>1279</v>
@@ -10582,7 +10582,7 @@
         <v>1151</v>
       </c>
       <c r="E109">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F109" t="s">
         <v>1279</v>
@@ -10617,7 +10617,7 @@
         <v>1151</v>
       </c>
       <c r="E110">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F110" t="s">
         <v>1279</v>
@@ -10652,7 +10652,7 @@
         <v>1152</v>
       </c>
       <c r="E111">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F111" t="s">
         <v>1279</v>
@@ -10687,7 +10687,7 @@
         <v>1153</v>
       </c>
       <c r="E112">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F112" t="s">
         <v>1279</v>
@@ -10722,7 +10722,7 @@
         <v>1153</v>
       </c>
       <c r="E113">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F113" t="s">
         <v>1279</v>
@@ -10757,7 +10757,7 @@
         <v>1154</v>
       </c>
       <c r="E114">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F114" t="s">
         <v>1279</v>
@@ -10792,7 +10792,7 @@
         <v>1155</v>
       </c>
       <c r="E115">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F115" t="s">
         <v>1279</v>
@@ -10830,7 +10830,7 @@
         <v>1155</v>
       </c>
       <c r="E116">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F116" t="s">
         <v>1279</v>
@@ -10865,7 +10865,7 @@
         <v>1155</v>
       </c>
       <c r="E117">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F117" t="s">
         <v>1279</v>
@@ -10900,7 +10900,7 @@
         <v>1155</v>
       </c>
       <c r="E118">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F118" t="s">
         <v>1279</v>
@@ -10935,7 +10935,7 @@
         <v>1156</v>
       </c>
       <c r="E119">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F119" t="s">
         <v>1280</v>
@@ -10970,7 +10970,7 @@
         <v>1157</v>
       </c>
       <c r="E120">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F120" t="s">
         <v>1279</v>
@@ -11005,7 +11005,7 @@
         <v>1157</v>
       </c>
       <c r="E121">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F121" t="s">
         <v>1279</v>
@@ -11040,7 +11040,7 @@
         <v>1157</v>
       </c>
       <c r="E122">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F122" t="s">
         <v>1279</v>
@@ -11075,7 +11075,7 @@
         <v>1157</v>
       </c>
       <c r="E123">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F123" t="s">
         <v>1279</v>
@@ -11110,7 +11110,7 @@
         <v>1158</v>
       </c>
       <c r="E124">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F124" t="s">
         <v>1279</v>
@@ -11145,7 +11145,7 @@
         <v>1158</v>
       </c>
       <c r="E125">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F125" t="s">
         <v>1279</v>
@@ -11180,7 +11180,7 @@
         <v>1158</v>
       </c>
       <c r="E126">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F126" t="s">
         <v>1279</v>
@@ -11215,7 +11215,7 @@
         <v>1158</v>
       </c>
       <c r="E127">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F127" t="s">
         <v>1279</v>
@@ -11250,7 +11250,7 @@
         <v>1158</v>
       </c>
       <c r="E128">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F128" t="s">
         <v>1279</v>
@@ -11285,7 +11285,7 @@
         <v>1158</v>
       </c>
       <c r="E129">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F129" t="s">
         <v>1279</v>
@@ -11320,7 +11320,7 @@
         <v>1158</v>
       </c>
       <c r="E130">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F130" t="s">
         <v>1279</v>
@@ -11355,7 +11355,7 @@
         <v>1159</v>
       </c>
       <c r="E131">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F131" t="s">
         <v>1279</v>
@@ -11390,7 +11390,7 @@
         <v>1159</v>
       </c>
       <c r="E132">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F132" t="s">
         <v>1279</v>
@@ -11425,7 +11425,7 @@
         <v>1160</v>
       </c>
       <c r="E133">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F133" t="s">
         <v>1279</v>
@@ -11460,7 +11460,7 @@
         <v>1161</v>
       </c>
       <c r="E134">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F134" t="s">
         <v>1279</v>
@@ -11495,7 +11495,7 @@
         <v>1161</v>
       </c>
       <c r="E135">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F135" t="s">
         <v>1279</v>
@@ -11530,7 +11530,7 @@
         <v>1161</v>
       </c>
       <c r="E136">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F136" t="s">
         <v>1279</v>
@@ -11565,7 +11565,7 @@
         <v>1162</v>
       </c>
       <c r="E137">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F137" t="s">
         <v>1279</v>
@@ -11600,7 +11600,7 @@
         <v>1162</v>
       </c>
       <c r="E138">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F138" t="s">
         <v>1279</v>
@@ -11635,7 +11635,7 @@
         <v>1162</v>
       </c>
       <c r="E139">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F139" t="s">
         <v>1279</v>
@@ -11670,7 +11670,7 @@
         <v>1162</v>
       </c>
       <c r="E140">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F140" t="s">
         <v>1279</v>
@@ -11705,7 +11705,7 @@
         <v>1162</v>
       </c>
       <c r="E141">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F141" t="s">
         <v>1279</v>
@@ -11740,7 +11740,7 @@
         <v>1162</v>
       </c>
       <c r="E142">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F142" t="s">
         <v>1279</v>
@@ -11775,7 +11775,7 @@
         <v>1162</v>
       </c>
       <c r="E143">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F143" t="s">
         <v>1279</v>
@@ -11810,7 +11810,7 @@
         <v>1162</v>
       </c>
       <c r="E144">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F144" t="s">
         <v>1279</v>
@@ -11845,7 +11845,7 @@
         <v>1162</v>
       </c>
       <c r="E145">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F145" t="s">
         <v>1279</v>
@@ -11880,7 +11880,7 @@
         <v>1163</v>
       </c>
       <c r="E146">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F146" t="s">
         <v>1279</v>
@@ -11915,7 +11915,7 @@
         <v>1163</v>
       </c>
       <c r="E147">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F147" t="s">
         <v>1279</v>
@@ -11950,7 +11950,7 @@
         <v>1163</v>
       </c>
       <c r="E148">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F148" t="s">
         <v>1279</v>
@@ -11985,7 +11985,7 @@
         <v>1164</v>
       </c>
       <c r="E149">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F149" t="s">
         <v>1279</v>
@@ -12020,7 +12020,7 @@
         <v>1164</v>
       </c>
       <c r="E150">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F150" t="s">
         <v>1280</v>
@@ -12055,7 +12055,7 @@
         <v>1164</v>
       </c>
       <c r="E151">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F151" t="s">
         <v>1279</v>
@@ -12090,7 +12090,7 @@
         <v>1165</v>
       </c>
       <c r="E152">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F152" t="s">
         <v>1279</v>
@@ -12125,7 +12125,7 @@
         <v>1165</v>
       </c>
       <c r="E153">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F153" t="s">
         <v>1279</v>
@@ -12160,7 +12160,7 @@
         <v>1166</v>
       </c>
       <c r="E154">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F154" t="s">
         <v>1279</v>
@@ -12195,7 +12195,7 @@
         <v>1166</v>
       </c>
       <c r="E155">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F155" t="s">
         <v>1279</v>
@@ -12230,7 +12230,7 @@
         <v>1167</v>
       </c>
       <c r="E156">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F156" t="s">
         <v>1279</v>
@@ -12265,7 +12265,7 @@
         <v>1167</v>
       </c>
       <c r="E157">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F157" t="s">
         <v>1279</v>
@@ -12300,7 +12300,7 @@
         <v>1168</v>
       </c>
       <c r="E158">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F158" t="s">
         <v>1279</v>
@@ -12335,7 +12335,7 @@
         <v>1168</v>
       </c>
       <c r="E159">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F159" t="s">
         <v>1279</v>
@@ -12370,7 +12370,7 @@
         <v>1168</v>
       </c>
       <c r="E160">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F160" t="s">
         <v>1279</v>
@@ -12405,7 +12405,7 @@
         <v>1169</v>
       </c>
       <c r="E161">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F161" t="s">
         <v>1279</v>
@@ -12440,7 +12440,7 @@
         <v>1169</v>
       </c>
       <c r="E162">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F162" t="s">
         <v>1279</v>
@@ -12475,7 +12475,7 @@
         <v>1170</v>
       </c>
       <c r="E163">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F163" t="s">
         <v>1279</v>
@@ -12510,7 +12510,7 @@
         <v>1171</v>
       </c>
       <c r="E164">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F164" t="s">
         <v>1279</v>
@@ -12545,7 +12545,7 @@
         <v>1171</v>
       </c>
       <c r="E165">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F165" t="s">
         <v>1279</v>
@@ -12580,7 +12580,7 @@
         <v>1171</v>
       </c>
       <c r="E166">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F166" t="s">
         <v>1279</v>
@@ -12615,7 +12615,7 @@
         <v>1171</v>
       </c>
       <c r="E167">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F167" t="s">
         <v>1279</v>
@@ -12650,7 +12650,7 @@
         <v>1172</v>
       </c>
       <c r="E168">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F168" t="s">
         <v>1279</v>
@@ -12685,7 +12685,7 @@
         <v>1173</v>
       </c>
       <c r="E169">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F169" t="s">
         <v>1279</v>
@@ -12720,7 +12720,7 @@
         <v>1173</v>
       </c>
       <c r="E170">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F170" t="s">
         <v>1279</v>
@@ -12755,7 +12755,7 @@
         <v>1173</v>
       </c>
       <c r="E171">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F171" t="s">
         <v>1279</v>
@@ -12790,7 +12790,7 @@
         <v>1173</v>
       </c>
       <c r="E172">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F172" t="s">
         <v>1279</v>
@@ -12825,7 +12825,7 @@
         <v>1173</v>
       </c>
       <c r="E173">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F173" t="s">
         <v>1279</v>
@@ -12860,7 +12860,7 @@
         <v>1174</v>
       </c>
       <c r="E174">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F174" t="s">
         <v>1279</v>
@@ -12895,7 +12895,7 @@
         <v>1174</v>
       </c>
       <c r="E175">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F175" t="s">
         <v>1279</v>
@@ -12930,7 +12930,7 @@
         <v>1174</v>
       </c>
       <c r="E176">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F176" t="s">
         <v>1279</v>
@@ -12965,7 +12965,7 @@
         <v>1174</v>
       </c>
       <c r="E177">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F177" t="s">
         <v>1279</v>
@@ -13000,7 +13000,7 @@
         <v>1174</v>
       </c>
       <c r="E178">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F178" t="s">
         <v>1279</v>
@@ -13035,7 +13035,7 @@
         <v>1174</v>
       </c>
       <c r="E179">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F179" t="s">
         <v>1279</v>
@@ -13070,7 +13070,7 @@
         <v>1175</v>
       </c>
       <c r="E180">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F180" t="s">
         <v>1279</v>
@@ -13105,7 +13105,7 @@
         <v>1175</v>
       </c>
       <c r="E181">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F181" t="s">
         <v>1279</v>
@@ -13140,7 +13140,7 @@
         <v>1175</v>
       </c>
       <c r="E182">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F182" t="s">
         <v>1279</v>
@@ -13175,7 +13175,7 @@
         <v>1175</v>
       </c>
       <c r="E183">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F183" t="s">
         <v>1279</v>
@@ -13210,7 +13210,7 @@
         <v>1176</v>
       </c>
       <c r="E184">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F184" t="s">
         <v>1279</v>
@@ -13245,7 +13245,7 @@
         <v>1176</v>
       </c>
       <c r="E185">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F185" t="s">
         <v>1279</v>
@@ -13280,7 +13280,7 @@
         <v>1177</v>
       </c>
       <c r="E186">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F186" t="s">
         <v>1279</v>
@@ -13315,7 +13315,7 @@
         <v>1178</v>
       </c>
       <c r="E187">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F187" t="s">
         <v>1279</v>
@@ -13350,7 +13350,7 @@
         <v>1178</v>
       </c>
       <c r="E188">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F188" t="s">
         <v>1279</v>
@@ -13385,7 +13385,7 @@
         <v>1179</v>
       </c>
       <c r="E189">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F189" t="s">
         <v>1279</v>
@@ -13420,7 +13420,7 @@
         <v>1180</v>
       </c>
       <c r="E190">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F190" t="s">
         <v>1279</v>
@@ -13455,7 +13455,7 @@
         <v>1180</v>
       </c>
       <c r="E191">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F191" t="s">
         <v>1279</v>
@@ -13490,7 +13490,7 @@
         <v>1181</v>
       </c>
       <c r="E192">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F192" t="s">
         <v>1279</v>
@@ -13525,7 +13525,7 @@
         <v>1181</v>
       </c>
       <c r="E193">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F193" t="s">
         <v>1279</v>
@@ -13560,7 +13560,7 @@
         <v>1182</v>
       </c>
       <c r="E194">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F194" t="s">
         <v>1279</v>
@@ -13595,7 +13595,7 @@
         <v>1183</v>
       </c>
       <c r="E195">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F195" t="s">
         <v>1279</v>
@@ -13630,7 +13630,7 @@
         <v>1183</v>
       </c>
       <c r="E196">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F196" t="s">
         <v>1279</v>
@@ -13665,7 +13665,7 @@
         <v>1183</v>
       </c>
       <c r="E197">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F197" t="s">
         <v>1279</v>
@@ -13700,7 +13700,7 @@
         <v>1184</v>
       </c>
       <c r="E198">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F198" t="s">
         <v>1279</v>
@@ -13735,7 +13735,7 @@
         <v>1184</v>
       </c>
       <c r="E199">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F199" t="s">
         <v>1279</v>
@@ -13770,7 +13770,7 @@
         <v>1185</v>
       </c>
       <c r="E200">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F200" t="s">
         <v>1279</v>
@@ -13805,7 +13805,7 @@
         <v>1186</v>
       </c>
       <c r="E201">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F201" t="s">
         <v>1279</v>
@@ -13840,7 +13840,7 @@
         <v>1186</v>
       </c>
       <c r="E202">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F202" t="s">
         <v>1279</v>
@@ -13875,7 +13875,7 @@
         <v>1186</v>
       </c>
       <c r="E203">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F203" t="s">
         <v>1279</v>
@@ -13910,7 +13910,7 @@
         <v>1187</v>
       </c>
       <c r="E204">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F204" t="s">
         <v>1279</v>
@@ -13945,7 +13945,7 @@
         <v>1187</v>
       </c>
       <c r="E205">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F205" t="s">
         <v>1279</v>
@@ -13980,7 +13980,7 @@
         <v>1188</v>
       </c>
       <c r="E206">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F206" t="s">
         <v>1279</v>
@@ -14015,7 +14015,7 @@
         <v>1188</v>
       </c>
       <c r="E207">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F207" t="s">
         <v>1281</v>
@@ -14050,7 +14050,7 @@
         <v>1188</v>
       </c>
       <c r="E208">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F208" t="s">
         <v>1279</v>
@@ -14085,7 +14085,7 @@
         <v>1189</v>
       </c>
       <c r="E209">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F209" t="s">
         <v>1279</v>
@@ -14120,7 +14120,7 @@
         <v>1189</v>
       </c>
       <c r="E210">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F210" t="s">
         <v>1279</v>
@@ -14158,7 +14158,7 @@
         <v>1189</v>
       </c>
       <c r="E211">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F211" t="s">
         <v>1279</v>
@@ -14193,7 +14193,7 @@
         <v>1189</v>
       </c>
       <c r="E212">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F212" t="s">
         <v>1279</v>
@@ -14228,7 +14228,7 @@
         <v>1189</v>
       </c>
       <c r="E213">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F213" t="s">
         <v>1279</v>
@@ -14263,7 +14263,7 @@
         <v>1189</v>
       </c>
       <c r="E214">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F214" t="s">
         <v>1279</v>
@@ -14298,7 +14298,7 @@
         <v>1190</v>
       </c>
       <c r="E215">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F215" t="s">
         <v>1279</v>
@@ -14333,7 +14333,7 @@
         <v>1190</v>
       </c>
       <c r="E216">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F216" t="s">
         <v>1279</v>
@@ -14368,7 +14368,7 @@
         <v>1190</v>
       </c>
       <c r="E217">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F217" t="s">
         <v>1279</v>
@@ -14403,7 +14403,7 @@
         <v>1191</v>
       </c>
       <c r="E218">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F218" t="s">
         <v>1279</v>
@@ -14438,7 +14438,7 @@
         <v>1191</v>
       </c>
       <c r="E219">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F219" t="s">
         <v>1279</v>
@@ -14473,7 +14473,7 @@
         <v>1191</v>
       </c>
       <c r="E220">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F220" t="s">
         <v>1279</v>
@@ -14508,7 +14508,7 @@
         <v>1192</v>
       </c>
       <c r="E221">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F221" t="s">
         <v>1279</v>
@@ -14543,7 +14543,7 @@
         <v>1192</v>
       </c>
       <c r="E222">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F222" t="s">
         <v>1279</v>
@@ -14578,7 +14578,7 @@
         <v>1192</v>
       </c>
       <c r="E223">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F223" t="s">
         <v>1279</v>
@@ -14613,7 +14613,7 @@
         <v>1193</v>
       </c>
       <c r="E224">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F224" t="s">
         <v>1279</v>
@@ -14648,7 +14648,7 @@
         <v>1193</v>
       </c>
       <c r="E225">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F225" t="s">
         <v>1279</v>
@@ -14683,7 +14683,7 @@
         <v>1193</v>
       </c>
       <c r="E226">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F226" t="s">
         <v>1279</v>
@@ -14718,7 +14718,7 @@
         <v>1193</v>
       </c>
       <c r="E227">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F227" t="s">
         <v>1279</v>
@@ -14753,7 +14753,7 @@
         <v>1193</v>
       </c>
       <c r="E228">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F228" t="s">
         <v>1279</v>
@@ -14788,7 +14788,7 @@
         <v>1193</v>
       </c>
       <c r="E229">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F229" t="s">
         <v>1279</v>
@@ -14823,7 +14823,7 @@
         <v>1194</v>
       </c>
       <c r="E230">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F230" t="s">
         <v>1279</v>
@@ -14858,7 +14858,7 @@
         <v>1195</v>
       </c>
       <c r="E231">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F231" t="s">
         <v>1279</v>
@@ -14893,7 +14893,7 @@
         <v>1195</v>
       </c>
       <c r="E232">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F232" t="s">
         <v>1282</v>
@@ -14928,7 +14928,7 @@
         <v>1195</v>
       </c>
       <c r="E233">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F233" t="s">
         <v>1279</v>
@@ -14963,7 +14963,7 @@
         <v>1195</v>
       </c>
       <c r="E234">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F234" t="s">
         <v>1279</v>
@@ -14998,7 +14998,7 @@
         <v>1196</v>
       </c>
       <c r="E235">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F235" t="s">
         <v>1279</v>
@@ -15033,7 +15033,7 @@
         <v>1196</v>
       </c>
       <c r="E236">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F236" t="s">
         <v>1279</v>
@@ -15068,7 +15068,7 @@
         <v>1196</v>
       </c>
       <c r="E237">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F237" t="s">
         <v>1279</v>
@@ -15103,7 +15103,7 @@
         <v>1196</v>
       </c>
       <c r="E238">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F238" t="s">
         <v>1279</v>
@@ -15138,7 +15138,7 @@
         <v>1197</v>
       </c>
       <c r="E239">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F239" t="s">
         <v>1279</v>
@@ -15176,7 +15176,7 @@
         <v>1198</v>
       </c>
       <c r="E240">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F240" t="s">
         <v>1279</v>
@@ -15211,7 +15211,7 @@
         <v>1198</v>
       </c>
       <c r="E241">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F241" t="s">
         <v>1279</v>
@@ -15246,7 +15246,7 @@
         <v>1198</v>
       </c>
       <c r="E242">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F242" t="s">
         <v>1279</v>
@@ -15281,7 +15281,7 @@
         <v>1198</v>
       </c>
       <c r="E243">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F243" t="s">
         <v>1279</v>
@@ -15319,7 +15319,7 @@
         <v>1198</v>
       </c>
       <c r="E244">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F244" t="s">
         <v>1279</v>
@@ -15354,7 +15354,7 @@
         <v>1199</v>
       </c>
       <c r="E245">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F245" t="s">
         <v>1279</v>
@@ -15389,7 +15389,7 @@
         <v>1199</v>
       </c>
       <c r="E246">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F246" t="s">
         <v>1279</v>
@@ -15424,7 +15424,7 @@
         <v>1200</v>
       </c>
       <c r="E247">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F247" t="s">
         <v>1279</v>
@@ -15459,7 +15459,7 @@
         <v>1200</v>
       </c>
       <c r="E248">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F248" t="s">
         <v>1279</v>
@@ -15494,7 +15494,7 @@
         <v>1200</v>
       </c>
       <c r="E249">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F249" t="s">
         <v>1279</v>
@@ -15529,7 +15529,7 @@
         <v>1201</v>
       </c>
       <c r="E250">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F250" t="s">
         <v>1279</v>
@@ -15564,7 +15564,7 @@
         <v>1201</v>
       </c>
       <c r="E251">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F251" t="s">
         <v>1279</v>
@@ -15599,7 +15599,7 @@
         <v>1202</v>
       </c>
       <c r="E252">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F252" t="s">
         <v>1279</v>
@@ -15634,7 +15634,7 @@
         <v>1203</v>
       </c>
       <c r="E253">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F253" t="s">
         <v>1279</v>
@@ -15669,7 +15669,7 @@
         <v>1203</v>
       </c>
       <c r="E254">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F254" t="s">
         <v>1279</v>
@@ -15704,7 +15704,7 @@
         <v>1203</v>
       </c>
       <c r="E255">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F255" t="s">
         <v>1279</v>
@@ -15739,7 +15739,7 @@
         <v>1203</v>
       </c>
       <c r="E256">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F256" t="s">
         <v>1279</v>
@@ -15774,7 +15774,7 @@
         <v>1204</v>
       </c>
       <c r="E257">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F257" t="s">
         <v>1279</v>
@@ -15809,7 +15809,7 @@
         <v>1204</v>
       </c>
       <c r="E258">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F258" t="s">
         <v>1279</v>
@@ -15844,7 +15844,7 @@
         <v>1204</v>
       </c>
       <c r="E259">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F259" t="s">
         <v>1279</v>
@@ -15879,7 +15879,7 @@
         <v>1205</v>
       </c>
       <c r="E260">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F260" t="s">
         <v>1279</v>
@@ -15914,7 +15914,7 @@
         <v>1206</v>
       </c>
       <c r="E261">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F261" t="s">
         <v>1279</v>
@@ -15949,7 +15949,7 @@
         <v>1206</v>
       </c>
       <c r="E262">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F262" t="s">
         <v>1279</v>
@@ -15984,7 +15984,7 @@
         <v>1206</v>
       </c>
       <c r="E263">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F263" t="s">
         <v>1279</v>
@@ -16019,7 +16019,7 @@
         <v>1207</v>
       </c>
       <c r="E264">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F264" t="s">
         <v>1279</v>
@@ -16054,7 +16054,7 @@
         <v>1207</v>
       </c>
       <c r="E265">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F265" t="s">
         <v>1279</v>
@@ -16089,7 +16089,7 @@
         <v>1207</v>
       </c>
       <c r="E266">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F266" t="s">
         <v>1279</v>
@@ -16124,7 +16124,7 @@
         <v>1208</v>
       </c>
       <c r="E267">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F267" t="s">
         <v>1279</v>
@@ -16159,7 +16159,7 @@
         <v>1209</v>
       </c>
       <c r="E268">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F268" t="s">
         <v>1279</v>
@@ -16194,7 +16194,7 @@
         <v>1210</v>
       </c>
       <c r="E269">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F269" t="s">
         <v>1279</v>
@@ -16229,7 +16229,7 @@
         <v>1210</v>
       </c>
       <c r="E270">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F270" t="s">
         <v>1279</v>
@@ -16264,7 +16264,7 @@
         <v>1210</v>
       </c>
       <c r="E271">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F271" t="s">
         <v>1279</v>
@@ -16299,7 +16299,7 @@
         <v>1210</v>
       </c>
       <c r="E272">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F272" t="s">
         <v>1279</v>
@@ -16334,7 +16334,7 @@
         <v>1211</v>
       </c>
       <c r="E273">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F273" t="s">
         <v>1279</v>
@@ -16369,7 +16369,7 @@
         <v>1212</v>
       </c>
       <c r="E274">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F274" t="s">
         <v>1279</v>
@@ -16404,7 +16404,7 @@
         <v>1212</v>
       </c>
       <c r="E275">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F275" t="s">
         <v>1279</v>
@@ -16439,7 +16439,7 @@
         <v>1213</v>
       </c>
       <c r="E276">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F276" t="s">
         <v>1279</v>
@@ -16474,7 +16474,7 @@
         <v>1214</v>
       </c>
       <c r="E277">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F277" t="s">
         <v>1279</v>
@@ -16509,7 +16509,7 @@
         <v>1215</v>
       </c>
       <c r="E278">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F278" t="s">
         <v>1279</v>
@@ -16544,7 +16544,7 @@
         <v>1215</v>
       </c>
       <c r="E279">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F279" t="s">
         <v>1279</v>
@@ -16579,7 +16579,7 @@
         <v>1216</v>
       </c>
       <c r="E280">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F280" t="s">
         <v>1279</v>
@@ -16614,7 +16614,7 @@
         <v>1216</v>
       </c>
       <c r="E281">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F281" t="s">
         <v>1279</v>
@@ -16649,7 +16649,7 @@
         <v>1216</v>
       </c>
       <c r="E282">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F282" t="s">
         <v>1279</v>
@@ -16684,7 +16684,7 @@
         <v>1217</v>
       </c>
       <c r="E283">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F283" t="s">
         <v>1279</v>
@@ -16719,7 +16719,7 @@
         <v>1217</v>
       </c>
       <c r="E284">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F284" t="s">
         <v>1279</v>
@@ -16754,7 +16754,7 @@
         <v>1217</v>
       </c>
       <c r="E285">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F285" t="s">
         <v>1279</v>
@@ -16789,7 +16789,7 @@
         <v>1217</v>
       </c>
       <c r="E286">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F286" t="s">
         <v>1279</v>
@@ -16824,7 +16824,7 @@
         <v>1217</v>
       </c>
       <c r="E287">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F287" t="s">
         <v>1279</v>
@@ -16859,7 +16859,7 @@
         <v>1217</v>
       </c>
       <c r="E288">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F288" t="s">
         <v>1279</v>
@@ -16894,7 +16894,7 @@
         <v>1217</v>
       </c>
       <c r="E289">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F289" t="s">
         <v>1279</v>
@@ -16929,7 +16929,7 @@
         <v>1217</v>
       </c>
       <c r="E290">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F290" t="s">
         <v>1279</v>
@@ -16964,7 +16964,7 @@
         <v>1218</v>
       </c>
       <c r="E291">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F291" t="s">
         <v>1279</v>
@@ -16999,7 +16999,7 @@
         <v>1218</v>
       </c>
       <c r="E292">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F292" t="s">
         <v>1279</v>
@@ -17034,7 +17034,7 @@
         <v>1218</v>
       </c>
       <c r="E293">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F293" t="s">
         <v>1279</v>
@@ -17069,7 +17069,7 @@
         <v>1219</v>
       </c>
       <c r="E294">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F294" t="s">
         <v>1279</v>
@@ -17104,7 +17104,7 @@
         <v>1220</v>
       </c>
       <c r="E295">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F295" t="s">
         <v>1279</v>
@@ -17139,7 +17139,7 @@
         <v>1220</v>
       </c>
       <c r="E296">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F296" t="s">
         <v>1279</v>
@@ -17174,7 +17174,7 @@
         <v>1220</v>
       </c>
       <c r="E297">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F297" t="s">
         <v>1279</v>
@@ -17209,7 +17209,7 @@
         <v>1220</v>
       </c>
       <c r="E298">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F298" t="s">
         <v>1283</v>
@@ -17247,7 +17247,7 @@
         <v>1220</v>
       </c>
       <c r="E299">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F299" t="s">
         <v>1279</v>
@@ -17282,7 +17282,7 @@
         <v>1220</v>
       </c>
       <c r="E300">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F300" t="s">
         <v>1279</v>
@@ -17317,7 +17317,7 @@
         <v>1221</v>
       </c>
       <c r="E301">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F301" t="s">
         <v>1279</v>
@@ -17352,7 +17352,7 @@
         <v>1221</v>
       </c>
       <c r="E302">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F302" t="s">
         <v>1279</v>
@@ -17387,7 +17387,7 @@
         <v>1221</v>
       </c>
       <c r="E303">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F303" t="s">
         <v>1279</v>
@@ -17425,7 +17425,7 @@
         <v>1221</v>
       </c>
       <c r="E304">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F304" t="s">
         <v>1279</v>
@@ -17460,7 +17460,7 @@
         <v>1221</v>
       </c>
       <c r="E305">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F305" t="s">
         <v>1279</v>
@@ -17495,7 +17495,7 @@
         <v>1221</v>
       </c>
       <c r="E306">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F306" t="s">
         <v>1279</v>
@@ -17530,7 +17530,7 @@
         <v>1221</v>
       </c>
       <c r="E307">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F307" t="s">
         <v>1279</v>
@@ -17565,7 +17565,7 @@
         <v>1221</v>
       </c>
       <c r="E308">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F308" t="s">
         <v>1279</v>
@@ -17600,7 +17600,7 @@
         <v>1222</v>
       </c>
       <c r="E309">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F309" t="s">
         <v>1280</v>
@@ -17635,7 +17635,7 @@
         <v>1223</v>
       </c>
       <c r="E310">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F310" t="s">
         <v>1283</v>
@@ -17670,7 +17670,7 @@
         <v>1224</v>
       </c>
       <c r="E311">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F311" t="s">
         <v>1279</v>
@@ -17705,7 +17705,7 @@
         <v>1224</v>
       </c>
       <c r="E312">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F312" t="s">
         <v>1279</v>
@@ -17740,7 +17740,7 @@
         <v>1225</v>
       </c>
       <c r="E313">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F313" t="s">
         <v>1279</v>
@@ -17775,7 +17775,7 @@
         <v>1226</v>
       </c>
       <c r="E314">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F314" t="s">
         <v>1282</v>
@@ -17810,7 +17810,7 @@
         <v>1226</v>
       </c>
       <c r="E315">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F315" t="s">
         <v>1279</v>
@@ -17845,7 +17845,7 @@
         <v>1226</v>
       </c>
       <c r="E316">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F316" t="s">
         <v>1279</v>
@@ -17880,7 +17880,7 @@
         <v>1226</v>
       </c>
       <c r="E317">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F317" t="s">
         <v>1279</v>
@@ -17915,7 +17915,7 @@
         <v>1227</v>
       </c>
       <c r="E318">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F318" t="s">
         <v>1279</v>
@@ -17950,7 +17950,7 @@
         <v>1228</v>
       </c>
       <c r="E319">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F319" t="s">
         <v>1279</v>
@@ -17985,7 +17985,7 @@
         <v>1228</v>
       </c>
       <c r="E320">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F320" t="s">
         <v>1279</v>
@@ -18020,7 +18020,7 @@
         <v>1229</v>
       </c>
       <c r="E321">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F321" t="s">
         <v>1279</v>
@@ -18055,7 +18055,7 @@
         <v>1230</v>
       </c>
       <c r="E322">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F322" t="s">
         <v>1279</v>
@@ -18090,7 +18090,7 @@
         <v>1230</v>
       </c>
       <c r="E323">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F323" t="s">
         <v>1279</v>
@@ -18125,7 +18125,7 @@
         <v>1230</v>
       </c>
       <c r="E324">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F324" t="s">
         <v>1279</v>
@@ -18160,7 +18160,7 @@
         <v>1230</v>
       </c>
       <c r="E325">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F325" t="s">
         <v>1279</v>
@@ -18195,7 +18195,7 @@
         <v>1230</v>
       </c>
       <c r="E326">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F326" t="s">
         <v>1279</v>
@@ -18230,7 +18230,7 @@
         <v>1230</v>
       </c>
       <c r="E327">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F327" t="s">
         <v>1279</v>
@@ -18265,7 +18265,7 @@
         <v>1230</v>
       </c>
       <c r="E328">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F328" t="s">
         <v>1279</v>
@@ -18300,7 +18300,7 @@
         <v>1231</v>
       </c>
       <c r="E329">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F329" t="s">
         <v>1279</v>
@@ -18335,7 +18335,7 @@
         <v>1231</v>
       </c>
       <c r="E330">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F330" t="s">
         <v>1279</v>
@@ -18370,7 +18370,7 @@
         <v>1231</v>
       </c>
       <c r="E331">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F331" t="s">
         <v>1280</v>
@@ -18405,7 +18405,7 @@
         <v>1232</v>
       </c>
       <c r="E332">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F332" t="s">
         <v>1279</v>
@@ -18440,7 +18440,7 @@
         <v>1232</v>
       </c>
       <c r="E333">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F333" t="s">
         <v>1279</v>
@@ -18475,7 +18475,7 @@
         <v>1232</v>
       </c>
       <c r="E334">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F334" t="s">
         <v>1279</v>
@@ -18510,7 +18510,7 @@
         <v>1232</v>
       </c>
       <c r="E335">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F335" t="s">
         <v>1279</v>
@@ -18545,7 +18545,7 @@
         <v>1232</v>
       </c>
       <c r="E336">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F336" t="s">
         <v>1279</v>
@@ -18580,7 +18580,7 @@
         <v>1232</v>
       </c>
       <c r="E337">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F337" t="s">
         <v>1282</v>
@@ -18615,7 +18615,7 @@
         <v>1233</v>
       </c>
       <c r="E338">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F338" t="s">
         <v>1279</v>
@@ -18650,7 +18650,7 @@
         <v>1233</v>
       </c>
       <c r="E339">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F339" t="s">
         <v>1279</v>
@@ -18685,7 +18685,7 @@
         <v>1233</v>
       </c>
       <c r="E340">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F340" t="s">
         <v>1279</v>
@@ -18720,7 +18720,7 @@
         <v>1234</v>
       </c>
       <c r="E341">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F341" t="s">
         <v>1282</v>
@@ -18755,7 +18755,7 @@
         <v>1234</v>
       </c>
       <c r="E342">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F342" t="s">
         <v>1279</v>
@@ -18790,7 +18790,7 @@
         <v>1234</v>
       </c>
       <c r="E343">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F343" t="s">
         <v>1279</v>
@@ -18825,7 +18825,7 @@
         <v>1235</v>
       </c>
       <c r="E344">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F344" t="s">
         <v>1279</v>
@@ -18860,7 +18860,7 @@
         <v>1235</v>
       </c>
       <c r="E345">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F345" t="s">
         <v>1279</v>
@@ -18895,7 +18895,7 @@
         <v>1235</v>
       </c>
       <c r="E346">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F346" t="s">
         <v>1279</v>
@@ -18930,7 +18930,7 @@
         <v>1235</v>
       </c>
       <c r="E347">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F347" t="s">
         <v>1279</v>
@@ -18965,7 +18965,7 @@
         <v>1235</v>
       </c>
       <c r="E348">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F348" t="s">
         <v>1281</v>
@@ -19000,7 +19000,7 @@
         <v>1235</v>
       </c>
       <c r="E349">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F349" t="s">
         <v>1279</v>
@@ -19035,7 +19035,7 @@
         <v>1236</v>
       </c>
       <c r="E350">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F350" t="s">
         <v>1279</v>
@@ -19070,7 +19070,7 @@
         <v>1236</v>
       </c>
       <c r="E351">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F351" t="s">
         <v>1279</v>
@@ -19105,7 +19105,7 @@
         <v>1236</v>
       </c>
       <c r="E352">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F352" t="s">
         <v>1279</v>
@@ -19140,7 +19140,7 @@
         <v>1236</v>
       </c>
       <c r="E353">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F353" t="s">
         <v>1279</v>
@@ -19175,7 +19175,7 @@
         <v>1237</v>
       </c>
       <c r="E354">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F354" t="s">
         <v>1279</v>
@@ -19210,7 +19210,7 @@
         <v>1237</v>
       </c>
       <c r="E355">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F355" t="s">
         <v>1279</v>
@@ -19245,7 +19245,7 @@
         <v>1237</v>
       </c>
       <c r="E356">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F356" t="s">
         <v>1279</v>
@@ -19280,7 +19280,7 @@
         <v>1237</v>
       </c>
       <c r="E357">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F357" t="s">
         <v>1279</v>
@@ -19315,7 +19315,7 @@
         <v>1237</v>
       </c>
       <c r="E358">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F358" t="s">
         <v>1279</v>
@@ -19353,7 +19353,7 @@
         <v>1238</v>
       </c>
       <c r="E359">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F359" t="s">
         <v>1279</v>
@@ -19388,7 +19388,7 @@
         <v>1238</v>
       </c>
       <c r="E360">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F360" t="s">
         <v>1279</v>
@@ -19423,7 +19423,7 @@
         <v>1238</v>
       </c>
       <c r="E361">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F361" t="s">
         <v>1279</v>
@@ -19458,7 +19458,7 @@
         <v>1238</v>
       </c>
       <c r="E362">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F362" t="s">
         <v>1279</v>
@@ -19493,7 +19493,7 @@
         <v>1238</v>
       </c>
       <c r="E363">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F363" t="s">
         <v>1279</v>
@@ -19528,7 +19528,7 @@
         <v>1238</v>
       </c>
       <c r="E364">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F364" t="s">
         <v>1279</v>
@@ -19563,7 +19563,7 @@
         <v>1239</v>
       </c>
       <c r="E365">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F365" t="s">
         <v>1280</v>
@@ -19598,7 +19598,7 @@
         <v>1240</v>
       </c>
       <c r="E366">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F366" t="s">
         <v>1279</v>
@@ -19633,7 +19633,7 @@
         <v>1241</v>
       </c>
       <c r="E367">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F367" t="s">
         <v>1281</v>
@@ -19671,7 +19671,7 @@
         <v>1242</v>
       </c>
       <c r="E368">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F368" t="s">
         <v>1279</v>
@@ -19706,7 +19706,7 @@
         <v>1242</v>
       </c>
       <c r="E369">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F369" t="s">
         <v>1279</v>
@@ -19741,7 +19741,7 @@
         <v>1242</v>
       </c>
       <c r="E370">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F370" t="s">
         <v>1279</v>
@@ -19776,7 +19776,7 @@
         <v>1243</v>
       </c>
       <c r="E371">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F371" t="s">
         <v>1279</v>
@@ -19811,7 +19811,7 @@
         <v>1243</v>
       </c>
       <c r="E372">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F372" t="s">
         <v>1279</v>
@@ -19846,7 +19846,7 @@
         <v>1244</v>
       </c>
       <c r="E373">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F373" t="s">
         <v>1279</v>
@@ -19881,7 +19881,7 @@
         <v>1244</v>
       </c>
       <c r="E374">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F374" t="s">
         <v>1283</v>
@@ -19919,7 +19919,7 @@
         <v>1244</v>
       </c>
       <c r="E375">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F375" t="s">
         <v>1279</v>
@@ -19954,7 +19954,7 @@
         <v>1244</v>
       </c>
       <c r="E376">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F376" t="s">
         <v>1283</v>
@@ -19989,7 +19989,7 @@
         <v>1245</v>
       </c>
       <c r="E377">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F377" t="s">
         <v>1279</v>
@@ -20024,7 +20024,7 @@
         <v>1246</v>
       </c>
       <c r="E378">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F378" t="s">
         <v>1279</v>
@@ -20059,7 +20059,7 @@
         <v>1246</v>
       </c>
       <c r="E379">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F379" t="s">
         <v>1279</v>
@@ -20094,7 +20094,7 @@
         <v>1246</v>
       </c>
       <c r="E380">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F380" t="s">
         <v>1279</v>
@@ -20129,7 +20129,7 @@
         <v>1246</v>
       </c>
       <c r="E381">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F381" t="s">
         <v>1279</v>
@@ -20164,7 +20164,7 @@
         <v>1247</v>
       </c>
       <c r="E382">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F382" t="s">
         <v>1283</v>
@@ -20199,7 +20199,7 @@
         <v>1247</v>
       </c>
       <c r="E383">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F383" t="s">
         <v>1279</v>
@@ -20234,7 +20234,7 @@
         <v>1247</v>
       </c>
       <c r="E384">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F384" t="s">
         <v>1279</v>
@@ -20269,7 +20269,7 @@
         <v>1248</v>
       </c>
       <c r="E385">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F385" t="s">
         <v>1279</v>
@@ -20304,7 +20304,7 @@
         <v>1249</v>
       </c>
       <c r="E386">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F386" t="s">
         <v>1279</v>
@@ -20339,7 +20339,7 @@
         <v>1249</v>
       </c>
       <c r="E387">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F387" t="s">
         <v>1279</v>
@@ -20374,7 +20374,7 @@
         <v>1250</v>
       </c>
       <c r="E388">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F388" t="s">
         <v>1279</v>
@@ -20409,7 +20409,7 @@
         <v>1250</v>
       </c>
       <c r="E389">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F389" t="s">
         <v>1279</v>
@@ -20444,7 +20444,7 @@
         <v>1250</v>
       </c>
       <c r="E390">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F390" t="s">
         <v>1279</v>
@@ -20479,7 +20479,7 @@
         <v>1250</v>
       </c>
       <c r="E391">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F391" t="s">
         <v>1279</v>
@@ -20514,7 +20514,7 @@
         <v>1250</v>
       </c>
       <c r="E392">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F392" t="s">
         <v>1279</v>
@@ -20549,7 +20549,7 @@
         <v>1250</v>
       </c>
       <c r="E393">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F393" t="s">
         <v>1279</v>
@@ -20584,7 +20584,7 @@
         <v>1250</v>
       </c>
       <c r="E394">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F394" t="s">
         <v>1279</v>
@@ -20619,7 +20619,7 @@
         <v>1250</v>
       </c>
       <c r="E395">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F395" t="s">
         <v>1279</v>
@@ -20654,7 +20654,7 @@
         <v>1250</v>
       </c>
       <c r="E396">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F396" t="s">
         <v>1279</v>
@@ -20689,7 +20689,7 @@
         <v>1250</v>
       </c>
       <c r="E397">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F397" t="s">
         <v>1279</v>
@@ -20724,7 +20724,7 @@
         <v>1250</v>
       </c>
       <c r="E398">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F398" t="s">
         <v>1279</v>
@@ -20759,7 +20759,7 @@
         <v>1250</v>
       </c>
       <c r="E399">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F399" t="s">
         <v>1279</v>
@@ -20794,7 +20794,7 @@
         <v>1250</v>
       </c>
       <c r="E400">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F400" t="s">
         <v>1279</v>
@@ -20829,7 +20829,7 @@
         <v>1250</v>
       </c>
       <c r="E401">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F401" t="s">
         <v>1279</v>
@@ -20864,7 +20864,7 @@
         <v>1250</v>
       </c>
       <c r="E402">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F402" t="s">
         <v>1279</v>
@@ -20899,7 +20899,7 @@
         <v>1250</v>
       </c>
       <c r="E403">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F403" t="s">
         <v>1279</v>
@@ -20934,7 +20934,7 @@
         <v>1250</v>
       </c>
       <c r="E404">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F404" t="s">
         <v>1279</v>
@@ -20969,7 +20969,7 @@
         <v>1250</v>
       </c>
       <c r="E405">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F405" t="s">
         <v>1279</v>
@@ -21004,7 +21004,7 @@
         <v>1250</v>
       </c>
       <c r="E406">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F406" t="s">
         <v>1279</v>
@@ -21039,7 +21039,7 @@
         <v>1250</v>
       </c>
       <c r="E407">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F407" t="s">
         <v>1279</v>
@@ -21074,7 +21074,7 @@
         <v>1250</v>
       </c>
       <c r="E408">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F408" t="s">
         <v>1279</v>
@@ -21109,7 +21109,7 @@
         <v>1250</v>
       </c>
       <c r="E409">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F409" t="s">
         <v>1279</v>
@@ -21144,7 +21144,7 @@
         <v>1251</v>
       </c>
       <c r="E410">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F410" t="s">
         <v>1279</v>
@@ -21179,7 +21179,7 @@
         <v>1251</v>
       </c>
       <c r="E411">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F411" t="s">
         <v>1279</v>
@@ -21214,7 +21214,7 @@
         <v>1251</v>
       </c>
       <c r="E412">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F412" t="s">
         <v>1283</v>
@@ -21249,7 +21249,7 @@
         <v>1252</v>
       </c>
       <c r="E413">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F413" t="s">
         <v>1279</v>
@@ -21284,7 +21284,7 @@
         <v>1253</v>
       </c>
       <c r="E414">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F414" t="s">
         <v>1281</v>
@@ -21322,7 +21322,7 @@
         <v>1253</v>
       </c>
       <c r="E415">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F415" t="s">
         <v>1279</v>
@@ -21357,7 +21357,7 @@
         <v>1253</v>
       </c>
       <c r="E416">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F416" t="s">
         <v>1279</v>
@@ -21392,7 +21392,7 @@
         <v>1253</v>
       </c>
       <c r="E417">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F417" t="s">
         <v>1279</v>
@@ -21427,7 +21427,7 @@
         <v>1254</v>
       </c>
       <c r="E418">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F418" t="s">
         <v>1279</v>
@@ -21465,7 +21465,7 @@
         <v>1254</v>
       </c>
       <c r="E419">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F419" t="s">
         <v>1283</v>
@@ -21500,7 +21500,7 @@
         <v>1254</v>
       </c>
       <c r="E420">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F420" t="s">
         <v>1281</v>
@@ -21535,7 +21535,7 @@
         <v>1254</v>
       </c>
       <c r="E421">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F421" t="s">
         <v>1279</v>
@@ -21570,7 +21570,7 @@
         <v>1254</v>
       </c>
       <c r="E422">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F422" t="s">
         <v>1279</v>
@@ -21605,7 +21605,7 @@
         <v>1254</v>
       </c>
       <c r="E423">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F423" t="s">
         <v>1279</v>
@@ -21640,7 +21640,7 @@
         <v>1254</v>
       </c>
       <c r="E424">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F424" t="s">
         <v>1279</v>
@@ -21675,7 +21675,7 @@
         <v>1255</v>
       </c>
       <c r="E425">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F425" t="s">
         <v>1283</v>
@@ -21713,7 +21713,7 @@
         <v>1256</v>
       </c>
       <c r="E426">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F426" t="s">
         <v>1279</v>
@@ -21748,7 +21748,7 @@
         <v>1256</v>
       </c>
       <c r="E427">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F427" t="s">
         <v>1279</v>
@@ -21783,7 +21783,7 @@
         <v>1256</v>
       </c>
       <c r="E428">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F428" t="s">
         <v>1279</v>
@@ -21818,7 +21818,7 @@
         <v>1257</v>
       </c>
       <c r="E429">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F429" t="s">
         <v>1279</v>
@@ -21853,7 +21853,7 @@
         <v>1257</v>
       </c>
       <c r="E430">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F430" t="s">
         <v>1279</v>
@@ -21888,7 +21888,7 @@
         <v>1257</v>
       </c>
       <c r="E431">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F431" t="s">
         <v>1279</v>
@@ -21923,7 +21923,7 @@
         <v>1257</v>
       </c>
       <c r="E432">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F432" t="s">
         <v>1281</v>
@@ -21958,7 +21958,7 @@
         <v>1257</v>
       </c>
       <c r="E433">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F433" t="s">
         <v>1279</v>
@@ -21993,7 +21993,7 @@
         <v>1258</v>
       </c>
       <c r="E434">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F434" t="s">
         <v>1279</v>
@@ -22028,7 +22028,7 @@
         <v>1258</v>
       </c>
       <c r="E435">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F435" t="s">
         <v>1279</v>
@@ -22063,7 +22063,7 @@
         <v>1258</v>
       </c>
       <c r="E436">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F436" t="s">
         <v>1279</v>
@@ -22098,7 +22098,7 @@
         <v>1258</v>
       </c>
       <c r="E437">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F437" t="s">
         <v>1279</v>
@@ -22133,7 +22133,7 @@
         <v>1258</v>
       </c>
       <c r="E438">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F438" t="s">
         <v>1279</v>
@@ -22171,7 +22171,7 @@
         <v>1258</v>
       </c>
       <c r="E439">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F439" t="s">
         <v>1281</v>
@@ -22209,7 +22209,7 @@
         <v>1258</v>
       </c>
       <c r="E440">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F440" t="s">
         <v>1281</v>
@@ -22244,7 +22244,7 @@
         <v>1259</v>
       </c>
       <c r="E441">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F441" t="s">
         <v>1279</v>
@@ -22279,7 +22279,7 @@
         <v>1259</v>
       </c>
       <c r="E442">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F442" t="s">
         <v>1279</v>
@@ -22314,7 +22314,7 @@
         <v>1259</v>
       </c>
       <c r="E443">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F443" t="s">
         <v>1279</v>
@@ -22349,7 +22349,7 @@
         <v>1260</v>
       </c>
       <c r="E444">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F444" t="s">
         <v>1279</v>
@@ -22384,7 +22384,7 @@
         <v>1260</v>
       </c>
       <c r="E445">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F445" t="s">
         <v>1279</v>
@@ -22419,7 +22419,7 @@
         <v>1260</v>
       </c>
       <c r="E446">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F446" t="s">
         <v>1281</v>
@@ -22457,7 +22457,7 @@
         <v>1260</v>
       </c>
       <c r="E447">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F447" t="s">
         <v>1279</v>
@@ -22492,7 +22492,7 @@
         <v>1261</v>
       </c>
       <c r="E448">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F448" t="s">
         <v>1279</v>
@@ -22527,7 +22527,7 @@
         <v>1261</v>
       </c>
       <c r="E449">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F449" t="s">
         <v>1279</v>
@@ -22562,7 +22562,7 @@
         <v>1262</v>
       </c>
       <c r="E450">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F450" t="s">
         <v>1281</v>
@@ -22600,7 +22600,7 @@
         <v>1262</v>
       </c>
       <c r="E451">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F451" t="s">
         <v>1279</v>
@@ -22635,7 +22635,7 @@
         <v>1262</v>
       </c>
       <c r="E452">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F452" t="s">
         <v>1279</v>
@@ -22670,7 +22670,7 @@
         <v>1263</v>
       </c>
       <c r="E453">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F453" t="s">
         <v>1281</v>
@@ -22705,7 +22705,7 @@
         <v>1263</v>
       </c>
       <c r="E454">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F454" t="s">
         <v>1279</v>
@@ -22740,7 +22740,7 @@
         <v>1263</v>
       </c>
       <c r="E455">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F455" t="s">
         <v>1281</v>
@@ -22778,7 +22778,7 @@
         <v>1263</v>
       </c>
       <c r="E456">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F456" t="s">
         <v>1279</v>
@@ -22813,7 +22813,7 @@
         <v>1263</v>
       </c>
       <c r="E457">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F457" t="s">
         <v>1279</v>
@@ -22848,7 +22848,7 @@
         <v>1264</v>
       </c>
       <c r="E458">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F458" t="s">
         <v>1279</v>
@@ -22883,7 +22883,7 @@
         <v>1264</v>
       </c>
       <c r="E459">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F459" t="s">
         <v>1279</v>
@@ -22918,7 +22918,7 @@
         <v>1265</v>
       </c>
       <c r="E460">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F460" t="s">
         <v>1279</v>
@@ -22953,7 +22953,7 @@
         <v>1265</v>
       </c>
       <c r="E461">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F461" t="s">
         <v>1279</v>
@@ -22988,7 +22988,7 @@
         <v>1265</v>
       </c>
       <c r="E462">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F462" t="s">
         <v>1279</v>
@@ -23023,7 +23023,7 @@
         <v>1265</v>
       </c>
       <c r="E463">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F463" t="s">
         <v>1281</v>
@@ -23061,7 +23061,7 @@
         <v>1266</v>
       </c>
       <c r="E464">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F464" t="s">
         <v>1279</v>
@@ -23096,7 +23096,7 @@
         <v>1266</v>
       </c>
       <c r="E465">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F465" t="s">
         <v>1283</v>
@@ -23134,7 +23134,7 @@
         <v>1266</v>
       </c>
       <c r="E466">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F466" t="s">
         <v>1279</v>
@@ -23169,7 +23169,7 @@
         <v>1266</v>
       </c>
       <c r="E467">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F467" t="s">
         <v>1279</v>
@@ -23204,7 +23204,7 @@
         <v>1267</v>
       </c>
       <c r="E468">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F468" t="s">
         <v>1279</v>
@@ -23239,7 +23239,7 @@
         <v>1267</v>
       </c>
       <c r="E469">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F469" t="s">
         <v>1279</v>
@@ -23274,7 +23274,7 @@
         <v>1267</v>
       </c>
       <c r="E470">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F470" t="s">
         <v>1279</v>
@@ -23309,7 +23309,7 @@
         <v>1267</v>
       </c>
       <c r="E471">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F471" t="s">
         <v>1279</v>
@@ -23344,7 +23344,7 @@
         <v>1267</v>
       </c>
       <c r="E472">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F472" t="s">
         <v>1279</v>
@@ -23379,7 +23379,7 @@
         <v>1267</v>
       </c>
       <c r="E473">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F473" t="s">
         <v>1281</v>
@@ -23417,7 +23417,7 @@
         <v>1268</v>
       </c>
       <c r="E474">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F474" t="s">
         <v>1279</v>
@@ -23452,7 +23452,7 @@
         <v>1268</v>
       </c>
       <c r="E475">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F475" t="s">
         <v>1281</v>
@@ -23487,7 +23487,7 @@
         <v>1269</v>
       </c>
       <c r="E476">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F476" t="s">
         <v>1281</v>
@@ -23525,7 +23525,7 @@
         <v>1269</v>
       </c>
       <c r="E477">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F477" t="s">
         <v>1281</v>
@@ -23563,7 +23563,7 @@
         <v>1269</v>
       </c>
       <c r="E478">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F478" t="s">
         <v>1279</v>
@@ -23598,7 +23598,7 @@
         <v>1269</v>
       </c>
       <c r="E479">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F479" t="s">
         <v>1279</v>
@@ -23633,7 +23633,7 @@
         <v>1270</v>
       </c>
       <c r="E480">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F480" t="s">
         <v>1279</v>
@@ -23668,7 +23668,7 @@
         <v>1271</v>
       </c>
       <c r="E481">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F481" t="s">
         <v>1279</v>
@@ -23703,7 +23703,7 @@
         <v>1271</v>
       </c>
       <c r="E482">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F482" t="s">
         <v>1279</v>
@@ -23738,7 +23738,7 @@
         <v>1271</v>
       </c>
       <c r="E483">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F483" t="s">
         <v>1279</v>
@@ -23773,7 +23773,7 @@
         <v>1271</v>
       </c>
       <c r="E484">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F484" t="s">
         <v>1279</v>
@@ -23808,7 +23808,7 @@
         <v>1271</v>
       </c>
       <c r="E485">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F485" t="s">
         <v>1279</v>
@@ -23843,7 +23843,7 @@
         <v>1271</v>
       </c>
       <c r="E486">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F486" t="s">
         <v>1279</v>
@@ -23878,7 +23878,7 @@
         <v>1271</v>
       </c>
       <c r="E487">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F487" t="s">
         <v>1279</v>
@@ -23913,7 +23913,7 @@
         <v>1271</v>
       </c>
       <c r="E488">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F488" t="s">
         <v>1281</v>
@@ -23951,7 +23951,7 @@
         <v>1272</v>
       </c>
       <c r="E489">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F489" t="s">
         <v>1279</v>
@@ -23986,7 +23986,7 @@
         <v>1272</v>
       </c>
       <c r="E490">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F490" t="s">
         <v>1279</v>
@@ -24021,7 +24021,7 @@
         <v>1272</v>
       </c>
       <c r="E491">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F491" t="s">
         <v>1279</v>
@@ -24056,7 +24056,7 @@
         <v>1272</v>
       </c>
       <c r="E492">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F492" t="s">
         <v>1281</v>
@@ -24094,7 +24094,7 @@
         <v>1272</v>
       </c>
       <c r="E493">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F493" t="s">
         <v>1281</v>
@@ -24132,7 +24132,7 @@
         <v>1272</v>
       </c>
       <c r="E494">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F494" t="s">
         <v>1281</v>
@@ -24170,7 +24170,7 @@
         <v>1272</v>
       </c>
       <c r="E495">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F495" t="s">
         <v>1279</v>
@@ -24205,7 +24205,7 @@
         <v>1273</v>
       </c>
       <c r="E496">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F496" t="s">
         <v>1281</v>
@@ -24243,7 +24243,7 @@
         <v>1273</v>
       </c>
       <c r="E497">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F497" t="s">
         <v>1281</v>
@@ -24281,7 +24281,7 @@
         <v>1274</v>
       </c>
       <c r="E498">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F498" t="s">
         <v>1281</v>
@@ -24319,7 +24319,7 @@
         <v>1274</v>
       </c>
       <c r="E499">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F499" t="s">
         <v>1279</v>
@@ -24354,7 +24354,7 @@
         <v>1275</v>
       </c>
       <c r="E500">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F500" t="s">
         <v>1279</v>
@@ -24389,7 +24389,7 @@
         <v>1275</v>
       </c>
       <c r="E501">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F501" t="s">
         <v>1279</v>
@@ -24427,7 +24427,7 @@
         <v>1275</v>
       </c>
       <c r="E502">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F502" t="s">
         <v>1281</v>
@@ -24465,7 +24465,7 @@
         <v>1276</v>
       </c>
       <c r="E503">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F503" t="s">
         <v>1279</v>
@@ -24503,7 +24503,7 @@
         <v>1276</v>
       </c>
       <c r="E504">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F504" t="s">
         <v>1279</v>
@@ -24538,7 +24538,7 @@
         <v>1276</v>
       </c>
       <c r="E505">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F505" t="s">
         <v>1279</v>
@@ -24573,7 +24573,7 @@
         <v>1276</v>
       </c>
       <c r="E506">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F506" t="s">
         <v>1279</v>
@@ -24608,7 +24608,7 @@
         <v>1276</v>
       </c>
       <c r="E507">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F507" t="s">
         <v>1279</v>
@@ -24643,7 +24643,7 @@
         <v>1276</v>
       </c>
       <c r="E508">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F508" t="s">
         <v>1281</v>
@@ -24681,7 +24681,7 @@
         <v>1277</v>
       </c>
       <c r="E509">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F509" t="s">
         <v>1279</v>
@@ -24716,7 +24716,7 @@
         <v>1277</v>
       </c>
       <c r="E510">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F510" t="s">
         <v>1279</v>
@@ -24751,7 +24751,7 @@
         <v>1277</v>
       </c>
       <c r="E511">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F511" t="s">
         <v>1279</v>
@@ -24786,7 +24786,7 @@
         <v>1277</v>
       </c>
       <c r="E512">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F512" t="s">
         <v>1279</v>
@@ -24821,7 +24821,7 @@
         <v>1277</v>
       </c>
       <c r="E513">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F513" t="s">
         <v>1279</v>
@@ -24856,7 +24856,7 @@
         <v>1277</v>
       </c>
       <c r="E514">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F514" t="s">
         <v>1279</v>
@@ -24891,7 +24891,7 @@
         <v>1278</v>
       </c>
       <c r="E515">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F515" t="s">
         <v>1279</v>
@@ -24929,7 +24929,7 @@
         <v>1278</v>
       </c>
       <c r="E516">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F516" t="s">
         <v>1279</v>
@@ -24964,7 +24964,7 @@
         <v>1278</v>
       </c>
       <c r="E517">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F517" t="s">
         <v>1279</v>
@@ -24999,7 +24999,7 @@
         <v>1278</v>
       </c>
       <c r="E518">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F518" t="s">
         <v>1279</v>
@@ -25037,7 +25037,7 @@
         <v>1278</v>
       </c>
       <c r="E519">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F519" t="s">
         <v>1279</v>
@@ -25072,7 +25072,7 @@
         <v>1278</v>
       </c>
       <c r="E520">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F520" t="s">
         <v>1281</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-21 00:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -6834,7 +6834,7 @@
         <v>1073</v>
       </c>
       <c r="E2">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="F2" t="s">
         <v>1279</v>
@@ -6869,7 +6869,7 @@
         <v>1074</v>
       </c>
       <c r="E3">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F3" t="s">
         <v>1279</v>
@@ -6904,7 +6904,7 @@
         <v>1075</v>
       </c>
       <c r="E4">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F4" t="s">
         <v>1279</v>
@@ -6939,7 +6939,7 @@
         <v>1076</v>
       </c>
       <c r="E5">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F5" t="s">
         <v>1279</v>
@@ -6974,7 +6974,7 @@
         <v>1077</v>
       </c>
       <c r="E6">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F6" t="s">
         <v>1279</v>
@@ -7009,7 +7009,7 @@
         <v>1078</v>
       </c>
       <c r="E7">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F7" t="s">
         <v>1279</v>
@@ -7044,7 +7044,7 @@
         <v>1079</v>
       </c>
       <c r="E8">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="F8" t="s">
         <v>1279</v>
@@ -7079,7 +7079,7 @@
         <v>1080</v>
       </c>
       <c r="E9">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="F9" t="s">
         <v>1279</v>
@@ -7114,7 +7114,7 @@
         <v>1081</v>
       </c>
       <c r="E10">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F10" t="s">
         <v>1279</v>
@@ -7149,7 +7149,7 @@
         <v>1081</v>
       </c>
       <c r="E11">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F11" t="s">
         <v>1279</v>
@@ -7184,7 +7184,7 @@
         <v>1082</v>
       </c>
       <c r="E12">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F12" t="s">
         <v>1279</v>
@@ -7219,7 +7219,7 @@
         <v>1083</v>
       </c>
       <c r="E13">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F13" t="s">
         <v>1279</v>
@@ -7254,7 +7254,7 @@
         <v>1084</v>
       </c>
       <c r="E14">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F14" t="s">
         <v>1279</v>
@@ -7289,7 +7289,7 @@
         <v>1084</v>
       </c>
       <c r="E15">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F15" t="s">
         <v>1279</v>
@@ -7324,7 +7324,7 @@
         <v>1085</v>
       </c>
       <c r="E16">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F16" t="s">
         <v>1279</v>
@@ -7359,7 +7359,7 @@
         <v>1085</v>
       </c>
       <c r="E17">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F17" t="s">
         <v>1279</v>
@@ -7394,7 +7394,7 @@
         <v>1086</v>
       </c>
       <c r="E18">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F18" t="s">
         <v>1279</v>
@@ -7429,7 +7429,7 @@
         <v>1087</v>
       </c>
       <c r="E19">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F19" t="s">
         <v>1279</v>
@@ -7464,7 +7464,7 @@
         <v>1088</v>
       </c>
       <c r="E20">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F20" t="s">
         <v>1279</v>
@@ -7499,7 +7499,7 @@
         <v>1089</v>
       </c>
       <c r="E21">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F21" t="s">
         <v>1279</v>
@@ -7534,7 +7534,7 @@
         <v>1090</v>
       </c>
       <c r="E22">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F22" t="s">
         <v>1279</v>
@@ -7572,7 +7572,7 @@
         <v>1091</v>
       </c>
       <c r="E23">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F23" t="s">
         <v>1279</v>
@@ -7607,7 +7607,7 @@
         <v>1092</v>
       </c>
       <c r="E24">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F24" t="s">
         <v>1279</v>
@@ -7642,7 +7642,7 @@
         <v>1093</v>
       </c>
       <c r="E25">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F25" t="s">
         <v>1279</v>
@@ -7677,7 +7677,7 @@
         <v>1094</v>
       </c>
       <c r="E26">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F26" t="s">
         <v>1279</v>
@@ -7712,7 +7712,7 @@
         <v>1095</v>
       </c>
       <c r="E27">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F27" t="s">
         <v>1279</v>
@@ -7747,7 +7747,7 @@
         <v>1096</v>
       </c>
       <c r="E28">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F28" t="s">
         <v>1279</v>
@@ -7782,7 +7782,7 @@
         <v>1097</v>
       </c>
       <c r="E29">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F29" t="s">
         <v>1279</v>
@@ -7817,7 +7817,7 @@
         <v>1098</v>
       </c>
       <c r="E30">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F30" t="s">
         <v>1279</v>
@@ -7852,7 +7852,7 @@
         <v>1099</v>
       </c>
       <c r="E31">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F31" t="s">
         <v>1279</v>
@@ -7887,7 +7887,7 @@
         <v>1100</v>
       </c>
       <c r="E32">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F32" t="s">
         <v>1279</v>
@@ -7922,7 +7922,7 @@
         <v>1101</v>
       </c>
       <c r="E33">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F33" t="s">
         <v>1279</v>
@@ -7957,7 +7957,7 @@
         <v>1102</v>
       </c>
       <c r="E34">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F34" t="s">
         <v>1279</v>
@@ -7992,7 +7992,7 @@
         <v>1103</v>
       </c>
       <c r="E35">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F35" t="s">
         <v>1279</v>
@@ -8027,7 +8027,7 @@
         <v>1104</v>
       </c>
       <c r="E36">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F36" t="s">
         <v>1279</v>
@@ -8062,7 +8062,7 @@
         <v>1104</v>
       </c>
       <c r="E37">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F37" t="s">
         <v>1279</v>
@@ -8097,7 +8097,7 @@
         <v>1105</v>
       </c>
       <c r="E38">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F38" t="s">
         <v>1279</v>
@@ -8132,7 +8132,7 @@
         <v>1106</v>
       </c>
       <c r="E39">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F39" t="s">
         <v>1279</v>
@@ -8167,7 +8167,7 @@
         <v>1107</v>
       </c>
       <c r="E40">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F40" t="s">
         <v>1279</v>
@@ -8202,7 +8202,7 @@
         <v>1107</v>
       </c>
       <c r="E41">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F41" t="s">
         <v>1279</v>
@@ -8237,7 +8237,7 @@
         <v>1108</v>
       </c>
       <c r="E42">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F42" t="s">
         <v>1279</v>
@@ -8272,7 +8272,7 @@
         <v>1108</v>
       </c>
       <c r="E43">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F43" t="s">
         <v>1279</v>
@@ -8307,7 +8307,7 @@
         <v>1109</v>
       </c>
       <c r="E44">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F44" t="s">
         <v>1279</v>
@@ -8342,7 +8342,7 @@
         <v>1110</v>
       </c>
       <c r="E45">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="F45" t="s">
         <v>1279</v>
@@ -8377,7 +8377,7 @@
         <v>1111</v>
       </c>
       <c r="E46">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F46" t="s">
         <v>1279</v>
@@ -8412,7 +8412,7 @@
         <v>1112</v>
       </c>
       <c r="E47">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F47" t="s">
         <v>1279</v>
@@ -8447,7 +8447,7 @@
         <v>1112</v>
       </c>
       <c r="E48">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F48" t="s">
         <v>1279</v>
@@ -8482,7 +8482,7 @@
         <v>1113</v>
       </c>
       <c r="E49">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F49" t="s">
         <v>1279</v>
@@ -8517,7 +8517,7 @@
         <v>1114</v>
       </c>
       <c r="E50">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F50" t="s">
         <v>1279</v>
@@ -8552,7 +8552,7 @@
         <v>1115</v>
       </c>
       <c r="E51">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F51" t="s">
         <v>1279</v>
@@ -8587,7 +8587,7 @@
         <v>1116</v>
       </c>
       <c r="E52">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F52" t="s">
         <v>1279</v>
@@ -8622,7 +8622,7 @@
         <v>1117</v>
       </c>
       <c r="E53">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F53" t="s">
         <v>1279</v>
@@ -8657,7 +8657,7 @@
         <v>1118</v>
       </c>
       <c r="E54">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F54" t="s">
         <v>1279</v>
@@ -8692,7 +8692,7 @@
         <v>1119</v>
       </c>
       <c r="E55">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F55" t="s">
         <v>1279</v>
@@ -8727,7 +8727,7 @@
         <v>1119</v>
       </c>
       <c r="E56">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F56" t="s">
         <v>1279</v>
@@ -8762,7 +8762,7 @@
         <v>1119</v>
       </c>
       <c r="E57">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F57" t="s">
         <v>1279</v>
@@ -8797,7 +8797,7 @@
         <v>1120</v>
       </c>
       <c r="E58">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F58" t="s">
         <v>1279</v>
@@ -8832,7 +8832,7 @@
         <v>1121</v>
       </c>
       <c r="E59">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F59" t="s">
         <v>1279</v>
@@ -8867,7 +8867,7 @@
         <v>1122</v>
       </c>
       <c r="E60">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F60" t="s">
         <v>1279</v>
@@ -8902,7 +8902,7 @@
         <v>1122</v>
       </c>
       <c r="E61">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F61" t="s">
         <v>1279</v>
@@ -8937,7 +8937,7 @@
         <v>1123</v>
       </c>
       <c r="E62">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F62" t="s">
         <v>1279</v>
@@ -8972,7 +8972,7 @@
         <v>1124</v>
       </c>
       <c r="E63">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F63" t="s">
         <v>1279</v>
@@ -9007,7 +9007,7 @@
         <v>1124</v>
       </c>
       <c r="E64">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F64" t="s">
         <v>1279</v>
@@ -9042,7 +9042,7 @@
         <v>1124</v>
       </c>
       <c r="E65">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F65" t="s">
         <v>1279</v>
@@ -9077,7 +9077,7 @@
         <v>1125</v>
       </c>
       <c r="E66">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F66" t="s">
         <v>1279</v>
@@ -9112,7 +9112,7 @@
         <v>1126</v>
       </c>
       <c r="E67">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F67" t="s">
         <v>1279</v>
@@ -9147,7 +9147,7 @@
         <v>1126</v>
       </c>
       <c r="E68">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F68" t="s">
         <v>1279</v>
@@ -9182,7 +9182,7 @@
         <v>1126</v>
       </c>
       <c r="E69">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F69" t="s">
         <v>1280</v>
@@ -9217,7 +9217,7 @@
         <v>1126</v>
       </c>
       <c r="E70">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F70" t="s">
         <v>1279</v>
@@ -9252,7 +9252,7 @@
         <v>1127</v>
       </c>
       <c r="E71">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F71" t="s">
         <v>1279</v>
@@ -9287,7 +9287,7 @@
         <v>1128</v>
       </c>
       <c r="E72">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F72" t="s">
         <v>1279</v>
@@ -9322,7 +9322,7 @@
         <v>1128</v>
       </c>
       <c r="E73">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="F73" t="s">
         <v>1279</v>
@@ -9357,7 +9357,7 @@
         <v>1129</v>
       </c>
       <c r="E74">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F74" t="s">
         <v>1279</v>
@@ -9392,7 +9392,7 @@
         <v>1130</v>
       </c>
       <c r="E75">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F75" t="s">
         <v>1279</v>
@@ -9427,7 +9427,7 @@
         <v>1131</v>
       </c>
       <c r="E76">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F76" t="s">
         <v>1279</v>
@@ -9462,7 +9462,7 @@
         <v>1132</v>
       </c>
       <c r="E77">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F77" t="s">
         <v>1279</v>
@@ -9497,7 +9497,7 @@
         <v>1132</v>
       </c>
       <c r="E78">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F78" t="s">
         <v>1279</v>
@@ -9532,7 +9532,7 @@
         <v>1132</v>
       </c>
       <c r="E79">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F79" t="s">
         <v>1279</v>
@@ -9567,7 +9567,7 @@
         <v>1132</v>
       </c>
       <c r="E80">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F80" t="s">
         <v>1279</v>
@@ -9602,7 +9602,7 @@
         <v>1132</v>
       </c>
       <c r="E81">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F81" t="s">
         <v>1279</v>
@@ -9637,7 +9637,7 @@
         <v>1132</v>
       </c>
       <c r="E82">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F82" t="s">
         <v>1279</v>
@@ -9672,7 +9672,7 @@
         <v>1133</v>
       </c>
       <c r="E83">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F83" t="s">
         <v>1279</v>
@@ -9707,7 +9707,7 @@
         <v>1134</v>
       </c>
       <c r="E84">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F84" t="s">
         <v>1279</v>
@@ -9742,7 +9742,7 @@
         <v>1135</v>
       </c>
       <c r="E85">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F85" t="s">
         <v>1279</v>
@@ -9777,7 +9777,7 @@
         <v>1135</v>
       </c>
       <c r="E86">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F86" t="s">
         <v>1279</v>
@@ -9812,7 +9812,7 @@
         <v>1136</v>
       </c>
       <c r="E87">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F87" t="s">
         <v>1281</v>
@@ -9847,7 +9847,7 @@
         <v>1137</v>
       </c>
       <c r="E88">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F88" t="s">
         <v>1279</v>
@@ -9882,7 +9882,7 @@
         <v>1138</v>
       </c>
       <c r="E89">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F89" t="s">
         <v>1279</v>
@@ -9917,7 +9917,7 @@
         <v>1138</v>
       </c>
       <c r="E90">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F90" t="s">
         <v>1279</v>
@@ -9952,7 +9952,7 @@
         <v>1139</v>
       </c>
       <c r="E91">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F91" t="s">
         <v>1279</v>
@@ -9987,7 +9987,7 @@
         <v>1140</v>
       </c>
       <c r="E92">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F92" t="s">
         <v>1279</v>
@@ -10022,7 +10022,7 @@
         <v>1141</v>
       </c>
       <c r="E93">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F93" t="s">
         <v>1279</v>
@@ -10057,7 +10057,7 @@
         <v>1142</v>
       </c>
       <c r="E94">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F94" t="s">
         <v>1279</v>
@@ -10092,7 +10092,7 @@
         <v>1143</v>
       </c>
       <c r="E95">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F95" t="s">
         <v>1279</v>
@@ -10127,7 +10127,7 @@
         <v>1143</v>
       </c>
       <c r="E96">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F96" t="s">
         <v>1279</v>
@@ -10162,7 +10162,7 @@
         <v>1144</v>
       </c>
       <c r="E97">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F97" t="s">
         <v>1279</v>
@@ -10197,7 +10197,7 @@
         <v>1144</v>
       </c>
       <c r="E98">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F98" t="s">
         <v>1279</v>
@@ -10232,7 +10232,7 @@
         <v>1144</v>
       </c>
       <c r="E99">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F99" t="s">
         <v>1279</v>
@@ -10267,7 +10267,7 @@
         <v>1145</v>
       </c>
       <c r="E100">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F100" t="s">
         <v>1279</v>
@@ -10302,7 +10302,7 @@
         <v>1145</v>
       </c>
       <c r="E101">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F101" t="s">
         <v>1279</v>
@@ -10337,7 +10337,7 @@
         <v>1146</v>
       </c>
       <c r="E102">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F102" t="s">
         <v>1279</v>
@@ -10372,7 +10372,7 @@
         <v>1147</v>
       </c>
       <c r="E103">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F103" t="s">
         <v>1279</v>
@@ -10407,7 +10407,7 @@
         <v>1148</v>
       </c>
       <c r="E104">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F104" t="s">
         <v>1279</v>
@@ -10442,7 +10442,7 @@
         <v>1148</v>
       </c>
       <c r="E105">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F105" t="s">
         <v>1279</v>
@@ -10477,7 +10477,7 @@
         <v>1149</v>
       </c>
       <c r="E106">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F106" t="s">
         <v>1279</v>
@@ -10512,7 +10512,7 @@
         <v>1149</v>
       </c>
       <c r="E107">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F107" t="s">
         <v>1279</v>
@@ -10547,7 +10547,7 @@
         <v>1150</v>
       </c>
       <c r="E108">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F108" t="s">
         <v>1279</v>
@@ -10582,7 +10582,7 @@
         <v>1151</v>
       </c>
       <c r="E109">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F109" t="s">
         <v>1279</v>
@@ -10617,7 +10617,7 @@
         <v>1151</v>
       </c>
       <c r="E110">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F110" t="s">
         <v>1279</v>
@@ -10652,7 +10652,7 @@
         <v>1152</v>
       </c>
       <c r="E111">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F111" t="s">
         <v>1279</v>
@@ -10687,7 +10687,7 @@
         <v>1153</v>
       </c>
       <c r="E112">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F112" t="s">
         <v>1279</v>
@@ -10722,7 +10722,7 @@
         <v>1153</v>
       </c>
       <c r="E113">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F113" t="s">
         <v>1279</v>
@@ -10757,7 +10757,7 @@
         <v>1154</v>
       </c>
       <c r="E114">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F114" t="s">
         <v>1279</v>
@@ -10792,7 +10792,7 @@
         <v>1155</v>
       </c>
       <c r="E115">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F115" t="s">
         <v>1279</v>
@@ -10830,7 +10830,7 @@
         <v>1155</v>
       </c>
       <c r="E116">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F116" t="s">
         <v>1279</v>
@@ -10865,7 +10865,7 @@
         <v>1155</v>
       </c>
       <c r="E117">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F117" t="s">
         <v>1279</v>
@@ -10900,7 +10900,7 @@
         <v>1155</v>
       </c>
       <c r="E118">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F118" t="s">
         <v>1279</v>
@@ -10935,7 +10935,7 @@
         <v>1156</v>
       </c>
       <c r="E119">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F119" t="s">
         <v>1280</v>
@@ -10970,7 +10970,7 @@
         <v>1157</v>
       </c>
       <c r="E120">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F120" t="s">
         <v>1279</v>
@@ -11005,7 +11005,7 @@
         <v>1157</v>
       </c>
       <c r="E121">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F121" t="s">
         <v>1279</v>
@@ -11040,7 +11040,7 @@
         <v>1157</v>
       </c>
       <c r="E122">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F122" t="s">
         <v>1279</v>
@@ -11075,7 +11075,7 @@
         <v>1157</v>
       </c>
       <c r="E123">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F123" t="s">
         <v>1279</v>
@@ -11110,7 +11110,7 @@
         <v>1158</v>
       </c>
       <c r="E124">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F124" t="s">
         <v>1279</v>
@@ -11145,7 +11145,7 @@
         <v>1158</v>
       </c>
       <c r="E125">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F125" t="s">
         <v>1279</v>
@@ -11180,7 +11180,7 @@
         <v>1158</v>
       </c>
       <c r="E126">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F126" t="s">
         <v>1279</v>
@@ -11215,7 +11215,7 @@
         <v>1158</v>
       </c>
       <c r="E127">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F127" t="s">
         <v>1279</v>
@@ -11250,7 +11250,7 @@
         <v>1158</v>
       </c>
       <c r="E128">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F128" t="s">
         <v>1279</v>
@@ -11285,7 +11285,7 @@
         <v>1158</v>
       </c>
       <c r="E129">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F129" t="s">
         <v>1279</v>
@@ -11320,7 +11320,7 @@
         <v>1158</v>
       </c>
       <c r="E130">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F130" t="s">
         <v>1279</v>
@@ -11355,7 +11355,7 @@
         <v>1159</v>
       </c>
       <c r="E131">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F131" t="s">
         <v>1279</v>
@@ -11390,7 +11390,7 @@
         <v>1159</v>
       </c>
       <c r="E132">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F132" t="s">
         <v>1279</v>
@@ -11425,7 +11425,7 @@
         <v>1160</v>
       </c>
       <c r="E133">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F133" t="s">
         <v>1279</v>
@@ -11460,7 +11460,7 @@
         <v>1161</v>
       </c>
       <c r="E134">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F134" t="s">
         <v>1279</v>
@@ -11495,7 +11495,7 @@
         <v>1161</v>
       </c>
       <c r="E135">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F135" t="s">
         <v>1279</v>
@@ -11530,7 +11530,7 @@
         <v>1161</v>
       </c>
       <c r="E136">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F136" t="s">
         <v>1279</v>
@@ -11565,7 +11565,7 @@
         <v>1162</v>
       </c>
       <c r="E137">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F137" t="s">
         <v>1279</v>
@@ -11600,7 +11600,7 @@
         <v>1162</v>
       </c>
       <c r="E138">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F138" t="s">
         <v>1279</v>
@@ -11635,7 +11635,7 @@
         <v>1162</v>
       </c>
       <c r="E139">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F139" t="s">
         <v>1279</v>
@@ -11670,7 +11670,7 @@
         <v>1162</v>
       </c>
       <c r="E140">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F140" t="s">
         <v>1279</v>
@@ -11705,7 +11705,7 @@
         <v>1162</v>
       </c>
       <c r="E141">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F141" t="s">
         <v>1279</v>
@@ -11740,7 +11740,7 @@
         <v>1162</v>
       </c>
       <c r="E142">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F142" t="s">
         <v>1279</v>
@@ -11775,7 +11775,7 @@
         <v>1162</v>
       </c>
       <c r="E143">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F143" t="s">
         <v>1279</v>
@@ -11810,7 +11810,7 @@
         <v>1162</v>
       </c>
       <c r="E144">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F144" t="s">
         <v>1279</v>
@@ -11845,7 +11845,7 @@
         <v>1162</v>
       </c>
       <c r="E145">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F145" t="s">
         <v>1279</v>
@@ -11880,7 +11880,7 @@
         <v>1163</v>
       </c>
       <c r="E146">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F146" t="s">
         <v>1279</v>
@@ -11915,7 +11915,7 @@
         <v>1163</v>
       </c>
       <c r="E147">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F147" t="s">
         <v>1279</v>
@@ -11950,7 +11950,7 @@
         <v>1163</v>
       </c>
       <c r="E148">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F148" t="s">
         <v>1279</v>
@@ -11985,7 +11985,7 @@
         <v>1164</v>
       </c>
       <c r="E149">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F149" t="s">
         <v>1279</v>
@@ -12020,7 +12020,7 @@
         <v>1164</v>
       </c>
       <c r="E150">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F150" t="s">
         <v>1280</v>
@@ -12055,7 +12055,7 @@
         <v>1164</v>
       </c>
       <c r="E151">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F151" t="s">
         <v>1279</v>
@@ -12090,7 +12090,7 @@
         <v>1165</v>
       </c>
       <c r="E152">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F152" t="s">
         <v>1279</v>
@@ -12125,7 +12125,7 @@
         <v>1165</v>
       </c>
       <c r="E153">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F153" t="s">
         <v>1279</v>
@@ -12160,7 +12160,7 @@
         <v>1166</v>
       </c>
       <c r="E154">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F154" t="s">
         <v>1279</v>
@@ -12195,7 +12195,7 @@
         <v>1166</v>
       </c>
       <c r="E155">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F155" t="s">
         <v>1279</v>
@@ -12230,7 +12230,7 @@
         <v>1167</v>
       </c>
       <c r="E156">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F156" t="s">
         <v>1279</v>
@@ -12265,7 +12265,7 @@
         <v>1167</v>
       </c>
       <c r="E157">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F157" t="s">
         <v>1279</v>
@@ -12300,7 +12300,7 @@
         <v>1168</v>
       </c>
       <c r="E158">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F158" t="s">
         <v>1279</v>
@@ -12335,7 +12335,7 @@
         <v>1168</v>
       </c>
       <c r="E159">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F159" t="s">
         <v>1279</v>
@@ -12370,7 +12370,7 @@
         <v>1168</v>
       </c>
       <c r="E160">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F160" t="s">
         <v>1279</v>
@@ -12405,7 +12405,7 @@
         <v>1169</v>
       </c>
       <c r="E161">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F161" t="s">
         <v>1279</v>
@@ -12440,7 +12440,7 @@
         <v>1169</v>
       </c>
       <c r="E162">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F162" t="s">
         <v>1279</v>
@@ -12475,7 +12475,7 @@
         <v>1170</v>
       </c>
       <c r="E163">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F163" t="s">
         <v>1279</v>
@@ -12510,7 +12510,7 @@
         <v>1171</v>
       </c>
       <c r="E164">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F164" t="s">
         <v>1279</v>
@@ -12545,7 +12545,7 @@
         <v>1171</v>
       </c>
       <c r="E165">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F165" t="s">
         <v>1279</v>
@@ -12580,7 +12580,7 @@
         <v>1171</v>
       </c>
       <c r="E166">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F166" t="s">
         <v>1279</v>
@@ -12615,7 +12615,7 @@
         <v>1171</v>
       </c>
       <c r="E167">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F167" t="s">
         <v>1279</v>
@@ -12650,7 +12650,7 @@
         <v>1172</v>
       </c>
       <c r="E168">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F168" t="s">
         <v>1279</v>
@@ -12685,7 +12685,7 @@
         <v>1173</v>
       </c>
       <c r="E169">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F169" t="s">
         <v>1279</v>
@@ -12720,7 +12720,7 @@
         <v>1173</v>
       </c>
       <c r="E170">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F170" t="s">
         <v>1279</v>
@@ -12755,7 +12755,7 @@
         <v>1173</v>
       </c>
       <c r="E171">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F171" t="s">
         <v>1279</v>
@@ -12790,7 +12790,7 @@
         <v>1173</v>
       </c>
       <c r="E172">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F172" t="s">
         <v>1279</v>
@@ -12825,7 +12825,7 @@
         <v>1173</v>
       </c>
       <c r="E173">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F173" t="s">
         <v>1279</v>
@@ -12860,7 +12860,7 @@
         <v>1174</v>
       </c>
       <c r="E174">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F174" t="s">
         <v>1279</v>
@@ -12895,7 +12895,7 @@
         <v>1174</v>
       </c>
       <c r="E175">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F175" t="s">
         <v>1279</v>
@@ -12930,7 +12930,7 @@
         <v>1174</v>
       </c>
       <c r="E176">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F176" t="s">
         <v>1279</v>
@@ -12965,7 +12965,7 @@
         <v>1174</v>
       </c>
       <c r="E177">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F177" t="s">
         <v>1279</v>
@@ -13000,7 +13000,7 @@
         <v>1174</v>
       </c>
       <c r="E178">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F178" t="s">
         <v>1279</v>
@@ -13035,7 +13035,7 @@
         <v>1174</v>
       </c>
       <c r="E179">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F179" t="s">
         <v>1279</v>
@@ -13070,7 +13070,7 @@
         <v>1175</v>
       </c>
       <c r="E180">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F180" t="s">
         <v>1279</v>
@@ -13105,7 +13105,7 @@
         <v>1175</v>
       </c>
       <c r="E181">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F181" t="s">
         <v>1279</v>
@@ -13140,7 +13140,7 @@
         <v>1175</v>
       </c>
       <c r="E182">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F182" t="s">
         <v>1279</v>
@@ -13175,7 +13175,7 @@
         <v>1175</v>
       </c>
       <c r="E183">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F183" t="s">
         <v>1279</v>
@@ -13210,7 +13210,7 @@
         <v>1176</v>
       </c>
       <c r="E184">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F184" t="s">
         <v>1279</v>
@@ -13245,7 +13245,7 @@
         <v>1176</v>
       </c>
       <c r="E185">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F185" t="s">
         <v>1279</v>
@@ -13280,7 +13280,7 @@
         <v>1177</v>
       </c>
       <c r="E186">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F186" t="s">
         <v>1279</v>
@@ -13315,7 +13315,7 @@
         <v>1178</v>
       </c>
       <c r="E187">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F187" t="s">
         <v>1279</v>
@@ -13350,7 +13350,7 @@
         <v>1178</v>
       </c>
       <c r="E188">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F188" t="s">
         <v>1279</v>
@@ -13385,7 +13385,7 @@
         <v>1179</v>
       </c>
       <c r="E189">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F189" t="s">
         <v>1279</v>
@@ -13420,7 +13420,7 @@
         <v>1180</v>
       </c>
       <c r="E190">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F190" t="s">
         <v>1279</v>
@@ -13455,7 +13455,7 @@
         <v>1180</v>
       </c>
       <c r="E191">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F191" t="s">
         <v>1279</v>
@@ -13490,7 +13490,7 @@
         <v>1181</v>
       </c>
       <c r="E192">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F192" t="s">
         <v>1279</v>
@@ -13525,7 +13525,7 @@
         <v>1181</v>
       </c>
       <c r="E193">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F193" t="s">
         <v>1279</v>
@@ -13560,7 +13560,7 @@
         <v>1182</v>
       </c>
       <c r="E194">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F194" t="s">
         <v>1279</v>
@@ -13595,7 +13595,7 @@
         <v>1183</v>
       </c>
       <c r="E195">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F195" t="s">
         <v>1279</v>
@@ -13630,7 +13630,7 @@
         <v>1183</v>
       </c>
       <c r="E196">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F196" t="s">
         <v>1279</v>
@@ -13665,7 +13665,7 @@
         <v>1183</v>
       </c>
       <c r="E197">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F197" t="s">
         <v>1279</v>
@@ -13700,7 +13700,7 @@
         <v>1184</v>
       </c>
       <c r="E198">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F198" t="s">
         <v>1279</v>
@@ -13735,7 +13735,7 @@
         <v>1184</v>
       </c>
       <c r="E199">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="F199" t="s">
         <v>1279</v>
@@ -13770,7 +13770,7 @@
         <v>1185</v>
       </c>
       <c r="E200">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F200" t="s">
         <v>1279</v>
@@ -13805,7 +13805,7 @@
         <v>1186</v>
       </c>
       <c r="E201">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F201" t="s">
         <v>1279</v>
@@ -13840,7 +13840,7 @@
         <v>1186</v>
       </c>
       <c r="E202">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F202" t="s">
         <v>1279</v>
@@ -13875,7 +13875,7 @@
         <v>1186</v>
       </c>
       <c r="E203">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F203" t="s">
         <v>1279</v>
@@ -13910,7 +13910,7 @@
         <v>1187</v>
       </c>
       <c r="E204">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F204" t="s">
         <v>1279</v>
@@ -13945,7 +13945,7 @@
         <v>1187</v>
       </c>
       <c r="E205">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F205" t="s">
         <v>1279</v>
@@ -13980,7 +13980,7 @@
         <v>1188</v>
       </c>
       <c r="E206">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F206" t="s">
         <v>1279</v>
@@ -14015,7 +14015,7 @@
         <v>1188</v>
       </c>
       <c r="E207">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F207" t="s">
         <v>1281</v>
@@ -14050,7 +14050,7 @@
         <v>1188</v>
       </c>
       <c r="E208">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F208" t="s">
         <v>1279</v>
@@ -14085,7 +14085,7 @@
         <v>1189</v>
       </c>
       <c r="E209">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F209" t="s">
         <v>1279</v>
@@ -14120,7 +14120,7 @@
         <v>1189</v>
       </c>
       <c r="E210">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F210" t="s">
         <v>1279</v>
@@ -14158,7 +14158,7 @@
         <v>1189</v>
       </c>
       <c r="E211">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F211" t="s">
         <v>1279</v>
@@ -14193,7 +14193,7 @@
         <v>1189</v>
       </c>
       <c r="E212">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F212" t="s">
         <v>1279</v>
@@ -14228,7 +14228,7 @@
         <v>1189</v>
       </c>
       <c r="E213">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F213" t="s">
         <v>1279</v>
@@ -14263,7 +14263,7 @@
         <v>1189</v>
       </c>
       <c r="E214">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F214" t="s">
         <v>1279</v>
@@ -14298,7 +14298,7 @@
         <v>1190</v>
       </c>
       <c r="E215">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F215" t="s">
         <v>1279</v>
@@ -14333,7 +14333,7 @@
         <v>1190</v>
       </c>
       <c r="E216">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F216" t="s">
         <v>1279</v>
@@ -14368,7 +14368,7 @@
         <v>1190</v>
       </c>
       <c r="E217">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F217" t="s">
         <v>1279</v>
@@ -14403,7 +14403,7 @@
         <v>1191</v>
       </c>
       <c r="E218">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F218" t="s">
         <v>1279</v>
@@ -14438,7 +14438,7 @@
         <v>1191</v>
       </c>
       <c r="E219">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F219" t="s">
         <v>1279</v>
@@ -14473,7 +14473,7 @@
         <v>1191</v>
       </c>
       <c r="E220">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F220" t="s">
         <v>1279</v>
@@ -14508,7 +14508,7 @@
         <v>1192</v>
       </c>
       <c r="E221">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F221" t="s">
         <v>1279</v>
@@ -14543,7 +14543,7 @@
         <v>1192</v>
       </c>
       <c r="E222">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F222" t="s">
         <v>1279</v>
@@ -14578,7 +14578,7 @@
         <v>1192</v>
       </c>
       <c r="E223">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F223" t="s">
         <v>1279</v>
@@ -14613,7 +14613,7 @@
         <v>1193</v>
       </c>
       <c r="E224">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F224" t="s">
         <v>1279</v>
@@ -14648,7 +14648,7 @@
         <v>1193</v>
       </c>
       <c r="E225">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F225" t="s">
         <v>1279</v>
@@ -14683,7 +14683,7 @@
         <v>1193</v>
       </c>
       <c r="E226">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F226" t="s">
         <v>1279</v>
@@ -14718,7 +14718,7 @@
         <v>1193</v>
       </c>
       <c r="E227">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F227" t="s">
         <v>1279</v>
@@ -14753,7 +14753,7 @@
         <v>1193</v>
       </c>
       <c r="E228">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F228" t="s">
         <v>1279</v>
@@ -14788,7 +14788,7 @@
         <v>1193</v>
       </c>
       <c r="E229">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F229" t="s">
         <v>1279</v>
@@ -14823,7 +14823,7 @@
         <v>1194</v>
       </c>
       <c r="E230">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F230" t="s">
         <v>1279</v>
@@ -14858,7 +14858,7 @@
         <v>1195</v>
       </c>
       <c r="E231">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F231" t="s">
         <v>1279</v>
@@ -14893,7 +14893,7 @@
         <v>1195</v>
       </c>
       <c r="E232">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F232" t="s">
         <v>1282</v>
@@ -14928,7 +14928,7 @@
         <v>1195</v>
       </c>
       <c r="E233">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F233" t="s">
         <v>1279</v>
@@ -14963,7 +14963,7 @@
         <v>1195</v>
       </c>
       <c r="E234">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F234" t="s">
         <v>1279</v>
@@ -14998,7 +14998,7 @@
         <v>1196</v>
       </c>
       <c r="E235">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F235" t="s">
         <v>1279</v>
@@ -15033,7 +15033,7 @@
         <v>1196</v>
       </c>
       <c r="E236">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F236" t="s">
         <v>1279</v>
@@ -15068,7 +15068,7 @@
         <v>1196</v>
       </c>
       <c r="E237">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F237" t="s">
         <v>1279</v>
@@ -15103,7 +15103,7 @@
         <v>1196</v>
       </c>
       <c r="E238">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F238" t="s">
         <v>1279</v>
@@ -15138,7 +15138,7 @@
         <v>1197</v>
       </c>
       <c r="E239">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F239" t="s">
         <v>1279</v>
@@ -15176,7 +15176,7 @@
         <v>1198</v>
       </c>
       <c r="E240">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F240" t="s">
         <v>1279</v>
@@ -15211,7 +15211,7 @@
         <v>1198</v>
       </c>
       <c r="E241">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F241" t="s">
         <v>1279</v>
@@ -15246,7 +15246,7 @@
         <v>1198</v>
       </c>
       <c r="E242">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F242" t="s">
         <v>1279</v>
@@ -15281,7 +15281,7 @@
         <v>1198</v>
       </c>
       <c r="E243">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F243" t="s">
         <v>1279</v>
@@ -15319,7 +15319,7 @@
         <v>1198</v>
       </c>
       <c r="E244">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F244" t="s">
         <v>1279</v>
@@ -15354,7 +15354,7 @@
         <v>1199</v>
       </c>
       <c r="E245">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F245" t="s">
         <v>1279</v>
@@ -15389,7 +15389,7 @@
         <v>1199</v>
       </c>
       <c r="E246">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F246" t="s">
         <v>1279</v>
@@ -15424,7 +15424,7 @@
         <v>1200</v>
       </c>
       <c r="E247">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F247" t="s">
         <v>1279</v>
@@ -15459,7 +15459,7 @@
         <v>1200</v>
       </c>
       <c r="E248">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F248" t="s">
         <v>1279</v>
@@ -15494,7 +15494,7 @@
         <v>1200</v>
       </c>
       <c r="E249">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F249" t="s">
         <v>1279</v>
@@ -15529,7 +15529,7 @@
         <v>1201</v>
       </c>
       <c r="E250">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F250" t="s">
         <v>1279</v>
@@ -15564,7 +15564,7 @@
         <v>1201</v>
       </c>
       <c r="E251">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F251" t="s">
         <v>1279</v>
@@ -15599,7 +15599,7 @@
         <v>1202</v>
       </c>
       <c r="E252">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F252" t="s">
         <v>1279</v>
@@ -15634,7 +15634,7 @@
         <v>1203</v>
       </c>
       <c r="E253">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F253" t="s">
         <v>1279</v>
@@ -15669,7 +15669,7 @@
         <v>1203</v>
       </c>
       <c r="E254">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F254" t="s">
         <v>1279</v>
@@ -15704,7 +15704,7 @@
         <v>1203</v>
       </c>
       <c r="E255">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F255" t="s">
         <v>1279</v>
@@ -15739,7 +15739,7 @@
         <v>1203</v>
       </c>
       <c r="E256">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F256" t="s">
         <v>1279</v>
@@ -15774,7 +15774,7 @@
         <v>1204</v>
       </c>
       <c r="E257">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F257" t="s">
         <v>1279</v>
@@ -15809,7 +15809,7 @@
         <v>1204</v>
       </c>
       <c r="E258">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F258" t="s">
         <v>1279</v>
@@ -15844,7 +15844,7 @@
         <v>1204</v>
       </c>
       <c r="E259">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F259" t="s">
         <v>1279</v>
@@ -15879,7 +15879,7 @@
         <v>1205</v>
       </c>
       <c r="E260">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F260" t="s">
         <v>1279</v>
@@ -15914,7 +15914,7 @@
         <v>1206</v>
       </c>
       <c r="E261">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F261" t="s">
         <v>1279</v>
@@ -15949,7 +15949,7 @@
         <v>1206</v>
       </c>
       <c r="E262">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F262" t="s">
         <v>1279</v>
@@ -15984,7 +15984,7 @@
         <v>1206</v>
       </c>
       <c r="E263">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F263" t="s">
         <v>1279</v>
@@ -16019,7 +16019,7 @@
         <v>1207</v>
       </c>
       <c r="E264">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F264" t="s">
         <v>1279</v>
@@ -16054,7 +16054,7 @@
         <v>1207</v>
       </c>
       <c r="E265">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F265" t="s">
         <v>1279</v>
@@ -16089,7 +16089,7 @@
         <v>1207</v>
       </c>
       <c r="E266">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F266" t="s">
         <v>1279</v>
@@ -16124,7 +16124,7 @@
         <v>1208</v>
       </c>
       <c r="E267">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F267" t="s">
         <v>1279</v>
@@ -16159,7 +16159,7 @@
         <v>1209</v>
       </c>
       <c r="E268">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F268" t="s">
         <v>1279</v>
@@ -16194,7 +16194,7 @@
         <v>1210</v>
       </c>
       <c r="E269">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F269" t="s">
         <v>1279</v>
@@ -16229,7 +16229,7 @@
         <v>1210</v>
       </c>
       <c r="E270">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F270" t="s">
         <v>1279</v>
@@ -16264,7 +16264,7 @@
         <v>1210</v>
       </c>
       <c r="E271">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F271" t="s">
         <v>1279</v>
@@ -16299,7 +16299,7 @@
         <v>1210</v>
       </c>
       <c r="E272">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F272" t="s">
         <v>1279</v>
@@ -16334,7 +16334,7 @@
         <v>1211</v>
       </c>
       <c r="E273">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F273" t="s">
         <v>1279</v>
@@ -16369,7 +16369,7 @@
         <v>1212</v>
       </c>
       <c r="E274">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F274" t="s">
         <v>1279</v>
@@ -16404,7 +16404,7 @@
         <v>1212</v>
       </c>
       <c r="E275">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F275" t="s">
         <v>1279</v>
@@ -16439,7 +16439,7 @@
         <v>1213</v>
       </c>
       <c r="E276">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F276" t="s">
         <v>1279</v>
@@ -16474,7 +16474,7 @@
         <v>1214</v>
       </c>
       <c r="E277">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F277" t="s">
         <v>1279</v>
@@ -16509,7 +16509,7 @@
         <v>1215</v>
       </c>
       <c r="E278">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F278" t="s">
         <v>1279</v>
@@ -16544,7 +16544,7 @@
         <v>1215</v>
       </c>
       <c r="E279">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F279" t="s">
         <v>1279</v>
@@ -16579,7 +16579,7 @@
         <v>1216</v>
       </c>
       <c r="E280">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F280" t="s">
         <v>1279</v>
@@ -16614,7 +16614,7 @@
         <v>1216</v>
       </c>
       <c r="E281">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F281" t="s">
         <v>1279</v>
@@ -16649,7 +16649,7 @@
         <v>1216</v>
       </c>
       <c r="E282">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F282" t="s">
         <v>1279</v>
@@ -16684,7 +16684,7 @@
         <v>1217</v>
       </c>
       <c r="E283">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F283" t="s">
         <v>1279</v>
@@ -16719,7 +16719,7 @@
         <v>1217</v>
       </c>
       <c r="E284">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F284" t="s">
         <v>1279</v>
@@ -16754,7 +16754,7 @@
         <v>1217</v>
       </c>
       <c r="E285">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F285" t="s">
         <v>1279</v>
@@ -16789,7 +16789,7 @@
         <v>1217</v>
       </c>
       <c r="E286">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F286" t="s">
         <v>1279</v>
@@ -16824,7 +16824,7 @@
         <v>1217</v>
       </c>
       <c r="E287">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F287" t="s">
         <v>1279</v>
@@ -16859,7 +16859,7 @@
         <v>1217</v>
       </c>
       <c r="E288">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F288" t="s">
         <v>1279</v>
@@ -16894,7 +16894,7 @@
         <v>1217</v>
       </c>
       <c r="E289">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F289" t="s">
         <v>1279</v>
@@ -16929,7 +16929,7 @@
         <v>1217</v>
       </c>
       <c r="E290">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F290" t="s">
         <v>1279</v>
@@ -16964,7 +16964,7 @@
         <v>1218</v>
       </c>
       <c r="E291">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F291" t="s">
         <v>1279</v>
@@ -16999,7 +16999,7 @@
         <v>1218</v>
       </c>
       <c r="E292">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F292" t="s">
         <v>1279</v>
@@ -17034,7 +17034,7 @@
         <v>1218</v>
       </c>
       <c r="E293">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F293" t="s">
         <v>1279</v>
@@ -17069,7 +17069,7 @@
         <v>1219</v>
       </c>
       <c r="E294">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F294" t="s">
         <v>1279</v>
@@ -17104,7 +17104,7 @@
         <v>1220</v>
       </c>
       <c r="E295">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F295" t="s">
         <v>1279</v>
@@ -17139,7 +17139,7 @@
         <v>1220</v>
       </c>
       <c r="E296">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F296" t="s">
         <v>1279</v>
@@ -17174,7 +17174,7 @@
         <v>1220</v>
       </c>
       <c r="E297">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F297" t="s">
         <v>1279</v>
@@ -17209,7 +17209,7 @@
         <v>1220</v>
       </c>
       <c r="E298">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F298" t="s">
         <v>1283</v>
@@ -17247,7 +17247,7 @@
         <v>1220</v>
       </c>
       <c r="E299">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F299" t="s">
         <v>1279</v>
@@ -17282,7 +17282,7 @@
         <v>1220</v>
       </c>
       <c r="E300">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F300" t="s">
         <v>1279</v>
@@ -17317,7 +17317,7 @@
         <v>1221</v>
       </c>
       <c r="E301">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F301" t="s">
         <v>1279</v>
@@ -17352,7 +17352,7 @@
         <v>1221</v>
       </c>
       <c r="E302">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F302" t="s">
         <v>1279</v>
@@ -17387,7 +17387,7 @@
         <v>1221</v>
       </c>
       <c r="E303">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F303" t="s">
         <v>1279</v>
@@ -17425,7 +17425,7 @@
         <v>1221</v>
       </c>
       <c r="E304">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F304" t="s">
         <v>1279</v>
@@ -17460,7 +17460,7 @@
         <v>1221</v>
       </c>
       <c r="E305">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F305" t="s">
         <v>1279</v>
@@ -17495,7 +17495,7 @@
         <v>1221</v>
       </c>
       <c r="E306">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F306" t="s">
         <v>1279</v>
@@ -17530,7 +17530,7 @@
         <v>1221</v>
       </c>
       <c r="E307">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F307" t="s">
         <v>1279</v>
@@ -17565,7 +17565,7 @@
         <v>1221</v>
       </c>
       <c r="E308">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F308" t="s">
         <v>1279</v>
@@ -17600,7 +17600,7 @@
         <v>1222</v>
       </c>
       <c r="E309">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F309" t="s">
         <v>1280</v>
@@ -17635,7 +17635,7 @@
         <v>1223</v>
       </c>
       <c r="E310">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F310" t="s">
         <v>1283</v>
@@ -17670,7 +17670,7 @@
         <v>1224</v>
       </c>
       <c r="E311">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F311" t="s">
         <v>1279</v>
@@ -17705,7 +17705,7 @@
         <v>1224</v>
       </c>
       <c r="E312">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F312" t="s">
         <v>1279</v>
@@ -17740,7 +17740,7 @@
         <v>1225</v>
       </c>
       <c r="E313">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F313" t="s">
         <v>1279</v>
@@ -17775,7 +17775,7 @@
         <v>1226</v>
       </c>
       <c r="E314">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F314" t="s">
         <v>1282</v>
@@ -17810,7 +17810,7 @@
         <v>1226</v>
       </c>
       <c r="E315">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F315" t="s">
         <v>1279</v>
@@ -17845,7 +17845,7 @@
         <v>1226</v>
       </c>
       <c r="E316">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F316" t="s">
         <v>1279</v>
@@ -17880,7 +17880,7 @@
         <v>1226</v>
       </c>
       <c r="E317">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F317" t="s">
         <v>1279</v>
@@ -17915,7 +17915,7 @@
         <v>1227</v>
       </c>
       <c r="E318">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F318" t="s">
         <v>1279</v>
@@ -17950,7 +17950,7 @@
         <v>1228</v>
       </c>
       <c r="E319">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F319" t="s">
         <v>1279</v>
@@ -17985,7 +17985,7 @@
         <v>1228</v>
       </c>
       <c r="E320">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F320" t="s">
         <v>1279</v>
@@ -18020,7 +18020,7 @@
         <v>1229</v>
       </c>
       <c r="E321">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F321" t="s">
         <v>1279</v>
@@ -18055,7 +18055,7 @@
         <v>1230</v>
       </c>
       <c r="E322">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F322" t="s">
         <v>1279</v>
@@ -18090,7 +18090,7 @@
         <v>1230</v>
       </c>
       <c r="E323">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F323" t="s">
         <v>1279</v>
@@ -18125,7 +18125,7 @@
         <v>1230</v>
       </c>
       <c r="E324">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F324" t="s">
         <v>1279</v>
@@ -18160,7 +18160,7 @@
         <v>1230</v>
       </c>
       <c r="E325">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F325" t="s">
         <v>1279</v>
@@ -18195,7 +18195,7 @@
         <v>1230</v>
       </c>
       <c r="E326">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F326" t="s">
         <v>1279</v>
@@ -18230,7 +18230,7 @@
         <v>1230</v>
       </c>
       <c r="E327">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F327" t="s">
         <v>1279</v>
@@ -18265,7 +18265,7 @@
         <v>1230</v>
       </c>
       <c r="E328">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F328" t="s">
         <v>1279</v>
@@ -18300,7 +18300,7 @@
         <v>1231</v>
       </c>
       <c r="E329">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F329" t="s">
         <v>1279</v>
@@ -18335,7 +18335,7 @@
         <v>1231</v>
       </c>
       <c r="E330">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F330" t="s">
         <v>1279</v>
@@ -18370,7 +18370,7 @@
         <v>1231</v>
       </c>
       <c r="E331">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F331" t="s">
         <v>1280</v>
@@ -18405,7 +18405,7 @@
         <v>1232</v>
       </c>
       <c r="E332">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F332" t="s">
         <v>1279</v>
@@ -18440,7 +18440,7 @@
         <v>1232</v>
       </c>
       <c r="E333">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F333" t="s">
         <v>1279</v>
@@ -18475,7 +18475,7 @@
         <v>1232</v>
       </c>
       <c r="E334">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F334" t="s">
         <v>1279</v>
@@ -18510,7 +18510,7 @@
         <v>1232</v>
       </c>
       <c r="E335">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F335" t="s">
         <v>1279</v>
@@ -18545,7 +18545,7 @@
         <v>1232</v>
       </c>
       <c r="E336">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F336" t="s">
         <v>1279</v>
@@ -18580,7 +18580,7 @@
         <v>1232</v>
       </c>
       <c r="E337">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F337" t="s">
         <v>1282</v>
@@ -18615,7 +18615,7 @@
         <v>1233</v>
       </c>
       <c r="E338">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F338" t="s">
         <v>1279</v>
@@ -18650,7 +18650,7 @@
         <v>1233</v>
       </c>
       <c r="E339">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F339" t="s">
         <v>1279</v>
@@ -18685,7 +18685,7 @@
         <v>1233</v>
       </c>
       <c r="E340">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F340" t="s">
         <v>1279</v>
@@ -18720,7 +18720,7 @@
         <v>1234</v>
       </c>
       <c r="E341">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F341" t="s">
         <v>1282</v>
@@ -18755,7 +18755,7 @@
         <v>1234</v>
       </c>
       <c r="E342">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F342" t="s">
         <v>1279</v>
@@ -18790,7 +18790,7 @@
         <v>1234</v>
       </c>
       <c r="E343">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F343" t="s">
         <v>1279</v>
@@ -18825,7 +18825,7 @@
         <v>1235</v>
       </c>
       <c r="E344">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F344" t="s">
         <v>1279</v>
@@ -18860,7 +18860,7 @@
         <v>1235</v>
       </c>
       <c r="E345">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F345" t="s">
         <v>1279</v>
@@ -18895,7 +18895,7 @@
         <v>1235</v>
       </c>
       <c r="E346">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F346" t="s">
         <v>1279</v>
@@ -18930,7 +18930,7 @@
         <v>1235</v>
       </c>
       <c r="E347">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F347" t="s">
         <v>1279</v>
@@ -18965,7 +18965,7 @@
         <v>1235</v>
       </c>
       <c r="E348">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F348" t="s">
         <v>1281</v>
@@ -19000,7 +19000,7 @@
         <v>1235</v>
       </c>
       <c r="E349">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F349" t="s">
         <v>1279</v>
@@ -19035,7 +19035,7 @@
         <v>1236</v>
       </c>
       <c r="E350">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F350" t="s">
         <v>1279</v>
@@ -19070,7 +19070,7 @@
         <v>1236</v>
       </c>
       <c r="E351">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F351" t="s">
         <v>1279</v>
@@ -19105,7 +19105,7 @@
         <v>1236</v>
       </c>
       <c r="E352">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F352" t="s">
         <v>1279</v>
@@ -19140,7 +19140,7 @@
         <v>1236</v>
       </c>
       <c r="E353">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F353" t="s">
         <v>1279</v>
@@ -19175,7 +19175,7 @@
         <v>1237</v>
       </c>
       <c r="E354">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F354" t="s">
         <v>1279</v>
@@ -19210,7 +19210,7 @@
         <v>1237</v>
       </c>
       <c r="E355">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F355" t="s">
         <v>1279</v>
@@ -19245,7 +19245,7 @@
         <v>1237</v>
       </c>
       <c r="E356">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F356" t="s">
         <v>1279</v>
@@ -19280,7 +19280,7 @@
         <v>1237</v>
       </c>
       <c r="E357">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F357" t="s">
         <v>1279</v>
@@ -19315,7 +19315,7 @@
         <v>1237</v>
       </c>
       <c r="E358">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F358" t="s">
         <v>1279</v>
@@ -19353,7 +19353,7 @@
         <v>1238</v>
       </c>
       <c r="E359">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F359" t="s">
         <v>1279</v>
@@ -19388,7 +19388,7 @@
         <v>1238</v>
       </c>
       <c r="E360">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F360" t="s">
         <v>1279</v>
@@ -19423,7 +19423,7 @@
         <v>1238</v>
       </c>
       <c r="E361">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F361" t="s">
         <v>1279</v>
@@ -19458,7 +19458,7 @@
         <v>1238</v>
       </c>
       <c r="E362">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F362" t="s">
         <v>1279</v>
@@ -19493,7 +19493,7 @@
         <v>1238</v>
       </c>
       <c r="E363">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F363" t="s">
         <v>1279</v>
@@ -19528,7 +19528,7 @@
         <v>1238</v>
       </c>
       <c r="E364">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F364" t="s">
         <v>1279</v>
@@ -19563,7 +19563,7 @@
         <v>1239</v>
       </c>
       <c r="E365">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F365" t="s">
         <v>1280</v>
@@ -19598,7 +19598,7 @@
         <v>1240</v>
       </c>
       <c r="E366">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F366" t="s">
         <v>1279</v>
@@ -19633,7 +19633,7 @@
         <v>1241</v>
       </c>
       <c r="E367">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F367" t="s">
         <v>1281</v>
@@ -19671,7 +19671,7 @@
         <v>1242</v>
       </c>
       <c r="E368">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F368" t="s">
         <v>1279</v>
@@ -19706,7 +19706,7 @@
         <v>1242</v>
       </c>
       <c r="E369">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F369" t="s">
         <v>1279</v>
@@ -19741,7 +19741,7 @@
         <v>1242</v>
       </c>
       <c r="E370">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F370" t="s">
         <v>1279</v>
@@ -19776,7 +19776,7 @@
         <v>1243</v>
       </c>
       <c r="E371">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F371" t="s">
         <v>1279</v>
@@ -19811,7 +19811,7 @@
         <v>1243</v>
       </c>
       <c r="E372">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F372" t="s">
         <v>1279</v>
@@ -19846,7 +19846,7 @@
         <v>1244</v>
       </c>
       <c r="E373">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F373" t="s">
         <v>1279</v>
@@ -19881,7 +19881,7 @@
         <v>1244</v>
       </c>
       <c r="E374">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F374" t="s">
         <v>1283</v>
@@ -19919,7 +19919,7 @@
         <v>1244</v>
       </c>
       <c r="E375">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F375" t="s">
         <v>1279</v>
@@ -19954,7 +19954,7 @@
         <v>1244</v>
       </c>
       <c r="E376">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F376" t="s">
         <v>1283</v>
@@ -19989,7 +19989,7 @@
         <v>1245</v>
       </c>
       <c r="E377">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F377" t="s">
         <v>1279</v>
@@ -20024,7 +20024,7 @@
         <v>1246</v>
       </c>
       <c r="E378">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F378" t="s">
         <v>1279</v>
@@ -20059,7 +20059,7 @@
         <v>1246</v>
       </c>
       <c r="E379">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F379" t="s">
         <v>1279</v>
@@ -20094,7 +20094,7 @@
         <v>1246</v>
       </c>
       <c r="E380">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F380" t="s">
         <v>1279</v>
@@ -20129,7 +20129,7 @@
         <v>1246</v>
       </c>
       <c r="E381">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F381" t="s">
         <v>1279</v>
@@ -20164,7 +20164,7 @@
         <v>1247</v>
       </c>
       <c r="E382">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F382" t="s">
         <v>1283</v>
@@ -20199,7 +20199,7 @@
         <v>1247</v>
       </c>
       <c r="E383">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F383" t="s">
         <v>1279</v>
@@ -20234,7 +20234,7 @@
         <v>1247</v>
       </c>
       <c r="E384">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F384" t="s">
         <v>1279</v>
@@ -20269,7 +20269,7 @@
         <v>1248</v>
       </c>
       <c r="E385">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F385" t="s">
         <v>1279</v>
@@ -20304,7 +20304,7 @@
         <v>1249</v>
       </c>
       <c r="E386">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F386" t="s">
         <v>1279</v>
@@ -20339,7 +20339,7 @@
         <v>1249</v>
       </c>
       <c r="E387">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F387" t="s">
         <v>1279</v>
@@ -20374,7 +20374,7 @@
         <v>1250</v>
       </c>
       <c r="E388">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F388" t="s">
         <v>1279</v>
@@ -20409,7 +20409,7 @@
         <v>1250</v>
       </c>
       <c r="E389">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F389" t="s">
         <v>1279</v>
@@ -20444,7 +20444,7 @@
         <v>1250</v>
       </c>
       <c r="E390">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F390" t="s">
         <v>1279</v>
@@ -20479,7 +20479,7 @@
         <v>1250</v>
       </c>
       <c r="E391">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F391" t="s">
         <v>1279</v>
@@ -20514,7 +20514,7 @@
         <v>1250</v>
       </c>
       <c r="E392">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F392" t="s">
         <v>1279</v>
@@ -20549,7 +20549,7 @@
         <v>1250</v>
       </c>
       <c r="E393">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F393" t="s">
         <v>1279</v>
@@ -20584,7 +20584,7 @@
         <v>1250</v>
       </c>
       <c r="E394">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F394" t="s">
         <v>1279</v>
@@ -20619,7 +20619,7 @@
         <v>1250</v>
       </c>
       <c r="E395">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F395" t="s">
         <v>1279</v>
@@ -20654,7 +20654,7 @@
         <v>1250</v>
       </c>
       <c r="E396">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F396" t="s">
         <v>1279</v>
@@ -20689,7 +20689,7 @@
         <v>1250</v>
       </c>
       <c r="E397">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F397" t="s">
         <v>1279</v>
@@ -20724,7 +20724,7 @@
         <v>1250</v>
       </c>
       <c r="E398">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F398" t="s">
         <v>1279</v>
@@ -20759,7 +20759,7 @@
         <v>1250</v>
       </c>
       <c r="E399">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F399" t="s">
         <v>1279</v>
@@ -20794,7 +20794,7 @@
         <v>1250</v>
       </c>
       <c r="E400">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F400" t="s">
         <v>1279</v>
@@ -20829,7 +20829,7 @@
         <v>1250</v>
       </c>
       <c r="E401">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F401" t="s">
         <v>1279</v>
@@ -20864,7 +20864,7 @@
         <v>1250</v>
       </c>
       <c r="E402">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F402" t="s">
         <v>1279</v>
@@ -20899,7 +20899,7 @@
         <v>1250</v>
       </c>
       <c r="E403">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F403" t="s">
         <v>1279</v>
@@ -20934,7 +20934,7 @@
         <v>1250</v>
       </c>
       <c r="E404">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F404" t="s">
         <v>1279</v>
@@ -20969,7 +20969,7 @@
         <v>1250</v>
       </c>
       <c r="E405">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F405" t="s">
         <v>1279</v>
@@ -21004,7 +21004,7 @@
         <v>1250</v>
       </c>
       <c r="E406">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F406" t="s">
         <v>1279</v>
@@ -21039,7 +21039,7 @@
         <v>1250</v>
       </c>
       <c r="E407">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F407" t="s">
         <v>1279</v>
@@ -21074,7 +21074,7 @@
         <v>1250</v>
       </c>
       <c r="E408">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F408" t="s">
         <v>1279</v>
@@ -21109,7 +21109,7 @@
         <v>1250</v>
       </c>
       <c r="E409">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F409" t="s">
         <v>1279</v>
@@ -21144,7 +21144,7 @@
         <v>1251</v>
       </c>
       <c r="E410">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F410" t="s">
         <v>1279</v>
@@ -21179,7 +21179,7 @@
         <v>1251</v>
       </c>
       <c r="E411">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F411" t="s">
         <v>1279</v>
@@ -21214,7 +21214,7 @@
         <v>1251</v>
       </c>
       <c r="E412">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F412" t="s">
         <v>1283</v>
@@ -21249,7 +21249,7 @@
         <v>1252</v>
       </c>
       <c r="E413">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F413" t="s">
         <v>1279</v>
@@ -21284,7 +21284,7 @@
         <v>1253</v>
       </c>
       <c r="E414">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F414" t="s">
         <v>1281</v>
@@ -21322,7 +21322,7 @@
         <v>1253</v>
       </c>
       <c r="E415">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F415" t="s">
         <v>1279</v>
@@ -21357,7 +21357,7 @@
         <v>1253</v>
       </c>
       <c r="E416">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F416" t="s">
         <v>1279</v>
@@ -21392,7 +21392,7 @@
         <v>1253</v>
       </c>
       <c r="E417">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F417" t="s">
         <v>1279</v>
@@ -21427,7 +21427,7 @@
         <v>1254</v>
       </c>
       <c r="E418">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F418" t="s">
         <v>1279</v>
@@ -21465,7 +21465,7 @@
         <v>1254</v>
       </c>
       <c r="E419">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F419" t="s">
         <v>1283</v>
@@ -21500,7 +21500,7 @@
         <v>1254</v>
       </c>
       <c r="E420">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F420" t="s">
         <v>1281</v>
@@ -21535,7 +21535,7 @@
         <v>1254</v>
       </c>
       <c r="E421">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F421" t="s">
         <v>1279</v>
@@ -21570,7 +21570,7 @@
         <v>1254</v>
       </c>
       <c r="E422">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F422" t="s">
         <v>1279</v>
@@ -21605,7 +21605,7 @@
         <v>1254</v>
       </c>
       <c r="E423">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F423" t="s">
         <v>1279</v>
@@ -21640,7 +21640,7 @@
         <v>1254</v>
       </c>
       <c r="E424">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F424" t="s">
         <v>1279</v>
@@ -21675,7 +21675,7 @@
         <v>1255</v>
       </c>
       <c r="E425">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F425" t="s">
         <v>1283</v>
@@ -21713,7 +21713,7 @@
         <v>1256</v>
       </c>
       <c r="E426">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F426" t="s">
         <v>1279</v>
@@ -21748,7 +21748,7 @@
         <v>1256</v>
       </c>
       <c r="E427">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F427" t="s">
         <v>1279</v>
@@ -21783,7 +21783,7 @@
         <v>1256</v>
       </c>
       <c r="E428">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F428" t="s">
         <v>1279</v>
@@ -21818,7 +21818,7 @@
         <v>1257</v>
       </c>
       <c r="E429">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F429" t="s">
         <v>1279</v>
@@ -21853,7 +21853,7 @@
         <v>1257</v>
       </c>
       <c r="E430">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F430" t="s">
         <v>1279</v>
@@ -21888,7 +21888,7 @@
         <v>1257</v>
       </c>
       <c r="E431">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F431" t="s">
         <v>1279</v>
@@ -21923,7 +21923,7 @@
         <v>1257</v>
       </c>
       <c r="E432">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F432" t="s">
         <v>1281</v>
@@ -21958,7 +21958,7 @@
         <v>1257</v>
       </c>
       <c r="E433">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F433" t="s">
         <v>1279</v>
@@ -21993,7 +21993,7 @@
         <v>1258</v>
       </c>
       <c r="E434">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F434" t="s">
         <v>1279</v>
@@ -22028,7 +22028,7 @@
         <v>1258</v>
       </c>
       <c r="E435">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F435" t="s">
         <v>1279</v>
@@ -22063,7 +22063,7 @@
         <v>1258</v>
       </c>
       <c r="E436">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F436" t="s">
         <v>1279</v>
@@ -22098,7 +22098,7 @@
         <v>1258</v>
       </c>
       <c r="E437">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F437" t="s">
         <v>1279</v>
@@ -22133,7 +22133,7 @@
         <v>1258</v>
       </c>
       <c r="E438">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F438" t="s">
         <v>1279</v>
@@ -22171,7 +22171,7 @@
         <v>1258</v>
       </c>
       <c r="E439">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F439" t="s">
         <v>1281</v>
@@ -22209,7 +22209,7 @@
         <v>1258</v>
       </c>
       <c r="E440">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F440" t="s">
         <v>1281</v>
@@ -22244,7 +22244,7 @@
         <v>1259</v>
       </c>
       <c r="E441">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F441" t="s">
         <v>1279</v>
@@ -22279,7 +22279,7 @@
         <v>1259</v>
       </c>
       <c r="E442">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F442" t="s">
         <v>1279</v>
@@ -22314,7 +22314,7 @@
         <v>1259</v>
       </c>
       <c r="E443">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F443" t="s">
         <v>1279</v>
@@ -22349,7 +22349,7 @@
         <v>1260</v>
       </c>
       <c r="E444">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F444" t="s">
         <v>1279</v>
@@ -22384,7 +22384,7 @@
         <v>1260</v>
       </c>
       <c r="E445">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F445" t="s">
         <v>1279</v>
@@ -22419,7 +22419,7 @@
         <v>1260</v>
       </c>
       <c r="E446">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F446" t="s">
         <v>1281</v>
@@ -22457,7 +22457,7 @@
         <v>1260</v>
       </c>
       <c r="E447">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F447" t="s">
         <v>1279</v>
@@ -22492,7 +22492,7 @@
         <v>1261</v>
       </c>
       <c r="E448">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F448" t="s">
         <v>1279</v>
@@ -22527,7 +22527,7 @@
         <v>1261</v>
       </c>
       <c r="E449">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F449" t="s">
         <v>1279</v>
@@ -22562,7 +22562,7 @@
         <v>1262</v>
       </c>
       <c r="E450">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F450" t="s">
         <v>1281</v>
@@ -22600,7 +22600,7 @@
         <v>1262</v>
       </c>
       <c r="E451">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F451" t="s">
         <v>1279</v>
@@ -22635,7 +22635,7 @@
         <v>1262</v>
       </c>
       <c r="E452">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F452" t="s">
         <v>1279</v>
@@ -22670,7 +22670,7 @@
         <v>1263</v>
       </c>
       <c r="E453">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F453" t="s">
         <v>1281</v>
@@ -22705,7 +22705,7 @@
         <v>1263</v>
       </c>
       <c r="E454">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F454" t="s">
         <v>1279</v>
@@ -22740,7 +22740,7 @@
         <v>1263</v>
       </c>
       <c r="E455">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F455" t="s">
         <v>1281</v>
@@ -22778,7 +22778,7 @@
         <v>1263</v>
       </c>
       <c r="E456">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F456" t="s">
         <v>1279</v>
@@ -22813,7 +22813,7 @@
         <v>1263</v>
       </c>
       <c r="E457">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F457" t="s">
         <v>1279</v>
@@ -22848,7 +22848,7 @@
         <v>1264</v>
       </c>
       <c r="E458">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F458" t="s">
         <v>1279</v>
@@ -22883,7 +22883,7 @@
         <v>1264</v>
       </c>
       <c r="E459">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F459" t="s">
         <v>1279</v>
@@ -22918,7 +22918,7 @@
         <v>1265</v>
       </c>
       <c r="E460">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F460" t="s">
         <v>1279</v>
@@ -22953,7 +22953,7 @@
         <v>1265</v>
       </c>
       <c r="E461">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F461" t="s">
         <v>1279</v>
@@ -22988,7 +22988,7 @@
         <v>1265</v>
       </c>
       <c r="E462">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F462" t="s">
         <v>1279</v>
@@ -23023,7 +23023,7 @@
         <v>1265</v>
       </c>
       <c r="E463">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F463" t="s">
         <v>1281</v>
@@ -23061,7 +23061,7 @@
         <v>1266</v>
       </c>
       <c r="E464">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F464" t="s">
         <v>1279</v>
@@ -23096,7 +23096,7 @@
         <v>1266</v>
       </c>
       <c r="E465">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F465" t="s">
         <v>1283</v>
@@ -23134,7 +23134,7 @@
         <v>1266</v>
       </c>
       <c r="E466">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F466" t="s">
         <v>1279</v>
@@ -23169,7 +23169,7 @@
         <v>1266</v>
       </c>
       <c r="E467">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F467" t="s">
         <v>1279</v>
@@ -23204,7 +23204,7 @@
         <v>1267</v>
       </c>
       <c r="E468">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F468" t="s">
         <v>1279</v>
@@ -23239,7 +23239,7 @@
         <v>1267</v>
       </c>
       <c r="E469">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F469" t="s">
         <v>1279</v>
@@ -23274,7 +23274,7 @@
         <v>1267</v>
       </c>
       <c r="E470">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F470" t="s">
         <v>1279</v>
@@ -23309,7 +23309,7 @@
         <v>1267</v>
       </c>
       <c r="E471">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F471" t="s">
         <v>1279</v>
@@ -23344,7 +23344,7 @@
         <v>1267</v>
       </c>
       <c r="E472">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F472" t="s">
         <v>1279</v>
@@ -23379,7 +23379,7 @@
         <v>1267</v>
       </c>
       <c r="E473">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F473" t="s">
         <v>1281</v>
@@ -23417,7 +23417,7 @@
         <v>1268</v>
       </c>
       <c r="E474">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F474" t="s">
         <v>1279</v>
@@ -23452,7 +23452,7 @@
         <v>1268</v>
       </c>
       <c r="E475">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F475" t="s">
         <v>1281</v>
@@ -23487,7 +23487,7 @@
         <v>1269</v>
       </c>
       <c r="E476">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F476" t="s">
         <v>1281</v>
@@ -23525,7 +23525,7 @@
         <v>1269</v>
       </c>
       <c r="E477">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F477" t="s">
         <v>1281</v>
@@ -23563,7 +23563,7 @@
         <v>1269</v>
       </c>
       <c r="E478">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F478" t="s">
         <v>1279</v>
@@ -23598,7 +23598,7 @@
         <v>1269</v>
       </c>
       <c r="E479">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F479" t="s">
         <v>1279</v>
@@ -23633,7 +23633,7 @@
         <v>1270</v>
       </c>
       <c r="E480">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F480" t="s">
         <v>1279</v>
@@ -23668,7 +23668,7 @@
         <v>1271</v>
       </c>
       <c r="E481">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F481" t="s">
         <v>1279</v>
@@ -23703,7 +23703,7 @@
         <v>1271</v>
       </c>
       <c r="E482">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F482" t="s">
         <v>1279</v>
@@ -23738,7 +23738,7 @@
         <v>1271</v>
       </c>
       <c r="E483">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F483" t="s">
         <v>1279</v>
@@ -23773,7 +23773,7 @@
         <v>1271</v>
       </c>
       <c r="E484">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F484" t="s">
         <v>1279</v>
@@ -23808,7 +23808,7 @@
         <v>1271</v>
       </c>
       <c r="E485">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F485" t="s">
         <v>1279</v>
@@ -23843,7 +23843,7 @@
         <v>1271</v>
       </c>
       <c r="E486">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F486" t="s">
         <v>1279</v>
@@ -23878,7 +23878,7 @@
         <v>1271</v>
       </c>
       <c r="E487">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F487" t="s">
         <v>1279</v>
@@ -23913,7 +23913,7 @@
         <v>1271</v>
       </c>
       <c r="E488">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F488" t="s">
         <v>1281</v>
@@ -23951,7 +23951,7 @@
         <v>1272</v>
       </c>
       <c r="E489">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F489" t="s">
         <v>1279</v>
@@ -23986,7 +23986,7 @@
         <v>1272</v>
       </c>
       <c r="E490">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F490" t="s">
         <v>1279</v>
@@ -24021,7 +24021,7 @@
         <v>1272</v>
       </c>
       <c r="E491">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F491" t="s">
         <v>1279</v>
@@ -24056,7 +24056,7 @@
         <v>1272</v>
       </c>
       <c r="E492">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F492" t="s">
         <v>1281</v>
@@ -24094,7 +24094,7 @@
         <v>1272</v>
       </c>
       <c r="E493">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F493" t="s">
         <v>1281</v>
@@ -24132,7 +24132,7 @@
         <v>1272</v>
       </c>
       <c r="E494">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F494" t="s">
         <v>1281</v>
@@ -24170,7 +24170,7 @@
         <v>1272</v>
       </c>
       <c r="E495">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F495" t="s">
         <v>1279</v>
@@ -24205,7 +24205,7 @@
         <v>1273</v>
       </c>
       <c r="E496">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F496" t="s">
         <v>1281</v>
@@ -24243,7 +24243,7 @@
         <v>1273</v>
       </c>
       <c r="E497">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F497" t="s">
         <v>1281</v>
@@ -24281,7 +24281,7 @@
         <v>1274</v>
       </c>
       <c r="E498">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F498" t="s">
         <v>1281</v>
@@ -24319,7 +24319,7 @@
         <v>1274</v>
       </c>
       <c r="E499">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F499" t="s">
         <v>1279</v>
@@ -24354,7 +24354,7 @@
         <v>1275</v>
       </c>
       <c r="E500">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F500" t="s">
         <v>1279</v>
@@ -24389,7 +24389,7 @@
         <v>1275</v>
       </c>
       <c r="E501">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F501" t="s">
         <v>1279</v>
@@ -24427,7 +24427,7 @@
         <v>1275</v>
       </c>
       <c r="E502">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F502" t="s">
         <v>1281</v>
@@ -24465,7 +24465,7 @@
         <v>1276</v>
       </c>
       <c r="E503">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F503" t="s">
         <v>1279</v>
@@ -24503,7 +24503,7 @@
         <v>1276</v>
       </c>
       <c r="E504">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F504" t="s">
         <v>1279</v>
@@ -24538,7 +24538,7 @@
         <v>1276</v>
       </c>
       <c r="E505">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F505" t="s">
         <v>1279</v>
@@ -24573,7 +24573,7 @@
         <v>1276</v>
       </c>
       <c r="E506">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F506" t="s">
         <v>1279</v>
@@ -24608,7 +24608,7 @@
         <v>1276</v>
       </c>
       <c r="E507">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F507" t="s">
         <v>1279</v>
@@ -24643,7 +24643,7 @@
         <v>1276</v>
       </c>
       <c r="E508">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F508" t="s">
         <v>1281</v>
@@ -24681,7 +24681,7 @@
         <v>1277</v>
       </c>
       <c r="E509">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F509" t="s">
         <v>1279</v>
@@ -24716,7 +24716,7 @@
         <v>1277</v>
       </c>
       <c r="E510">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F510" t="s">
         <v>1279</v>
@@ -24751,7 +24751,7 @@
         <v>1277</v>
       </c>
       <c r="E511">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F511" t="s">
         <v>1279</v>
@@ -24786,7 +24786,7 @@
         <v>1277</v>
       </c>
       <c r="E512">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F512" t="s">
         <v>1279</v>
@@ -24821,7 +24821,7 @@
         <v>1277</v>
       </c>
       <c r="E513">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F513" t="s">
         <v>1279</v>
@@ -24856,7 +24856,7 @@
         <v>1277</v>
       </c>
       <c r="E514">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F514" t="s">
         <v>1279</v>
@@ -24891,7 +24891,7 @@
         <v>1278</v>
       </c>
       <c r="E515">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F515" t="s">
         <v>1279</v>
@@ -24929,7 +24929,7 @@
         <v>1278</v>
       </c>
       <c r="E516">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F516" t="s">
         <v>1279</v>
@@ -24964,7 +24964,7 @@
         <v>1278</v>
       </c>
       <c r="E517">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F517" t="s">
         <v>1279</v>
@@ -24999,7 +24999,7 @@
         <v>1278</v>
       </c>
       <c r="E518">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F518" t="s">
         <v>1279</v>
@@ -25037,7 +25037,7 @@
         <v>1278</v>
       </c>
       <c r="E519">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F519" t="s">
         <v>1279</v>
@@ -25072,7 +25072,7 @@
         <v>1278</v>
       </c>
       <c r="E520">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F520" t="s">
         <v>1281</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-21 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7450,9 +7450,6 @@
     <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
-    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
     <t>PATRIMÔNIO HISTÓRICO E CULTURAL,URBANISMO</t>
   </si>
   <si>
@@ -7474,40 +7471,43 @@
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>VALORAÇÃO DANOS AMBIENTAIS,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
+  </si>
+  <si>
+    <t>URBANISMO,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>FARMÁCIA,SAÚDE</t>
+  </si>
+  <si>
+    <t>ENGENHARIA AMBIENTAL,BIOLOGIA</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>RECURSOS HÍDRICOS,VALORAÇÃO DANOS AMBIENTAIS</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
-  </si>
-  <si>
-    <t>URBANISMO,BIOLOGIA</t>
-  </si>
-  <si>
-    <t>FARMÁCIA,SAÚDE</t>
-  </si>
-  <si>
-    <t>ENGENHARIA AMBIENTAL,BIOLOGIA</t>
-  </si>
-  <si>
     <t>BIOLOGIA,GEOLOGIA</t>
   </si>
   <si>
-    <t>BIOLOGIA,RECURSOS HÍDRICOS,MOBILIDADE E TRANSPORTE,URBANISMO</t>
+    <t>MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS,BIOLOGIA,URBANISMO</t>
   </si>
   <si>
     <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
@@ -7516,16 +7516,16 @@
     <t>GEOLOGIA,ENGENHARIA QUÍMICA</t>
   </si>
   <si>
-    <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ENGENHARIA CIVIL</t>
   </si>
   <si>
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ORÇAMENTO,SAÚDE,PSICOLOGIA,SAÚDE MENTAL,MOBILIDADE E TRANSPORTE,ECONOMICIDADE CONTÁBIL,URBANISMO,ASSISTÊNCIA SOCIAL,ECONOMIA</t>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>SAÚDE MENTAL,SAÚDE,ECONOMICIDADE CONTÁBIL,AVALIAÇÃO DE IMÓVEIS,ECONOMIA,URBANISMO,MOBILIDADE E TRANSPORTE,PSICOLOGIA,ASSISTÊNCIA SOCIAL,ORÇAMENTO</t>
   </si>
 </sst>
 </file>
@@ -19667,7 +19667,7 @@
         <v>2329</v>
       </c>
       <c r="L336" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="337" spans="1:12">
@@ -20440,7 +20440,7 @@
         <v>2327</v>
       </c>
       <c r="L358" t="s">
-        <v>2479</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="359" spans="1:12">
@@ -20475,7 +20475,7 @@
         <v>2336</v>
       </c>
       <c r="L359" t="s">
-        <v>2480</v>
+        <v>2479</v>
       </c>
     </row>
     <row r="360" spans="1:12">
@@ -20580,7 +20580,7 @@
         <v>2318</v>
       </c>
       <c r="L362" t="s">
-        <v>2481</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="363" spans="1:12">
@@ -20895,7 +20895,7 @@
         <v>2387</v>
       </c>
       <c r="L371" t="s">
-        <v>2482</v>
+        <v>2481</v>
       </c>
     </row>
     <row r="372" spans="1:12">
@@ -21490,7 +21490,7 @@
         <v>2335</v>
       </c>
       <c r="L388" t="s">
-        <v>2483</v>
+        <v>2482</v>
       </c>
     </row>
     <row r="389" spans="1:12">
@@ -21595,7 +21595,7 @@
         <v>2351</v>
       </c>
       <c r="L391" t="s">
-        <v>2484</v>
+        <v>2483</v>
       </c>
     </row>
     <row r="392" spans="1:12">
@@ -21913,7 +21913,7 @@
         <v>2336</v>
       </c>
       <c r="L400" t="s">
-        <v>2480</v>
+        <v>2479</v>
       </c>
     </row>
     <row r="401" spans="1:12">
@@ -23494,7 +23494,7 @@
         <v>2356</v>
       </c>
       <c r="L445" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="446" spans="1:12">
@@ -23529,7 +23529,7 @@
         <v>2399</v>
       </c>
       <c r="L446" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="447" spans="1:12">
@@ -23564,7 +23564,7 @@
         <v>2399</v>
       </c>
       <c r="L447" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="448" spans="1:12">
@@ -23599,7 +23599,7 @@
         <v>2399</v>
       </c>
       <c r="L448" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="449" spans="1:12">
@@ -23634,7 +23634,7 @@
         <v>2399</v>
       </c>
       <c r="L449" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="450" spans="1:12">
@@ -23669,7 +23669,7 @@
         <v>2399</v>
       </c>
       <c r="L450" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="451" spans="1:12">
@@ -23704,7 +23704,7 @@
         <v>2399</v>
       </c>
       <c r="L451" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="452" spans="1:12">
@@ -23739,7 +23739,7 @@
         <v>2399</v>
       </c>
       <c r="L452" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="453" spans="1:12">
@@ -23774,7 +23774,7 @@
         <v>2399</v>
       </c>
       <c r="L453" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="454" spans="1:12">
@@ -23809,7 +23809,7 @@
         <v>2399</v>
       </c>
       <c r="L454" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="455" spans="1:12">
@@ -23844,7 +23844,7 @@
         <v>2399</v>
       </c>
       <c r="L455" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="456" spans="1:12">
@@ -23879,7 +23879,7 @@
         <v>2399</v>
       </c>
       <c r="L456" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="457" spans="1:12">
@@ -23914,7 +23914,7 @@
         <v>2399</v>
       </c>
       <c r="L457" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="458" spans="1:12">
@@ -23949,7 +23949,7 @@
         <v>2399</v>
       </c>
       <c r="L458" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="459" spans="1:12">
@@ -23984,7 +23984,7 @@
         <v>2399</v>
       </c>
       <c r="L459" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="460" spans="1:12">
@@ -24019,7 +24019,7 @@
         <v>2399</v>
       </c>
       <c r="L460" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="461" spans="1:12">
@@ -24054,7 +24054,7 @@
         <v>2399</v>
       </c>
       <c r="L461" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="462" spans="1:12">
@@ -24089,7 +24089,7 @@
         <v>2399</v>
       </c>
       <c r="L462" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="463" spans="1:12">
@@ -24124,7 +24124,7 @@
         <v>2399</v>
       </c>
       <c r="L463" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="464" spans="1:12">
@@ -24299,7 +24299,7 @@
         <v>2388</v>
       </c>
       <c r="L468" t="s">
-        <v>2486</v>
+        <v>2485</v>
       </c>
     </row>
     <row r="469" spans="1:12">
@@ -24655,7 +24655,7 @@
         <v>2316</v>
       </c>
       <c r="L478" t="s">
-        <v>2487</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="479" spans="1:12">
@@ -24690,7 +24690,7 @@
         <v>2356</v>
       </c>
       <c r="L479" t="s">
-        <v>2488</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="480" spans="1:12">
@@ -25323,7 +25323,7 @@
         <v>2334</v>
       </c>
       <c r="L497" t="s">
-        <v>2432</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="498" spans="1:12">
@@ -25428,7 +25428,7 @@
         <v>2357</v>
       </c>
       <c r="L500" t="s">
-        <v>2489</v>
+        <v>2488</v>
       </c>
     </row>
     <row r="501" spans="1:12">
@@ -25463,7 +25463,7 @@
         <v>2311</v>
       </c>
       <c r="L501" t="s">
-        <v>2488</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="502" spans="1:12">
@@ -25854,7 +25854,7 @@
         <v>2307</v>
       </c>
       <c r="L512" t="s">
-        <v>2490</v>
+        <v>2489</v>
       </c>
     </row>
     <row r="513" spans="1:12">
@@ -26134,7 +26134,7 @@
         <v>2332</v>
       </c>
       <c r="L520" t="s">
-        <v>2491</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="521" spans="1:12">
@@ -26169,7 +26169,7 @@
         <v>2326</v>
       </c>
       <c r="L521" t="s">
-        <v>2492</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="522" spans="1:12">
@@ -26417,7 +26417,7 @@
         <v>2405</v>
       </c>
       <c r="L528" t="s">
-        <v>2493</v>
+        <v>2492</v>
       </c>
     </row>
     <row r="529" spans="1:12">
@@ -26557,7 +26557,7 @@
         <v>2344</v>
       </c>
       <c r="L532" t="s">
-        <v>2494</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="533" spans="1:12">
@@ -27056,7 +27056,7 @@
         <v>2334</v>
       </c>
       <c r="L546" t="s">
-        <v>2434</v>
+        <v>2492</v>
       </c>
     </row>
     <row r="547" spans="1:12">
@@ -27126,7 +27126,7 @@
         <v>2334</v>
       </c>
       <c r="L548" t="s">
-        <v>2495</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="549" spans="1:12">
@@ -27196,7 +27196,7 @@
         <v>2338</v>
       </c>
       <c r="L550" t="s">
-        <v>2486</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="551" spans="1:12">
@@ -27371,7 +27371,7 @@
         <v>2350</v>
       </c>
       <c r="L555" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="556" spans="1:12">
@@ -27657,7 +27657,7 @@
         <v>2409</v>
       </c>
       <c r="L563" t="s">
-        <v>2481</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="564" spans="1:12">
@@ -27692,7 +27692,7 @@
         <v>2409</v>
       </c>
       <c r="L564" t="s">
-        <v>2488</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="565" spans="1:12">
@@ -27940,7 +27940,7 @@
         <v>2323</v>
       </c>
       <c r="L571" t="s">
-        <v>2492</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="572" spans="1:12">
@@ -29192,7 +29192,7 @@
         <v>2323</v>
       </c>
       <c r="L606" t="s">
-        <v>2481</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="607" spans="1:12">
@@ -29227,7 +29227,7 @@
         <v>2349</v>
       </c>
       <c r="L607" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="608" spans="1:12">
@@ -29691,7 +29691,7 @@
         <v>2412</v>
       </c>
       <c r="L620" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="621" spans="1:12">
@@ -29726,7 +29726,7 @@
         <v>2336</v>
       </c>
       <c r="L621" t="s">
-        <v>2500</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="622" spans="1:12">
@@ -29764,7 +29764,7 @@
         <v>2413</v>
       </c>
       <c r="L622" t="s">
-        <v>2481</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="623" spans="1:12">
@@ -29834,7 +29834,7 @@
         <v>2414</v>
       </c>
       <c r="L624" t="s">
-        <v>2501</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="625" spans="1:12">
@@ -29869,7 +29869,7 @@
         <v>2346</v>
       </c>
       <c r="L625" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="626" spans="1:12">
@@ -30044,7 +30044,7 @@
         <v>2416</v>
       </c>
       <c r="L630" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="631" spans="1:12">
@@ -30082,7 +30082,7 @@
         <v>2417</v>
       </c>
       <c r="L631" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="632" spans="1:12">
@@ -30117,7 +30117,7 @@
         <v>2308</v>
       </c>
       <c r="L632" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="633" spans="1:12">
@@ -30152,7 +30152,7 @@
         <v>2308</v>
       </c>
       <c r="L633" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="634" spans="1:12">
@@ -30260,7 +30260,7 @@
         <v>2418</v>
       </c>
       <c r="L636" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="637" spans="1:12">
@@ -30295,7 +30295,7 @@
         <v>2353</v>
       </c>
       <c r="L637" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
     </row>
     <row r="638" spans="1:12">
@@ -30327,7 +30327,7 @@
         <v>2419</v>
       </c>
       <c r="L638" t="s">
-        <v>2438</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="639" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-23 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6490" uniqueCount="2509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6490" uniqueCount="2512">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7498,49 +7498,58 @@
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
+  </si>
+  <si>
+    <t>FARMÁCIA,SAÚDE</t>
+  </si>
+  <si>
+    <t>URBANISMO,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA AMBIENTAL,BIOLOGIA</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
-  </si>
-  <si>
-    <t>FARMÁCIA,SAÚDE</t>
-  </si>
-  <si>
-    <t>URBANISMO,BIOLOGIA</t>
+    <t>BIOLOGIA,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>URBANISMO,MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
     <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
-    <t>BIOLOGIA,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,URBANISMO,MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA AMBIENTAL,BIOLOGIA</t>
-  </si>
-  <si>
     <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,ASSISTÊNCIA SOCIAL,SAÚDE,URBANISMO,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,MOBILIDADE E TRANSPORTE,ECONOMIA,SAÚDE MENTAL,ORÇAMENTO</t>
+    <t>ENGENHARIA FLORESTAL,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>PSICOLOGIA,URBANISMO,ASSISTÊNCIA SOCIAL,SAÚDE,MOBILIDADE E TRANSPORTE,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS,SAÚDE MENTAL,ECONOMIA,ECONOMICIDADE CONTÁBIL</t>
   </si>
 </sst>
 </file>
@@ -15755,7 +15764,7 @@
     </row>
     <row r="225" spans="1:12">
       <c r="A225" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B225" t="s">
         <v>264</v>
@@ -15776,7 +15785,7 @@
         <v>1542</v>
       </c>
       <c r="I225" t="s">
-        <v>1632</v>
+        <v>1574</v>
       </c>
       <c r="J225" t="s">
         <v>1903</v>
@@ -16318,7 +16327,7 @@
     </row>
     <row r="241" spans="1:12">
       <c r="A241" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B241" t="s">
         <v>280</v>
@@ -16342,7 +16351,7 @@
         <v>1547</v>
       </c>
       <c r="I241" t="s">
-        <v>1632</v>
+        <v>1574</v>
       </c>
       <c r="J241" t="s">
         <v>1919</v>
@@ -26779,7 +26788,7 @@
         <v>2348</v>
       </c>
       <c r="L538" t="s">
-        <v>2494</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="539" spans="1:12">
@@ -27634,7 +27643,7 @@
         <v>2352</v>
       </c>
       <c r="L562" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="563" spans="1:12">
@@ -27914,7 +27923,7 @@
         <v>2319</v>
       </c>
       <c r="L570" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="571" spans="1:12">
@@ -28197,7 +28206,7 @@
         <v>2314</v>
       </c>
       <c r="L578" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="579" spans="1:12">
@@ -29201,7 +29210,7 @@
         <v>2346</v>
       </c>
       <c r="L606" t="s">
-        <v>2506</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="607" spans="1:12">
@@ -29309,7 +29318,7 @@
         <v>2424</v>
       </c>
       <c r="L609" t="s">
-        <v>2507</v>
+        <v>2508</v>
       </c>
     </row>
     <row r="610" spans="1:12">
@@ -29983,7 +29992,7 @@
         <v>2364</v>
       </c>
       <c r="L628" t="s">
-        <v>2493</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -30453,7 +30462,7 @@
         <v>2314</v>
       </c>
       <c r="L641" t="s">
-        <v>2484</v>
+        <v>2509</v>
       </c>
     </row>
     <row r="642" spans="1:12">
@@ -30558,7 +30567,7 @@
         <v>2428</v>
       </c>
       <c r="L644" t="s">
-        <v>2447</v>
+        <v>2510</v>
       </c>
     </row>
     <row r="645" spans="1:12">
@@ -30590,7 +30599,7 @@
         <v>2428</v>
       </c>
       <c r="L645" t="s">
-        <v>2508</v>
+        <v>2511</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-24 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6395" uniqueCount="2476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6395" uniqueCount="2474">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7369,9 +7369,6 @@
     <t>ECONOMICIDADE OBRAS,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
-    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
     <t>PATRIMÔNIO HISTÓRICO E CULTURAL,URBANISMO</t>
   </si>
   <si>
@@ -7405,6 +7402,9 @@
     <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
+    <t>URBANISMO,BIOLOGIA</t>
+  </si>
+  <si>
     <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
@@ -7414,34 +7414,28 @@
     <t>ENGENHARIA FLORESTAL,URBANISMO</t>
   </si>
   <si>
-    <t>URBANISMO,BIOLOGIA</t>
-  </si>
-  <si>
     <t>FARMÁCIA,SAÚDE</t>
   </si>
   <si>
     <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
-    <t>URBANISMO,ENGENHARIA FLORESTAL</t>
-  </si>
-  <si>
     <t>BIOLOGIA,GEOLOGIA</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,BIOLOGIA,URBANISMO,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,BIOLOGIA,URBANISMO,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA AMBIENTAL,BIOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
-  </si>
-  <si>
-    <t>SAÚDE MENTAL,MOBILIDADE E TRANSPORTE,SAÚDE,ASSISTÊNCIA SOCIAL,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,URBANISMO,ECONOMIA,ECONOMICIDADE CONTÁBIL</t>
+    <t>MOBILIDADE E TRANSPORTE,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>MOBILIDADE E TRANSPORTE,SAÚDE MENTAL,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,URBANISMO,ORÇAMENTO,ECONOMICIDADE CONTÁBIL,ECONOMIA,SAÚDE,PSICOLOGIA</t>
   </si>
 </sst>
 </file>
@@ -19122,7 +19116,7 @@
         <v>2306</v>
       </c>
       <c r="L323" t="s">
-        <v>2451</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="324" spans="1:12">
@@ -19895,7 +19889,7 @@
         <v>2304</v>
       </c>
       <c r="L345" t="s">
-        <v>2452</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="346" spans="1:12">
@@ -19930,7 +19924,7 @@
         <v>2312</v>
       </c>
       <c r="L346" t="s">
-        <v>2453</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="347" spans="1:12">
@@ -20035,7 +20029,7 @@
         <v>2297</v>
       </c>
       <c r="L349" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="350" spans="1:12">
@@ -20350,7 +20344,7 @@
         <v>2365</v>
       </c>
       <c r="L358" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="359" spans="1:12">
@@ -20735,7 +20729,7 @@
         <v>2358</v>
       </c>
       <c r="L369" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="370" spans="1:12">
@@ -20840,7 +20834,7 @@
         <v>2341</v>
       </c>
       <c r="L372" t="s">
-        <v>2457</v>
+        <v>2456</v>
       </c>
     </row>
     <row r="373" spans="1:12">
@@ -20945,7 +20939,7 @@
         <v>2328</v>
       </c>
       <c r="L375" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="376" spans="1:12">
@@ -21228,7 +21222,7 @@
         <v>2312</v>
       </c>
       <c r="L383" t="s">
-        <v>2453</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="384" spans="1:12">
@@ -21298,7 +21292,7 @@
         <v>2371</v>
       </c>
       <c r="L385" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="386" spans="1:12">
@@ -21581,7 +21575,7 @@
         <v>2372</v>
       </c>
       <c r="L393" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="394" spans="1:12">
@@ -21651,7 +21645,7 @@
         <v>2372</v>
       </c>
       <c r="L395" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="396" spans="1:12">
@@ -22774,7 +22768,7 @@
         <v>2334</v>
       </c>
       <c r="L427" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="428" spans="1:12">
@@ -22809,7 +22803,7 @@
         <v>2375</v>
       </c>
       <c r="L428" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="429" spans="1:12">
@@ -22844,7 +22838,7 @@
         <v>2375</v>
       </c>
       <c r="L429" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="430" spans="1:12">
@@ -22879,7 +22873,7 @@
         <v>2375</v>
       </c>
       <c r="L430" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="431" spans="1:12">
@@ -22914,7 +22908,7 @@
         <v>2375</v>
       </c>
       <c r="L431" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="432" spans="1:12">
@@ -22949,7 +22943,7 @@
         <v>2375</v>
       </c>
       <c r="L432" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="433" spans="1:12">
@@ -22984,7 +22978,7 @@
         <v>2375</v>
       </c>
       <c r="L433" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="434" spans="1:12">
@@ -23019,7 +23013,7 @@
         <v>2375</v>
       </c>
       <c r="L434" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="435" spans="1:12">
@@ -23054,7 +23048,7 @@
         <v>2375</v>
       </c>
       <c r="L435" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="436" spans="1:12">
@@ -23089,7 +23083,7 @@
         <v>2375</v>
       </c>
       <c r="L436" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="437" spans="1:12">
@@ -23124,7 +23118,7 @@
         <v>2375</v>
       </c>
       <c r="L437" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="438" spans="1:12">
@@ -23159,7 +23153,7 @@
         <v>2375</v>
       </c>
       <c r="L438" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="439" spans="1:12">
@@ -23194,7 +23188,7 @@
         <v>2375</v>
       </c>
       <c r="L439" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="440" spans="1:12">
@@ -23229,7 +23223,7 @@
         <v>2375</v>
       </c>
       <c r="L440" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="441" spans="1:12">
@@ -23264,7 +23258,7 @@
         <v>2375</v>
       </c>
       <c r="L441" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="442" spans="1:12">
@@ -23299,7 +23293,7 @@
         <v>2375</v>
       </c>
       <c r="L442" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="443" spans="1:12">
@@ -23334,7 +23328,7 @@
         <v>2375</v>
       </c>
       <c r="L443" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="444" spans="1:12">
@@ -23369,7 +23363,7 @@
         <v>2375</v>
       </c>
       <c r="L444" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="445" spans="1:12">
@@ -23404,7 +23398,7 @@
         <v>2375</v>
       </c>
       <c r="L445" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="446" spans="1:12">
@@ -23474,7 +23468,7 @@
         <v>2376</v>
       </c>
       <c r="L447" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="448" spans="1:12">
@@ -23579,7 +23573,7 @@
         <v>2366</v>
       </c>
       <c r="L450" t="s">
-        <v>2460</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="451" spans="1:12">
@@ -23935,7 +23929,7 @@
         <v>2295</v>
       </c>
       <c r="L460" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="461" spans="1:12">
@@ -23970,7 +23964,7 @@
         <v>2334</v>
       </c>
       <c r="L461" t="s">
-        <v>2462</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="462" spans="1:12">
@@ -24040,7 +24034,7 @@
         <v>2378</v>
       </c>
       <c r="L463" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="464" spans="1:12">
@@ -24358,7 +24352,7 @@
         <v>2379</v>
       </c>
       <c r="L472" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="473" spans="1:12">
@@ -24463,7 +24457,7 @@
         <v>2291</v>
       </c>
       <c r="L475" t="s">
-        <v>2447</v>
+        <v>2403</v>
       </c>
     </row>
     <row r="476" spans="1:12">
@@ -24533,7 +24527,7 @@
         <v>2319</v>
       </c>
       <c r="L477" t="s">
-        <v>2431</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="478" spans="1:12">
@@ -24568,7 +24562,7 @@
         <v>2358</v>
       </c>
       <c r="L478" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="479" spans="1:12">
@@ -24743,7 +24737,7 @@
         <v>2290</v>
       </c>
       <c r="L483" t="s">
-        <v>2462</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="484" spans="1:12">
@@ -24813,7 +24807,7 @@
         <v>2380</v>
       </c>
       <c r="L485" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="486" spans="1:12">
@@ -25548,7 +25542,7 @@
         <v>2382</v>
       </c>
       <c r="L506" t="s">
-        <v>2466</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="507" spans="1:12">
@@ -25688,7 +25682,7 @@
         <v>2321</v>
       </c>
       <c r="L510" t="s">
-        <v>2467</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="511" spans="1:12">
@@ -26152,7 +26146,7 @@
         <v>2310</v>
       </c>
       <c r="L523" t="s">
-        <v>2466</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="524" spans="1:12">
@@ -26222,7 +26216,7 @@
         <v>2310</v>
       </c>
       <c r="L525" t="s">
-        <v>2468</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="526" spans="1:12">
@@ -26292,7 +26286,7 @@
         <v>2314</v>
       </c>
       <c r="L527" t="s">
-        <v>2460</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="528" spans="1:12">
@@ -26467,7 +26461,7 @@
         <v>2327</v>
       </c>
       <c r="L532" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="533" spans="1:12">
@@ -26683,7 +26677,7 @@
         <v>2378</v>
       </c>
       <c r="L538" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="539" spans="1:12">
@@ -26753,7 +26747,7 @@
         <v>2386</v>
       </c>
       <c r="L540" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="541" spans="1:12">
@@ -27001,7 +26995,7 @@
         <v>2316</v>
       </c>
       <c r="L547" t="s">
-        <v>2469</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="548" spans="1:12">
@@ -27147,7 +27141,7 @@
         <v>2318</v>
       </c>
       <c r="L551" t="s">
-        <v>2470</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="552" spans="1:12">
@@ -27427,7 +27421,7 @@
         <v>2286</v>
       </c>
       <c r="L559" t="s">
-        <v>2471</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="560" spans="1:12">
@@ -27710,7 +27704,7 @@
         <v>2281</v>
       </c>
       <c r="L567" t="s">
-        <v>2472</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="568" spans="1:12">
@@ -28180,7 +28174,7 @@
         <v>2316</v>
       </c>
       <c r="L580" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="581" spans="1:12">
@@ -28215,7 +28209,7 @@
         <v>2326</v>
       </c>
       <c r="L581" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="582" spans="1:12">
@@ -28539,7 +28533,7 @@
         <v>2388</v>
       </c>
       <c r="L590" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="591" spans="1:12">
@@ -28679,7 +28673,7 @@
         <v>2389</v>
       </c>
       <c r="L594" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -28714,7 +28708,7 @@
         <v>2312</v>
       </c>
       <c r="L595" t="s">
-        <v>2473</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="596" spans="1:12">
@@ -28784,7 +28778,7 @@
         <v>2390</v>
       </c>
       <c r="L597" t="s">
-        <v>2474</v>
+        <v>2471</v>
       </c>
     </row>
     <row r="598" spans="1:12">
@@ -28819,7 +28813,7 @@
         <v>2323</v>
       </c>
       <c r="L598" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="599" spans="1:12">
@@ -28959,7 +28953,7 @@
         <v>2391</v>
       </c>
       <c r="L602" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="603" spans="1:12">
@@ -28997,7 +28991,7 @@
         <v>2392</v>
       </c>
       <c r="L603" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="604" spans="1:12">
@@ -29175,7 +29169,7 @@
         <v>2330</v>
       </c>
       <c r="L608" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="609" spans="1:12">
@@ -29210,7 +29204,7 @@
         <v>2353</v>
       </c>
       <c r="L609" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="610" spans="1:12">
@@ -30129,7 +30123,7 @@
         <v>2393</v>
       </c>
       <c r="L635" t="s">
-        <v>2412</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="636" spans="1:12">
@@ -30161,7 +30155,7 @@
         <v>2393</v>
       </c>
       <c r="L636" t="s">
-        <v>2475</v>
+        <v>2473</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-25 20:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6391" uniqueCount="2477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6391" uniqueCount="2479">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7402,49 +7402,55 @@
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
+  </si>
+  <si>
+    <t>FARMÁCIA,SAÚDE</t>
+  </si>
+  <si>
+    <t>URBANISMO,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
-  </si>
-  <si>
-    <t>URBANISMO,BIOLOGIA</t>
-  </si>
-  <si>
-    <t>FARMÁCIA,SAÚDE</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE,URBANISMO,BIOLOGIA,RECURSOS HÍDRICOS</t>
+    <t>URBANISMO,ENGENHARIA FLORESTAL</t>
+  </si>
+  <si>
+    <t>URBANISMO,BIOLOGIA,MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA AMBIENTAL,BIOLOGIA</t>
-  </si>
-  <si>
     <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
+    <t>ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE</t>
+  </si>
+  <si>
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>ORÇAMENTO,ECONOMICIDADE CONTÁBIL,AVALIAÇÃO DE IMÓVEIS,SAÚDE,SAÚDE MENTAL,URBANISMO,ECONOMIA,PSICOLOGIA,MOBILIDADE E TRANSPORTE,ASSISTÊNCIA SOCIAL</t>
+    <t>ASSISTÊNCIA SOCIAL,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL,SAÚDE,ECONOMIA,SAÚDE MENTAL,PSICOLOGIA,URBANISMO,ORÇAMENTO</t>
   </si>
 </sst>
 </file>
@@ -25411,7 +25417,7 @@
         <v>2383</v>
       </c>
       <c r="L502" t="s">
-        <v>2468</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="503" spans="1:12">
@@ -25551,7 +25557,7 @@
         <v>2321</v>
       </c>
       <c r="L506" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="507" spans="1:12">
@@ -25977,7 +25983,7 @@
         <v>2310</v>
       </c>
       <c r="L518" t="s">
-        <v>2407</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="519" spans="1:12">
@@ -26117,7 +26123,7 @@
         <v>2315</v>
       </c>
       <c r="L522" t="s">
-        <v>2462</v>
+        <v>2471</v>
       </c>
     </row>
     <row r="523" spans="1:12">
@@ -26826,7 +26832,7 @@
         <v>2317</v>
       </c>
       <c r="L542" t="s">
-        <v>2467</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="543" spans="1:12">
@@ -27214,7 +27220,7 @@
         <v>2286</v>
       </c>
       <c r="L553" t="s">
-        <v>2471</v>
+        <v>2473</v>
       </c>
     </row>
     <row r="554" spans="1:12">
@@ -27497,7 +27503,7 @@
         <v>2281</v>
       </c>
       <c r="L561" t="s">
-        <v>2472</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="562" spans="1:12">
@@ -28387,7 +28393,7 @@
         <v>2312</v>
       </c>
       <c r="L586" t="s">
-        <v>2473</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="587" spans="1:12">
@@ -28457,7 +28463,7 @@
         <v>2391</v>
       </c>
       <c r="L588" t="s">
-        <v>2474</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="589" spans="1:12">
@@ -29875,7 +29881,7 @@
         <v>2325</v>
       </c>
       <c r="L628" t="s">
-        <v>2432</v>
+        <v>2476</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -30120,7 +30126,7 @@
         <v>2394</v>
       </c>
       <c r="L635" t="s">
-        <v>2475</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="636" spans="1:12">
@@ -30152,7 +30158,7 @@
         <v>2394</v>
       </c>
       <c r="L636" t="s">
-        <v>2476</v>
+        <v>2478</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-28 22:30:05
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4822,64 +4822,64 @@
     <t>HUDSON DE OLIVEIRA SACRAMENTO</t>
   </si>
   <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA</t>
+  </si>
+  <si>
+    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>PABLO GINIO VIMERCATI SIMAS</t>
+  </si>
+  <si>
+    <t>THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>FERNANDA FERREIRA FONTES,JULIANA MARTINS BAHIENSE,RODRIGO VALENTE SERRA</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
+  </si>
+  <si>
+    <t>RODRIGO VENTURA MARRA,THIAGO JOSÉ DUPRAT FORTES</t>
+  </si>
+  <si>
+    <t>CHRISTIANA ROSA FERREIRA</t>
+  </si>
+  <si>
+    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
+  </si>
+  <si>
+    <t>JULIANA MARTINS BAHIENSE,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
+  </si>
+  <si>
+    <t>MARINA DE AQUINO PARREIRA XAVIER, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>EDUARDO COUTO SOLEDADE</t>
+  </si>
+  <si>
+    <t>HELENA FERREIRA DE LIMA</t>
+  </si>
+  <si>
+    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
+    <t>SEZISNANDO JOSE PRIMO PAES</t>
+  </si>
+  <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
+    <t>DIANA DELGADO DA COSTA DA SILVA,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>DIANA DELGADO DA COSTA DA SILVA</t>
+  </si>
+  <si>
+    <t>RANAILLA LIMA BANDEIRA DOS SANTOS, _SEM USUARIO ATRIBUIDO</t>
+  </si>
+  <si>
     <t>GLAUCO CASTILHO DE ALMEIDA</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA</t>
-  </si>
-  <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,ALEXANDER MAGNO BORGES GOMES DA SILVA,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>PABLO GINIO VIMERCATI SIMAS</t>
-  </si>
-  <si>
-    <t>THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>FERNANDA FERREIRA FONTES,JULIANA MARTINS BAHIENSE,RODRIGO VALENTE SERRA</t>
-  </si>
-  <si>
-    <t>PEDRO HENRIQUE DE MESQUITA MAGALHÃES</t>
-  </si>
-  <si>
-    <t>RODRIGO VENTURA MARRA,THIAGO JOSÉ DUPRAT FORTES</t>
-  </si>
-  <si>
-    <t>CHRISTIANA ROSA FERREIRA</t>
-  </si>
-  <si>
-    <t>HEITOR DE FÁTIMA BARBOSA DA SILVA</t>
-  </si>
-  <si>
-    <t>JULIANA MARTINS BAHIENSE,MARIA JOSÉ LOPES DE ARAUJO SAROLDI</t>
-  </si>
-  <si>
-    <t>MARINA DE AQUINO PARREIRA XAVIER, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>EDUARDO COUTO SOLEDADE</t>
-  </si>
-  <si>
-    <t>HELENA FERREIRA DE LIMA</t>
-  </si>
-  <si>
-    <t>LUIZ FRANCISCO PERALTA BRAGA,MARCELO SILVA DE AZEVEDO, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>SEZISNANDO JOSE PRIMO PAES</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
-  </si>
-  <si>
-    <t>DIANA DELGADO DA COSTA DA SILVA,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>DIANA DELGADO DA COSTA DA SILVA</t>
-  </si>
-  <si>
-    <t>RANAILLA LIMA BANDEIRA DOS SANTOS, _SEM USUARIO ATRIBUIDO</t>
   </si>
   <si>
     <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
@@ -13751,7 +13751,7 @@
     </row>
     <row r="171" spans="1:12">
       <c r="A171" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="B171" t="s">
         <v>211</v>
@@ -13772,7 +13772,7 @@
         <v>1514</v>
       </c>
       <c r="I171" t="s">
-        <v>1602</v>
+        <v>1546</v>
       </c>
       <c r="J171" t="s">
         <v>1822</v>
@@ -13947,7 +13947,7 @@
         <v>1514</v>
       </c>
       <c r="I176" t="s">
-        <v>1603</v>
+        <v>1602</v>
       </c>
       <c r="J176" t="s">
         <v>1827</v>
@@ -13982,7 +13982,7 @@
         <v>1514</v>
       </c>
       <c r="I177" t="s">
-        <v>1604</v>
+        <v>1603</v>
       </c>
       <c r="J177" t="s">
         <v>1828</v>
@@ -14157,7 +14157,7 @@
         <v>1514</v>
       </c>
       <c r="I182" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J182" t="s">
         <v>1833</v>
@@ -14192,7 +14192,7 @@
         <v>1514</v>
       </c>
       <c r="I183" t="s">
-        <v>1606</v>
+        <v>1605</v>
       </c>
       <c r="J183" t="s">
         <v>1834</v>
@@ -14332,7 +14332,7 @@
         <v>1514</v>
       </c>
       <c r="I187" t="s">
-        <v>1607</v>
+        <v>1606</v>
       </c>
       <c r="J187" t="s">
         <v>1838</v>
@@ -14402,7 +14402,7 @@
         <v>1514</v>
       </c>
       <c r="I189" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J189" t="s">
         <v>1840</v>
@@ -14437,7 +14437,7 @@
         <v>1514</v>
       </c>
       <c r="I190" t="s">
-        <v>1609</v>
+        <v>1608</v>
       </c>
       <c r="J190" t="s">
         <v>1841</v>
@@ -14615,7 +14615,7 @@
         <v>1514</v>
       </c>
       <c r="I195" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="J195" t="s">
         <v>1846</v>
@@ -14650,7 +14650,7 @@
         <v>1514</v>
       </c>
       <c r="I196" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J196" t="s">
         <v>1847</v>
@@ -14685,7 +14685,7 @@
         <v>1514</v>
       </c>
       <c r="I197" t="s">
-        <v>1612</v>
+        <v>1611</v>
       </c>
       <c r="J197" t="s">
         <v>1848</v>
@@ -14965,7 +14965,7 @@
         <v>1514</v>
       </c>
       <c r="I205" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J205" t="s">
         <v>1856</v>
@@ -15035,7 +15035,7 @@
         <v>1514</v>
       </c>
       <c r="I207" t="s">
-        <v>1614</v>
+        <v>1613</v>
       </c>
       <c r="J207" t="s">
         <v>1858</v>
@@ -15245,7 +15245,7 @@
         <v>1514</v>
       </c>
       <c r="I213" t="s">
-        <v>1615</v>
+        <v>1614</v>
       </c>
       <c r="J213" t="s">
         <v>1864</v>
@@ -15315,7 +15315,7 @@
         <v>1514</v>
       </c>
       <c r="I215" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J215" t="s">
         <v>1866</v>
@@ -15350,7 +15350,7 @@
         <v>1514</v>
       </c>
       <c r="I216" t="s">
-        <v>1616</v>
+        <v>1615</v>
       </c>
       <c r="J216" t="s">
         <v>1867</v>
@@ -15525,7 +15525,7 @@
         <v>1514</v>
       </c>
       <c r="I221" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J221" t="s">
         <v>1872</v>
@@ -15563,7 +15563,7 @@
         <v>1436</v>
       </c>
       <c r="I222" t="s">
-        <v>1617</v>
+        <v>1616</v>
       </c>
       <c r="J222" t="s">
         <v>1873</v>
@@ -15633,7 +15633,7 @@
         <v>1514</v>
       </c>
       <c r="I224" t="s">
-        <v>1618</v>
+        <v>1617</v>
       </c>
       <c r="J224" t="s">
         <v>1875</v>
@@ -15773,7 +15773,7 @@
         <v>1514</v>
       </c>
       <c r="I228" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J228" t="s">
         <v>1879</v>
@@ -15808,7 +15808,7 @@
         <v>1514</v>
       </c>
       <c r="I229" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J229" t="s">
         <v>1880</v>
@@ -15878,7 +15878,7 @@
         <v>1514</v>
       </c>
       <c r="I231" t="s">
-        <v>1619</v>
+        <v>1618</v>
       </c>
       <c r="J231" t="s">
         <v>1882</v>
@@ -15948,7 +15948,7 @@
         <v>1514</v>
       </c>
       <c r="I233" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="J233" t="s">
         <v>1884</v>
@@ -15983,7 +15983,7 @@
         <v>1514</v>
       </c>
       <c r="I234" t="s">
-        <v>1621</v>
+        <v>1620</v>
       </c>
       <c r="J234" t="s">
         <v>1885</v>
@@ -16018,7 +16018,7 @@
         <v>1514</v>
       </c>
       <c r="I235" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J235" t="s">
         <v>1886</v>
@@ -16333,7 +16333,7 @@
         <v>1514</v>
       </c>
       <c r="I244" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J244" t="s">
         <v>1895</v>
@@ -16403,7 +16403,7 @@
         <v>1514</v>
       </c>
       <c r="I246" t="s">
-        <v>1602</v>
+        <v>1621</v>
       </c>
       <c r="J246" t="s">
         <v>1897</v>
@@ -16473,7 +16473,7 @@
         <v>1514</v>
       </c>
       <c r="I248" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J248" t="s">
         <v>1899</v>
@@ -16823,7 +16823,7 @@
         <v>1514</v>
       </c>
       <c r="I258" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J258" t="s">
         <v>1909</v>
@@ -16928,7 +16928,7 @@
         <v>1514</v>
       </c>
       <c r="I261" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J261" t="s">
         <v>1912</v>
@@ -17033,7 +17033,7 @@
         <v>1514</v>
       </c>
       <c r="I264" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="J264" t="s">
         <v>1915</v>
@@ -17383,7 +17383,7 @@
         <v>1514</v>
       </c>
       <c r="I274" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J274" t="s">
         <v>1925</v>
@@ -17768,7 +17768,7 @@
         <v>1514</v>
       </c>
       <c r="I285" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J285" t="s">
         <v>1936</v>
@@ -17908,7 +17908,7 @@
         <v>1514</v>
       </c>
       <c r="I289" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J289" t="s">
         <v>1940</v>
@@ -18296,7 +18296,7 @@
         <v>1514</v>
       </c>
       <c r="I300" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J300" t="s">
         <v>1951</v>
@@ -18611,7 +18611,7 @@
         <v>1514</v>
       </c>
       <c r="I309" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J309" t="s">
         <v>1960</v>
@@ -18754,7 +18754,7 @@
         <v>1520</v>
       </c>
       <c r="I313" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J313" t="s">
         <v>1964</v>
@@ -18824,7 +18824,7 @@
         <v>1514</v>
       </c>
       <c r="I315" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J315" t="s">
         <v>1966</v>
@@ -18859,7 +18859,7 @@
         <v>1514</v>
       </c>
       <c r="I316" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J316" t="s">
         <v>1967</v>
@@ -18964,7 +18964,7 @@
         <v>1514</v>
       </c>
       <c r="I319" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J319" t="s">
         <v>1970</v>
@@ -19034,7 +19034,7 @@
         <v>1514</v>
       </c>
       <c r="I321" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J321" t="s">
         <v>1972</v>
@@ -19139,7 +19139,7 @@
         <v>1514</v>
       </c>
       <c r="I324" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J324" t="s">
         <v>1975</v>
@@ -19244,7 +19244,7 @@
         <v>1514</v>
       </c>
       <c r="I327" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J327" t="s">
         <v>1978</v>
@@ -19979,7 +19979,7 @@
         <v>1514</v>
       </c>
       <c r="I348" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J348" t="s">
         <v>1999</v>
@@ -20049,7 +20049,7 @@
         <v>1514</v>
       </c>
       <c r="I350" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J350" t="s">
         <v>2001</v>
@@ -20329,7 +20329,7 @@
         <v>1514</v>
       </c>
       <c r="I358" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J358" t="s">
         <v>2009</v>
@@ -20364,7 +20364,7 @@
         <v>1514</v>
       </c>
       <c r="I359" t="s">
-        <v>1606</v>
+        <v>1605</v>
       </c>
       <c r="J359" t="s">
         <v>2010</v>
@@ -20787,7 +20787,7 @@
         <v>1514</v>
       </c>
       <c r="I371" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J371" t="s">
         <v>2022</v>
@@ -20930,7 +20930,7 @@
         <v>1480</v>
       </c>
       <c r="I375" t="s">
-        <v>1602</v>
+        <v>1621</v>
       </c>
       <c r="J375" t="s">
         <v>2026</v>
@@ -21245,7 +21245,7 @@
         <v>1514</v>
       </c>
       <c r="I384" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J384" t="s">
         <v>2035</v>
@@ -21280,7 +21280,7 @@
         <v>1514</v>
       </c>
       <c r="I385" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J385" t="s">
         <v>2036</v>
@@ -21315,7 +21315,7 @@
         <v>1514</v>
       </c>
       <c r="I386" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J386" t="s">
         <v>2037</v>
@@ -21350,7 +21350,7 @@
         <v>1514</v>
       </c>
       <c r="I387" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J387" t="s">
         <v>2038</v>
@@ -21385,7 +21385,7 @@
         <v>1514</v>
       </c>
       <c r="I388" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J388" t="s">
         <v>2009</v>
@@ -21668,7 +21668,7 @@
         <v>1514</v>
       </c>
       <c r="I396" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J396" t="s">
         <v>2046</v>
@@ -21843,7 +21843,7 @@
         <v>1514</v>
       </c>
       <c r="I401" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J401" t="s">
         <v>2051</v>
@@ -21878,7 +21878,7 @@
         <v>1514</v>
       </c>
       <c r="I402" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J402" t="s">
         <v>2052</v>
@@ -21913,7 +21913,7 @@
         <v>1514</v>
       </c>
       <c r="I403" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J403" t="s">
         <v>2053</v>
@@ -21948,7 +21948,7 @@
         <v>1514</v>
       </c>
       <c r="I404" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J404" t="s">
         <v>2054</v>
@@ -22963,7 +22963,7 @@
         <v>1514</v>
       </c>
       <c r="I433" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J433" t="s">
         <v>2083</v>
@@ -23208,7 +23208,7 @@
         <v>1514</v>
       </c>
       <c r="I440" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J440" t="s">
         <v>2087</v>
@@ -23421,7 +23421,7 @@
         <v>1514</v>
       </c>
       <c r="I446" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J446" t="s">
         <v>2093</v>
@@ -23777,7 +23777,7 @@
         <v>1522</v>
       </c>
       <c r="I456" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J456" t="s">
         <v>2103</v>
@@ -24302,7 +24302,7 @@
         <v>1514</v>
       </c>
       <c r="I471" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J471" t="s">
         <v>2118</v>
@@ -24477,7 +24477,7 @@
         <v>1514</v>
       </c>
       <c r="I476" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J476" t="s">
         <v>2123</v>
@@ -24582,7 +24582,7 @@
         <v>1514</v>
       </c>
       <c r="I479" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J479" t="s">
         <v>2126</v>
@@ -24967,7 +24967,7 @@
         <v>1514</v>
       </c>
       <c r="I490" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J490" t="s">
         <v>2137</v>
@@ -25037,7 +25037,7 @@
         <v>1514</v>
       </c>
       <c r="I492" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J492" t="s">
         <v>2139</v>
@@ -25107,7 +25107,7 @@
         <v>1514</v>
       </c>
       <c r="I494" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J494" t="s">
         <v>2141</v>
@@ -25247,7 +25247,7 @@
         <v>1514</v>
       </c>
       <c r="I498" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J498" t="s">
         <v>2042</v>
@@ -25460,7 +25460,7 @@
         <v>1514</v>
       </c>
       <c r="I504" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J504" t="s">
         <v>2150</v>
@@ -26907,7 +26907,7 @@
         <v>1514</v>
       </c>
       <c r="I545" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J545" t="s">
         <v>2190</v>
@@ -27050,7 +27050,7 @@
         <v>1514</v>
       </c>
       <c r="I549" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J549" t="s">
         <v>2194</v>
@@ -27333,7 +27333,7 @@
         <v>1514</v>
       </c>
       <c r="I557" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J557" t="s">
         <v>2201</v>
@@ -27549,7 +27549,7 @@
         <v>1514</v>
       </c>
       <c r="I563" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J563" t="s">
         <v>2207</v>
@@ -27654,7 +27654,7 @@
         <v>1514</v>
       </c>
       <c r="I566" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J566" t="s">
         <v>2210</v>
@@ -27870,7 +27870,7 @@
         <v>1514</v>
       </c>
       <c r="I572" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J572" t="s">
         <v>2216</v>
@@ -28220,7 +28220,7 @@
         <v>1514</v>
       </c>
       <c r="I582" t="s">
-        <v>1620</v>
+        <v>1619</v>
       </c>
       <c r="J582" t="s">
         <v>2226</v>
@@ -28401,7 +28401,7 @@
         <v>1514</v>
       </c>
       <c r="I587" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J587" t="s">
         <v>2229</v>
@@ -28827,7 +28827,7 @@
         <v>1534</v>
       </c>
       <c r="I599" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J599" t="s">
         <v>2241</v>
@@ -28862,7 +28862,7 @@
         <v>1514</v>
       </c>
       <c r="I600" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J600" t="s">
         <v>2242</v>
@@ -28967,7 +28967,7 @@
         <v>1514</v>
       </c>
       <c r="I603" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J603" t="s">
         <v>2244</v>
@@ -29145,7 +29145,7 @@
         <v>1514</v>
       </c>
       <c r="I608" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J608" t="s">
         <v>2248</v>
@@ -29215,7 +29215,7 @@
         <v>1514</v>
       </c>
       <c r="I610" t="s">
-        <v>1608</v>
+        <v>1607</v>
       </c>
       <c r="J610" t="s">
         <v>2250</v>
@@ -29250,7 +29250,7 @@
         <v>1514</v>
       </c>
       <c r="I611" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J611" t="s">
         <v>2251</v>
@@ -29495,7 +29495,7 @@
         <v>1514</v>
       </c>
       <c r="I618" t="s">
-        <v>1605</v>
+        <v>1604</v>
       </c>
       <c r="J618" t="s">
         <v>2258</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-30 10:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -26831,7 +26831,7 @@
     </row>
     <row r="543" spans="1:12">
       <c r="A543" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B543" t="s">
         <v>582</v>
@@ -26855,7 +26855,7 @@
         <v>1528</v>
       </c>
       <c r="I543" t="s">
-        <v>1552</v>
+        <v>1548</v>
       </c>
       <c r="J543" t="s">
         <v>2190</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-09-30 22:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7486,34 +7486,37 @@
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
+  </si>
+  <si>
+    <t>URBANISMO,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>FARMÁCIA,SAÚDE</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>URBANISMO,BIOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
-  </si>
-  <si>
-    <t>FARMÁCIA,SAÚDE</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS,URBANISMO,BIOLOGIA</t>
+    <t>RECURSOS HÍDRICOS,MOBILIDADE E TRANSPORTE,BIOLOGIA,URBANISMO</t>
   </si>
   <si>
     <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
@@ -7525,13 +7528,10 @@
     <t>ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
-    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
     <t>ECONOMICIDADE CONTÁBIL,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMIA,ASSISTÊNCIA SOCIAL,SAÚDE MENTAL,ORÇAMENTO,PSICOLOGIA,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS,URBANISMO,SAÚDE</t>
+    <t>URBANISMO,PSICOLOGIA,SAÚDE,ASSISTÊNCIA SOCIAL,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,ECONOMIA,ORÇAMENTO,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
 </sst>
 </file>
@@ -23888,7 +23888,7 @@
         <v>2344</v>
       </c>
       <c r="L456" t="s">
-        <v>2493</v>
+        <v>2436</v>
       </c>
     </row>
     <row r="457" spans="1:12">
@@ -24063,7 +24063,7 @@
         <v>2404</v>
       </c>
       <c r="L461" t="s">
-        <v>2494</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="462" spans="1:12">
@@ -24658,7 +24658,7 @@
         <v>2335</v>
       </c>
       <c r="L478" t="s">
-        <v>2495</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="479" spans="1:12">
@@ -24693,7 +24693,7 @@
         <v>2337</v>
       </c>
       <c r="L479" t="s">
-        <v>2496</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="480" spans="1:12">
@@ -24903,7 +24903,7 @@
         <v>2408</v>
       </c>
       <c r="L485" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="486" spans="1:12">
@@ -25431,7 +25431,7 @@
         <v>2336</v>
       </c>
       <c r="L500" t="s">
-        <v>2493</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="501" spans="1:12">
@@ -25571,7 +25571,7 @@
         <v>2340</v>
       </c>
       <c r="L504" t="s">
-        <v>2490</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="505" spans="1:12">
@@ -26172,7 +26172,7 @@
         <v>2342</v>
       </c>
       <c r="L521" t="s">
-        <v>2496</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="522" spans="1:12">
@@ -26560,7 +26560,7 @@
         <v>2312</v>
       </c>
       <c r="L532" t="s">
-        <v>2499</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="533" spans="1:12">
@@ -26843,7 +26843,7 @@
         <v>2307</v>
       </c>
       <c r="L540" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="541" spans="1:12">
@@ -27689,7 +27689,7 @@
         <v>2415</v>
       </c>
       <c r="L564" t="s">
-        <v>2501</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="565" spans="1:12">
@@ -29034,7 +29034,7 @@
         <v>2350</v>
       </c>
       <c r="L602" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="603" spans="1:12">
@@ -29282,7 +29282,7 @@
         <v>2418</v>
       </c>
       <c r="L609" t="s">
-        <v>2503</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="610" spans="1:12">
@@ -30347,7 +30347,7 @@
         <v>2409</v>
       </c>
       <c r="L639" t="s">
-        <v>2489</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="640" spans="1:12">
@@ -30449,7 +30449,7 @@
         <v>2423</v>
       </c>
       <c r="L642" t="s">
-        <v>2503</v>
+        <v>2442</v>
       </c>
     </row>
     <row r="643" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-01 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -7498,7 +7498,7 @@
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
@@ -7516,19 +7516,16 @@
     <t>ENGENHARIA FLORESTAL,URBANISMO</t>
   </si>
   <si>
-    <t>URBANISMO,BIOLOGIA</t>
-  </si>
-  <si>
     <t>FARMÁCIA,SAÚDE</t>
   </si>
   <si>
     <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>RECURSOS HÍDRICOS,MOBILIDADE E TRANSPORTE,BIOLOGIA,URBANISMO</t>
+    <t>URBANISMO,ENGENHARIA FLORESTAL</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,URBANISMO,MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
@@ -7537,13 +7534,16 @@
     <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
     <t>ECONOMICIDADE CONTÁBIL,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
-    <t>URBANISMO,PSICOLOGIA,SAÚDE,ASSISTÊNCIA SOCIAL,SAÚDE MENTAL,ECONOMICIDADE CONTÁBIL,ECONOMIA,ORÇAMENTO,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS</t>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>PSICOLOGIA,AVALIAÇÃO DE IMÓVEIS,ORÇAMENTO,SAÚDE MENTAL,ASSISTÊNCIA SOCIAL,SAÚDE,URBANISMO,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,ECONOMIA</t>
   </si>
 </sst>
 </file>
@@ -24915,7 +24915,7 @@
         <v>2412</v>
       </c>
       <c r="L485" t="s">
-        <v>2500</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="486" spans="1:12">
@@ -25055,7 +25055,7 @@
         <v>2350</v>
       </c>
       <c r="L489" t="s">
-        <v>2501</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="490" spans="1:12">
@@ -25443,7 +25443,7 @@
         <v>2340</v>
       </c>
       <c r="L500" t="s">
-        <v>2500</v>
+        <v>2440</v>
       </c>
     </row>
     <row r="501" spans="1:12">
@@ -25513,7 +25513,7 @@
         <v>2340</v>
       </c>
       <c r="L502" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="503" spans="1:12">
@@ -25583,7 +25583,7 @@
         <v>2344</v>
       </c>
       <c r="L504" t="s">
-        <v>2503</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="505" spans="1:12">
@@ -26184,7 +26184,7 @@
         <v>2346</v>
       </c>
       <c r="L521" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="522" spans="1:12">
@@ -26572,7 +26572,7 @@
         <v>2316</v>
       </c>
       <c r="L532" t="s">
-        <v>2504</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="533" spans="1:12">
@@ -26855,7 +26855,7 @@
         <v>2311</v>
       </c>
       <c r="L540" t="s">
-        <v>2505</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="541" spans="1:12">
@@ -27631,7 +27631,7 @@
         <v>2342</v>
       </c>
       <c r="L562" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="563" spans="1:12">
@@ -27701,7 +27701,7 @@
         <v>2419</v>
       </c>
       <c r="L564" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="565" spans="1:12">
@@ -29046,7 +29046,7 @@
         <v>2354</v>
       </c>
       <c r="L602" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="603" spans="1:12">
@@ -29650,7 +29650,7 @@
         <v>2344</v>
       </c>
       <c r="L619" t="s">
-        <v>2508</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="620" spans="1:12">
@@ -29790,7 +29790,7 @@
         <v>2357</v>
       </c>
       <c r="L623" t="s">
-        <v>2493</v>
+        <v>2445</v>
       </c>
     </row>
     <row r="624" spans="1:12">
@@ -30324,7 +30324,7 @@
         <v>2426</v>
       </c>
       <c r="L638" t="s">
-        <v>2493</v>
+        <v>2445</v>
       </c>
     </row>
     <row r="639" spans="1:12">
@@ -30394,7 +30394,7 @@
         <v>2413</v>
       </c>
       <c r="L640" t="s">
-        <v>2499</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="641" spans="1:12">
@@ -30496,7 +30496,7 @@
         <v>2427</v>
       </c>
       <c r="L643" t="s">
-        <v>2446</v>
+        <v>2508</v>
       </c>
     </row>
     <row r="644" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-02 02:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -73,7 +73,7 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIA DE DADOS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
-    <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
+    <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS, SECRETARIA GERAL DO GATE</t>
   </si>
   <si>
     <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE ENGENHARIA</t>
@@ -4822,7 +4822,7 @@
     <t>CAIO EDUARDO BARBOSA DOS SANTOS FERREIRA,EDIWAN SOUSA DA SILVA</t>
   </si>
   <si>
-    <t>ALESSANDRA ALMEIDA DIAS DA SILVA,LILIAN ALVES DE ARAUJO,SIMONE MANNHEIMER DE ALVARENGA</t>
+    <t>LILIAN ALVES DE ARAUJO,SIMONE MANNHEIMER DE ALVARENGA, _SEM USUARIO ATRIBUIDO</t>
   </si>
   <si>
     <t>MARINA DE AQUINO PARREIRA XAVIER,SERGIO PEDRO LOPES</t>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-08 02:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -8771,7 +8771,7 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B30" t="s">
         <v>70</v>
@@ -8792,7 +8792,7 @@
         <v>1502</v>
       </c>
       <c r="I30" t="s">
-        <v>1529</v>
+        <v>1535</v>
       </c>
       <c r="J30" t="s">
         <v>1674</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-08 22:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6256" uniqueCount="2435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6256" uniqueCount="2436">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7264,37 +7264,43 @@
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
+  </si>
+  <si>
+    <t>FARMÁCIA,SAÚDE</t>
+  </si>
+  <si>
+    <t>URBANISMO,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
-  </si>
-  <si>
-    <t>FARMÁCIA,SAÚDE</t>
-  </si>
-  <si>
-    <t>URBANISMO,BIOLOGIA</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE,URBANISMO,BIOLOGIA,RECURSOS HÍDRICOS</t>
+    <t>URBANISMO,ENGENHARIA FLORESTAL</t>
+  </si>
+  <si>
+    <t>URBANISMO,BIOLOGIA,MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
@@ -7315,10 +7321,7 @@
     <t>ECONOMICIDADE CONTÁBIL,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,ENGENHARIA QUÍMICA</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,SAÚDE MENTAL,SAÚDE,ECONOMIA,ORÇAMENTO,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,PSICOLOGIA,URBANISMO,MOBILIDADE E TRANSPORTE</t>
+    <t>ASSISTÊNCIA SOCIAL,SAÚDE,SAÚDE MENTAL,URBANISMO,ECONOMIA,ORÇAMENTO,AVALIAÇÃO DE IMÓVEIS,MOBILIDADE E TRANSPORTE,PSICOLOGIA,ECONOMICIDADE CONTÁBIL</t>
   </si>
 </sst>
 </file>
@@ -23809,7 +23812,7 @@
         <v>2273</v>
       </c>
       <c r="L460" t="s">
-        <v>2416</v>
+        <v>2426</v>
       </c>
     </row>
     <row r="461" spans="1:12">
@@ -24337,7 +24340,7 @@
         <v>2275</v>
       </c>
       <c r="L475" t="s">
-        <v>2422</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="476" spans="1:12">
@@ -24652,7 +24655,7 @@
         <v>2246</v>
       </c>
       <c r="L484" t="s">
-        <v>2426</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="485" spans="1:12">
@@ -24862,7 +24865,7 @@
         <v>2241</v>
       </c>
       <c r="L490" t="s">
-        <v>2427</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="491" spans="1:12">
@@ -25568,7 +25571,7 @@
         <v>2345</v>
       </c>
       <c r="L510" t="s">
-        <v>2428</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="511" spans="1:12">
@@ -26840,7 +26843,7 @@
         <v>2283</v>
       </c>
       <c r="L546" t="s">
-        <v>2429</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="547" spans="1:12">
@@ -27444,7 +27447,7 @@
         <v>2273</v>
       </c>
       <c r="L563" t="s">
-        <v>2430</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="564" spans="1:12">
@@ -28188,7 +28191,7 @@
         <v>2341</v>
       </c>
       <c r="L584" t="s">
-        <v>2422</v>
+        <v>2427</v>
       </c>
     </row>
     <row r="585" spans="1:12">
@@ -28334,7 +28337,7 @@
         <v>2246</v>
       </c>
       <c r="L588" t="s">
-        <v>2431</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="589" spans="1:12">
@@ -28518,7 +28521,7 @@
         <v>2267</v>
       </c>
       <c r="L593" t="s">
-        <v>2432</v>
+        <v>2434</v>
       </c>
     </row>
     <row r="594" spans="1:12">
@@ -28851,7 +28854,7 @@
         <v>2241</v>
       </c>
       <c r="L602" t="s">
-        <v>2433</v>
+        <v>2384</v>
       </c>
     </row>
     <row r="603" spans="1:12">
@@ -29452,7 +29455,7 @@
         <v>2243</v>
       </c>
       <c r="L619" t="s">
-        <v>2415</v>
+        <v>2390</v>
       </c>
     </row>
     <row r="620" spans="1:12">
@@ -29551,7 +29554,7 @@
         <v>2354</v>
       </c>
       <c r="L622" t="s">
-        <v>2434</v>
+        <v>2435</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-09 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -85,6 +85,9 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE</t>
   </si>
   <si>
+    <t>SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS DA SAÚDE, SECRETARIA GERAL DO GATE</t>
   </si>
   <si>
@@ -121,9 +124,6 @@
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS, NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
-    <t>SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ECONOMIA</t>
   </si>
   <si>
@@ -4657,36 +4657,39 @@
     <t>EDIWAN SOUSA DA SILVA</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
+    <t>VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>GIULIANA DE ANDRADE CERVAI</t>
+  </si>
+  <si>
+    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
+  </si>
+  <si>
+    <t>CELSO BARBOSA MONTENEGRO,CLAUDIA DA SILVA LUNARDI</t>
+  </si>
+  <si>
+    <t>JULIANA MARTINS BAHIENSE,RODRIGO VENTURA MARRA</t>
+  </si>
+  <si>
+    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA FERNANDES LEÃO</t>
+  </si>
+  <si>
+    <t>RENATA PASCOAL FREIRE,ROSEMARY PROVENZANO THAMI</t>
+  </si>
+  <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO, RENATA PASCOAL FREIRE</t>
+  </si>
+  <si>
+    <t>RODRIGO VALENTE SERRA</t>
+  </si>
+  <si>
     <t>CARLOS FELIPE DA GRAÇA SILVA</t>
   </si>
   <si>
-    <t>VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>GIULIANA DE ANDRADE CERVAI</t>
-  </si>
-  <si>
-    <t>MARCELO TEIXEIRA SANTANA,MARIA JOSÉ LOPES DE ARAUJO SAROLDI,SIMONE MANNHEIMER DE ALVARENGA</t>
-  </si>
-  <si>
-    <t>CELSO BARBOSA MONTENEGRO,CLAUDIA DA SILVA LUNARDI</t>
-  </si>
-  <si>
-    <t>JULIANA MARTINS BAHIENSE,RODRIGO VENTURA MARRA</t>
-  </si>
-  <si>
-    <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA FERNANDES LEÃO</t>
-  </si>
-  <si>
-    <t>RENATA PASCOAL FREIRE,ROSEMARY PROVENZANO THAMI</t>
-  </si>
-  <si>
-    <t>RENATA PASCOAL FREIRE, _SEM USUARIO ATRIBUIDO</t>
-  </si>
-  <si>
-    <t>RODRIGO VALENTE SERRA</t>
-  </si>
-  <si>
     <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
   </si>
   <si>
@@ -4907,9 +4910,6 @@
   </si>
   <si>
     <t>LUIZ FRANCISCO PERALTA BRAGA,RONALDO PEIXOTO VELLOSO</t>
-  </si>
-  <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
   </si>
   <si>
     <t>201701021184</t>
@@ -8977,7 +8977,7 @@
         <v>1652</v>
       </c>
       <c r="K37" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="L37" t="s">
         <v>2357</v>
@@ -10805,7 +10805,7 @@
     </row>
     <row r="90" spans="1:12">
       <c r="A90" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="B90" t="s">
         <v>130</v>
@@ -11225,7 +11225,7 @@
     </row>
     <row r="102" spans="1:12">
       <c r="A102" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B102" t="s">
         <v>142</v>
@@ -11400,7 +11400,7 @@
     </row>
     <row r="107" spans="1:12">
       <c r="A107" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B107" t="s">
         <v>147</v>
@@ -11456,7 +11456,7 @@
         <v>1488</v>
       </c>
       <c r="I108" t="s">
-        <v>1547</v>
+        <v>1557</v>
       </c>
       <c r="J108" t="s">
         <v>1736</v>
@@ -11505,7 +11505,7 @@
     </row>
     <row r="110" spans="1:12">
       <c r="A110" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B110" t="s">
         <v>150</v>
@@ -11526,7 +11526,7 @@
         <v>1488</v>
       </c>
       <c r="I110" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="J110" t="s">
         <v>1738</v>
@@ -11610,7 +11610,7 @@
     </row>
     <row r="113" spans="1:12">
       <c r="A113" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B113" t="s">
         <v>153</v>
@@ -11666,7 +11666,7 @@
         <v>1488</v>
       </c>
       <c r="I114" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="J114" t="s">
         <v>1742</v>
@@ -11680,7 +11680,7 @@
     </row>
     <row r="115" spans="1:12">
       <c r="A115" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B115" t="s">
         <v>155</v>
@@ -11701,7 +11701,7 @@
         <v>1488</v>
       </c>
       <c r="I115" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="J115" t="s">
         <v>1743</v>
@@ -11750,7 +11750,7 @@
     </row>
     <row r="117" spans="1:12">
       <c r="A117" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B117" t="s">
         <v>157</v>
@@ -11785,7 +11785,7 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B118" t="s">
         <v>158</v>
@@ -12016,7 +12016,7 @@
         <v>1488</v>
       </c>
       <c r="I124" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="J124" t="s">
         <v>1752</v>
@@ -12065,7 +12065,7 @@
     </row>
     <row r="126" spans="1:12">
       <c r="A126" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B126" t="s">
         <v>166</v>
@@ -12156,7 +12156,7 @@
         <v>1488</v>
       </c>
       <c r="I128" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="J128" t="s">
         <v>1756</v>
@@ -12191,7 +12191,7 @@
         <v>1488</v>
       </c>
       <c r="I129" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="J129" t="s">
         <v>1757</v>
@@ -12261,7 +12261,7 @@
         <v>1488</v>
       </c>
       <c r="I131" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="J131" t="s">
         <v>1759</v>
@@ -12401,7 +12401,7 @@
         <v>1488</v>
       </c>
       <c r="I135" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
       <c r="J135" t="s">
         <v>1763</v>
@@ -12415,7 +12415,7 @@
     </row>
     <row r="136" spans="1:12">
       <c r="A136" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B136" t="s">
         <v>176</v>
@@ -12471,7 +12471,7 @@
         <v>1488</v>
       </c>
       <c r="I137" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="J137" t="s">
         <v>1765</v>
@@ -12576,7 +12576,7 @@
         <v>1488</v>
       </c>
       <c r="I140" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
       <c r="J140" t="s">
         <v>1768</v>
@@ -12751,7 +12751,7 @@
         <v>1488</v>
       </c>
       <c r="I145" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="J145" t="s">
         <v>1773</v>
@@ -12821,7 +12821,7 @@
         <v>1488</v>
       </c>
       <c r="I147" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
       <c r="J147" t="s">
         <v>1775</v>
@@ -12856,7 +12856,7 @@
         <v>1488</v>
       </c>
       <c r="I148" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="J148" t="s">
         <v>1776</v>
@@ -12996,7 +12996,7 @@
         <v>1488</v>
       </c>
       <c r="I152" t="s">
-        <v>1570</v>
+        <v>1571</v>
       </c>
       <c r="J152" t="s">
         <v>1780</v>
@@ -13101,7 +13101,7 @@
         <v>1488</v>
       </c>
       <c r="I155" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="J155" t="s">
         <v>1783</v>
@@ -13276,7 +13276,7 @@
         <v>1488</v>
       </c>
       <c r="I160" t="s">
-        <v>1572</v>
+        <v>1573</v>
       </c>
       <c r="J160" t="s">
         <v>1788</v>
@@ -13395,7 +13395,7 @@
     </row>
     <row r="164" spans="1:12">
       <c r="A164" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B164" t="s">
         <v>204</v>
@@ -13416,7 +13416,7 @@
         <v>1488</v>
       </c>
       <c r="I164" t="s">
-        <v>1573</v>
+        <v>1574</v>
       </c>
       <c r="J164" t="s">
         <v>1792</v>
@@ -13465,7 +13465,7 @@
     </row>
     <row r="166" spans="1:12">
       <c r="A166" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B166" t="s">
         <v>206</v>
@@ -13486,7 +13486,7 @@
         <v>1488</v>
       </c>
       <c r="I166" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J166" t="s">
         <v>1794</v>
@@ -13521,7 +13521,7 @@
         <v>1488</v>
       </c>
       <c r="I167" t="s">
-        <v>1575</v>
+        <v>1576</v>
       </c>
       <c r="J167" t="s">
         <v>1795</v>
@@ -13535,7 +13535,7 @@
     </row>
     <row r="168" spans="1:12">
       <c r="A168" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B168" t="s">
         <v>208</v>
@@ -13605,7 +13605,7 @@
     </row>
     <row r="170" spans="1:12">
       <c r="A170" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B170" t="s">
         <v>210</v>
@@ -13678,7 +13678,7 @@
     </row>
     <row r="172" spans="1:12">
       <c r="A172" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B172" t="s">
         <v>212</v>
@@ -13699,7 +13699,7 @@
         <v>1488</v>
       </c>
       <c r="I172" t="s">
-        <v>1576</v>
+        <v>1577</v>
       </c>
       <c r="J172" t="s">
         <v>1800</v>
@@ -13734,7 +13734,7 @@
         <v>1488</v>
       </c>
       <c r="I173" t="s">
-        <v>1577</v>
+        <v>1578</v>
       </c>
       <c r="J173" t="s">
         <v>1801</v>
@@ -13769,7 +13769,7 @@
         <v>1488</v>
       </c>
       <c r="I174" t="s">
-        <v>1578</v>
+        <v>1579</v>
       </c>
       <c r="J174" t="s">
         <v>1802</v>
@@ -13783,7 +13783,7 @@
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B175" t="s">
         <v>215</v>
@@ -13993,7 +13993,7 @@
     </row>
     <row r="181" spans="1:12">
       <c r="A181" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B181" t="s">
         <v>221</v>
@@ -14014,7 +14014,7 @@
         <v>1488</v>
       </c>
       <c r="I181" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="J181" t="s">
         <v>1809</v>
@@ -14084,7 +14084,7 @@
         <v>1488</v>
       </c>
       <c r="I183" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="J183" t="s">
         <v>1811</v>
@@ -14294,7 +14294,7 @@
         <v>1488</v>
       </c>
       <c r="I189" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="J189" t="s">
         <v>1817</v>
@@ -14308,7 +14308,7 @@
     </row>
     <row r="190" spans="1:12">
       <c r="A190" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B190" t="s">
         <v>230</v>
@@ -14329,7 +14329,7 @@
         <v>1488</v>
       </c>
       <c r="I190" t="s">
-        <v>1576</v>
+        <v>1577</v>
       </c>
       <c r="J190" t="s">
         <v>1818</v>
@@ -14469,7 +14469,7 @@
         <v>1488</v>
       </c>
       <c r="I194" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="J194" t="s">
         <v>1822</v>
@@ -14518,7 +14518,7 @@
     </row>
     <row r="196" spans="1:12">
       <c r="A196" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B196" t="s">
         <v>236</v>
@@ -14539,7 +14539,7 @@
         <v>1488</v>
       </c>
       <c r="I196" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J196" t="s">
         <v>1824</v>
@@ -14577,7 +14577,7 @@
         <v>1406</v>
       </c>
       <c r="I197" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="J197" t="s">
         <v>1825</v>
@@ -14766,7 +14766,7 @@
     </row>
     <row r="203" spans="1:12">
       <c r="A203" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B203" t="s">
         <v>243</v>
@@ -14787,7 +14787,7 @@
         <v>1488</v>
       </c>
       <c r="I203" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J203" t="s">
         <v>1831</v>
@@ -14857,7 +14857,7 @@
         <v>1488</v>
       </c>
       <c r="I205" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
       <c r="J205" t="s">
         <v>1833</v>
@@ -14906,7 +14906,7 @@
     </row>
     <row r="207" spans="1:12">
       <c r="A207" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B207" t="s">
         <v>247</v>
@@ -14927,7 +14927,7 @@
         <v>1488</v>
       </c>
       <c r="I207" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J207" t="s">
         <v>1835</v>
@@ -14941,7 +14941,7 @@
     </row>
     <row r="208" spans="1:12">
       <c r="A208" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B208" t="s">
         <v>248</v>
@@ -15207,7 +15207,7 @@
         <v>1488</v>
       </c>
       <c r="I215" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="J215" t="s">
         <v>1843</v>
@@ -15291,7 +15291,7 @@
     </row>
     <row r="218" spans="1:12">
       <c r="A218" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B218" t="s">
         <v>258</v>
@@ -15312,7 +15312,7 @@
         <v>1488</v>
       </c>
       <c r="I218" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J218" t="s">
         <v>1846</v>
@@ -15431,7 +15431,7 @@
     </row>
     <row r="222" spans="1:12">
       <c r="A222" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B222" t="s">
         <v>262</v>
@@ -15452,7 +15452,7 @@
         <v>1488</v>
       </c>
       <c r="I222" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="J222" t="s">
         <v>1850</v>
@@ -15536,7 +15536,7 @@
     </row>
     <row r="225" spans="1:12">
       <c r="A225" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B225" t="s">
         <v>265</v>
@@ -15557,7 +15557,7 @@
         <v>1488</v>
       </c>
       <c r="I225" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J225" t="s">
         <v>1853</v>
@@ -15641,7 +15641,7 @@
     </row>
     <row r="228" spans="1:12">
       <c r="A228" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B228" t="s">
         <v>268</v>
@@ -15662,7 +15662,7 @@
         <v>1488</v>
       </c>
       <c r="I228" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J228" t="s">
         <v>1856</v>
@@ -16012,7 +16012,7 @@
         <v>1488</v>
       </c>
       <c r="I238" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
       <c r="J238" t="s">
         <v>1866</v>
@@ -16026,7 +16026,7 @@
     </row>
     <row r="239" spans="1:12">
       <c r="A239" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B239" t="s">
         <v>279</v>
@@ -16047,7 +16047,7 @@
         <v>1488</v>
       </c>
       <c r="I239" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J239" t="s">
         <v>1867</v>
@@ -16152,7 +16152,7 @@
         <v>1488</v>
       </c>
       <c r="I242" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="J242" t="s">
         <v>1870</v>
@@ -16201,7 +16201,7 @@
     </row>
     <row r="244" spans="1:12">
       <c r="A244" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B244" t="s">
         <v>284</v>
@@ -16222,7 +16222,7 @@
         <v>1488</v>
       </c>
       <c r="I244" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
       <c r="J244" t="s">
         <v>1872</v>
@@ -16236,7 +16236,7 @@
     </row>
     <row r="245" spans="1:12">
       <c r="A245" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B245" t="s">
         <v>285</v>
@@ -16327,7 +16327,7 @@
         <v>1488</v>
       </c>
       <c r="I247" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
       <c r="J247" t="s">
         <v>1875</v>
@@ -16376,7 +16376,7 @@
     </row>
     <row r="249" spans="1:12">
       <c r="A249" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B249" t="s">
         <v>289</v>
@@ -16397,7 +16397,7 @@
         <v>1488</v>
       </c>
       <c r="I249" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J249" t="s">
         <v>1877</v>
@@ -16432,7 +16432,7 @@
         <v>1488</v>
       </c>
       <c r="I250" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="J250" t="s">
         <v>1878</v>
@@ -16502,7 +16502,7 @@
         <v>1488</v>
       </c>
       <c r="I252" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J252" t="s">
         <v>1880</v>
@@ -16540,7 +16540,7 @@
         <v>1492</v>
       </c>
       <c r="I253" t="s">
-        <v>1592</v>
+        <v>1593</v>
       </c>
       <c r="J253" t="s">
         <v>1881</v>
@@ -16575,7 +16575,7 @@
         <v>1488</v>
       </c>
       <c r="I254" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="J254" t="s">
         <v>1882</v>
@@ -16610,7 +16610,7 @@
         <v>1488</v>
       </c>
       <c r="I255" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="J255" t="s">
         <v>1883</v>
@@ -16680,7 +16680,7 @@
         <v>1488</v>
       </c>
       <c r="I257" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="J257" t="s">
         <v>1885</v>
@@ -16799,7 +16799,7 @@
     </row>
     <row r="261" spans="1:12">
       <c r="A261" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B261" t="s">
         <v>301</v>
@@ -17065,7 +17065,7 @@
         <v>1488</v>
       </c>
       <c r="I268" t="s">
-        <v>1572</v>
+        <v>1573</v>
       </c>
       <c r="J268" t="s">
         <v>1896</v>
@@ -17100,7 +17100,7 @@
         <v>1488</v>
       </c>
       <c r="I269" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
       <c r="J269" t="s">
         <v>1897</v>
@@ -17114,7 +17114,7 @@
     </row>
     <row r="270" spans="1:12">
       <c r="A270" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B270" t="s">
         <v>310</v>
@@ -17135,7 +17135,7 @@
         <v>1488</v>
       </c>
       <c r="I270" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J270" t="s">
         <v>1898</v>
@@ -17170,7 +17170,7 @@
         <v>1488</v>
       </c>
       <c r="I271" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
       <c r="J271" t="s">
         <v>1899</v>
@@ -17184,7 +17184,7 @@
     </row>
     <row r="272" spans="1:12">
       <c r="A272" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B272" t="s">
         <v>312</v>
@@ -17205,7 +17205,7 @@
         <v>1488</v>
       </c>
       <c r="I272" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J272" t="s">
         <v>1900</v>
@@ -17219,7 +17219,7 @@
     </row>
     <row r="273" spans="1:12">
       <c r="A273" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B273" t="s">
         <v>313</v>
@@ -17240,7 +17240,7 @@
         <v>1488</v>
       </c>
       <c r="I273" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J273" t="s">
         <v>1901</v>
@@ -17254,7 +17254,7 @@
     </row>
     <row r="274" spans="1:12">
       <c r="A274" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B274" t="s">
         <v>314</v>
@@ -17275,7 +17275,7 @@
         <v>1488</v>
       </c>
       <c r="I274" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J274" t="s">
         <v>1902</v>
@@ -17324,7 +17324,7 @@
     </row>
     <row r="276" spans="1:12">
       <c r="A276" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B276" t="s">
         <v>316</v>
@@ -17345,7 +17345,7 @@
         <v>1488</v>
       </c>
       <c r="I276" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J276" t="s">
         <v>1904</v>
@@ -17499,7 +17499,7 @@
     </row>
     <row r="281" spans="1:12">
       <c r="A281" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B281" t="s">
         <v>321</v>
@@ -17520,7 +17520,7 @@
         <v>1488</v>
       </c>
       <c r="I281" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J281" t="s">
         <v>1909</v>
@@ -17604,7 +17604,7 @@
     </row>
     <row r="284" spans="1:12">
       <c r="A284" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B284" t="s">
         <v>324</v>
@@ -17625,7 +17625,7 @@
         <v>1488</v>
       </c>
       <c r="I284" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J284" t="s">
         <v>1912</v>
@@ -17800,7 +17800,7 @@
         <v>1488</v>
       </c>
       <c r="I289" t="s">
-        <v>1596</v>
+        <v>1597</v>
       </c>
       <c r="J289" t="s">
         <v>1917</v>
@@ -17849,7 +17849,7 @@
     </row>
     <row r="291" spans="1:12">
       <c r="A291" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B291" t="s">
         <v>331</v>
@@ -17870,7 +17870,7 @@
         <v>1490</v>
       </c>
       <c r="I291" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J291" t="s">
         <v>1919</v>
@@ -17905,7 +17905,7 @@
         <v>1488</v>
       </c>
       <c r="I292" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
       <c r="J292" t="s">
         <v>1920</v>
@@ -18094,7 +18094,7 @@
     </row>
     <row r="298" spans="1:12">
       <c r="A298" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B298" t="s">
         <v>338</v>
@@ -18115,7 +18115,7 @@
         <v>1488</v>
       </c>
       <c r="I298" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J298" t="s">
         <v>1926</v>
@@ -18164,7 +18164,7 @@
     </row>
     <row r="300" spans="1:12">
       <c r="A300" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B300" t="s">
         <v>340</v>
@@ -18234,7 +18234,7 @@
     </row>
     <row r="302" spans="1:12">
       <c r="A302" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B302" t="s">
         <v>342</v>
@@ -18304,7 +18304,7 @@
     </row>
     <row r="304" spans="1:12">
       <c r="A304" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B304" t="s">
         <v>344</v>
@@ -18325,7 +18325,7 @@
         <v>1488</v>
       </c>
       <c r="I304" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J304" t="s">
         <v>1932</v>
@@ -18374,7 +18374,7 @@
     </row>
     <row r="306" spans="1:12">
       <c r="A306" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B306" t="s">
         <v>346</v>
@@ -18395,7 +18395,7 @@
         <v>1488</v>
       </c>
       <c r="I306" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J306" t="s">
         <v>1934</v>
@@ -18654,7 +18654,7 @@
     </row>
     <row r="314" spans="1:12">
       <c r="A314" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B314" t="s">
         <v>354</v>
@@ -18675,7 +18675,7 @@
         <v>1488</v>
       </c>
       <c r="I314" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J314" t="s">
         <v>1942</v>
@@ -18710,7 +18710,7 @@
         <v>1488</v>
       </c>
       <c r="I315" t="s">
-        <v>1572</v>
+        <v>1573</v>
       </c>
       <c r="J315" t="s">
         <v>1943</v>
@@ -18780,7 +18780,7 @@
         <v>1488</v>
       </c>
       <c r="I317" t="s">
-        <v>1600</v>
+        <v>1601</v>
       </c>
       <c r="J317" t="s">
         <v>1945</v>
@@ -18902,7 +18902,7 @@
     </row>
     <row r="321" spans="1:12">
       <c r="A321" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B321" t="s">
         <v>361</v>
@@ -18972,7 +18972,7 @@
     </row>
     <row r="323" spans="1:12">
       <c r="A323" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B323" t="s">
         <v>363</v>
@@ -19063,7 +19063,7 @@
         <v>1488</v>
       </c>
       <c r="I325" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="J325" t="s">
         <v>1953</v>
@@ -19182,7 +19182,7 @@
     </row>
     <row r="329" spans="1:12">
       <c r="A329" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B329" t="s">
         <v>369</v>
@@ -19203,7 +19203,7 @@
         <v>1488</v>
       </c>
       <c r="I329" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J329" t="s">
         <v>1957</v>
@@ -19322,7 +19322,7 @@
     </row>
     <row r="333" spans="1:12">
       <c r="A333" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B333" t="s">
         <v>373</v>
@@ -19343,7 +19343,7 @@
         <v>1488</v>
       </c>
       <c r="I333" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J333" t="s">
         <v>1961</v>
@@ -19378,7 +19378,7 @@
         <v>1488</v>
       </c>
       <c r="I334" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="J334" t="s">
         <v>1962</v>
@@ -19427,7 +19427,7 @@
     </row>
     <row r="336" spans="1:12">
       <c r="A336" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B336" t="s">
         <v>376</v>
@@ -19448,7 +19448,7 @@
         <v>1488</v>
       </c>
       <c r="I336" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J336" t="s">
         <v>1964</v>
@@ -19462,7 +19462,7 @@
     </row>
     <row r="337" spans="1:12">
       <c r="A337" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B337" t="s">
         <v>377</v>
@@ -19483,7 +19483,7 @@
         <v>1488</v>
       </c>
       <c r="I337" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J337" t="s">
         <v>1965</v>
@@ -19497,7 +19497,7 @@
     </row>
     <row r="338" spans="1:12">
       <c r="A338" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B338" t="s">
         <v>378</v>
@@ -19518,7 +19518,7 @@
         <v>1488</v>
       </c>
       <c r="I338" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J338" t="s">
         <v>1966</v>
@@ -19532,7 +19532,7 @@
     </row>
     <row r="339" spans="1:12">
       <c r="A339" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B339" t="s">
         <v>379</v>
@@ -19553,7 +19553,7 @@
         <v>1488</v>
       </c>
       <c r="I339" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J339" t="s">
         <v>1942</v>
@@ -19780,7 +19780,7 @@
     </row>
     <row r="346" spans="1:12">
       <c r="A346" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B346" t="s">
         <v>386</v>
@@ -19801,7 +19801,7 @@
         <v>1488</v>
       </c>
       <c r="I346" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J346" t="s">
         <v>1973</v>
@@ -19906,7 +19906,7 @@
         <v>1488</v>
       </c>
       <c r="I349" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="J349" t="s">
         <v>1976</v>
@@ -19920,7 +19920,7 @@
     </row>
     <row r="350" spans="1:12">
       <c r="A350" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B350" t="s">
         <v>390</v>
@@ -19941,7 +19941,7 @@
         <v>1488</v>
       </c>
       <c r="I350" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J350" t="s">
         <v>1977</v>
@@ -19955,7 +19955,7 @@
     </row>
     <row r="351" spans="1:12">
       <c r="A351" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B351" t="s">
         <v>391</v>
@@ -19976,7 +19976,7 @@
         <v>1488</v>
       </c>
       <c r="I351" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J351" t="s">
         <v>1978</v>
@@ -19990,7 +19990,7 @@
     </row>
     <row r="352" spans="1:12">
       <c r="A352" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B352" t="s">
         <v>392</v>
@@ -20011,7 +20011,7 @@
         <v>1488</v>
       </c>
       <c r="I352" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J352" t="s">
         <v>1979</v>
@@ -20025,7 +20025,7 @@
     </row>
     <row r="353" spans="1:12">
       <c r="A353" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B353" t="s">
         <v>393</v>
@@ -20046,7 +20046,7 @@
         <v>1488</v>
       </c>
       <c r="I353" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J353" t="s">
         <v>1980</v>
@@ -20060,7 +20060,7 @@
     </row>
     <row r="354" spans="1:12">
       <c r="A354" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B354" t="s">
         <v>394</v>
@@ -20081,7 +20081,7 @@
         <v>1488</v>
       </c>
       <c r="I354" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J354" t="s">
         <v>1981</v>
@@ -20130,7 +20130,7 @@
     </row>
     <row r="356" spans="1:12">
       <c r="A356" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B356" t="s">
         <v>396</v>
@@ -20165,7 +20165,7 @@
     </row>
     <row r="357" spans="1:12">
       <c r="A357" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B357" t="s">
         <v>397</v>
@@ -20186,7 +20186,7 @@
         <v>1488</v>
       </c>
       <c r="I357" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J357" t="s">
         <v>1984</v>
@@ -20200,7 +20200,7 @@
     </row>
     <row r="358" spans="1:12">
       <c r="A358" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B358" t="s">
         <v>398</v>
@@ -20221,7 +20221,7 @@
         <v>1488</v>
       </c>
       <c r="I358" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J358" t="s">
         <v>1985</v>
@@ -20270,7 +20270,7 @@
     </row>
     <row r="360" spans="1:12">
       <c r="A360" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B360" t="s">
         <v>400</v>
@@ -20291,7 +20291,7 @@
         <v>1488</v>
       </c>
       <c r="I360" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J360" t="s">
         <v>1987</v>
@@ -20361,7 +20361,7 @@
         <v>1488</v>
       </c>
       <c r="I362" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="J362" t="s">
         <v>1989</v>
@@ -20375,7 +20375,7 @@
     </row>
     <row r="363" spans="1:12">
       <c r="A363" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B363" t="s">
         <v>403</v>
@@ -20396,7 +20396,7 @@
         <v>1488</v>
       </c>
       <c r="I363" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J363" t="s">
         <v>1990</v>
@@ -20410,7 +20410,7 @@
     </row>
     <row r="364" spans="1:12">
       <c r="A364" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B364" t="s">
         <v>404</v>
@@ -20431,7 +20431,7 @@
         <v>1488</v>
       </c>
       <c r="I364" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J364" t="s">
         <v>1991</v>
@@ -20445,7 +20445,7 @@
     </row>
     <row r="365" spans="1:12">
       <c r="A365" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B365" t="s">
         <v>405</v>
@@ -20466,7 +20466,7 @@
         <v>1488</v>
       </c>
       <c r="I365" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J365" t="s">
         <v>1992</v>
@@ -20480,7 +20480,7 @@
     </row>
     <row r="366" spans="1:12">
       <c r="A366" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B366" t="s">
         <v>406</v>
@@ -20501,7 +20501,7 @@
         <v>1488</v>
       </c>
       <c r="I366" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J366" t="s">
         <v>1993</v>
@@ -20515,7 +20515,7 @@
     </row>
     <row r="367" spans="1:12">
       <c r="A367" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B367" t="s">
         <v>407</v>
@@ -20536,7 +20536,7 @@
         <v>1488</v>
       </c>
       <c r="I367" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J367" t="s">
         <v>1994</v>
@@ -20550,7 +20550,7 @@
     </row>
     <row r="368" spans="1:12">
       <c r="A368" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B368" t="s">
         <v>408</v>
@@ -20571,7 +20571,7 @@
         <v>1488</v>
       </c>
       <c r="I368" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J368" t="s">
         <v>1995</v>
@@ -20585,7 +20585,7 @@
     </row>
     <row r="369" spans="1:12">
       <c r="A369" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B369" t="s">
         <v>409</v>
@@ -20606,7 +20606,7 @@
         <v>1488</v>
       </c>
       <c r="I369" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J369" t="s">
         <v>1996</v>
@@ -20620,7 +20620,7 @@
     </row>
     <row r="370" spans="1:12">
       <c r="A370" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B370" t="s">
         <v>410</v>
@@ -20641,7 +20641,7 @@
         <v>1488</v>
       </c>
       <c r="I370" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J370" t="s">
         <v>1997</v>
@@ -20655,7 +20655,7 @@
     </row>
     <row r="371" spans="1:12">
       <c r="A371" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B371" t="s">
         <v>411</v>
@@ -20676,7 +20676,7 @@
         <v>1488</v>
       </c>
       <c r="I371" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J371" t="s">
         <v>1998</v>
@@ -20690,7 +20690,7 @@
     </row>
     <row r="372" spans="1:12">
       <c r="A372" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B372" t="s">
         <v>412</v>
@@ -20711,7 +20711,7 @@
         <v>1488</v>
       </c>
       <c r="I372" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J372" t="s">
         <v>1999</v>
@@ -20725,7 +20725,7 @@
     </row>
     <row r="373" spans="1:12">
       <c r="A373" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B373" t="s">
         <v>413</v>
@@ -20746,7 +20746,7 @@
         <v>1488</v>
       </c>
       <c r="I373" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J373" t="s">
         <v>2000</v>
@@ -20760,7 +20760,7 @@
     </row>
     <row r="374" spans="1:12">
       <c r="A374" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B374" t="s">
         <v>414</v>
@@ -20781,7 +20781,7 @@
         <v>1488</v>
       </c>
       <c r="I374" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J374" t="s">
         <v>2001</v>
@@ -20795,7 +20795,7 @@
     </row>
     <row r="375" spans="1:12">
       <c r="A375" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B375" t="s">
         <v>415</v>
@@ -20816,7 +20816,7 @@
         <v>1488</v>
       </c>
       <c r="I375" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J375" t="s">
         <v>2002</v>
@@ -20830,7 +20830,7 @@
     </row>
     <row r="376" spans="1:12">
       <c r="A376" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B376" t="s">
         <v>416</v>
@@ -20851,7 +20851,7 @@
         <v>1488</v>
       </c>
       <c r="I376" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J376" t="s">
         <v>2003</v>
@@ -20865,7 +20865,7 @@
     </row>
     <row r="377" spans="1:12">
       <c r="A377" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B377" t="s">
         <v>417</v>
@@ -20886,7 +20886,7 @@
         <v>1488</v>
       </c>
       <c r="I377" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J377" t="s">
         <v>2004</v>
@@ -20900,7 +20900,7 @@
     </row>
     <row r="378" spans="1:12">
       <c r="A378" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B378" t="s">
         <v>418</v>
@@ -20921,7 +20921,7 @@
         <v>1488</v>
       </c>
       <c r="I378" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J378" t="s">
         <v>2005</v>
@@ -20935,7 +20935,7 @@
     </row>
     <row r="379" spans="1:12">
       <c r="A379" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B379" t="s">
         <v>419</v>
@@ -20956,7 +20956,7 @@
         <v>1488</v>
       </c>
       <c r="I379" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J379" t="s">
         <v>2006</v>
@@ -20970,7 +20970,7 @@
     </row>
     <row r="380" spans="1:12">
       <c r="A380" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B380" t="s">
         <v>420</v>
@@ -20991,7 +20991,7 @@
         <v>1488</v>
       </c>
       <c r="I380" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J380" t="s">
         <v>2007</v>
@@ -21005,7 +21005,7 @@
     </row>
     <row r="381" spans="1:12">
       <c r="A381" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B381" t="s">
         <v>421</v>
@@ -21026,7 +21026,7 @@
         <v>1488</v>
       </c>
       <c r="I381" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J381" t="s">
         <v>2008</v>
@@ -21040,7 +21040,7 @@
     </row>
     <row r="382" spans="1:12">
       <c r="A382" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B382" t="s">
         <v>422</v>
@@ -21061,7 +21061,7 @@
         <v>1488</v>
       </c>
       <c r="I382" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J382" t="s">
         <v>2009</v>
@@ -21075,7 +21075,7 @@
     </row>
     <row r="383" spans="1:12">
       <c r="A383" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B383" t="s">
         <v>423</v>
@@ -21096,7 +21096,7 @@
         <v>1488</v>
       </c>
       <c r="I383" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J383" t="s">
         <v>2010</v>
@@ -21145,7 +21145,7 @@
     </row>
     <row r="385" spans="1:12">
       <c r="A385" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B385" t="s">
         <v>425</v>
@@ -21166,7 +21166,7 @@
         <v>1488</v>
       </c>
       <c r="I385" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J385" t="s">
         <v>2012</v>
@@ -21180,7 +21180,7 @@
     </row>
     <row r="386" spans="1:12">
       <c r="A386" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B386" t="s">
         <v>426</v>
@@ -21201,7 +21201,7 @@
         <v>1488</v>
       </c>
       <c r="I386" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J386" t="s">
         <v>2012</v>
@@ -21215,7 +21215,7 @@
     </row>
     <row r="387" spans="1:12">
       <c r="A387" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B387" t="s">
         <v>427</v>
@@ -21236,7 +21236,7 @@
         <v>1488</v>
       </c>
       <c r="I387" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J387" t="s">
         <v>2012</v>
@@ -21271,7 +21271,7 @@
         <v>1488</v>
       </c>
       <c r="I388" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J388" t="s">
         <v>2013</v>
@@ -21306,7 +21306,7 @@
         <v>1488</v>
       </c>
       <c r="I389" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J389" t="s">
         <v>2013</v>
@@ -21320,7 +21320,7 @@
     </row>
     <row r="390" spans="1:12">
       <c r="A390" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B390" t="s">
         <v>429</v>
@@ -21341,7 +21341,7 @@
         <v>1488</v>
       </c>
       <c r="I390" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J390" t="s">
         <v>2014</v>
@@ -21390,7 +21390,7 @@
     </row>
     <row r="392" spans="1:12">
       <c r="A392" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B392" t="s">
         <v>431</v>
@@ -21533,7 +21533,7 @@
     </row>
     <row r="396" spans="1:12">
       <c r="A396" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B396" t="s">
         <v>435</v>
@@ -21554,7 +21554,7 @@
         <v>1488</v>
       </c>
       <c r="I396" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J396" t="s">
         <v>2020</v>
@@ -21568,7 +21568,7 @@
     </row>
     <row r="397" spans="1:12">
       <c r="A397" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B397" t="s">
         <v>436</v>
@@ -21627,7 +21627,7 @@
         <v>1488</v>
       </c>
       <c r="I398" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
       <c r="J398" t="s">
         <v>2022</v>
@@ -21662,7 +21662,7 @@
         <v>1488</v>
       </c>
       <c r="I399" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="J399" t="s">
         <v>2023</v>
@@ -21676,7 +21676,7 @@
     </row>
     <row r="400" spans="1:12">
       <c r="A400" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B400" t="s">
         <v>439</v>
@@ -21697,7 +21697,7 @@
         <v>1488</v>
       </c>
       <c r="I400" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J400" t="s">
         <v>2024</v>
@@ -21781,7 +21781,7 @@
     </row>
     <row r="403" spans="1:12">
       <c r="A403" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B403" t="s">
         <v>442</v>
@@ -21802,7 +21802,7 @@
         <v>1488</v>
       </c>
       <c r="I403" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J403" t="s">
         <v>2027</v>
@@ -21875,7 +21875,7 @@
         <v>1494</v>
       </c>
       <c r="I405" t="s">
-        <v>1577</v>
+        <v>1578</v>
       </c>
       <c r="J405" t="s">
         <v>2029</v>
@@ -21889,7 +21889,7 @@
     </row>
     <row r="406" spans="1:12">
       <c r="A406" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B406" t="s">
         <v>445</v>
@@ -21910,7 +21910,7 @@
         <v>1488</v>
       </c>
       <c r="I406" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J406" t="s">
         <v>2030</v>
@@ -21924,7 +21924,7 @@
     </row>
     <row r="407" spans="1:12">
       <c r="A407" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B407" t="s">
         <v>446</v>
@@ -21945,7 +21945,7 @@
         <v>1488</v>
       </c>
       <c r="I407" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J407" t="s">
         <v>2031</v>
@@ -21994,7 +21994,7 @@
     </row>
     <row r="409" spans="1:12">
       <c r="A409" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B409" t="s">
         <v>448</v>
@@ -22015,7 +22015,7 @@
         <v>1488</v>
       </c>
       <c r="I409" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="J409" t="s">
         <v>2033</v>
@@ -22064,7 +22064,7 @@
     </row>
     <row r="411" spans="1:12">
       <c r="A411" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B411" t="s">
         <v>450</v>
@@ -22085,7 +22085,7 @@
         <v>1488</v>
       </c>
       <c r="I411" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J411" t="s">
         <v>2035</v>
@@ -22134,7 +22134,7 @@
     </row>
     <row r="413" spans="1:12">
       <c r="A413" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B413" t="s">
         <v>452</v>
@@ -22155,7 +22155,7 @@
         <v>1488</v>
       </c>
       <c r="I413" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J413" t="s">
         <v>2037</v>
@@ -22204,7 +22204,7 @@
     </row>
     <row r="415" spans="1:12">
       <c r="A415" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B415" t="s">
         <v>454</v>
@@ -22225,7 +22225,7 @@
         <v>1488</v>
       </c>
       <c r="I415" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J415" t="s">
         <v>2039</v>
@@ -22330,7 +22330,7 @@
         <v>1488</v>
       </c>
       <c r="I418" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
       <c r="J418" t="s">
         <v>2042</v>
@@ -22379,7 +22379,7 @@
     </row>
     <row r="420" spans="1:12">
       <c r="A420" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B420" t="s">
         <v>459</v>
@@ -22400,7 +22400,7 @@
         <v>1488</v>
       </c>
       <c r="I420" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J420" t="s">
         <v>2044</v>
@@ -22484,7 +22484,7 @@
     </row>
     <row r="423" spans="1:12">
       <c r="A423" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B423" t="s">
         <v>462</v>
@@ -22505,7 +22505,7 @@
         <v>1488</v>
       </c>
       <c r="I423" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J423" t="s">
         <v>2047</v>
@@ -22519,7 +22519,7 @@
     </row>
     <row r="424" spans="1:12">
       <c r="A424" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B424" t="s">
         <v>463</v>
@@ -22540,7 +22540,7 @@
         <v>1488</v>
       </c>
       <c r="I424" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J424" t="s">
         <v>2048</v>
@@ -22554,7 +22554,7 @@
     </row>
     <row r="425" spans="1:12">
       <c r="A425" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B425" t="s">
         <v>464</v>
@@ -22575,7 +22575,7 @@
         <v>1488</v>
       </c>
       <c r="I425" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J425" t="s">
         <v>2049</v>
@@ -22610,7 +22610,7 @@
         <v>1488</v>
       </c>
       <c r="I426" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="J426" t="s">
         <v>2050</v>
@@ -22659,7 +22659,7 @@
     </row>
     <row r="428" spans="1:12">
       <c r="A428" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B428" t="s">
         <v>467</v>
@@ -22680,7 +22680,7 @@
         <v>1488</v>
       </c>
       <c r="I428" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J428" t="s">
         <v>2052</v>
@@ -22729,7 +22729,7 @@
     </row>
     <row r="430" spans="1:12">
       <c r="A430" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B430" t="s">
         <v>469</v>
@@ -22750,7 +22750,7 @@
         <v>1488</v>
       </c>
       <c r="I430" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J430" t="s">
         <v>2054</v>
@@ -22799,7 +22799,7 @@
     </row>
     <row r="432" spans="1:12">
       <c r="A432" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B432" t="s">
         <v>471</v>
@@ -22820,7 +22820,7 @@
         <v>1488</v>
       </c>
       <c r="I432" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J432" t="s">
         <v>2056</v>
@@ -22834,7 +22834,7 @@
     </row>
     <row r="433" spans="1:12">
       <c r="A433" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B433" t="s">
         <v>472</v>
@@ -22939,7 +22939,7 @@
     </row>
     <row r="436" spans="1:12">
       <c r="A436" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B436" t="s">
         <v>475</v>
@@ -23044,7 +23044,7 @@
     </row>
     <row r="439" spans="1:12">
       <c r="A439" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B439" t="s">
         <v>478</v>
@@ -23065,7 +23065,7 @@
         <v>1488</v>
       </c>
       <c r="I439" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J439" t="s">
         <v>2063</v>
@@ -23079,7 +23079,7 @@
     </row>
     <row r="440" spans="1:12">
       <c r="A440" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B440" t="s">
         <v>479</v>
@@ -23100,7 +23100,7 @@
         <v>1488</v>
       </c>
       <c r="I440" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J440" t="s">
         <v>2064</v>
@@ -23114,7 +23114,7 @@
     </row>
     <row r="441" spans="1:12">
       <c r="A441" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B441" t="s">
         <v>480</v>
@@ -23135,7 +23135,7 @@
         <v>1488</v>
       </c>
       <c r="I441" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J441" t="s">
         <v>2065</v>
@@ -23149,7 +23149,7 @@
     </row>
     <row r="442" spans="1:12">
       <c r="A442" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B442" t="s">
         <v>481</v>
@@ -23170,7 +23170,7 @@
         <v>1488</v>
       </c>
       <c r="I442" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J442" t="s">
         <v>2066</v>
@@ -23184,7 +23184,7 @@
     </row>
     <row r="443" spans="1:12">
       <c r="A443" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B443" t="s">
         <v>482</v>
@@ -23205,7 +23205,7 @@
         <v>1488</v>
       </c>
       <c r="I443" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J443" t="s">
         <v>2067</v>
@@ -23219,7 +23219,7 @@
     </row>
     <row r="444" spans="1:12">
       <c r="A444" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B444" t="s">
         <v>483</v>
@@ -23240,7 +23240,7 @@
         <v>1488</v>
       </c>
       <c r="I444" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J444" t="s">
         <v>2068</v>
@@ -23289,7 +23289,7 @@
     </row>
     <row r="446" spans="1:12">
       <c r="A446" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B446" t="s">
         <v>485</v>
@@ -23310,7 +23310,7 @@
         <v>1488</v>
       </c>
       <c r="I446" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J446" t="s">
         <v>1970</v>
@@ -23324,7 +23324,7 @@
     </row>
     <row r="447" spans="1:12">
       <c r="A447" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B447" t="s">
         <v>486</v>
@@ -23348,7 +23348,7 @@
         <v>1496</v>
       </c>
       <c r="I447" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J447" t="s">
         <v>2070</v>
@@ -23397,7 +23397,7 @@
     </row>
     <row r="449" spans="1:12">
       <c r="A449" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B449" t="s">
         <v>488</v>
@@ -23418,7 +23418,7 @@
         <v>1488</v>
       </c>
       <c r="I449" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J449" t="s">
         <v>2072</v>
@@ -23502,7 +23502,7 @@
     </row>
     <row r="452" spans="1:12">
       <c r="A452" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B452" t="s">
         <v>491</v>
@@ -23523,7 +23523,7 @@
         <v>1488</v>
       </c>
       <c r="I452" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J452" t="s">
         <v>2075</v>
@@ -23642,7 +23642,7 @@
     </row>
     <row r="456" spans="1:12">
       <c r="A456" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B456" t="s">
         <v>495</v>
@@ -23663,7 +23663,7 @@
         <v>1488</v>
       </c>
       <c r="I456" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J456" t="s">
         <v>2079</v>
@@ -23677,7 +23677,7 @@
     </row>
     <row r="457" spans="1:12">
       <c r="A457" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B457" t="s">
         <v>496</v>
@@ -23698,7 +23698,7 @@
         <v>1488</v>
       </c>
       <c r="I457" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J457" t="s">
         <v>2080</v>
@@ -23733,7 +23733,7 @@
         <v>1488</v>
       </c>
       <c r="I458" t="s">
-        <v>1611</v>
+        <v>1612</v>
       </c>
       <c r="J458" t="s">
         <v>2081</v>
@@ -23747,7 +23747,7 @@
     </row>
     <row r="459" spans="1:12">
       <c r="A459" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B459" t="s">
         <v>498</v>
@@ -23768,7 +23768,7 @@
         <v>1488</v>
       </c>
       <c r="I459" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J459" t="s">
         <v>2082</v>
@@ -23887,7 +23887,7 @@
     </row>
     <row r="463" spans="1:12">
       <c r="A463" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B463" t="s">
         <v>502</v>
@@ -23908,7 +23908,7 @@
         <v>1488</v>
       </c>
       <c r="I463" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J463" t="s">
         <v>2086</v>
@@ -23922,7 +23922,7 @@
     </row>
     <row r="464" spans="1:12">
       <c r="A464" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B464" t="s">
         <v>503</v>
@@ -23943,7 +23943,7 @@
         <v>1488</v>
       </c>
       <c r="I464" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J464" t="s">
         <v>2087</v>
@@ -24205,7 +24205,7 @@
     </row>
     <row r="472" spans="1:12">
       <c r="A472" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B472" t="s">
         <v>511</v>
@@ -24240,7 +24240,7 @@
     </row>
     <row r="473" spans="1:12">
       <c r="A473" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B473" t="s">
         <v>512</v>
@@ -24261,7 +24261,7 @@
         <v>1488</v>
       </c>
       <c r="I473" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J473" t="s">
         <v>2096</v>
@@ -24275,7 +24275,7 @@
     </row>
     <row r="474" spans="1:12">
       <c r="A474" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B474" t="s">
         <v>513</v>
@@ -24296,7 +24296,7 @@
         <v>1488</v>
       </c>
       <c r="I474" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J474" t="s">
         <v>2097</v>
@@ -24310,7 +24310,7 @@
     </row>
     <row r="475" spans="1:12">
       <c r="A475" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B475" t="s">
         <v>514</v>
@@ -24331,7 +24331,7 @@
         <v>1488</v>
       </c>
       <c r="I475" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J475" t="s">
         <v>2098</v>
@@ -24541,7 +24541,7 @@
         <v>1488</v>
       </c>
       <c r="I481" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="J481" t="s">
         <v>2104</v>
@@ -24625,7 +24625,7 @@
     </row>
     <row r="484" spans="1:12">
       <c r="A484" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B484" t="s">
         <v>523</v>
@@ -24646,7 +24646,7 @@
         <v>1488</v>
       </c>
       <c r="I484" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J484" t="s">
         <v>2106</v>
@@ -24660,7 +24660,7 @@
     </row>
     <row r="485" spans="1:12">
       <c r="A485" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B485" t="s">
         <v>524</v>
@@ -24681,7 +24681,7 @@
         <v>1488</v>
       </c>
       <c r="I485" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J485" t="s">
         <v>2107</v>
@@ -24716,7 +24716,7 @@
         <v>1488</v>
       </c>
       <c r="I486" t="s">
-        <v>1613</v>
+        <v>1614</v>
       </c>
       <c r="J486" t="s">
         <v>2108</v>
@@ -24730,7 +24730,7 @@
     </row>
     <row r="487" spans="1:12">
       <c r="A487" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B487" t="s">
         <v>526</v>
@@ -24751,7 +24751,7 @@
         <v>1488</v>
       </c>
       <c r="I487" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J487" t="s">
         <v>2109</v>
@@ -24800,7 +24800,7 @@
     </row>
     <row r="489" spans="1:12">
       <c r="A489" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B489" t="s">
         <v>528</v>
@@ -24821,7 +24821,7 @@
         <v>1488</v>
       </c>
       <c r="I489" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J489" t="s">
         <v>2111</v>
@@ -24856,7 +24856,7 @@
         <v>1488</v>
       </c>
       <c r="I490" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
       <c r="J490" t="s">
         <v>2112</v>
@@ -24870,7 +24870,7 @@
     </row>
     <row r="491" spans="1:12">
       <c r="A491" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B491" t="s">
         <v>530</v>
@@ -24891,7 +24891,7 @@
         <v>1488</v>
       </c>
       <c r="I491" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J491" t="s">
         <v>2113</v>
@@ -24975,7 +24975,7 @@
     </row>
     <row r="494" spans="1:12">
       <c r="A494" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B494" t="s">
         <v>533</v>
@@ -24996,7 +24996,7 @@
         <v>1488</v>
       </c>
       <c r="I494" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J494" t="s">
         <v>2116</v>
@@ -25010,7 +25010,7 @@
     </row>
     <row r="495" spans="1:12">
       <c r="A495" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B495" t="s">
         <v>534</v>
@@ -25048,7 +25048,7 @@
     </row>
     <row r="496" spans="1:12">
       <c r="A496" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B496" t="s">
         <v>535</v>
@@ -25069,7 +25069,7 @@
         <v>1488</v>
       </c>
       <c r="I496" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J496" t="s">
         <v>2118</v>
@@ -25083,7 +25083,7 @@
     </row>
     <row r="497" spans="1:12">
       <c r="A497" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B497" t="s">
         <v>536</v>
@@ -25104,7 +25104,7 @@
         <v>1488</v>
       </c>
       <c r="I497" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J497" t="s">
         <v>2119</v>
@@ -25118,7 +25118,7 @@
     </row>
     <row r="498" spans="1:12">
       <c r="A498" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B498" t="s">
         <v>537</v>
@@ -25139,7 +25139,7 @@
         <v>1488</v>
       </c>
       <c r="I498" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J498" t="s">
         <v>2120</v>
@@ -25153,7 +25153,7 @@
     </row>
     <row r="499" spans="1:12">
       <c r="A499" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B499" t="s">
         <v>538</v>
@@ -25174,7 +25174,7 @@
         <v>1488</v>
       </c>
       <c r="I499" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J499" t="s">
         <v>2121</v>
@@ -25188,7 +25188,7 @@
     </row>
     <row r="500" spans="1:12">
       <c r="A500" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B500" t="s">
         <v>539</v>
@@ -25209,7 +25209,7 @@
         <v>1488</v>
       </c>
       <c r="I500" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J500" t="s">
         <v>2122</v>
@@ -25223,7 +25223,7 @@
     </row>
     <row r="501" spans="1:12">
       <c r="A501" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B501" t="s">
         <v>540</v>
@@ -25244,7 +25244,7 @@
         <v>1488</v>
       </c>
       <c r="I501" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J501" t="s">
         <v>2123</v>
@@ -25279,7 +25279,7 @@
         <v>1488</v>
       </c>
       <c r="I502" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="J502" t="s">
         <v>2124</v>
@@ -25293,7 +25293,7 @@
     </row>
     <row r="503" spans="1:12">
       <c r="A503" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B503" t="s">
         <v>542</v>
@@ -25314,7 +25314,7 @@
         <v>1488</v>
       </c>
       <c r="I503" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J503" t="s">
         <v>2125</v>
@@ -25352,7 +25352,7 @@
         <v>1499</v>
       </c>
       <c r="I504" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J504" t="s">
         <v>2126</v>
@@ -25366,7 +25366,7 @@
     </row>
     <row r="505" spans="1:12">
       <c r="A505" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B505" t="s">
         <v>544</v>
@@ -25387,7 +25387,7 @@
         <v>1488</v>
       </c>
       <c r="I505" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J505" t="s">
         <v>2127</v>
@@ -25471,7 +25471,7 @@
     </row>
     <row r="508" spans="1:12">
       <c r="A508" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B508" t="s">
         <v>547</v>
@@ -25562,7 +25562,7 @@
         <v>1488</v>
       </c>
       <c r="I510" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="J510" t="s">
         <v>2132</v>
@@ -25576,7 +25576,7 @@
     </row>
     <row r="511" spans="1:12">
       <c r="A511" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B511" t="s">
         <v>550</v>
@@ -25597,7 +25597,7 @@
         <v>1488</v>
       </c>
       <c r="I511" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J511" t="s">
         <v>2133</v>
@@ -25611,7 +25611,7 @@
     </row>
     <row r="512" spans="1:12">
       <c r="A512" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B512" t="s">
         <v>551</v>
@@ -25632,7 +25632,7 @@
         <v>1488</v>
       </c>
       <c r="I512" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J512" t="s">
         <v>2134</v>
@@ -25646,7 +25646,7 @@
     </row>
     <row r="513" spans="1:12">
       <c r="A513" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B513" t="s">
         <v>552</v>
@@ -25667,7 +25667,7 @@
         <v>1488</v>
       </c>
       <c r="I513" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J513" t="s">
         <v>2135</v>
@@ -25681,7 +25681,7 @@
     </row>
     <row r="514" spans="1:12">
       <c r="A514" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B514" t="s">
         <v>553</v>
@@ -25702,7 +25702,7 @@
         <v>1488</v>
       </c>
       <c r="I514" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J514" t="s">
         <v>2136</v>
@@ -25737,7 +25737,7 @@
         <v>1488</v>
       </c>
       <c r="I515" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="J515" t="s">
         <v>2137</v>
@@ -25859,7 +25859,7 @@
     </row>
     <row r="519" spans="1:12">
       <c r="A519" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B519" t="s">
         <v>558</v>
@@ -25883,7 +25883,7 @@
         <v>1494</v>
       </c>
       <c r="I519" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J519" t="s">
         <v>2139</v>
@@ -25897,7 +25897,7 @@
     </row>
     <row r="520" spans="1:12">
       <c r="A520" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B520" t="s">
         <v>559</v>
@@ -25918,7 +25918,7 @@
         <v>1488</v>
       </c>
       <c r="I520" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J520" t="s">
         <v>2140</v>
@@ -25988,7 +25988,7 @@
         <v>1488</v>
       </c>
       <c r="I522" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="J522" t="s">
         <v>2142</v>
@@ -26110,7 +26110,7 @@
     </row>
     <row r="526" spans="1:12">
       <c r="A526" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B526" t="s">
         <v>565</v>
@@ -26131,7 +26131,7 @@
         <v>1488</v>
       </c>
       <c r="I526" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J526" t="s">
         <v>2146</v>
@@ -26166,7 +26166,7 @@
         <v>1488</v>
       </c>
       <c r="I527" t="s">
-        <v>1577</v>
+        <v>1578</v>
       </c>
       <c r="J527" t="s">
         <v>2147</v>
@@ -26180,7 +26180,7 @@
     </row>
     <row r="528" spans="1:12">
       <c r="A528" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B528" t="s">
         <v>567</v>
@@ -26201,7 +26201,7 @@
         <v>1488</v>
       </c>
       <c r="I528" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J528" t="s">
         <v>2148</v>
@@ -26215,7 +26215,7 @@
     </row>
     <row r="529" spans="1:12">
       <c r="A529" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B529" t="s">
         <v>568</v>
@@ -26236,7 +26236,7 @@
         <v>1488</v>
       </c>
       <c r="I529" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J529" t="s">
         <v>2149</v>
@@ -26250,7 +26250,7 @@
     </row>
     <row r="530" spans="1:12">
       <c r="A530" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B530" t="s">
         <v>569</v>
@@ -26271,7 +26271,7 @@
         <v>1488</v>
       </c>
       <c r="I530" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J530" t="s">
         <v>2150</v>
@@ -26285,7 +26285,7 @@
     </row>
     <row r="531" spans="1:12">
       <c r="A531" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B531" t="s">
         <v>570</v>
@@ -26306,7 +26306,7 @@
         <v>1488</v>
       </c>
       <c r="I531" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J531" t="s">
         <v>2151</v>
@@ -26320,7 +26320,7 @@
     </row>
     <row r="532" spans="1:12">
       <c r="A532" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B532" t="s">
         <v>571</v>
@@ -26344,7 +26344,7 @@
         <v>1502</v>
       </c>
       <c r="I532" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J532" t="s">
         <v>2152</v>
@@ -26358,7 +26358,7 @@
     </row>
     <row r="533" spans="1:12">
       <c r="A533" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B533" t="s">
         <v>572</v>
@@ -26379,7 +26379,7 @@
         <v>1488</v>
       </c>
       <c r="I533" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J533" t="s">
         <v>2153</v>
@@ -26393,7 +26393,7 @@
     </row>
     <row r="534" spans="1:12">
       <c r="A534" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B534" t="s">
         <v>573</v>
@@ -26414,7 +26414,7 @@
         <v>1488</v>
       </c>
       <c r="I534" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J534" t="s">
         <v>2154</v>
@@ -26428,7 +26428,7 @@
     </row>
     <row r="535" spans="1:12">
       <c r="A535" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B535" t="s">
         <v>573</v>
@@ -26449,7 +26449,7 @@
         <v>1488</v>
       </c>
       <c r="I535" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J535" t="s">
         <v>2154</v>
@@ -26463,7 +26463,7 @@
     </row>
     <row r="536" spans="1:12">
       <c r="A536" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B536" t="s">
         <v>574</v>
@@ -26484,7 +26484,7 @@
         <v>1488</v>
       </c>
       <c r="I536" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J536" t="s">
         <v>2155</v>
@@ -26498,7 +26498,7 @@
     </row>
     <row r="537" spans="1:12">
       <c r="A537" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B537" t="s">
         <v>575</v>
@@ -26519,7 +26519,7 @@
         <v>1488</v>
       </c>
       <c r="I537" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J537" t="s">
         <v>2156</v>
@@ -26533,7 +26533,7 @@
     </row>
     <row r="538" spans="1:12">
       <c r="A538" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B538" t="s">
         <v>576</v>
@@ -26554,7 +26554,7 @@
         <v>1488</v>
       </c>
       <c r="I538" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J538" t="s">
         <v>2157</v>
@@ -26568,7 +26568,7 @@
     </row>
     <row r="539" spans="1:12">
       <c r="A539" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B539" t="s">
         <v>577</v>
@@ -26589,7 +26589,7 @@
         <v>1488</v>
       </c>
       <c r="I539" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J539" t="s">
         <v>2158</v>
@@ -26603,7 +26603,7 @@
     </row>
     <row r="540" spans="1:12">
       <c r="A540" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B540" t="s">
         <v>578</v>
@@ -26624,7 +26624,7 @@
         <v>1488</v>
       </c>
       <c r="I540" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J540" t="s">
         <v>2159</v>
@@ -26638,7 +26638,7 @@
     </row>
     <row r="541" spans="1:12">
       <c r="A541" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B541" t="s">
         <v>579</v>
@@ -26659,7 +26659,7 @@
         <v>1488</v>
       </c>
       <c r="I541" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J541" t="s">
         <v>2160</v>
@@ -26673,7 +26673,7 @@
     </row>
     <row r="542" spans="1:12">
       <c r="A542" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B542" t="s">
         <v>580</v>
@@ -26694,7 +26694,7 @@
         <v>1488</v>
       </c>
       <c r="I542" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J542" t="s">
         <v>2161</v>
@@ -26708,7 +26708,7 @@
     </row>
     <row r="543" spans="1:12">
       <c r="A543" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B543" t="s">
         <v>581</v>
@@ -26729,7 +26729,7 @@
         <v>1488</v>
       </c>
       <c r="I543" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J543" t="s">
         <v>2162</v>
@@ -26743,7 +26743,7 @@
     </row>
     <row r="544" spans="1:12">
       <c r="A544" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B544" t="s">
         <v>582</v>
@@ -26764,7 +26764,7 @@
         <v>1488</v>
       </c>
       <c r="I544" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J544" t="s">
         <v>2163</v>
@@ -26778,7 +26778,7 @@
     </row>
     <row r="545" spans="1:12">
       <c r="A545" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B545" t="s">
         <v>583</v>
@@ -26799,7 +26799,7 @@
         <v>1488</v>
       </c>
       <c r="I545" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J545" t="s">
         <v>2164</v>
@@ -26813,7 +26813,7 @@
     </row>
     <row r="546" spans="1:12">
       <c r="A546" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B546" t="s">
         <v>584</v>
@@ -26834,7 +26834,7 @@
         <v>1488</v>
       </c>
       <c r="I546" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J546" t="s">
         <v>2165</v>
@@ -26848,7 +26848,7 @@
     </row>
     <row r="547" spans="1:12">
       <c r="A547" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B547" t="s">
         <v>585</v>
@@ -26869,7 +26869,7 @@
         <v>1488</v>
       </c>
       <c r="I547" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J547" t="s">
         <v>2166</v>
@@ -26883,7 +26883,7 @@
     </row>
     <row r="548" spans="1:12">
       <c r="A548" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B548" t="s">
         <v>586</v>
@@ -26904,7 +26904,7 @@
         <v>1488</v>
       </c>
       <c r="I548" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J548" t="s">
         <v>2167</v>
@@ -26918,7 +26918,7 @@
     </row>
     <row r="549" spans="1:12">
       <c r="A549" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B549" t="s">
         <v>587</v>
@@ -26942,7 +26942,7 @@
         <v>1503</v>
       </c>
       <c r="I549" t="s">
-        <v>1521</v>
+        <v>1547</v>
       </c>
       <c r="J549" t="s">
         <v>2168</v>
@@ -26956,7 +26956,7 @@
     </row>
     <row r="550" spans="1:12">
       <c r="A550" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B550" t="s">
         <v>588</v>
@@ -26977,7 +26977,7 @@
         <v>1488</v>
       </c>
       <c r="I550" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="J550" t="s">
         <v>2169</v>
@@ -27012,7 +27012,7 @@
         <v>1488</v>
       </c>
       <c r="I551" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J551" t="s">
         <v>2170</v>
@@ -27026,7 +27026,7 @@
     </row>
     <row r="552" spans="1:12">
       <c r="A552" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B552" t="s">
         <v>590</v>
@@ -27047,7 +27047,7 @@
         <v>1488</v>
       </c>
       <c r="I552" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J552" t="s">
         <v>2171</v>
@@ -27155,7 +27155,7 @@
         <v>1504</v>
       </c>
       <c r="I555" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
       <c r="J555" t="s">
         <v>2174</v>
@@ -27169,7 +27169,7 @@
     </row>
     <row r="556" spans="1:12">
       <c r="A556" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B556" t="s">
         <v>594</v>
@@ -27190,7 +27190,7 @@
         <v>1488</v>
       </c>
       <c r="I556" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J556" t="s">
         <v>2096</v>
@@ -27228,7 +27228,7 @@
         <v>1505</v>
       </c>
       <c r="I557" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
       <c r="J557" t="s">
         <v>2175</v>
@@ -27263,7 +27263,7 @@
         <v>1488</v>
       </c>
       <c r="I558" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
       <c r="J558" t="s">
         <v>2176</v>
@@ -27277,7 +27277,7 @@
     </row>
     <row r="559" spans="1:12">
       <c r="A559" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B559" t="s">
         <v>597</v>
@@ -27298,7 +27298,7 @@
         <v>1488</v>
       </c>
       <c r="I559" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J559" t="s">
         <v>2177</v>
@@ -27312,7 +27312,7 @@
     </row>
     <row r="560" spans="1:12">
       <c r="A560" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B560" t="s">
         <v>598</v>
@@ -27333,7 +27333,7 @@
         <v>1488</v>
       </c>
       <c r="I560" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J560" t="s">
         <v>2178</v>
@@ -27347,7 +27347,7 @@
     </row>
     <row r="561" spans="1:12">
       <c r="A561" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B561" t="s">
         <v>599</v>
@@ -27368,7 +27368,7 @@
         <v>1488</v>
       </c>
       <c r="I561" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J561" t="s">
         <v>2179</v>
@@ -27382,7 +27382,7 @@
     </row>
     <row r="562" spans="1:12">
       <c r="A562" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B562" t="s">
         <v>600</v>
@@ -27403,7 +27403,7 @@
         <v>1488</v>
       </c>
       <c r="I562" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J562" t="s">
         <v>2180</v>
@@ -27417,7 +27417,7 @@
     </row>
     <row r="563" spans="1:12">
       <c r="A563" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B563" t="s">
         <v>601</v>
@@ -27438,7 +27438,7 @@
         <v>1488</v>
       </c>
       <c r="I563" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J563" t="s">
         <v>2181</v>
@@ -27452,7 +27452,7 @@
     </row>
     <row r="564" spans="1:12">
       <c r="A564" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B564" t="s">
         <v>602</v>
@@ -27473,7 +27473,7 @@
         <v>1488</v>
       </c>
       <c r="I564" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J564" t="s">
         <v>2182</v>
@@ -27508,7 +27508,7 @@
         <v>1488</v>
       </c>
       <c r="I565" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="J565" t="s">
         <v>2183</v>
@@ -27557,7 +27557,7 @@
     </row>
     <row r="567" spans="1:12">
       <c r="A567" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B567" t="s">
         <v>605</v>
@@ -27578,7 +27578,7 @@
         <v>1488</v>
       </c>
       <c r="I567" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J567" t="s">
         <v>2185</v>
@@ -27616,7 +27616,7 @@
         <v>1506</v>
       </c>
       <c r="I568" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J568" t="s">
         <v>2186</v>
@@ -27668,7 +27668,7 @@
     </row>
     <row r="570" spans="1:12">
       <c r="A570" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B570" t="s">
         <v>608</v>
@@ -27689,7 +27689,7 @@
         <v>1488</v>
       </c>
       <c r="I570" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J570" t="s">
         <v>2188</v>
@@ -27703,7 +27703,7 @@
     </row>
     <row r="571" spans="1:12">
       <c r="A571" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B571" t="s">
         <v>609</v>
@@ -27724,7 +27724,7 @@
         <v>1488</v>
       </c>
       <c r="I571" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J571" t="s">
         <v>2189</v>
@@ -27738,7 +27738,7 @@
     </row>
     <row r="572" spans="1:12">
       <c r="A572" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B572" t="s">
         <v>610</v>
@@ -27759,7 +27759,7 @@
         <v>1488</v>
       </c>
       <c r="I572" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J572" t="s">
         <v>2190</v>
@@ -27794,7 +27794,7 @@
         <v>1488</v>
       </c>
       <c r="I573" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="J573" t="s">
         <v>2191</v>
@@ -27808,7 +27808,7 @@
     </row>
     <row r="574" spans="1:12">
       <c r="A574" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B574" t="s">
         <v>612</v>
@@ -27829,7 +27829,7 @@
         <v>1488</v>
       </c>
       <c r="I574" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J574" t="s">
         <v>2192</v>
@@ -27864,7 +27864,7 @@
         <v>1488</v>
       </c>
       <c r="I575" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="J575" t="s">
         <v>2193</v>
@@ -27899,7 +27899,7 @@
         <v>1488</v>
       </c>
       <c r="I576" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="J576" t="s">
         <v>2194</v>
@@ -27937,7 +27937,7 @@
         <v>1508</v>
       </c>
       <c r="I577" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
       <c r="J577" t="s">
         <v>2195</v>
@@ -27951,7 +27951,7 @@
     </row>
     <row r="578" spans="1:12">
       <c r="A578" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B578" t="s">
         <v>616</v>
@@ -27972,7 +27972,7 @@
         <v>1488</v>
       </c>
       <c r="I578" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J578" t="s">
         <v>2196</v>
@@ -27986,7 +27986,7 @@
     </row>
     <row r="579" spans="1:12">
       <c r="A579" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B579" t="s">
         <v>617</v>
@@ -28007,7 +28007,7 @@
         <v>1488</v>
       </c>
       <c r="I579" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J579" t="s">
         <v>2197</v>
@@ -28021,7 +28021,7 @@
     </row>
     <row r="580" spans="1:12">
       <c r="A580" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B580" t="s">
         <v>618</v>
@@ -28042,7 +28042,7 @@
         <v>1488</v>
       </c>
       <c r="I580" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J580" t="s">
         <v>2198</v>
@@ -28056,7 +28056,7 @@
     </row>
     <row r="581" spans="1:12">
       <c r="A581" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B581" t="s">
         <v>619</v>
@@ -28077,7 +28077,7 @@
         <v>1488</v>
       </c>
       <c r="I581" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J581" t="s">
         <v>2199</v>
@@ -28126,7 +28126,7 @@
     </row>
     <row r="583" spans="1:12">
       <c r="A583" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B583" t="s">
         <v>621</v>
@@ -28147,7 +28147,7 @@
         <v>1488</v>
       </c>
       <c r="I583" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J583" t="s">
         <v>2201</v>
@@ -28161,7 +28161,7 @@
     </row>
     <row r="584" spans="1:12">
       <c r="A584" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B584" t="s">
         <v>622</v>
@@ -28182,7 +28182,7 @@
         <v>1488</v>
       </c>
       <c r="I584" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J584" t="s">
         <v>2202</v>
@@ -28196,7 +28196,7 @@
     </row>
     <row r="585" spans="1:12">
       <c r="A585" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B585" t="s">
         <v>623</v>
@@ -28217,7 +28217,7 @@
         <v>1488</v>
       </c>
       <c r="I585" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J585" t="s">
         <v>2203</v>
@@ -28231,7 +28231,7 @@
     </row>
     <row r="586" spans="1:12">
       <c r="A586" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B586" t="s">
         <v>624</v>
@@ -28252,7 +28252,7 @@
         <v>1488</v>
       </c>
       <c r="I586" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J586" t="s">
         <v>2204</v>
@@ -28290,7 +28290,7 @@
         <v>1509</v>
       </c>
       <c r="I587" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J587" t="s">
         <v>2205</v>
@@ -28328,7 +28328,7 @@
         <v>1510</v>
       </c>
       <c r="I588" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="J588" t="s">
         <v>2206</v>
@@ -28366,7 +28366,7 @@
         <v>1509</v>
       </c>
       <c r="I589" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="J589" t="s">
         <v>2207</v>
@@ -28442,7 +28442,7 @@
         <v>1509</v>
       </c>
       <c r="I591" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J591" t="s">
         <v>2209</v>
@@ -28456,7 +28456,7 @@
     </row>
     <row r="592" spans="1:12">
       <c r="A592" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B592" t="s">
         <v>630</v>
@@ -28477,7 +28477,7 @@
         <v>1488</v>
       </c>
       <c r="I592" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J592" t="s">
         <v>2210</v>
@@ -28512,7 +28512,7 @@
         <v>1488</v>
       </c>
       <c r="I593" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J593" t="s">
         <v>2211</v>
@@ -28550,7 +28550,7 @@
         <v>1509</v>
       </c>
       <c r="I594" t="s">
-        <v>1628</v>
+        <v>1629</v>
       </c>
       <c r="J594" t="s">
         <v>2212</v>
@@ -28588,7 +28588,7 @@
         <v>1511</v>
       </c>
       <c r="I595" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="J595" t="s">
         <v>2213</v>
@@ -28626,7 +28626,7 @@
         <v>1512</v>
       </c>
       <c r="I596" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
       <c r="J596" t="s">
         <v>2214</v>
@@ -28678,7 +28678,7 @@
     </row>
     <row r="598" spans="1:12">
       <c r="A598" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B598" t="s">
         <v>636</v>
@@ -28702,7 +28702,7 @@
         <v>1512</v>
       </c>
       <c r="I598" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="J598" t="s">
         <v>2216</v>
@@ -28716,7 +28716,7 @@
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B599" t="s">
         <v>637</v>
@@ -28737,7 +28737,7 @@
         <v>1488</v>
       </c>
       <c r="I599" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J599" t="s">
         <v>2217</v>
@@ -28775,7 +28775,7 @@
         <v>1510</v>
       </c>
       <c r="I600" t="s">
-        <v>1630</v>
+        <v>1631</v>
       </c>
       <c r="J600" t="s">
         <v>2218</v>
@@ -28789,7 +28789,7 @@
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B601" t="s">
         <v>639</v>
@@ -28810,7 +28810,7 @@
         <v>1488</v>
       </c>
       <c r="I601" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J601" t="s">
         <v>2219</v>
@@ -28824,7 +28824,7 @@
     </row>
     <row r="602" spans="1:12">
       <c r="A602" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B602" t="s">
         <v>640</v>
@@ -28845,7 +28845,7 @@
         <v>1488</v>
       </c>
       <c r="I602" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J602" t="s">
         <v>2220</v>
@@ -28859,7 +28859,7 @@
     </row>
     <row r="603" spans="1:12">
       <c r="A603" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B603" t="s">
         <v>641</v>
@@ -28880,7 +28880,7 @@
         <v>1488</v>
       </c>
       <c r="I603" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J603" t="s">
         <v>2221</v>
@@ -28894,7 +28894,7 @@
     </row>
     <row r="604" spans="1:12">
       <c r="A604" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B604" t="s">
         <v>642</v>
@@ -28915,7 +28915,7 @@
         <v>1488</v>
       </c>
       <c r="I604" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J604" t="s">
         <v>2222</v>
@@ -28929,7 +28929,7 @@
     </row>
     <row r="605" spans="1:12">
       <c r="A605" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B605" t="s">
         <v>643</v>
@@ -28950,7 +28950,7 @@
         <v>1488</v>
       </c>
       <c r="I605" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J605" t="s">
         <v>2223</v>
@@ -28964,7 +28964,7 @@
     </row>
     <row r="606" spans="1:12">
       <c r="A606" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B606" t="s">
         <v>644</v>
@@ -28985,7 +28985,7 @@
         <v>1488</v>
       </c>
       <c r="I606" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J606" t="s">
         <v>2224</v>
@@ -28999,7 +28999,7 @@
     </row>
     <row r="607" spans="1:12">
       <c r="A607" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B607" t="s">
         <v>645</v>
@@ -29020,7 +29020,7 @@
         <v>1488</v>
       </c>
       <c r="I607" t="s">
-        <v>1631</v>
+        <v>1547</v>
       </c>
       <c r="J607" t="s">
         <v>2225</v>
@@ -29034,7 +29034,7 @@
     </row>
     <row r="608" spans="1:12">
       <c r="A608" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B608" t="s">
         <v>646</v>
@@ -29055,7 +29055,7 @@
         <v>1488</v>
       </c>
       <c r="I608" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J608" t="s">
         <v>2226</v>
@@ -29069,7 +29069,7 @@
     </row>
     <row r="609" spans="1:12">
       <c r="A609" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B609" t="s">
         <v>647</v>
@@ -29090,7 +29090,7 @@
         <v>1488</v>
       </c>
       <c r="I609" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J609" t="s">
         <v>2227</v>
@@ -29104,7 +29104,7 @@
     </row>
     <row r="610" spans="1:12">
       <c r="A610" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B610" t="s">
         <v>648</v>
@@ -29125,7 +29125,7 @@
         <v>1488</v>
       </c>
       <c r="I610" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J610" t="s">
         <v>2228</v>
@@ -29139,7 +29139,7 @@
     </row>
     <row r="611" spans="1:12">
       <c r="A611" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B611" t="s">
         <v>649</v>
@@ -29160,7 +29160,7 @@
         <v>1488</v>
       </c>
       <c r="I611" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J611" t="s">
         <v>2229</v>
@@ -29174,7 +29174,7 @@
     </row>
     <row r="612" spans="1:12">
       <c r="A612" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B612" t="s">
         <v>650</v>
@@ -29195,7 +29195,7 @@
         <v>1488</v>
       </c>
       <c r="I612" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J612" t="s">
         <v>2230</v>
@@ -29209,7 +29209,7 @@
     </row>
     <row r="613" spans="1:12">
       <c r="A613" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B613" t="s">
         <v>651</v>
@@ -29230,7 +29230,7 @@
         <v>1488</v>
       </c>
       <c r="I613" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J613" t="s">
         <v>2230</v>
@@ -29244,7 +29244,7 @@
     </row>
     <row r="614" spans="1:12">
       <c r="A614" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B614" t="s">
         <v>652</v>
@@ -29268,7 +29268,7 @@
         <v>1510</v>
       </c>
       <c r="I614" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="J614" t="s">
         <v>2231</v>
@@ -29282,7 +29282,7 @@
     </row>
     <row r="615" spans="1:12">
       <c r="A615" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B615" t="s">
         <v>653</v>
@@ -29303,7 +29303,7 @@
         <v>1488</v>
       </c>
       <c r="I615" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J615" t="s">
         <v>2232</v>
@@ -29317,7 +29317,7 @@
     </row>
     <row r="616" spans="1:12">
       <c r="A616" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B616" t="s">
         <v>654</v>
@@ -29355,7 +29355,7 @@
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B617" t="s">
         <v>655</v>
@@ -29376,7 +29376,7 @@
         <v>1488</v>
       </c>
       <c r="I617" t="s">
-        <v>1629</v>
+        <v>1630</v>
       </c>
       <c r="J617" t="s">
         <v>2234</v>
@@ -29390,7 +29390,7 @@
     </row>
     <row r="618" spans="1:12">
       <c r="A618" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B618" t="s">
         <v>656</v>
@@ -29411,7 +29411,7 @@
         <v>1488</v>
       </c>
       <c r="I618" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J618" t="s">
         <v>2235</v>
@@ -29425,7 +29425,7 @@
     </row>
     <row r="619" spans="1:12">
       <c r="A619" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B619" t="s">
         <v>657</v>
@@ -29446,7 +29446,7 @@
         <v>1488</v>
       </c>
       <c r="I619" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J619" t="s">
         <v>2236</v>
@@ -29460,7 +29460,7 @@
     </row>
     <row r="620" spans="1:12">
       <c r="A620" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B620" t="s">
         <v>658</v>
@@ -29481,7 +29481,7 @@
         <v>1488</v>
       </c>
       <c r="I620" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J620" t="s">
         <v>2237</v>
@@ -29495,7 +29495,7 @@
     </row>
     <row r="621" spans="1:12">
       <c r="A621" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B621" t="s">
         <v>659</v>
@@ -29513,7 +29513,7 @@
         <v>1488</v>
       </c>
       <c r="I621" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J621" t="s">
         <v>2238</v>
@@ -29527,7 +29527,7 @@
     </row>
     <row r="622" spans="1:12">
       <c r="A622" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B622" t="s">
         <v>660</v>
@@ -29545,7 +29545,7 @@
         <v>1488</v>
       </c>
       <c r="I622" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J622" t="s">
         <v>2239</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-13 02:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4612,13 +4612,13 @@
     <t>MOEMA BELLONI SCHMIDT</t>
   </si>
   <si>
+    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
+  </si>
+  <si>
+    <t>LUZIA LAMOSA ARANTES</t>
+  </si>
+  <si>
     <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
-  </si>
-  <si>
-    <t>LUZIA LAMOSA ARANTES</t>
   </si>
   <si>
     <t>EDIWAN SOUSA DA SILVA</t>
@@ -10343,7 +10343,7 @@
     </row>
     <row r="78" spans="1:12">
       <c r="A78" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B78" t="s">
         <v>118</v>
@@ -10364,7 +10364,7 @@
         <v>1479</v>
       </c>
       <c r="I78" t="s">
-        <v>1532</v>
+        <v>1507</v>
       </c>
       <c r="J78" t="s">
         <v>1695</v>
@@ -10399,7 +10399,7 @@
         <v>1479</v>
       </c>
       <c r="I79" t="s">
-        <v>1533</v>
+        <v>1532</v>
       </c>
       <c r="J79" t="s">
         <v>1696</v>
@@ -10469,7 +10469,7 @@
         <v>1479</v>
       </c>
       <c r="I81" t="s">
-        <v>1534</v>
+        <v>1533</v>
       </c>
       <c r="J81" t="s">
         <v>1698</v>
@@ -10539,7 +10539,7 @@
         <v>1479</v>
       </c>
       <c r="I83" t="s">
-        <v>1532</v>
+        <v>1534</v>
       </c>
       <c r="J83" t="s">
         <v>1700</v>
@@ -10819,7 +10819,7 @@
         <v>1479</v>
       </c>
       <c r="I91" t="s">
-        <v>1534</v>
+        <v>1533</v>
       </c>
       <c r="J91" t="s">
         <v>1708</v>
@@ -19269,7 +19269,7 @@
         <v>1485</v>
       </c>
       <c r="I332" t="s">
-        <v>1532</v>
+        <v>1534</v>
       </c>
       <c r="J332" t="s">
         <v>1947</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-14 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -1825,9 +1825,6 @@
     <t>20.22.0001.0069984.2026-96</t>
   </si>
   <si>
-    <t>20.22.0001.0069982.2026-53</t>
-  </si>
-  <si>
     <t>20.22.0001.0054367.2025-02</t>
   </si>
   <si>
@@ -1933,6 +1930,9 @@
     <t>20.22.0001.0014000.2026-16</t>
   </si>
   <si>
+    <t>20.22.0001.0073504.2026-19</t>
+  </si>
+  <si>
     <t>20.22.0001.0073419.2026-83</t>
   </si>
   <si>
@@ -3643,9 +3643,6 @@
     <t>2026.1222</t>
   </si>
   <si>
-    <t>2026.1220</t>
-  </si>
-  <si>
     <t>2025.0963</t>
   </si>
   <si>
@@ -3751,6 +3748,9 @@
     <t>2026.0204</t>
   </si>
   <si>
+    <t>2026.1272</t>
+  </si>
+  <si>
     <t>2026.1271</t>
   </si>
   <si>
@@ -4465,9 +4465,6 @@
     <t>15/10/2026</t>
   </si>
   <si>
-    <t>16/10/2026</t>
-  </si>
-  <si>
     <t>20/10/2026</t>
   </si>
   <si>
@@ -4477,6 +4474,9 @@
     <t>30/10/2026</t>
   </si>
   <si>
+    <t>27/10/2026</t>
+  </si>
+  <si>
     <t>CASSIA CRISTINA DA SILVA,EDIWAN SOUSA DA SILVA</t>
   </si>
   <si>
@@ -6475,9 +6475,6 @@
     <t>202200681790</t>
   </si>
   <si>
-    <t>201900042656</t>
-  </si>
-  <si>
     <t>202400714998</t>
   </si>
   <si>
@@ -6578,6 +6575,9 @@
   </si>
   <si>
     <t>202500624023</t>
+  </si>
+  <si>
+    <t>202500141011</t>
   </si>
   <si>
     <t>201700677509</t>
@@ -22603,7 +22603,7 @@
     </row>
     <row r="430" spans="1:12">
       <c r="A430" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="B430" t="s">
         <v>469</v>
@@ -22624,7 +22624,7 @@
         <v>1461</v>
       </c>
       <c r="I430" t="s">
-        <v>1492</v>
+        <v>1537</v>
       </c>
       <c r="J430" t="s">
         <v>2023</v>
@@ -27379,7 +27379,7 @@
     </row>
     <row r="565" spans="1:12">
       <c r="A565" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B565" t="s">
         <v>603</v>
@@ -27394,30 +27394,27 @@
         <v>13</v>
       </c>
       <c r="F565" t="s">
-        <v>1458</v>
+        <v>1456</v>
       </c>
       <c r="G565" t="s">
-        <v>1462</v>
-      </c>
-      <c r="H565" t="s">
-        <v>1483</v>
+        <v>1461</v>
       </c>
       <c r="I565" t="s">
-        <v>1492</v>
+        <v>1576</v>
       </c>
       <c r="J565" t="s">
         <v>2153</v>
       </c>
       <c r="K565" t="s">
-        <v>2199</v>
+        <v>2245</v>
       </c>
       <c r="L565" t="s">
-        <v>2313</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="566" spans="1:12">
       <c r="A566" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B566" t="s">
         <v>604</v>
@@ -27426,33 +27423,36 @@
         <v>1210</v>
       </c>
       <c r="D566" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="E566">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="F566" t="s">
-        <v>1456</v>
+        <v>1458</v>
       </c>
       <c r="G566" t="s">
-        <v>1461</v>
+        <v>1462</v>
+      </c>
+      <c r="H566" t="s">
+        <v>1483</v>
       </c>
       <c r="I566" t="s">
-        <v>1576</v>
+        <v>1598</v>
       </c>
       <c r="J566" t="s">
         <v>2154</v>
       </c>
       <c r="K566" t="s">
-        <v>2245</v>
+        <v>2308</v>
       </c>
       <c r="L566" t="s">
-        <v>2374</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="567" spans="1:12">
       <c r="A567" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B567" t="s">
         <v>605</v>
@@ -27467,25 +27467,22 @@
         <v>9</v>
       </c>
       <c r="F567" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
       <c r="G567" t="s">
-        <v>1462</v>
-      </c>
-      <c r="H567" t="s">
-        <v>1484</v>
+        <v>1461</v>
       </c>
       <c r="I567" t="s">
-        <v>1598</v>
+        <v>1492</v>
       </c>
       <c r="J567" t="s">
         <v>2155</v>
       </c>
       <c r="K567" t="s">
-        <v>2308</v>
+        <v>2212</v>
       </c>
       <c r="L567" t="s">
-        <v>2347</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="568" spans="1:12">
@@ -27493,10 +27490,10 @@
         <v>12</v>
       </c>
       <c r="B568" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="C568" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="D568" t="s">
         <v>1448</v>
@@ -27505,7 +27502,7 @@
         <v>9</v>
       </c>
       <c r="F568" t="s">
-        <v>1457</v>
+        <v>1458</v>
       </c>
       <c r="G568" t="s">
         <v>1461</v>
@@ -27514,7 +27511,7 @@
         <v>1492</v>
       </c>
       <c r="J568" t="s">
-        <v>2156</v>
+        <v>2155</v>
       </c>
       <c r="K568" t="s">
         <v>2212</v>
@@ -27525,7 +27522,7 @@
     </row>
     <row r="569" spans="1:12">
       <c r="A569" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="B569" t="s">
         <v>606</v>
@@ -27540,13 +27537,13 @@
         <v>9</v>
       </c>
       <c r="F569" t="s">
-        <v>1458</v>
+        <v>1456</v>
       </c>
       <c r="G569" t="s">
         <v>1461</v>
       </c>
       <c r="I569" t="s">
-        <v>1492</v>
+        <v>1576</v>
       </c>
       <c r="J569" t="s">
         <v>2156</v>
@@ -27555,7 +27552,7 @@
         <v>2212</v>
       </c>
       <c r="L569" t="s">
-        <v>2313</v>
+        <v>2392</v>
       </c>
     </row>
     <row r="570" spans="1:12">
@@ -27590,7 +27587,7 @@
         <v>2212</v>
       </c>
       <c r="L570" t="s">
-        <v>2392</v>
+        <v>2319</v>
       </c>
     </row>
     <row r="571" spans="1:12">
@@ -27616,16 +27613,16 @@
         <v>1461</v>
       </c>
       <c r="I571" t="s">
-        <v>1576</v>
+        <v>1565</v>
       </c>
       <c r="J571" t="s">
         <v>2158</v>
       </c>
       <c r="K571" t="s">
-        <v>2212</v>
+        <v>2227</v>
       </c>
       <c r="L571" t="s">
-        <v>2319</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="572" spans="1:12">
@@ -27651,7 +27648,7 @@
         <v>1461</v>
       </c>
       <c r="I572" t="s">
-        <v>1565</v>
+        <v>1553</v>
       </c>
       <c r="J572" t="s">
         <v>2159</v>
@@ -27660,7 +27657,7 @@
         <v>2227</v>
       </c>
       <c r="L572" t="s">
-        <v>2316</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="573" spans="1:12">
@@ -27686,7 +27683,7 @@
         <v>1461</v>
       </c>
       <c r="I573" t="s">
-        <v>1553</v>
+        <v>1565</v>
       </c>
       <c r="J573" t="s">
         <v>2160</v>
@@ -27695,12 +27692,12 @@
         <v>2227</v>
       </c>
       <c r="L573" t="s">
-        <v>2347</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="574" spans="1:12">
       <c r="A574" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B574" t="s">
         <v>611</v>
@@ -27721,7 +27718,7 @@
         <v>1461</v>
       </c>
       <c r="I574" t="s">
-        <v>1565</v>
+        <v>1599</v>
       </c>
       <c r="J574" t="s">
         <v>2161</v>
@@ -27730,12 +27727,12 @@
         <v>2227</v>
       </c>
       <c r="L574" t="s">
-        <v>2316</v>
+        <v>2373</v>
       </c>
     </row>
     <row r="575" spans="1:12">
       <c r="A575" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B575" t="s">
         <v>612</v>
@@ -27744,10 +27741,10 @@
         <v>1218</v>
       </c>
       <c r="D575" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="E575">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F575" t="s">
         <v>1456</v>
@@ -27756,21 +27753,21 @@
         <v>1461</v>
       </c>
       <c r="I575" t="s">
-        <v>1599</v>
+        <v>1568</v>
       </c>
       <c r="J575" t="s">
         <v>2162</v>
       </c>
       <c r="K575" t="s">
-        <v>2227</v>
+        <v>2263</v>
       </c>
       <c r="L575" t="s">
-        <v>2373</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="576" spans="1:12">
       <c r="A576" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B576" t="s">
         <v>613</v>
@@ -27791,13 +27788,13 @@
         <v>1461</v>
       </c>
       <c r="I576" t="s">
-        <v>1568</v>
+        <v>1590</v>
       </c>
       <c r="J576" t="s">
         <v>2163</v>
       </c>
       <c r="K576" t="s">
-        <v>2263</v>
+        <v>2229</v>
       </c>
       <c r="L576" t="s">
         <v>2374</v>
@@ -27805,7 +27802,7 @@
     </row>
     <row r="577" spans="1:12">
       <c r="A577" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B577" t="s">
         <v>614</v>
@@ -27826,16 +27823,16 @@
         <v>1461</v>
       </c>
       <c r="I577" t="s">
-        <v>1590</v>
+        <v>1576</v>
       </c>
       <c r="J577" t="s">
         <v>2164</v>
       </c>
       <c r="K577" t="s">
-        <v>2229</v>
+        <v>2296</v>
       </c>
       <c r="L577" t="s">
-        <v>2374</v>
+        <v>2369</v>
       </c>
     </row>
     <row r="578" spans="1:12">
@@ -27849,10 +27846,10 @@
         <v>1221</v>
       </c>
       <c r="D578" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
       <c r="E578">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F578" t="s">
         <v>1456</v>
@@ -27861,16 +27858,16 @@
         <v>1461</v>
       </c>
       <c r="I578" t="s">
-        <v>1576</v>
+        <v>1562</v>
       </c>
       <c r="J578" t="s">
         <v>2165</v>
       </c>
       <c r="K578" t="s">
-        <v>2296</v>
+        <v>2245</v>
       </c>
       <c r="L578" t="s">
-        <v>2369</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="579" spans="1:12">
@@ -27896,16 +27893,16 @@
         <v>1461</v>
       </c>
       <c r="I579" t="s">
-        <v>1562</v>
+        <v>1576</v>
       </c>
       <c r="J579" t="s">
-        <v>2166</v>
+        <v>2165</v>
       </c>
       <c r="K579" t="s">
         <v>2245</v>
       </c>
       <c r="L579" t="s">
-        <v>2313</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="580" spans="1:12">
@@ -27928,19 +27925,22 @@
         <v>1456</v>
       </c>
       <c r="G580" t="s">
-        <v>1461</v>
+        <v>1462</v>
+      </c>
+      <c r="H580" t="s">
+        <v>1483</v>
       </c>
       <c r="I580" t="s">
-        <v>1576</v>
+        <v>1541</v>
       </c>
       <c r="J580" t="s">
         <v>2166</v>
       </c>
       <c r="K580" t="s">
-        <v>2245</v>
+        <v>2215</v>
       </c>
       <c r="L580" t="s">
-        <v>2374</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="581" spans="1:12">
@@ -27963,19 +27963,16 @@
         <v>1456</v>
       </c>
       <c r="G581" t="s">
-        <v>1462</v>
-      </c>
-      <c r="H581" t="s">
-        <v>1484</v>
+        <v>1461</v>
       </c>
       <c r="I581" t="s">
-        <v>1541</v>
+        <v>1553</v>
       </c>
       <c r="J581" t="s">
         <v>2167</v>
       </c>
       <c r="K581" t="s">
-        <v>2215</v>
+        <v>2272</v>
       </c>
       <c r="L581" t="s">
         <v>2313</v>
@@ -27983,7 +27980,7 @@
     </row>
     <row r="582" spans="1:12">
       <c r="A582" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="B582" t="s">
         <v>619</v>
@@ -27992,33 +27989,36 @@
         <v>1225</v>
       </c>
       <c r="D582" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
       <c r="E582">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F582" t="s">
-        <v>1456</v>
+        <v>1458</v>
       </c>
       <c r="G582" t="s">
-        <v>1461</v>
+        <v>1462</v>
+      </c>
+      <c r="H582" t="s">
+        <v>1484</v>
       </c>
       <c r="I582" t="s">
-        <v>1553</v>
+        <v>1556</v>
       </c>
       <c r="J582" t="s">
         <v>2168</v>
       </c>
       <c r="K582" t="s">
-        <v>2272</v>
+        <v>2221</v>
       </c>
       <c r="L582" t="s">
-        <v>2313</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="583" spans="1:12">
       <c r="A583" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="B583" t="s">
         <v>620</v>
@@ -28033,22 +28033,19 @@
         <v>6</v>
       </c>
       <c r="F583" t="s">
-        <v>1458</v>
+        <v>1456</v>
       </c>
       <c r="G583" t="s">
-        <v>1462</v>
-      </c>
-      <c r="H583" t="s">
-        <v>1485</v>
+        <v>1461</v>
       </c>
       <c r="I583" t="s">
-        <v>1556</v>
+        <v>1565</v>
       </c>
       <c r="J583" t="s">
         <v>2169</v>
       </c>
       <c r="K583" t="s">
-        <v>2221</v>
+        <v>2215</v>
       </c>
       <c r="L583" t="s">
         <v>2347</v>
@@ -28056,7 +28053,7 @@
     </row>
     <row r="584" spans="1:12">
       <c r="A584" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B584" t="s">
         <v>621</v>
@@ -28077,21 +28074,21 @@
         <v>1461</v>
       </c>
       <c r="I584" t="s">
-        <v>1565</v>
+        <v>1590</v>
       </c>
       <c r="J584" t="s">
         <v>2170</v>
       </c>
       <c r="K584" t="s">
-        <v>2215</v>
+        <v>2228</v>
       </c>
       <c r="L584" t="s">
-        <v>2347</v>
+        <v>2335</v>
       </c>
     </row>
     <row r="585" spans="1:12">
       <c r="A585" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B585" t="s">
         <v>622</v>
@@ -28112,16 +28109,16 @@
         <v>1461</v>
       </c>
       <c r="I585" t="s">
-        <v>1590</v>
+        <v>1565</v>
       </c>
       <c r="J585" t="s">
         <v>2171</v>
       </c>
       <c r="K585" t="s">
-        <v>2228</v>
+        <v>2199</v>
       </c>
       <c r="L585" t="s">
-        <v>2335</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="586" spans="1:12">
@@ -28147,16 +28144,16 @@
         <v>1461</v>
       </c>
       <c r="I586" t="s">
-        <v>1565</v>
+        <v>1576</v>
       </c>
       <c r="J586" t="s">
         <v>2172</v>
       </c>
       <c r="K586" t="s">
-        <v>2199</v>
+        <v>2244</v>
       </c>
       <c r="L586" t="s">
-        <v>2347</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="587" spans="1:12">
@@ -28170,10 +28167,10 @@
         <v>1230</v>
       </c>
       <c r="D587" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
       <c r="E587">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F587" t="s">
         <v>1456</v>
@@ -28182,21 +28179,21 @@
         <v>1461</v>
       </c>
       <c r="I587" t="s">
-        <v>1576</v>
+        <v>1565</v>
       </c>
       <c r="J587" t="s">
         <v>2173</v>
       </c>
       <c r="K587" t="s">
-        <v>2244</v>
+        <v>2259</v>
       </c>
       <c r="L587" t="s">
-        <v>2374</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="588" spans="1:12">
       <c r="A588" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B588" t="s">
         <v>625</v>
@@ -28214,24 +28211,27 @@
         <v>1456</v>
       </c>
       <c r="G588" t="s">
-        <v>1461</v>
+        <v>1462</v>
+      </c>
+      <c r="H588" t="s">
+        <v>1485</v>
       </c>
       <c r="I588" t="s">
-        <v>1565</v>
+        <v>1600</v>
       </c>
       <c r="J588" t="s">
         <v>2174</v>
       </c>
       <c r="K588" t="s">
-        <v>2259</v>
+        <v>2253</v>
       </c>
       <c r="L588" t="s">
-        <v>2347</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="589" spans="1:12">
       <c r="A589" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B589" t="s">
         <v>626</v>
@@ -28249,27 +28249,24 @@
         <v>1456</v>
       </c>
       <c r="G589" t="s">
-        <v>1462</v>
-      </c>
-      <c r="H589" t="s">
-        <v>1486</v>
+        <v>1461</v>
       </c>
       <c r="I589" t="s">
-        <v>1600</v>
+        <v>1583</v>
       </c>
       <c r="J589" t="s">
         <v>2175</v>
       </c>
       <c r="K589" t="s">
-        <v>2253</v>
+        <v>2211</v>
       </c>
       <c r="L589" t="s">
-        <v>2360</v>
+        <v>2320</v>
       </c>
     </row>
     <row r="590" spans="1:12">
       <c r="A590" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="B590" t="s">
         <v>627</v>
@@ -28290,16 +28287,16 @@
         <v>1461</v>
       </c>
       <c r="I590" t="s">
-        <v>1583</v>
+        <v>1568</v>
       </c>
       <c r="J590" t="s">
         <v>2176</v>
       </c>
       <c r="K590" t="s">
-        <v>2211</v>
+        <v>2309</v>
       </c>
       <c r="L590" t="s">
-        <v>2320</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="591" spans="1:12">
@@ -28325,21 +28322,21 @@
         <v>1461</v>
       </c>
       <c r="I591" t="s">
-        <v>1568</v>
+        <v>1541</v>
       </c>
       <c r="J591" t="s">
         <v>2177</v>
       </c>
       <c r="K591" t="s">
-        <v>2309</v>
+        <v>2238</v>
       </c>
       <c r="L591" t="s">
-        <v>2347</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="592" spans="1:12">
       <c r="A592" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B592" t="s">
         <v>629</v>
@@ -28348,10 +28345,10 @@
         <v>1235</v>
       </c>
       <c r="D592" t="s">
-        <v>1452</v>
+        <v>1453</v>
       </c>
       <c r="E592">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F592" t="s">
         <v>1456</v>
@@ -28360,21 +28357,21 @@
         <v>1461</v>
       </c>
       <c r="I592" t="s">
-        <v>1541</v>
+        <v>1599</v>
       </c>
       <c r="J592" t="s">
         <v>2178</v>
       </c>
       <c r="K592" t="s">
-        <v>2238</v>
+        <v>2310</v>
       </c>
       <c r="L592" t="s">
-        <v>2313</v>
+        <v>2373</v>
       </c>
     </row>
     <row r="593" spans="1:12">
       <c r="A593" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B593" t="s">
         <v>630</v>
@@ -28395,21 +28392,21 @@
         <v>1461</v>
       </c>
       <c r="I593" t="s">
-        <v>1599</v>
+        <v>1553</v>
       </c>
       <c r="J593" t="s">
         <v>2179</v>
       </c>
       <c r="K593" t="s">
-        <v>2310</v>
+        <v>2309</v>
       </c>
       <c r="L593" t="s">
-        <v>2373</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="594" spans="1:12">
       <c r="A594" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B594" t="s">
         <v>631</v>
@@ -28418,10 +28415,10 @@
         <v>1237</v>
       </c>
       <c r="D594" t="s">
-        <v>1453</v>
+        <v>1454</v>
       </c>
       <c r="E594">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F594" t="s">
         <v>1456</v>
@@ -28430,16 +28427,16 @@
         <v>1461</v>
       </c>
       <c r="I594" t="s">
-        <v>1553</v>
+        <v>1571</v>
       </c>
       <c r="J594" t="s">
         <v>2180</v>
       </c>
       <c r="K594" t="s">
-        <v>2309</v>
+        <v>2208</v>
       </c>
       <c r="L594" t="s">
-        <v>2313</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -28465,13 +28462,13 @@
         <v>1461</v>
       </c>
       <c r="I595" t="s">
-        <v>1571</v>
+        <v>1599</v>
       </c>
       <c r="J595" t="s">
         <v>2181</v>
       </c>
       <c r="K595" t="s">
-        <v>2208</v>
+        <v>2305</v>
       </c>
       <c r="L595" t="s">
         <v>2374</v>
@@ -28500,13 +28497,13 @@
         <v>1461</v>
       </c>
       <c r="I596" t="s">
-        <v>1599</v>
+        <v>1590</v>
       </c>
       <c r="J596" t="s">
         <v>2182</v>
       </c>
       <c r="K596" t="s">
-        <v>2305</v>
+        <v>2311</v>
       </c>
       <c r="L596" t="s">
         <v>2374</v>
@@ -28514,7 +28511,7 @@
     </row>
     <row r="597" spans="1:12">
       <c r="A597" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B597" t="s">
         <v>634</v>
@@ -28535,21 +28532,21 @@
         <v>1461</v>
       </c>
       <c r="I597" t="s">
-        <v>1590</v>
+        <v>1568</v>
       </c>
       <c r="J597" t="s">
         <v>2183</v>
       </c>
       <c r="K597" t="s">
-        <v>2311</v>
+        <v>2252</v>
       </c>
       <c r="L597" t="s">
-        <v>2374</v>
+        <v>2347</v>
       </c>
     </row>
     <row r="598" spans="1:12">
       <c r="A598" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B598" t="s">
         <v>635</v>
@@ -28570,21 +28567,21 @@
         <v>1461</v>
       </c>
       <c r="I598" t="s">
-        <v>1568</v>
+        <v>1599</v>
       </c>
       <c r="J598" t="s">
         <v>2184</v>
       </c>
       <c r="K598" t="s">
-        <v>2252</v>
+        <v>2282</v>
       </c>
       <c r="L598" t="s">
-        <v>2347</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B599" t="s">
         <v>636</v>
@@ -28605,21 +28602,21 @@
         <v>1461</v>
       </c>
       <c r="I599" t="s">
-        <v>1599</v>
+        <v>1541</v>
       </c>
       <c r="J599" t="s">
         <v>2185</v>
       </c>
       <c r="K599" t="s">
-        <v>2282</v>
+        <v>2264</v>
       </c>
       <c r="L599" t="s">
-        <v>2374</v>
+        <v>2313</v>
       </c>
     </row>
     <row r="600" spans="1:12">
       <c r="A600" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="B600" t="s">
         <v>637</v>
@@ -28640,21 +28637,21 @@
         <v>1461</v>
       </c>
       <c r="I600" t="s">
-        <v>1541</v>
+        <v>1492</v>
       </c>
       <c r="J600" t="s">
         <v>2186</v>
       </c>
       <c r="K600" t="s">
-        <v>2264</v>
+        <v>2211</v>
       </c>
       <c r="L600" t="s">
-        <v>2313</v>
+        <v>2320</v>
       </c>
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="B601" t="s">
         <v>638</v>
@@ -28663,16 +28660,19 @@
         <v>1244</v>
       </c>
       <c r="D601" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
       <c r="E601">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F601" t="s">
         <v>1456</v>
       </c>
       <c r="G601" t="s">
-        <v>1461</v>
+        <v>1462</v>
+      </c>
+      <c r="H601" t="s">
+        <v>1486</v>
       </c>
       <c r="I601" t="s">
         <v>1492</v>
@@ -28681,10 +28681,10 @@
         <v>2187</v>
       </c>
       <c r="K601" t="s">
-        <v>2211</v>
+        <v>2230</v>
       </c>
       <c r="L601" t="s">
-        <v>2320</v>
+        <v>2374</v>
       </c>
     </row>
     <row r="602" spans="1:12">

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-15 22:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -27557,7 +27557,7 @@
     </row>
     <row r="567" spans="1:12">
       <c r="A567" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B567" t="s">
         <v>605</v>
@@ -27572,13 +27572,13 @@
         <v>10</v>
       </c>
       <c r="F567" t="s">
-        <v>1482</v>
+        <v>1486</v>
       </c>
       <c r="G567" t="s">
         <v>1487</v>
       </c>
       <c r="I567" t="s">
-        <v>1600</v>
+        <v>1557</v>
       </c>
       <c r="J567" t="s">
         <v>2183</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-16 04:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4570,18 +4570,18 @@
     <t>_SEM USUARIO ATRIBUIDO</t>
   </si>
   <si>
+    <t>CARLA CARVALHO DE LIMA CARNEIRO,FERNANDA ZUCOLOTTO</t>
+  </si>
+  <si>
+    <t>JULIANA MARTINS BAHIENSE</t>
+  </si>
+  <si>
+    <t>EDNELSON SILVEIRA DA SILVA</t>
+  </si>
+  <si>
     <t>PEDRO DE OLIVEIRA PERES</t>
   </si>
   <si>
-    <t>CARLA CARVALHO DE LIMA CARNEIRO,FERNANDA ZUCOLOTTO</t>
-  </si>
-  <si>
-    <t>JULIANA MARTINS BAHIENSE</t>
-  </si>
-  <si>
-    <t>EDNELSON SILVEIRA DA SILVA</t>
-  </si>
-  <si>
     <t>IZABEL REGINA BENITE AGUIAR DA SILVA</t>
   </si>
   <si>
@@ -4789,10 +4789,10 @@
     <t>FERNANDA TEIXEIRA ROSALBA</t>
   </si>
   <si>
+    <t>MARCIA PINHEIRO HENRIQUES SANDES</t>
+  </si>
+  <si>
     <t>CAROLINE OLIVEIRA DE MENEZES</t>
-  </si>
-  <si>
-    <t>MARCIA PINHEIRO HENRIQUES SANDES</t>
   </si>
   <si>
     <t>FERNANDA ZUCOLOTTO,MARINA DE AQUINO PARREIRA XAVIER</t>
@@ -8375,7 +8375,7 @@
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
         <v>62</v>
@@ -8396,7 +8396,7 @@
         <v>1487</v>
       </c>
       <c r="I21" t="s">
-        <v>1518</v>
+        <v>1517</v>
       </c>
       <c r="J21" t="s">
         <v>1648</v>
@@ -8431,7 +8431,7 @@
         <v>1487</v>
       </c>
       <c r="I22" t="s">
-        <v>1519</v>
+        <v>1518</v>
       </c>
       <c r="J22" t="s">
         <v>1649</v>
@@ -8466,7 +8466,7 @@
         <v>1487</v>
       </c>
       <c r="I23" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="J23" t="s">
         <v>1650</v>
@@ -8501,7 +8501,7 @@
         <v>1487</v>
       </c>
       <c r="I24" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="J24" t="s">
         <v>1651</v>
@@ -8536,7 +8536,7 @@
         <v>1487</v>
       </c>
       <c r="I25" t="s">
-        <v>1519</v>
+        <v>1518</v>
       </c>
       <c r="J25" t="s">
         <v>1652</v>
@@ -8606,7 +8606,7 @@
         <v>1487</v>
       </c>
       <c r="I27" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="J27" t="s">
         <v>1654</v>
@@ -8711,7 +8711,7 @@
         <v>1487</v>
       </c>
       <c r="I30" t="s">
-        <v>1518</v>
+        <v>1521</v>
       </c>
       <c r="J30" t="s">
         <v>1657</v>
@@ -8816,7 +8816,7 @@
         <v>1487</v>
       </c>
       <c r="I33" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="J33" t="s">
         <v>1660</v>
@@ -9026,7 +9026,7 @@
         <v>1487</v>
       </c>
       <c r="I39" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="J39" t="s">
         <v>1666</v>
@@ -9096,7 +9096,7 @@
         <v>1487</v>
       </c>
       <c r="I41" t="s">
-        <v>1518</v>
+        <v>1521</v>
       </c>
       <c r="J41" t="s">
         <v>1668</v>
@@ -9236,7 +9236,7 @@
         <v>1487</v>
       </c>
       <c r="I45" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="J45" t="s">
         <v>1672</v>
@@ -9411,7 +9411,7 @@
         <v>1487</v>
       </c>
       <c r="I50" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="J50" t="s">
         <v>1677</v>
@@ -9761,7 +9761,7 @@
         <v>1487</v>
       </c>
       <c r="I60" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="J60" t="s">
         <v>1687</v>
@@ -9936,7 +9936,7 @@
         <v>1487</v>
       </c>
       <c r="I65" t="s">
-        <v>1521</v>
+        <v>1520</v>
       </c>
       <c r="J65" t="s">
         <v>1692</v>
@@ -10636,7 +10636,7 @@
         <v>1487</v>
       </c>
       <c r="I85" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="J85" t="s">
         <v>1712</v>
@@ -10881,7 +10881,7 @@
         <v>1487</v>
       </c>
       <c r="I92" t="s">
-        <v>1518</v>
+        <v>1521</v>
       </c>
       <c r="J92" t="s">
         <v>1719</v>
@@ -10951,7 +10951,7 @@
         <v>1487</v>
       </c>
       <c r="I94" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="J94" t="s">
         <v>1721</v>
@@ -12246,7 +12246,7 @@
         <v>1487</v>
       </c>
       <c r="I131" t="s">
-        <v>1518</v>
+        <v>1521</v>
       </c>
       <c r="J131" t="s">
         <v>1758</v>
@@ -16434,7 +16434,7 @@
     </row>
     <row r="251" spans="1:12">
       <c r="A251" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="B251" t="s">
         <v>292</v>
@@ -16455,7 +16455,7 @@
         <v>1487</v>
       </c>
       <c r="I251" t="s">
-        <v>1591</v>
+        <v>1513</v>
       </c>
       <c r="J251" t="s">
         <v>1878</v>
@@ -16490,7 +16490,7 @@
         <v>1487</v>
       </c>
       <c r="I252" t="s">
-        <v>1592</v>
+        <v>1591</v>
       </c>
       <c r="J252" t="s">
         <v>1879</v>
@@ -16595,7 +16595,7 @@
         <v>1487</v>
       </c>
       <c r="I255" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J255" t="s">
         <v>1882</v>
@@ -19156,7 +19156,7 @@
         <v>1487</v>
       </c>
       <c r="I328" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J328" t="s">
         <v>1954</v>
@@ -19401,7 +19401,7 @@
         <v>1487</v>
       </c>
       <c r="I335" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J335" t="s">
         <v>1961</v>
@@ -20346,7 +20346,7 @@
         <v>1487</v>
       </c>
       <c r="I362" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J362" t="s">
         <v>1988</v>
@@ -20381,7 +20381,7 @@
         <v>1487</v>
       </c>
       <c r="I363" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J363" t="s">
         <v>1988</v>
@@ -21017,7 +21017,7 @@
         <v>1487</v>
       </c>
       <c r="I381" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J381" t="s">
         <v>2004</v>
@@ -22840,7 +22840,7 @@
         <v>1487</v>
       </c>
       <c r="I433" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J433" t="s">
         <v>2055</v>
@@ -25060,7 +25060,7 @@
         <v>1499</v>
       </c>
       <c r="I496" t="s">
-        <v>1520</v>
+        <v>1519</v>
       </c>
       <c r="J496" t="s">
         <v>2115</v>
@@ -25165,7 +25165,7 @@
         <v>1487</v>
       </c>
       <c r="I499" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J499" t="s">
         <v>2118</v>
@@ -25588,7 +25588,7 @@
         <v>1487</v>
       </c>
       <c r="I511" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J511" t="s">
         <v>2129</v>
@@ -25798,7 +25798,7 @@
         <v>1487</v>
       </c>
       <c r="I517" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J517" t="s">
         <v>2135</v>
@@ -25833,7 +25833,7 @@
         <v>1487</v>
       </c>
       <c r="I518" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J518" t="s">
         <v>2136</v>
@@ -25973,7 +25973,7 @@
         <v>1487</v>
       </c>
       <c r="I522" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J522" t="s">
         <v>2140</v>
@@ -26259,7 +26259,7 @@
         <v>1487</v>
       </c>
       <c r="I530" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J530" t="s">
         <v>2147</v>
@@ -26720,7 +26720,7 @@
         <v>1487</v>
       </c>
       <c r="I543" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J543" t="s">
         <v>2160</v>
@@ -27823,7 +27823,7 @@
         <v>1487</v>
       </c>
       <c r="I574" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J574" t="s">
         <v>2190</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-19 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14123,7 +14123,7 @@
     </row>
     <row r="183" spans="1:12">
       <c r="A183" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="B183" t="s">
         <v>226</v>
@@ -14144,7 +14144,7 @@
         <v>1501</v>
       </c>
       <c r="I183" t="s">
-        <v>1595</v>
+        <v>1528</v>
       </c>
       <c r="J183" t="s">
         <v>1833</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-20 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6423" uniqueCount="2487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6423" uniqueCount="2483">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7312,7 +7312,7 @@
     <t>BIOLOGIA,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>RECURSOS HÍDRICOS,ENGENHARIA QUÍMICA</t>
+    <t>ENGENHARIA QUÍMICA,RECURSOS HÍDRICOS</t>
   </si>
   <si>
     <t>BIOLOGIA,GEOLOGIA,URBANISMO</t>
@@ -7363,9 +7363,6 @@
     <t>BIOLOGIA,ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
   </si>
   <si>
-    <t>ENGENHARIA QUÍMICA,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
     <t>ENGENHARIA CIVIL,GEOTECNIA</t>
   </si>
   <si>
@@ -7417,7 +7414,7 @@
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
-    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
   </si>
   <si>
     <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
@@ -7444,37 +7441,28 @@
     <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS,URBANISMO,BIOLOGIA</t>
+    <t>BIOLOGIA,RECURSOS HÍDRICOS,MOBILIDADE E TRANSPORTE,URBANISMO</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
-    <t>ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL</t>
+    <t>MOBILIDADE E TRANSPORTE,ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
     <t>URBANISMO,ENGENHARIA FLORESTAL</t>
   </si>
   <si>
-    <t>ECONOMIA,ECONOMICIDADE CONTÁBIL</t>
-  </si>
-  <si>
-    <t>RECURSOS HÍDRICOS,ECONOMICIDADE OBRAS</t>
+    <t>ECONOMICIDADE CONTÁBIL,ECONOMIA</t>
   </si>
   <si>
     <t>URBANISMO,RECURSOS HÍDRICOS</t>
   </si>
   <si>
-    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMIA,AVALIAÇÃO DE IMÓVEIS,ASSISTÊNCIA SOCIAL,URBANISMO,SAÚDE MENTAL,PSICOLOGIA,MOBILIDADE E TRANSPORTE,SAÚDE,ORÇAMENTO</t>
+    <t>SAÚDE,ORÇAMENTO,ASSISTÊNCIA SOCIAL,AVALIAÇÃO DE IMÓVEIS,URBANISMO,SAÚDE MENTAL,PSICOLOGIA,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,ECONOMIA</t>
   </si>
 </sst>
 </file>
@@ -13651,7 +13639,7 @@
         <v>2330</v>
       </c>
       <c r="L166" t="s">
-        <v>2449</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="167" spans="1:12">
@@ -14529,7 +14517,7 @@
         <v>2318</v>
       </c>
       <c r="L191" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="192" spans="1:12">
@@ -14739,7 +14727,7 @@
         <v>2334</v>
       </c>
       <c r="L197" t="s">
-        <v>2451</v>
+        <v>2450</v>
       </c>
     </row>
     <row r="198" spans="1:12">
@@ -15019,7 +15007,7 @@
         <v>2318</v>
       </c>
       <c r="L205" t="s">
-        <v>2452</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="206" spans="1:12">
@@ -15054,7 +15042,7 @@
         <v>2317</v>
       </c>
       <c r="L206" t="s">
-        <v>2453</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="207" spans="1:12">
@@ -15194,7 +15182,7 @@
         <v>2326</v>
       </c>
       <c r="L210" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="211" spans="1:12">
@@ -15474,7 +15462,7 @@
         <v>2354</v>
       </c>
       <c r="L218" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="219" spans="1:12">
@@ -15509,7 +15497,7 @@
         <v>2330</v>
       </c>
       <c r="L219" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
     </row>
     <row r="220" spans="1:12">
@@ -15792,7 +15780,7 @@
         <v>2330</v>
       </c>
       <c r="L227" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="228" spans="1:12">
@@ -15897,7 +15885,7 @@
         <v>2311</v>
       </c>
       <c r="L230" t="s">
-        <v>2457</v>
+        <v>2456</v>
       </c>
     </row>
     <row r="231" spans="1:12">
@@ -16142,7 +16130,7 @@
         <v>2304</v>
       </c>
       <c r="L237" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="238" spans="1:12">
@@ -16177,7 +16165,7 @@
         <v>2298</v>
       </c>
       <c r="L238" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="239" spans="1:12">
@@ -16877,7 +16865,7 @@
         <v>2308</v>
       </c>
       <c r="L258" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="259" spans="1:12">
@@ -16912,7 +16900,7 @@
         <v>2311</v>
       </c>
       <c r="L259" t="s">
-        <v>2460</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="260" spans="1:12">
@@ -17017,7 +17005,7 @@
         <v>2296</v>
       </c>
       <c r="L262" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="263" spans="1:12">
@@ -17297,7 +17285,7 @@
         <v>2359</v>
       </c>
       <c r="L270" t="s">
-        <v>2462</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="271" spans="1:12">
@@ -17717,7 +17705,7 @@
         <v>2340</v>
       </c>
       <c r="L282" t="s">
-        <v>2463</v>
+        <v>2462</v>
       </c>
     </row>
     <row r="283" spans="1:12">
@@ -17822,7 +17810,7 @@
         <v>2328</v>
       </c>
       <c r="L285" t="s">
-        <v>2464</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="286" spans="1:12">
@@ -18105,7 +18093,7 @@
         <v>2311</v>
       </c>
       <c r="L293" t="s">
-        <v>2460</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="294" spans="1:12">
@@ -18175,7 +18163,7 @@
         <v>2367</v>
       </c>
       <c r="L295" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="296" spans="1:12">
@@ -18350,7 +18338,7 @@
         <v>2368</v>
       </c>
       <c r="L300" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="301" spans="1:12">
@@ -18385,7 +18373,7 @@
         <v>2368</v>
       </c>
       <c r="L301" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="302" spans="1:12">
@@ -19368,7 +19356,7 @@
         <v>2334</v>
       </c>
       <c r="L329" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="330" spans="1:12">
@@ -19403,7 +19391,7 @@
         <v>2370</v>
       </c>
       <c r="L330" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="331" spans="1:12">
@@ -19438,7 +19426,7 @@
         <v>2370</v>
       </c>
       <c r="L331" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="332" spans="1:12">
@@ -19473,7 +19461,7 @@
         <v>2370</v>
       </c>
       <c r="L332" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="333" spans="1:12">
@@ -19508,7 +19496,7 @@
         <v>2370</v>
       </c>
       <c r="L333" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="334" spans="1:12">
@@ -19543,7 +19531,7 @@
         <v>2370</v>
       </c>
       <c r="L334" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="335" spans="1:12">
@@ -19578,7 +19566,7 @@
         <v>2370</v>
       </c>
       <c r="L335" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="336" spans="1:12">
@@ -19613,7 +19601,7 @@
         <v>2370</v>
       </c>
       <c r="L336" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="337" spans="1:12">
@@ -19648,7 +19636,7 @@
         <v>2370</v>
       </c>
       <c r="L337" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="338" spans="1:12">
@@ -19683,7 +19671,7 @@
         <v>2370</v>
       </c>
       <c r="L338" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="339" spans="1:12">
@@ -19718,7 +19706,7 @@
         <v>2370</v>
       </c>
       <c r="L339" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="340" spans="1:12">
@@ -19753,7 +19741,7 @@
         <v>2370</v>
       </c>
       <c r="L340" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="341" spans="1:12">
@@ -19788,7 +19776,7 @@
         <v>2370</v>
       </c>
       <c r="L341" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="342" spans="1:12">
@@ -19823,7 +19811,7 @@
         <v>2370</v>
       </c>
       <c r="L342" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="343" spans="1:12">
@@ -19858,7 +19846,7 @@
         <v>2370</v>
       </c>
       <c r="L343" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="344" spans="1:12">
@@ -19893,7 +19881,7 @@
         <v>2370</v>
       </c>
       <c r="L344" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="345" spans="1:12">
@@ -19928,7 +19916,7 @@
         <v>2370</v>
       </c>
       <c r="L345" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="346" spans="1:12">
@@ -19963,7 +19951,7 @@
         <v>2370</v>
       </c>
       <c r="L346" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="347" spans="1:12">
@@ -19998,7 +19986,7 @@
         <v>2370</v>
       </c>
       <c r="L347" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="348" spans="1:12">
@@ -20068,7 +20056,7 @@
         <v>2371</v>
       </c>
       <c r="L349" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="350" spans="1:12">
@@ -20173,7 +20161,7 @@
         <v>2360</v>
       </c>
       <c r="L352" t="s">
-        <v>2467</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="353" spans="1:12">
@@ -20529,7 +20517,7 @@
         <v>2295</v>
       </c>
       <c r="L362" t="s">
-        <v>2468</v>
+        <v>2467</v>
       </c>
     </row>
     <row r="363" spans="1:12">
@@ -20564,7 +20552,7 @@
         <v>2334</v>
       </c>
       <c r="L363" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="364" spans="1:12">
@@ -20599,7 +20587,7 @@
         <v>2374</v>
       </c>
       <c r="L364" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="365" spans="1:12">
@@ -20844,7 +20832,7 @@
         <v>2375</v>
       </c>
       <c r="L371" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="372" spans="1:12">
@@ -21054,7 +21042,7 @@
         <v>2353</v>
       </c>
       <c r="L377" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="378" spans="1:12">
@@ -21089,7 +21077,7 @@
         <v>2309</v>
       </c>
       <c r="L378" t="s">
-        <v>2452</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="379" spans="1:12">
@@ -21194,7 +21182,7 @@
         <v>2376</v>
       </c>
       <c r="L381" t="s">
-        <v>2470</v>
+        <v>2469</v>
       </c>
     </row>
     <row r="382" spans="1:12">
@@ -21229,7 +21217,7 @@
         <v>2290</v>
       </c>
       <c r="L382" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="383" spans="1:12">
@@ -21299,7 +21287,7 @@
         <v>2377</v>
       </c>
       <c r="L384" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="385" spans="1:12">
@@ -21439,7 +21427,7 @@
         <v>2378</v>
       </c>
       <c r="L388" t="s">
-        <v>2471</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="389" spans="1:12">
@@ -21754,7 +21742,7 @@
         <v>2307</v>
       </c>
       <c r="L397" t="s">
-        <v>2472</v>
+        <v>2471</v>
       </c>
     </row>
     <row r="398" spans="1:12">
@@ -21789,7 +21777,7 @@
         <v>2310</v>
       </c>
       <c r="L398" t="s">
-        <v>2473</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="399" spans="1:12">
@@ -22104,7 +22092,7 @@
         <v>2320</v>
       </c>
       <c r="L407" t="s">
-        <v>2474</v>
+        <v>2473</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -22282,7 +22270,7 @@
         <v>2343</v>
       </c>
       <c r="L412" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="413" spans="1:12">
@@ -22317,7 +22305,7 @@
         <v>2340</v>
       </c>
       <c r="L413" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="414" spans="1:12">
@@ -22562,7 +22550,7 @@
         <v>2309</v>
       </c>
       <c r="L420" t="s">
-        <v>2475</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="421" spans="1:12">
@@ -22632,7 +22620,7 @@
         <v>2314</v>
       </c>
       <c r="L422" t="s">
-        <v>2476</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="423" spans="1:12">
@@ -22807,7 +22795,7 @@
         <v>2326</v>
       </c>
       <c r="L427" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="428" spans="1:12">
@@ -22947,7 +22935,7 @@
         <v>2374</v>
       </c>
       <c r="L431" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="432" spans="1:12">
@@ -23122,7 +23110,7 @@
         <v>2330</v>
       </c>
       <c r="L436" t="s">
-        <v>2473</v>
+        <v>2472</v>
       </c>
     </row>
     <row r="437" spans="1:12">
@@ -23437,7 +23425,7 @@
         <v>2316</v>
       </c>
       <c r="L445" t="s">
-        <v>2477</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="446" spans="1:12">
@@ -23822,7 +23810,7 @@
         <v>2330</v>
       </c>
       <c r="L456" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="457" spans="1:12">
@@ -24175,7 +24163,7 @@
         <v>2386</v>
       </c>
       <c r="L466" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="467" spans="1:12">
@@ -24210,7 +24198,7 @@
         <v>2311</v>
       </c>
       <c r="L467" t="s">
-        <v>2475</v>
+        <v>2474</v>
       </c>
     </row>
     <row r="468" spans="1:12">
@@ -24280,7 +24268,7 @@
         <v>2387</v>
       </c>
       <c r="L469" t="s">
-        <v>2478</v>
+        <v>2476</v>
       </c>
     </row>
     <row r="470" spans="1:12">
@@ -24315,7 +24303,7 @@
         <v>2322</v>
       </c>
       <c r="L470" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="471" spans="1:12">
@@ -24458,7 +24446,7 @@
         <v>2389</v>
       </c>
       <c r="L474" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="475" spans="1:12">
@@ -25447,7 +25435,7 @@
         <v>2324</v>
       </c>
       <c r="L502" t="s">
-        <v>2479</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="503" spans="1:12">
@@ -25657,7 +25645,7 @@
         <v>2390</v>
       </c>
       <c r="L508" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="509" spans="1:12">
@@ -25692,7 +25680,7 @@
         <v>2391</v>
       </c>
       <c r="L509" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="510" spans="1:12">
@@ -25765,7 +25753,7 @@
         <v>2324</v>
       </c>
       <c r="L511" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="512" spans="1:12">
@@ -25905,7 +25893,7 @@
         <v>2336</v>
       </c>
       <c r="L515" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="516" spans="1:12">
@@ -25940,7 +25928,7 @@
         <v>2314</v>
       </c>
       <c r="L516" t="s">
-        <v>2480</v>
+        <v>2478</v>
       </c>
     </row>
     <row r="517" spans="1:12">
@@ -26083,7 +26071,7 @@
         <v>2308</v>
       </c>
       <c r="L520" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="521" spans="1:12">
@@ -26261,7 +26249,7 @@
         <v>2392</v>
       </c>
       <c r="L525" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="526" spans="1:12">
@@ -26404,7 +26392,7 @@
         <v>2329</v>
       </c>
       <c r="L529" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="530" spans="1:12">
@@ -26439,7 +26427,7 @@
         <v>2329</v>
       </c>
       <c r="L530" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="531" spans="1:12">
@@ -26474,7 +26462,7 @@
         <v>2322</v>
       </c>
       <c r="L531" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="532" spans="1:12">
@@ -26614,7 +26602,7 @@
         <v>2382</v>
       </c>
       <c r="L535" t="s">
-        <v>2481</v>
+        <v>2479</v>
       </c>
     </row>
     <row r="536" spans="1:12">
@@ -27011,7 +26999,7 @@
         <v>2298</v>
       </c>
       <c r="L546" t="s">
-        <v>2449</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="547" spans="1:12">
@@ -27186,7 +27174,7 @@
         <v>2313</v>
       </c>
       <c r="L551" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="552" spans="1:12">
@@ -27221,7 +27209,7 @@
         <v>2349</v>
       </c>
       <c r="L552" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="553" spans="1:12">
@@ -27256,7 +27244,7 @@
         <v>2315</v>
       </c>
       <c r="L553" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="554" spans="1:12">
@@ -27291,7 +27279,7 @@
         <v>2382</v>
       </c>
       <c r="L554" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
     </row>
     <row r="555" spans="1:12">
@@ -27361,7 +27349,7 @@
         <v>2331</v>
       </c>
       <c r="L556" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="557" spans="1:12">
@@ -27574,7 +27562,7 @@
         <v>2330</v>
       </c>
       <c r="L562" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="563" spans="1:12">
@@ -27647,7 +27635,7 @@
         <v>2339</v>
       </c>
       <c r="L564" t="s">
-        <v>2453</v>
+        <v>2452</v>
       </c>
     </row>
     <row r="565" spans="1:12">
@@ -27787,7 +27775,7 @@
         <v>2396</v>
       </c>
       <c r="L568" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="569" spans="1:12">
@@ -27857,7 +27845,7 @@
         <v>2294</v>
       </c>
       <c r="L570" t="s">
-        <v>2452</v>
+        <v>2451</v>
       </c>
     </row>
     <row r="571" spans="1:12">
@@ -27892,7 +27880,7 @@
         <v>2392</v>
       </c>
       <c r="L571" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="572" spans="1:12">
@@ -27962,7 +27950,7 @@
         <v>2367</v>
       </c>
       <c r="L573" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="574" spans="1:12">
@@ -28245,7 +28233,7 @@
         <v>2312</v>
       </c>
       <c r="L581" t="s">
-        <v>2482</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="582" spans="1:12">
@@ -28636,7 +28624,7 @@
         <v>2308</v>
       </c>
       <c r="L592" t="s">
-        <v>2455</v>
+        <v>2454</v>
       </c>
     </row>
     <row r="593" spans="1:12">
@@ -28671,7 +28659,7 @@
         <v>2311</v>
       </c>
       <c r="L593" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="594" spans="1:12">
@@ -28706,7 +28694,7 @@
         <v>2311</v>
       </c>
       <c r="L594" t="s">
-        <v>2483</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="595" spans="1:12">
@@ -28741,7 +28729,7 @@
         <v>2311</v>
       </c>
       <c r="L595" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="596" spans="1:12">
@@ -29027,7 +29015,7 @@
         <v>2306</v>
       </c>
       <c r="L603" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="604" spans="1:12">
@@ -29062,7 +29050,7 @@
         <v>2306</v>
       </c>
       <c r="L604" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="605" spans="1:12">
@@ -29167,7 +29155,7 @@
         <v>2297</v>
       </c>
       <c r="L607" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="608" spans="1:12">
@@ -29237,7 +29225,7 @@
         <v>2297</v>
       </c>
       <c r="L609" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="610" spans="1:12">
@@ -29345,7 +29333,7 @@
         <v>2284</v>
       </c>
       <c r="L612" t="s">
-        <v>2484</v>
+        <v>2481</v>
       </c>
     </row>
     <row r="613" spans="1:12">
@@ -29383,7 +29371,7 @@
         <v>2285</v>
       </c>
       <c r="L613" t="s">
-        <v>2466</v>
+        <v>2437</v>
       </c>
     </row>
     <row r="614" spans="1:12">
@@ -29526,7 +29514,7 @@
         <v>2400</v>
       </c>
       <c r="L617" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="618" spans="1:12">
@@ -29561,7 +29549,7 @@
         <v>2329</v>
       </c>
       <c r="L618" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="619" spans="1:12">
@@ -29596,7 +29584,7 @@
         <v>2329</v>
       </c>
       <c r="L619" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="620" spans="1:12">
@@ -29809,7 +29797,7 @@
         <v>2285</v>
       </c>
       <c r="L625" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="626" spans="1:12">
@@ -29879,7 +29867,7 @@
         <v>2285</v>
       </c>
       <c r="L627" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="628" spans="1:12">
@@ -29949,7 +29937,7 @@
         <v>2285</v>
       </c>
       <c r="L629" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="630" spans="1:12">
@@ -29984,7 +29972,7 @@
         <v>2330</v>
       </c>
       <c r="L630" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="631" spans="1:12">
@@ -30019,7 +30007,7 @@
         <v>2330</v>
       </c>
       <c r="L631" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="632" spans="1:12">
@@ -30054,7 +30042,7 @@
         <v>2296</v>
       </c>
       <c r="L632" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="633" spans="1:12">
@@ -30089,7 +30077,7 @@
         <v>2296</v>
       </c>
       <c r="L633" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
     </row>
     <row r="634" spans="1:12">
@@ -30229,7 +30217,7 @@
         <v>2303</v>
       </c>
       <c r="L637" t="s">
-        <v>2467</v>
+        <v>2466</v>
       </c>
     </row>
     <row r="638" spans="1:12">
@@ -30261,7 +30249,7 @@
         <v>2404</v>
       </c>
       <c r="L638" t="s">
-        <v>2485</v>
+        <v>2449</v>
       </c>
     </row>
     <row r="639" spans="1:12">
@@ -30293,7 +30281,7 @@
         <v>2404</v>
       </c>
       <c r="L639" t="s">
-        <v>2486</v>
+        <v>2482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-20 10:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4762,6 +4762,9 @@
     <t>IZABEL REGINA BENITE AGUIAR DA SILVA,VANESSA FERNANDES LEÃO</t>
   </si>
   <si>
+    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
+  </si>
+  <si>
     <t>LEONARDO ARAÚJO DE SOUZA,MOEMA BELLONI SCHMIDT,RANAILLA LIMA BANDEIRA DOS SANTOS</t>
   </si>
   <si>
@@ -4900,6 +4903,9 @@
     <t>FERNANDA ZUCOLOTTO,MARINA DE AQUINO PARREIRA XAVIER</t>
   </si>
   <si>
+    <t>JOELSON SANTANA DE CARVALHO</t>
+  </si>
+  <si>
     <t>FERNANDA TEIXEIRA ROSALBA</t>
   </si>
   <si>
@@ -4990,13 +4996,7 @@
     <t>IZABEL REGINA BENITE AGUIAR DA SILVA,THIAGO JOSÉ DUPRAT FORTES</t>
   </si>
   <si>
-    <t>ANDRÉA SILVA ARAUJO DE MELLO</t>
-  </si>
-  <si>
     <t>ERIKA CANTANHEDE WUILLAUME,MARCELO TEIXEIRA SANTANA</t>
-  </si>
-  <si>
-    <t>JOELSON SANTANA DE CARVALHO</t>
   </si>
   <si>
     <t>ALEXANDER MAGNO BORGES GOMES DA SILVA, PATRICIA FONTES ESTEVES</t>
@@ -11107,7 +11107,7 @@
         <v>1521</v>
       </c>
       <c r="I94" t="s">
-        <v>1551</v>
+        <v>1582</v>
       </c>
       <c r="J94" t="s">
         <v>1758</v>
@@ -11177,7 +11177,7 @@
         <v>1521</v>
       </c>
       <c r="I96" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="J96" t="s">
         <v>1760</v>
@@ -11317,7 +11317,7 @@
         <v>1521</v>
       </c>
       <c r="I100" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="J100" t="s">
         <v>1764</v>
@@ -11387,7 +11387,7 @@
         <v>1521</v>
       </c>
       <c r="I102" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
       <c r="J102" t="s">
         <v>1766</v>
@@ -11422,7 +11422,7 @@
         <v>1521</v>
       </c>
       <c r="I103" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J103" t="s">
         <v>1767</v>
@@ -11527,7 +11527,7 @@
         <v>1521</v>
       </c>
       <c r="I106" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="J106" t="s">
         <v>1770</v>
@@ -11667,7 +11667,7 @@
         <v>1521</v>
       </c>
       <c r="I110" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J110" t="s">
         <v>1774</v>
@@ -11737,7 +11737,7 @@
         <v>1521</v>
       </c>
       <c r="I112" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="J112" t="s">
         <v>1776</v>
@@ -11807,7 +11807,7 @@
         <v>1521</v>
       </c>
       <c r="I114" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
       <c r="J114" t="s">
         <v>1778</v>
@@ -11877,7 +11877,7 @@
         <v>1521</v>
       </c>
       <c r="I116" t="s">
-        <v>1590</v>
+        <v>1591</v>
       </c>
       <c r="J116" t="s">
         <v>1780</v>
@@ -11912,7 +11912,7 @@
         <v>1521</v>
       </c>
       <c r="I117" t="s">
-        <v>1591</v>
+        <v>1592</v>
       </c>
       <c r="J117" t="s">
         <v>1781</v>
@@ -11947,7 +11947,7 @@
         <v>1521</v>
       </c>
       <c r="I118" t="s">
-        <v>1592</v>
+        <v>1593</v>
       </c>
       <c r="J118" t="s">
         <v>1782</v>
@@ -12017,7 +12017,7 @@
         <v>1521</v>
       </c>
       <c r="I120" t="s">
-        <v>1593</v>
+        <v>1594</v>
       </c>
       <c r="J120" t="s">
         <v>1784</v>
@@ -12122,7 +12122,7 @@
         <v>1521</v>
       </c>
       <c r="I123" t="s">
-        <v>1594</v>
+        <v>1595</v>
       </c>
       <c r="J123" t="s">
         <v>1787</v>
@@ -12262,7 +12262,7 @@
         <v>1521</v>
       </c>
       <c r="I127" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
       <c r="J127" t="s">
         <v>1791</v>
@@ -12297,7 +12297,7 @@
         <v>1521</v>
       </c>
       <c r="I128" t="s">
-        <v>1596</v>
+        <v>1597</v>
       </c>
       <c r="J128" t="s">
         <v>1792</v>
@@ -12367,7 +12367,7 @@
         <v>1521</v>
       </c>
       <c r="I130" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J130" t="s">
         <v>1794</v>
@@ -12507,7 +12507,7 @@
         <v>1521</v>
       </c>
       <c r="I134" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
       <c r="J134" t="s">
         <v>1798</v>
@@ -12612,7 +12612,7 @@
         <v>1521</v>
       </c>
       <c r="I137" t="s">
-        <v>1599</v>
+        <v>1600</v>
       </c>
       <c r="J137" t="s">
         <v>1801</v>
@@ -12717,7 +12717,7 @@
         <v>1521</v>
       </c>
       <c r="I140" t="s">
-        <v>1600</v>
+        <v>1601</v>
       </c>
       <c r="J140" t="s">
         <v>1804</v>
@@ -12787,7 +12787,7 @@
         <v>1521</v>
       </c>
       <c r="I142" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="J142" t="s">
         <v>1806</v>
@@ -12892,7 +12892,7 @@
         <v>1521</v>
       </c>
       <c r="I145" t="s">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="J145" t="s">
         <v>1809</v>
@@ -12927,7 +12927,7 @@
         <v>1521</v>
       </c>
       <c r="I146" t="s">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="J146" t="s">
         <v>1810</v>
@@ -12997,7 +12997,7 @@
         <v>1521</v>
       </c>
       <c r="I148" t="s">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="J148" t="s">
         <v>1812</v>
@@ -13067,7 +13067,7 @@
         <v>1521</v>
       </c>
       <c r="I150" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J150" t="s">
         <v>1814</v>
@@ -13175,7 +13175,7 @@
         <v>1521</v>
       </c>
       <c r="I153" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
       <c r="J153" t="s">
         <v>1817</v>
@@ -13210,7 +13210,7 @@
         <v>1521</v>
       </c>
       <c r="I154" t="s">
-        <v>1607</v>
+        <v>1608</v>
       </c>
       <c r="J154" t="s">
         <v>1818</v>
@@ -13385,7 +13385,7 @@
         <v>1521</v>
       </c>
       <c r="I159" t="s">
-        <v>1597</v>
+        <v>1598</v>
       </c>
       <c r="J159" t="s">
         <v>1823</v>
@@ -13455,7 +13455,7 @@
         <v>1521</v>
       </c>
       <c r="I161" t="s">
-        <v>1608</v>
+        <v>1609</v>
       </c>
       <c r="J161" t="s">
         <v>1825</v>
@@ -13700,7 +13700,7 @@
         <v>1521</v>
       </c>
       <c r="I168" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
       <c r="J168" t="s">
         <v>1832</v>
@@ -13735,7 +13735,7 @@
         <v>1521</v>
       </c>
       <c r="I169" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
       <c r="J169" t="s">
         <v>1833</v>
@@ -13770,7 +13770,7 @@
         <v>1521</v>
       </c>
       <c r="I170" t="s">
-        <v>1611</v>
+        <v>1612</v>
       </c>
       <c r="J170" t="s">
         <v>1834</v>
@@ -13910,7 +13910,7 @@
         <v>1521</v>
       </c>
       <c r="I174" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J174" t="s">
         <v>1838</v>
@@ -13948,7 +13948,7 @@
         <v>1433</v>
       </c>
       <c r="I175" t="s">
-        <v>1613</v>
+        <v>1614</v>
       </c>
       <c r="J175" t="s">
         <v>1839</v>
@@ -13983,7 +13983,7 @@
         <v>1521</v>
       </c>
       <c r="I176" t="s">
-        <v>1614</v>
+        <v>1615</v>
       </c>
       <c r="J176" t="s">
         <v>1840</v>
@@ -14123,7 +14123,7 @@
         <v>1521</v>
       </c>
       <c r="I180" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
       <c r="J180" t="s">
         <v>1844</v>
@@ -14193,7 +14193,7 @@
         <v>1521</v>
       </c>
       <c r="I182" t="s">
-        <v>1615</v>
+        <v>1616</v>
       </c>
       <c r="J182" t="s">
         <v>1846</v>
@@ -14473,7 +14473,7 @@
         <v>1521</v>
       </c>
       <c r="I190" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
       <c r="J190" t="s">
         <v>1854</v>
@@ -14578,7 +14578,7 @@
         <v>1521</v>
       </c>
       <c r="I193" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J193" t="s">
         <v>1857</v>
@@ -14718,7 +14718,7 @@
         <v>1521</v>
       </c>
       <c r="I197" t="s">
-        <v>1616</v>
+        <v>1617</v>
       </c>
       <c r="J197" t="s">
         <v>1861</v>
@@ -14823,7 +14823,7 @@
         <v>1521</v>
       </c>
       <c r="I200" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J200" t="s">
         <v>1864</v>
@@ -14928,7 +14928,7 @@
         <v>1521</v>
       </c>
       <c r="I203" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J203" t="s">
         <v>1867</v>
@@ -15278,7 +15278,7 @@
         <v>1521</v>
       </c>
       <c r="I213" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
       <c r="J213" t="s">
         <v>1877</v>
@@ -15313,7 +15313,7 @@
         <v>1521</v>
       </c>
       <c r="I214" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J214" t="s">
         <v>1878</v>
@@ -15453,7 +15453,7 @@
         <v>1521</v>
       </c>
       <c r="I218" t="s">
-        <v>1619</v>
+        <v>1620</v>
       </c>
       <c r="J218" t="s">
         <v>1882</v>
@@ -15558,7 +15558,7 @@
         <v>1521</v>
       </c>
       <c r="I221" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="J221" t="s">
         <v>1885</v>
@@ -15593,7 +15593,7 @@
         <v>1521</v>
       </c>
       <c r="I222" t="s">
-        <v>1618</v>
+        <v>1619</v>
       </c>
       <c r="J222" t="s">
         <v>1886</v>
@@ -15663,7 +15663,7 @@
         <v>1521</v>
       </c>
       <c r="I224" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J224" t="s">
         <v>1888</v>
@@ -15701,7 +15701,7 @@
         <v>1525</v>
       </c>
       <c r="I225" t="s">
-        <v>1622</v>
+        <v>1623</v>
       </c>
       <c r="J225" t="s">
         <v>1889</v>
@@ -15736,7 +15736,7 @@
         <v>1521</v>
       </c>
       <c r="I226" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="J226" t="s">
         <v>1890</v>
@@ -15806,7 +15806,7 @@
         <v>1521</v>
       </c>
       <c r="I228" t="s">
-        <v>1623</v>
+        <v>1624</v>
       </c>
       <c r="J228" t="s">
         <v>1892</v>
@@ -15841,7 +15841,7 @@
         <v>1521</v>
       </c>
       <c r="I229" t="s">
-        <v>1620</v>
+        <v>1621</v>
       </c>
       <c r="J229" t="s">
         <v>1893</v>
@@ -16086,7 +16086,7 @@
         <v>1521</v>
       </c>
       <c r="I236" t="s">
-        <v>1624</v>
+        <v>1625</v>
       </c>
       <c r="J236" t="s">
         <v>1900</v>
@@ -16191,7 +16191,7 @@
         <v>1521</v>
       </c>
       <c r="I239" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="J239" t="s">
         <v>1903</v>
@@ -16226,7 +16226,7 @@
         <v>1521</v>
       </c>
       <c r="I240" t="s">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="J240" t="s">
         <v>1904</v>
@@ -16261,7 +16261,7 @@
         <v>1521</v>
       </c>
       <c r="I241" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J241" t="s">
         <v>1905</v>
@@ -16296,7 +16296,7 @@
         <v>1521</v>
       </c>
       <c r="I242" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J242" t="s">
         <v>1906</v>
@@ -16331,7 +16331,7 @@
         <v>1521</v>
       </c>
       <c r="I243" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J243" t="s">
         <v>1907</v>
@@ -16401,7 +16401,7 @@
         <v>1521</v>
       </c>
       <c r="I245" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J245" t="s">
         <v>1909</v>
@@ -16576,7 +16576,7 @@
         <v>1521</v>
       </c>
       <c r="I250" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J250" t="s">
         <v>1914</v>
@@ -16681,7 +16681,7 @@
         <v>1521</v>
       </c>
       <c r="I253" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J253" t="s">
         <v>1917</v>
@@ -16856,7 +16856,7 @@
         <v>1521</v>
       </c>
       <c r="I258" t="s">
-        <v>1627</v>
+        <v>1628</v>
       </c>
       <c r="J258" t="s">
         <v>1922</v>
@@ -16961,7 +16961,7 @@
         <v>1521</v>
       </c>
       <c r="I261" t="s">
-        <v>1595</v>
+        <v>1596</v>
       </c>
       <c r="J261" t="s">
         <v>1925</v>
@@ -17066,7 +17066,7 @@
         <v>1521</v>
       </c>
       <c r="I264" t="s">
-        <v>1551</v>
+        <v>1582</v>
       </c>
       <c r="J264" t="s">
         <v>1928</v>
@@ -17171,7 +17171,7 @@
         <v>1521</v>
       </c>
       <c r="I267" t="s">
-        <v>1551</v>
+        <v>1629</v>
       </c>
       <c r="J267" t="s">
         <v>1931</v>
@@ -17346,7 +17346,7 @@
         <v>1521</v>
       </c>
       <c r="I272" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J272" t="s">
         <v>1936</v>
@@ -17416,7 +17416,7 @@
         <v>1521</v>
       </c>
       <c r="I274" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J274" t="s">
         <v>1938</v>
@@ -17521,7 +17521,7 @@
         <v>1521</v>
       </c>
       <c r="I277" t="s">
-        <v>1628</v>
+        <v>1630</v>
       </c>
       <c r="J277" t="s">
         <v>1941</v>
@@ -17661,7 +17661,7 @@
         <v>1521</v>
       </c>
       <c r="I281" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J281" t="s">
         <v>1945</v>
@@ -17696,7 +17696,7 @@
         <v>1521</v>
       </c>
       <c r="I282" t="s">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="J282" t="s">
         <v>1946</v>
@@ -17766,7 +17766,7 @@
         <v>1521</v>
       </c>
       <c r="I284" t="s">
-        <v>1605</v>
+        <v>1606</v>
       </c>
       <c r="J284" t="s">
         <v>1948</v>
@@ -18049,7 +18049,7 @@
         <v>1521</v>
       </c>
       <c r="I292" t="s">
-        <v>1629</v>
+        <v>1631</v>
       </c>
       <c r="J292" t="s">
         <v>1956</v>
@@ -18329,7 +18329,7 @@
         <v>1521</v>
       </c>
       <c r="I300" t="s">
-        <v>1630</v>
+        <v>1632</v>
       </c>
       <c r="J300" t="s">
         <v>1964</v>
@@ -18399,7 +18399,7 @@
         <v>1521</v>
       </c>
       <c r="I302" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J302" t="s">
         <v>1966</v>
@@ -18434,7 +18434,7 @@
         <v>1521</v>
       </c>
       <c r="I303" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J303" t="s">
         <v>1967</v>
@@ -18469,7 +18469,7 @@
         <v>1521</v>
       </c>
       <c r="I304" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J304" t="s">
         <v>1968</v>
@@ -18504,7 +18504,7 @@
         <v>1521</v>
       </c>
       <c r="I305" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J305" t="s">
         <v>1945</v>
@@ -18752,7 +18752,7 @@
         <v>1521</v>
       </c>
       <c r="I312" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J312" t="s">
         <v>1975</v>
@@ -18892,7 +18892,7 @@
         <v>1521</v>
       </c>
       <c r="I316" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J316" t="s">
         <v>1979</v>
@@ -18927,7 +18927,7 @@
         <v>1521</v>
       </c>
       <c r="I317" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J317" t="s">
         <v>1980</v>
@@ -18962,7 +18962,7 @@
         <v>1521</v>
       </c>
       <c r="I318" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J318" t="s">
         <v>1981</v>
@@ -18997,7 +18997,7 @@
         <v>1521</v>
       </c>
       <c r="I319" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J319" t="s">
         <v>1982</v>
@@ -19032,7 +19032,7 @@
         <v>1521</v>
       </c>
       <c r="I320" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J320" t="s">
         <v>1983</v>
@@ -19137,7 +19137,7 @@
         <v>1521</v>
       </c>
       <c r="I323" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J323" t="s">
         <v>1986</v>
@@ -19277,7 +19277,7 @@
         <v>1521</v>
       </c>
       <c r="I327" t="s">
-        <v>1631</v>
+        <v>1633</v>
       </c>
       <c r="J327" t="s">
         <v>1990</v>
@@ -19312,7 +19312,7 @@
         <v>1521</v>
       </c>
       <c r="I328" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J328" t="s">
         <v>1991</v>
@@ -19347,7 +19347,7 @@
         <v>1521</v>
       </c>
       <c r="I329" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J329" t="s">
         <v>1992</v>
@@ -19382,7 +19382,7 @@
         <v>1521</v>
       </c>
       <c r="I330" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J330" t="s">
         <v>1993</v>
@@ -19417,7 +19417,7 @@
         <v>1521</v>
       </c>
       <c r="I331" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J331" t="s">
         <v>1994</v>
@@ -19452,7 +19452,7 @@
         <v>1521</v>
       </c>
       <c r="I332" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J332" t="s">
         <v>1995</v>
@@ -19487,7 +19487,7 @@
         <v>1521</v>
       </c>
       <c r="I333" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J333" t="s">
         <v>1996</v>
@@ -19522,7 +19522,7 @@
         <v>1521</v>
       </c>
       <c r="I334" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J334" t="s">
         <v>1997</v>
@@ -19557,7 +19557,7 @@
         <v>1521</v>
       </c>
       <c r="I335" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J335" t="s">
         <v>1998</v>
@@ -19592,7 +19592,7 @@
         <v>1521</v>
       </c>
       <c r="I336" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J336" t="s">
         <v>1999</v>
@@ -19627,7 +19627,7 @@
         <v>1521</v>
       </c>
       <c r="I337" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J337" t="s">
         <v>2000</v>
@@ -19662,7 +19662,7 @@
         <v>1521</v>
       </c>
       <c r="I338" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J338" t="s">
         <v>2001</v>
@@ -19697,7 +19697,7 @@
         <v>1521</v>
       </c>
       <c r="I339" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J339" t="s">
         <v>2002</v>
@@ -19732,7 +19732,7 @@
         <v>1521</v>
       </c>
       <c r="I340" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J340" t="s">
         <v>2003</v>
@@ -19767,7 +19767,7 @@
         <v>1521</v>
       </c>
       <c r="I341" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J341" t="s">
         <v>2004</v>
@@ -19802,7 +19802,7 @@
         <v>1521</v>
       </c>
       <c r="I342" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J342" t="s">
         <v>2005</v>
@@ -19837,7 +19837,7 @@
         <v>1521</v>
       </c>
       <c r="I343" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J343" t="s">
         <v>2006</v>
@@ -19872,7 +19872,7 @@
         <v>1521</v>
       </c>
       <c r="I344" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J344" t="s">
         <v>2007</v>
@@ -19907,7 +19907,7 @@
         <v>1521</v>
       </c>
       <c r="I345" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J345" t="s">
         <v>2008</v>
@@ -19942,7 +19942,7 @@
         <v>1521</v>
       </c>
       <c r="I346" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J346" t="s">
         <v>2009</v>
@@ -19977,7 +19977,7 @@
         <v>1521</v>
       </c>
       <c r="I347" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J347" t="s">
         <v>2010</v>
@@ -20012,7 +20012,7 @@
         <v>1521</v>
       </c>
       <c r="I348" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J348" t="s">
         <v>2011</v>
@@ -20082,7 +20082,7 @@
         <v>1521</v>
       </c>
       <c r="I350" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J350" t="s">
         <v>2013</v>
@@ -20117,7 +20117,7 @@
         <v>1521</v>
       </c>
       <c r="I351" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J351" t="s">
         <v>2013</v>
@@ -20152,7 +20152,7 @@
         <v>1521</v>
       </c>
       <c r="I352" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J352" t="s">
         <v>2013</v>
@@ -20187,7 +20187,7 @@
         <v>1521</v>
       </c>
       <c r="I353" t="s">
-        <v>1635</v>
+        <v>1637</v>
       </c>
       <c r="J353" t="s">
         <v>2014</v>
@@ -20222,7 +20222,7 @@
         <v>1521</v>
       </c>
       <c r="I354" t="s">
-        <v>1635</v>
+        <v>1637</v>
       </c>
       <c r="J354" t="s">
         <v>2014</v>
@@ -20257,7 +20257,7 @@
         <v>1521</v>
       </c>
       <c r="I355" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J355" t="s">
         <v>2015</v>
@@ -20470,7 +20470,7 @@
         <v>1521</v>
       </c>
       <c r="I361" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J361" t="s">
         <v>2021</v>
@@ -20508,7 +20508,7 @@
         <v>1528</v>
       </c>
       <c r="I362" t="s">
-        <v>1636</v>
+        <v>1638</v>
       </c>
       <c r="J362" t="s">
         <v>2022</v>
@@ -20543,7 +20543,7 @@
         <v>1521</v>
       </c>
       <c r="I363" t="s">
-        <v>1637</v>
+        <v>1639</v>
       </c>
       <c r="J363" t="s">
         <v>2023</v>
@@ -20578,7 +20578,7 @@
         <v>1521</v>
       </c>
       <c r="I364" t="s">
-        <v>1630</v>
+        <v>1632</v>
       </c>
       <c r="J364" t="s">
         <v>2024</v>
@@ -20613,7 +20613,7 @@
         <v>1521</v>
       </c>
       <c r="I365" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J365" t="s">
         <v>2025</v>
@@ -20753,7 +20753,7 @@
         <v>1521</v>
       </c>
       <c r="I369" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J369" t="s">
         <v>2029</v>
@@ -20858,7 +20858,7 @@
         <v>1521</v>
       </c>
       <c r="I372" t="s">
-        <v>1638</v>
+        <v>1640</v>
       </c>
       <c r="J372" t="s">
         <v>2032</v>
@@ -20928,7 +20928,7 @@
         <v>1521</v>
       </c>
       <c r="I374" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J374" t="s">
         <v>2034</v>
@@ -21173,7 +21173,7 @@
         <v>1521</v>
       </c>
       <c r="I381" t="s">
-        <v>1640</v>
+        <v>1642</v>
       </c>
       <c r="J381" t="s">
         <v>2041</v>
@@ -21243,7 +21243,7 @@
         <v>1521</v>
       </c>
       <c r="I383" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J383" t="s">
         <v>2043</v>
@@ -21313,7 +21313,7 @@
         <v>1521</v>
       </c>
       <c r="I385" t="s">
-        <v>1600</v>
+        <v>1601</v>
       </c>
       <c r="J385" t="s">
         <v>2045</v>
@@ -21348,7 +21348,7 @@
         <v>1521</v>
       </c>
       <c r="I386" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J386" t="s">
         <v>2046</v>
@@ -21383,7 +21383,7 @@
         <v>1521</v>
       </c>
       <c r="I387" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J387" t="s">
         <v>2047</v>
@@ -21418,7 +21418,7 @@
         <v>1521</v>
       </c>
       <c r="I388" t="s">
-        <v>1641</v>
+        <v>1643</v>
       </c>
       <c r="J388" t="s">
         <v>2048</v>
@@ -21488,7 +21488,7 @@
         <v>1521</v>
       </c>
       <c r="I390" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J390" t="s">
         <v>2050</v>
@@ -21558,7 +21558,7 @@
         <v>1521</v>
       </c>
       <c r="I392" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J392" t="s">
         <v>2052</v>
@@ -21628,7 +21628,7 @@
         <v>1521</v>
       </c>
       <c r="I394" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J394" t="s">
         <v>2054</v>
@@ -21873,7 +21873,7 @@
         <v>1521</v>
       </c>
       <c r="I401" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J401" t="s">
         <v>2061</v>
@@ -21908,7 +21908,7 @@
         <v>1521</v>
       </c>
       <c r="I402" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J402" t="s">
         <v>2062</v>
@@ -21943,7 +21943,7 @@
         <v>1521</v>
       </c>
       <c r="I403" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J403" t="s">
         <v>2063</v>
@@ -21978,7 +21978,7 @@
         <v>1521</v>
       </c>
       <c r="I404" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J404" t="s">
         <v>2064</v>
@@ -22013,7 +22013,7 @@
         <v>1521</v>
       </c>
       <c r="I405" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J405" t="s">
         <v>2065</v>
@@ -22048,7 +22048,7 @@
         <v>1521</v>
       </c>
       <c r="I406" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J406" t="s">
         <v>2066</v>
@@ -22118,7 +22118,7 @@
         <v>1521</v>
       </c>
       <c r="I408" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J408" t="s">
         <v>1972</v>
@@ -22331,7 +22331,7 @@
         <v>1521</v>
       </c>
       <c r="I414" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J414" t="s">
         <v>2073</v>
@@ -22401,7 +22401,7 @@
         <v>1521</v>
       </c>
       <c r="I416" t="s">
-        <v>1598</v>
+        <v>1599</v>
       </c>
       <c r="J416" t="s">
         <v>2075</v>
@@ -22541,7 +22541,7 @@
         <v>1521</v>
       </c>
       <c r="I420" t="s">
-        <v>1642</v>
+        <v>1644</v>
       </c>
       <c r="J420" t="s">
         <v>2079</v>
@@ -22576,7 +22576,7 @@
         <v>1521</v>
       </c>
       <c r="I421" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J421" t="s">
         <v>2080</v>
@@ -23031,7 +23031,7 @@
         <v>1521</v>
       </c>
       <c r="I434" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J434" t="s">
         <v>2093</v>
@@ -23066,7 +23066,7 @@
         <v>1521</v>
       </c>
       <c r="I435" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J435" t="s">
         <v>2094</v>
@@ -23101,7 +23101,7 @@
         <v>1521</v>
       </c>
       <c r="I436" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J436" t="s">
         <v>2095</v>
@@ -23416,7 +23416,7 @@
         <v>1521</v>
       </c>
       <c r="I445" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J445" t="s">
         <v>2103</v>
@@ -23451,7 +23451,7 @@
         <v>1521</v>
       </c>
       <c r="I446" t="s">
-        <v>1643</v>
+        <v>1645</v>
       </c>
       <c r="J446" t="s">
         <v>2104</v>
@@ -23486,7 +23486,7 @@
         <v>1521</v>
       </c>
       <c r="I447" t="s">
-        <v>1644</v>
+        <v>1646</v>
       </c>
       <c r="J447" t="s">
         <v>2105</v>
@@ -23521,7 +23521,7 @@
         <v>1521</v>
       </c>
       <c r="I448" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J448" t="s">
         <v>2106</v>
@@ -23591,7 +23591,7 @@
         <v>1521</v>
       </c>
       <c r="I450" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J450" t="s">
         <v>2108</v>
@@ -23731,7 +23731,7 @@
         <v>1521</v>
       </c>
       <c r="I454" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J454" t="s">
         <v>2112</v>
@@ -23801,7 +23801,7 @@
         <v>1521</v>
       </c>
       <c r="I456" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J456" t="s">
         <v>2114</v>
@@ -23836,7 +23836,7 @@
         <v>1521</v>
       </c>
       <c r="I457" t="s">
-        <v>1645</v>
+        <v>1647</v>
       </c>
       <c r="J457" t="s">
         <v>2115</v>
@@ -23871,7 +23871,7 @@
         <v>1521</v>
       </c>
       <c r="I458" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J458" t="s">
         <v>2116</v>
@@ -23906,7 +23906,7 @@
         <v>1521</v>
       </c>
       <c r="I459" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J459" t="s">
         <v>2117</v>
@@ -23941,7 +23941,7 @@
         <v>1521</v>
       </c>
       <c r="I460" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J460" t="s">
         <v>2118</v>
@@ -24011,7 +24011,7 @@
         <v>1521</v>
       </c>
       <c r="I462" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J462" t="s">
         <v>2120</v>
@@ -24049,7 +24049,7 @@
         <v>1530</v>
       </c>
       <c r="I463" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="J463" t="s">
         <v>2121</v>
@@ -24084,7 +24084,7 @@
         <v>1521</v>
       </c>
       <c r="I464" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J464" t="s">
         <v>2122</v>
@@ -24259,7 +24259,7 @@
         <v>1521</v>
       </c>
       <c r="I469" t="s">
-        <v>1646</v>
+        <v>1648</v>
       </c>
       <c r="J469" t="s">
         <v>2127</v>
@@ -24294,7 +24294,7 @@
         <v>1521</v>
       </c>
       <c r="I470" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J470" t="s">
         <v>2128</v>
@@ -24329,7 +24329,7 @@
         <v>1521</v>
       </c>
       <c r="I471" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J471" t="s">
         <v>2129</v>
@@ -24364,7 +24364,7 @@
         <v>1521</v>
       </c>
       <c r="I472" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J472" t="s">
         <v>2130</v>
@@ -24399,7 +24399,7 @@
         <v>1521</v>
       </c>
       <c r="I473" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
       <c r="J473" t="s">
         <v>2131</v>
@@ -24545,7 +24545,7 @@
         <v>1527</v>
       </c>
       <c r="I477" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J477" t="s">
         <v>2133</v>
@@ -24580,7 +24580,7 @@
         <v>1521</v>
       </c>
       <c r="I478" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J478" t="s">
         <v>2134</v>
@@ -24758,7 +24758,7 @@
         <v>1521</v>
       </c>
       <c r="I483" t="s">
-        <v>1606</v>
+        <v>1607</v>
       </c>
       <c r="J483" t="s">
         <v>2139</v>
@@ -24793,7 +24793,7 @@
         <v>1521</v>
       </c>
       <c r="I484" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J484" t="s">
         <v>2140</v>
@@ -24828,7 +24828,7 @@
         <v>1521</v>
       </c>
       <c r="I485" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J485" t="s">
         <v>2141</v>
@@ -24863,7 +24863,7 @@
         <v>1521</v>
       </c>
       <c r="I486" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J486" t="s">
         <v>2142</v>
@@ -24898,7 +24898,7 @@
         <v>1521</v>
       </c>
       <c r="I487" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J487" t="s">
         <v>2143</v>
@@ -24936,7 +24936,7 @@
         <v>1533</v>
       </c>
       <c r="I488" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J488" t="s">
         <v>2144</v>
@@ -24971,7 +24971,7 @@
         <v>1521</v>
       </c>
       <c r="I489" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J489" t="s">
         <v>2145</v>
@@ -25076,7 +25076,7 @@
         <v>1521</v>
       </c>
       <c r="I492" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J492" t="s">
         <v>2147</v>
@@ -25111,7 +25111,7 @@
         <v>1521</v>
       </c>
       <c r="I493" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J493" t="s">
         <v>2148</v>
@@ -25181,7 +25181,7 @@
         <v>1521</v>
       </c>
       <c r="I495" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J495" t="s">
         <v>2150</v>
@@ -25216,7 +25216,7 @@
         <v>1521</v>
       </c>
       <c r="I496" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J496" t="s">
         <v>2151</v>
@@ -25251,7 +25251,7 @@
         <v>1521</v>
       </c>
       <c r="I497" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J497" t="s">
         <v>2152</v>
@@ -25286,7 +25286,7 @@
         <v>1521</v>
       </c>
       <c r="I498" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J498" t="s">
         <v>2153</v>
@@ -25321,7 +25321,7 @@
         <v>1521</v>
       </c>
       <c r="I499" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J499" t="s">
         <v>2154</v>
@@ -25356,7 +25356,7 @@
         <v>1521</v>
       </c>
       <c r="I500" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J500" t="s">
         <v>2155</v>
@@ -25391,7 +25391,7 @@
         <v>1521</v>
       </c>
       <c r="I501" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J501" t="s">
         <v>2156</v>
@@ -25426,7 +25426,7 @@
         <v>1521</v>
       </c>
       <c r="I502" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J502" t="s">
         <v>2157</v>
@@ -25461,7 +25461,7 @@
         <v>1521</v>
       </c>
       <c r="I503" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J503" t="s">
         <v>2158</v>
@@ -25496,7 +25496,7 @@
         <v>1521</v>
       </c>
       <c r="I504" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J504" t="s">
         <v>2159</v>
@@ -25531,7 +25531,7 @@
         <v>1521</v>
       </c>
       <c r="I505" t="s">
-        <v>1638</v>
+        <v>1640</v>
       </c>
       <c r="J505" t="s">
         <v>2160</v>
@@ -25566,7 +25566,7 @@
         <v>1521</v>
       </c>
       <c r="I506" t="s">
-        <v>1647</v>
+        <v>1649</v>
       </c>
       <c r="J506" t="s">
         <v>2161</v>
@@ -25601,7 +25601,7 @@
         <v>1521</v>
       </c>
       <c r="I507" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J507" t="s">
         <v>2162</v>
@@ -25636,7 +25636,7 @@
         <v>1521</v>
       </c>
       <c r="I508" t="s">
-        <v>1648</v>
+        <v>1650</v>
       </c>
       <c r="J508" t="s">
         <v>2163</v>
@@ -25706,7 +25706,7 @@
         <v>1521</v>
       </c>
       <c r="I510" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J510" t="s">
         <v>2093</v>
@@ -25744,7 +25744,7 @@
         <v>1534</v>
       </c>
       <c r="I511" t="s">
-        <v>1649</v>
+        <v>1651</v>
       </c>
       <c r="J511" t="s">
         <v>2165</v>
@@ -25779,7 +25779,7 @@
         <v>1521</v>
       </c>
       <c r="I512" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J512" t="s">
         <v>2166</v>
@@ -25849,7 +25849,7 @@
         <v>1521</v>
       </c>
       <c r="I514" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J514" t="s">
         <v>2168</v>
@@ -25919,7 +25919,7 @@
         <v>1521</v>
       </c>
       <c r="I516" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J516" t="s">
         <v>2170</v>
@@ -25954,7 +25954,7 @@
         <v>1521</v>
       </c>
       <c r="I517" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J517" t="s">
         <v>2171</v>
@@ -25989,7 +25989,7 @@
         <v>1521</v>
       </c>
       <c r="I518" t="s">
-        <v>1650</v>
+        <v>1652</v>
       </c>
       <c r="J518" t="s">
         <v>2172</v>
@@ -26062,7 +26062,7 @@
         <v>1535</v>
       </c>
       <c r="I520" t="s">
-        <v>1651</v>
+        <v>1653</v>
       </c>
       <c r="J520" t="s">
         <v>2174</v>
@@ -26100,7 +26100,7 @@
         <v>1536</v>
       </c>
       <c r="I521" t="s">
-        <v>1551</v>
+        <v>1582</v>
       </c>
       <c r="J521" t="s">
         <v>2175</v>
@@ -26135,7 +26135,7 @@
         <v>1521</v>
       </c>
       <c r="I522" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J522" t="s">
         <v>2176</v>
@@ -26170,7 +26170,7 @@
         <v>1521</v>
       </c>
       <c r="I523" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J523" t="s">
         <v>2177</v>
@@ -26205,7 +26205,7 @@
         <v>1521</v>
       </c>
       <c r="I524" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J524" t="s">
         <v>2178</v>
@@ -26240,7 +26240,7 @@
         <v>1521</v>
       </c>
       <c r="I525" t="s">
-        <v>1613</v>
+        <v>1614</v>
       </c>
       <c r="J525" t="s">
         <v>2179</v>
@@ -26275,7 +26275,7 @@
         <v>1521</v>
       </c>
       <c r="I526" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J526" t="s">
         <v>2180</v>
@@ -26310,7 +26310,7 @@
         <v>1521</v>
       </c>
       <c r="I527" t="s">
-        <v>1652</v>
+        <v>1654</v>
       </c>
       <c r="J527" t="s">
         <v>2181</v>
@@ -26383,7 +26383,7 @@
         <v>1537</v>
       </c>
       <c r="I529" t="s">
-        <v>1649</v>
+        <v>1651</v>
       </c>
       <c r="J529" t="s">
         <v>2183</v>
@@ -26418,7 +26418,7 @@
         <v>1521</v>
       </c>
       <c r="I530" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J530" t="s">
         <v>2184</v>
@@ -26453,7 +26453,7 @@
         <v>1521</v>
       </c>
       <c r="I531" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="J531" t="s">
         <v>2185</v>
@@ -26488,7 +26488,7 @@
         <v>1521</v>
       </c>
       <c r="I532" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J532" t="s">
         <v>2186</v>
@@ -26558,7 +26558,7 @@
         <v>1521</v>
       </c>
       <c r="I534" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J534" t="s">
         <v>2188</v>
@@ -26593,7 +26593,7 @@
         <v>1521</v>
       </c>
       <c r="I535" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J535" t="s">
         <v>2189</v>
@@ -26628,7 +26628,7 @@
         <v>1521</v>
       </c>
       <c r="I536" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J536" t="s">
         <v>2190</v>
@@ -26663,7 +26663,7 @@
         <v>1521</v>
       </c>
       <c r="I537" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J537" t="s">
         <v>2191</v>
@@ -26701,7 +26701,7 @@
         <v>1538</v>
       </c>
       <c r="I538" t="s">
-        <v>1621</v>
+        <v>1622</v>
       </c>
       <c r="J538" t="s">
         <v>2192</v>
@@ -26739,7 +26739,7 @@
         <v>1538</v>
       </c>
       <c r="I539" t="s">
-        <v>1654</v>
+        <v>1656</v>
       </c>
       <c r="J539" t="s">
         <v>2193</v>
@@ -26777,7 +26777,7 @@
         <v>1538</v>
       </c>
       <c r="I540" t="s">
-        <v>1655</v>
+        <v>1657</v>
       </c>
       <c r="J540" t="s">
         <v>2194</v>
@@ -26812,7 +26812,7 @@
         <v>1521</v>
       </c>
       <c r="I541" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="J541" t="s">
         <v>2195</v>
@@ -26850,7 +26850,7 @@
         <v>1538</v>
       </c>
       <c r="I542" t="s">
-        <v>1656</v>
+        <v>1658</v>
       </c>
       <c r="J542" t="s">
         <v>2196</v>
@@ -27060,7 +27060,7 @@
         <v>1521</v>
       </c>
       <c r="I548" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="J548" t="s">
         <v>2201</v>
@@ -27095,7 +27095,7 @@
         <v>1521</v>
       </c>
       <c r="I549" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J549" t="s">
         <v>2202</v>
@@ -27200,7 +27200,7 @@
         <v>1521</v>
       </c>
       <c r="I552" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J552" t="s">
         <v>2205</v>
@@ -27235,7 +27235,7 @@
         <v>1521</v>
       </c>
       <c r="I553" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="J553" t="s">
         <v>2206</v>
@@ -27270,7 +27270,7 @@
         <v>1521</v>
       </c>
       <c r="I554" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J554" t="s">
         <v>2207</v>
@@ -27305,7 +27305,7 @@
         <v>1521</v>
       </c>
       <c r="I555" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J555" t="s">
         <v>2208</v>
@@ -27340,7 +27340,7 @@
         <v>1521</v>
       </c>
       <c r="I556" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J556" t="s">
         <v>2208</v>
@@ -27378,7 +27378,7 @@
         <v>1539</v>
       </c>
       <c r="I557" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J557" t="s">
         <v>2209</v>
@@ -27413,7 +27413,7 @@
         <v>1521</v>
       </c>
       <c r="I558" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J558" t="s">
         <v>2210</v>
@@ -27448,7 +27448,7 @@
         <v>1521</v>
       </c>
       <c r="I559" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J559" t="s">
         <v>2211</v>
@@ -27483,7 +27483,7 @@
         <v>1521</v>
       </c>
       <c r="I560" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="J560" t="s">
         <v>2212</v>
@@ -27518,7 +27518,7 @@
         <v>1521</v>
       </c>
       <c r="I561" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J561" t="s">
         <v>2213</v>
@@ -27553,7 +27553,7 @@
         <v>1521</v>
       </c>
       <c r="I562" t="s">
-        <v>1639</v>
+        <v>1641</v>
       </c>
       <c r="J562" t="s">
         <v>2214</v>
@@ -27588,7 +27588,7 @@
         <v>1521</v>
       </c>
       <c r="I563" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J563" t="s">
         <v>2215</v>
@@ -27626,7 +27626,7 @@
         <v>1540</v>
       </c>
       <c r="I564" t="s">
-        <v>1657</v>
+        <v>1659</v>
       </c>
       <c r="J564" t="s">
         <v>2216</v>
@@ -27696,7 +27696,7 @@
         <v>1521</v>
       </c>
       <c r="I566" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J566" t="s">
         <v>2218</v>
@@ -27731,7 +27731,7 @@
         <v>1521</v>
       </c>
       <c r="I567" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J567" t="s">
         <v>2219</v>
@@ -27801,7 +27801,7 @@
         <v>1521</v>
       </c>
       <c r="I569" t="s">
-        <v>1617</v>
+        <v>1618</v>
       </c>
       <c r="J569" t="s">
         <v>2221</v>
@@ -27836,7 +27836,7 @@
         <v>1521</v>
       </c>
       <c r="I570" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J570" t="s">
         <v>2222</v>
@@ -27871,7 +27871,7 @@
         <v>1521</v>
       </c>
       <c r="I571" t="s">
-        <v>1658</v>
+        <v>1582</v>
       </c>
       <c r="J571" t="s">
         <v>2223</v>
@@ -27906,7 +27906,7 @@
         <v>1521</v>
       </c>
       <c r="I572" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J572" t="s">
         <v>2224</v>
@@ -27941,7 +27941,7 @@
         <v>1521</v>
       </c>
       <c r="I573" t="s">
-        <v>1658</v>
+        <v>1582</v>
       </c>
       <c r="J573" t="s">
         <v>2225</v>
@@ -27976,7 +27976,7 @@
         <v>1521</v>
       </c>
       <c r="I574" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J574" t="s">
         <v>2226</v>
@@ -28084,7 +28084,7 @@
         <v>1541</v>
       </c>
       <c r="I577" t="s">
-        <v>1659</v>
+        <v>1660</v>
       </c>
       <c r="J577" t="s">
         <v>2229</v>
@@ -28154,7 +28154,7 @@
         <v>1521</v>
       </c>
       <c r="I579" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J579" t="s">
         <v>2231</v>
@@ -28189,7 +28189,7 @@
         <v>1521</v>
       </c>
       <c r="I580" t="s">
-        <v>1660</v>
+        <v>1629</v>
       </c>
       <c r="J580" t="s">
         <v>2232</v>
@@ -28224,7 +28224,7 @@
         <v>1521</v>
       </c>
       <c r="I581" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J581" t="s">
         <v>2233</v>
@@ -28259,7 +28259,7 @@
         <v>1521</v>
       </c>
       <c r="I582" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J582" t="s">
         <v>2234</v>
@@ -28332,7 +28332,7 @@
         <v>1521</v>
       </c>
       <c r="I584" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J584" t="s">
         <v>2228</v>
@@ -28367,7 +28367,7 @@
         <v>1521</v>
       </c>
       <c r="I585" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J585" t="s">
         <v>2228</v>
@@ -28402,7 +28402,7 @@
         <v>1521</v>
       </c>
       <c r="I586" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J586" t="s">
         <v>2228</v>
@@ -28437,7 +28437,7 @@
         <v>1521</v>
       </c>
       <c r="I587" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J587" t="s">
         <v>2228</v>
@@ -28472,7 +28472,7 @@
         <v>1521</v>
       </c>
       <c r="I588" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J588" t="s">
         <v>2228</v>
@@ -28507,7 +28507,7 @@
         <v>1521</v>
       </c>
       <c r="I589" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J589" t="s">
         <v>2228</v>
@@ -28542,7 +28542,7 @@
         <v>1521</v>
       </c>
       <c r="I590" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J590" t="s">
         <v>2228</v>
@@ -28577,7 +28577,7 @@
         <v>1521</v>
       </c>
       <c r="I591" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J591" t="s">
         <v>2236</v>
@@ -28650,7 +28650,7 @@
         <v>1521</v>
       </c>
       <c r="I593" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J593" t="s">
         <v>2238</v>
@@ -28685,7 +28685,7 @@
         <v>1521</v>
       </c>
       <c r="I594" t="s">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="J594" t="s">
         <v>2239</v>
@@ -28720,7 +28720,7 @@
         <v>1521</v>
       </c>
       <c r="I595" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J595" t="s">
         <v>2240</v>
@@ -28793,7 +28793,7 @@
         <v>1521</v>
       </c>
       <c r="I597" t="s">
-        <v>1638</v>
+        <v>1640</v>
       </c>
       <c r="J597" t="s">
         <v>2242</v>
@@ -28828,7 +28828,7 @@
         <v>1521</v>
       </c>
       <c r="I598" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="J598" t="s">
         <v>2243</v>
@@ -28863,7 +28863,7 @@
         <v>1521</v>
       </c>
       <c r="I599" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J599" t="s">
         <v>2244</v>
@@ -28898,7 +28898,7 @@
         <v>1521</v>
       </c>
       <c r="I600" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J600" t="s">
         <v>2231</v>
@@ -28971,7 +28971,7 @@
         <v>1521</v>
       </c>
       <c r="I602" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J602" t="s">
         <v>2246</v>
@@ -29006,7 +29006,7 @@
         <v>1521</v>
       </c>
       <c r="I603" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J603" t="s">
         <v>2247</v>
@@ -29041,7 +29041,7 @@
         <v>1521</v>
       </c>
       <c r="I604" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J604" t="s">
         <v>2248</v>
@@ -29076,7 +29076,7 @@
         <v>1521</v>
       </c>
       <c r="I605" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J605" t="s">
         <v>2249</v>
@@ -29111,7 +29111,7 @@
         <v>1521</v>
       </c>
       <c r="I606" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J606" t="s">
         <v>2250</v>
@@ -29181,7 +29181,7 @@
         <v>1521</v>
       </c>
       <c r="I608" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J608" t="s">
         <v>2252</v>
@@ -29251,7 +29251,7 @@
         <v>1521</v>
       </c>
       <c r="I610" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J610" t="s">
         <v>2254</v>
@@ -29286,7 +29286,7 @@
         <v>1521</v>
       </c>
       <c r="I611" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J611" t="s">
         <v>2255</v>
@@ -29362,7 +29362,7 @@
         <v>1545</v>
       </c>
       <c r="I613" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J613" t="s">
         <v>2257</v>
@@ -29432,7 +29432,7 @@
         <v>1521</v>
       </c>
       <c r="I615" t="s">
-        <v>1658</v>
+        <v>1582</v>
       </c>
       <c r="J615" t="s">
         <v>2259</v>
@@ -29467,7 +29467,7 @@
         <v>1521</v>
       </c>
       <c r="I616" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J616" t="s">
         <v>2260</v>
@@ -29505,7 +29505,7 @@
         <v>1544</v>
       </c>
       <c r="I617" t="s">
-        <v>1551</v>
+        <v>1655</v>
       </c>
       <c r="J617" t="s">
         <v>2261</v>
@@ -29540,7 +29540,7 @@
         <v>1521</v>
       </c>
       <c r="I618" t="s">
-        <v>1551</v>
+        <v>1664</v>
       </c>
       <c r="J618" t="s">
         <v>2262</v>
@@ -29575,7 +29575,7 @@
         <v>1521</v>
       </c>
       <c r="I619" t="s">
-        <v>1551</v>
+        <v>1655</v>
       </c>
       <c r="J619" t="s">
         <v>2263</v>
@@ -29613,7 +29613,7 @@
         <v>1546</v>
       </c>
       <c r="I620" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J620" t="s">
         <v>2264</v>
@@ -29648,7 +29648,7 @@
         <v>1521</v>
       </c>
       <c r="I621" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="J621" t="s">
         <v>2265</v>
@@ -29683,7 +29683,7 @@
         <v>1521</v>
       </c>
       <c r="I622" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J622" t="s">
         <v>2266</v>
@@ -29718,7 +29718,7 @@
         <v>1521</v>
       </c>
       <c r="I623" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J623" t="s">
         <v>2267</v>
@@ -29753,7 +29753,7 @@
         <v>1521</v>
       </c>
       <c r="I624" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J624" t="s">
         <v>2268</v>
@@ -29823,7 +29823,7 @@
         <v>1521</v>
       </c>
       <c r="I626" t="s">
-        <v>1634</v>
+        <v>1636</v>
       </c>
       <c r="J626" t="s">
         <v>2270</v>
@@ -29893,7 +29893,7 @@
         <v>1521</v>
       </c>
       <c r="I628" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J628" t="s">
         <v>2272</v>
@@ -29928,7 +29928,7 @@
         <v>1521</v>
       </c>
       <c r="I629" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="J629" t="s">
         <v>2273</v>
@@ -29963,7 +29963,7 @@
         <v>1521</v>
       </c>
       <c r="I630" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J630" t="s">
         <v>2274</v>
@@ -29998,7 +29998,7 @@
         <v>1521</v>
       </c>
       <c r="I631" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J631" t="s">
         <v>2275</v>
@@ -30033,7 +30033,7 @@
         <v>1521</v>
       </c>
       <c r="I632" t="s">
-        <v>1633</v>
+        <v>1635</v>
       </c>
       <c r="J632" t="s">
         <v>2276</v>
@@ -30103,7 +30103,7 @@
         <v>1521</v>
       </c>
       <c r="I634" t="s">
-        <v>1632</v>
+        <v>1634</v>
       </c>
       <c r="J634" t="s">
         <v>2278</v>
@@ -30138,7 +30138,7 @@
         <v>1521</v>
       </c>
       <c r="I635" t="s">
-        <v>1638</v>
+        <v>1640</v>
       </c>
       <c r="J635" t="s">
         <v>2279</v>
@@ -30173,7 +30173,7 @@
         <v>1521</v>
       </c>
       <c r="I636" t="s">
-        <v>1658</v>
+        <v>1582</v>
       </c>
       <c r="J636" t="s">
         <v>2280</v>
@@ -30208,7 +30208,7 @@
         <v>1521</v>
       </c>
       <c r="I637" t="s">
-        <v>1626</v>
+        <v>1627</v>
       </c>
       <c r="J637" t="s">
         <v>2281</v>
@@ -30240,7 +30240,7 @@
         <v>1521</v>
       </c>
       <c r="I638" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="J638" t="s">
         <v>2282</v>
@@ -30272,7 +30272,7 @@
         <v>1521</v>
       </c>
       <c r="I639" t="s">
-        <v>1653</v>
+        <v>1655</v>
       </c>
       <c r="J639" t="s">
         <v>2283</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-27 08:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6548" uniqueCount="2524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6548" uniqueCount="2529">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7372,117 +7372,120 @@
     <t>AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
+    <t>URBANISMO,MOBILIDADE E TRANSPORTE</t>
+  </si>
+  <si>
+    <t>URBANISMO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA QUÍMICA</t>
+  </si>
+  <si>
+    <t>GEOLOGIA</t>
+  </si>
+  <si>
+    <t>EDIFICAÇÕES</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,PATRIMÔNIO HISTÓRICO E CULTURAL</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,URBANISMO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA QUÍMICA,GEOLOGIA,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
+    <t>RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
+    <t>SAÚDE MENTAL</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
+  </si>
+  <si>
+    <t>ASSISTÊNCIA SOCIAL</t>
+  </si>
+  <si>
+    <t>SAÚDE</t>
+  </si>
+  <si>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>FARMÁCIA</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,FARMÁCIA</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,GEOLOGIA,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA QUÍMICA,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,GEOLOGIA,URBANISMO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA QUÍMICA,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL</t>
+  </si>
+  <si>
+    <t>BIOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,GEOTECNIA,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>EDIFICAÇÕES,MOBILIDADE E TRANSPORTE</t>
+  </si>
+  <si>
+    <t>MOBILIDADE E TRANSPORTE</t>
+  </si>
+  <si>
+    <t>ECONOMIA,ENGENHARIA FLORESTAL,RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>RECURSOS HÍDRICOS,URBANISMO</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,GEOTECNIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO,MEDICINA LEGAL</t>
+  </si>
+  <si>
     <t>MOBILIDADE E TRANSPORTE,URBANISMO</t>
   </si>
   <si>
-    <t>URBANISMO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA QUÍMICA</t>
-  </si>
-  <si>
-    <t>GEOLOGIA</t>
-  </si>
-  <si>
-    <t>EDIFICAÇÕES</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,PATRIMÔNIO HISTÓRICO E CULTURAL</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,URBANISMO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA QUÍMICA,GEOLOGIA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>SAÚDE MENTAL</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
-  </si>
-  <si>
-    <t>ASSISTÊNCIA SOCIAL</t>
-  </si>
-  <si>
-    <t>SAÚDE</t>
-  </si>
-  <si>
-    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>FARMÁCIA</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,FARMÁCIA</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,GEOLOGIA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA QUÍMICA,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,GEOLOGIA,URBANISMO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA QUÍMICA,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL</t>
-  </si>
-  <si>
-    <t>BIOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,VALORAÇÃO DANOS AMBIENTAIS</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,GEOTECNIA,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>EDIFICAÇÕES,MOBILIDADE E TRANSPORTE</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE</t>
-  </si>
-  <si>
-    <t>ECONOMIA,ENGENHARIA FLORESTAL,RECURSOS HÍDRICOS</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>RECURSOS HÍDRICOS,URBANISMO</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,ENGENHARIA QUÍMICA,RESÍDUOS SÓLIDOS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,GEOTECNIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO,MEDICINA LEGAL</t>
-  </si>
-  <si>
     <t>ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
@@ -7555,7 +7558,10 @@
     <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
   </si>
   <si>
-    <t>BIOLOGIA,RECURSOS HÍDRICOS,URBANISMO,MOBILIDADE E TRANSPORTE</t>
+    <t>URBANISMO,ENGENHARIA FLORESTAL</t>
+  </si>
+  <si>
+    <t>MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS,URBANISMO,BIOLOGIA</t>
   </si>
   <si>
     <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
@@ -7573,6 +7579,9 @@
     <t>ENGENHARIA AMBIENTAL,ENGENHARIA FLORESTAL</t>
   </si>
   <si>
+    <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
     <t>GEOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
@@ -7582,10 +7591,16 @@
     <t>URBANISMO,BIOLOGIA</t>
   </si>
   <si>
+    <t>VALORAÇÃO DANOS AMBIENTAIS,BIOLOGIA</t>
+  </si>
+  <si>
     <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
-    <t>URBANISMO,PSICOLOGIA,ORÇAMENTO,ECONOMICIDADE CONTÁBIL,SAÚDE,MOBILIDADE E TRANSPORTE,AVALIAÇÃO DE IMÓVEIS,ECONOMIA,SAÚDE MENTAL,ASSISTÊNCIA SOCIAL</t>
+    <t>GEOTECNIA,ENGENHARIA CIVIL</t>
+  </si>
+  <si>
+    <t>URBANISMO,ASSISTÊNCIA SOCIAL,SAÚDE,MOBILIDADE E TRANSPORTE,ECONOMIA,SAÚDE MENTAL,AVALIAÇÃO DE IMÓVEIS,ORÇAMENTO,PSICOLOGIA,ECONOMICIDADE CONTÁBIL</t>
   </si>
 </sst>
 </file>
@@ -14815,7 +14830,7 @@
         <v>2370</v>
       </c>
       <c r="L196" t="s">
-        <v>2452</v>
+        <v>2489</v>
       </c>
     </row>
     <row r="197" spans="1:12">
@@ -14920,7 +14935,7 @@
         <v>2358</v>
       </c>
       <c r="L199" t="s">
-        <v>2489</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="200" spans="1:12">
@@ -14955,7 +14970,7 @@
         <v>2357</v>
       </c>
       <c r="L200" t="s">
-        <v>2490</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="201" spans="1:12">
@@ -15095,7 +15110,7 @@
         <v>2366</v>
       </c>
       <c r="L204" t="s">
-        <v>2491</v>
+        <v>2492</v>
       </c>
     </row>
     <row r="205" spans="1:12">
@@ -15375,7 +15390,7 @@
         <v>2370</v>
       </c>
       <c r="L212" t="s">
-        <v>2492</v>
+        <v>2493</v>
       </c>
     </row>
     <row r="213" spans="1:12">
@@ -15658,7 +15673,7 @@
         <v>2370</v>
       </c>
       <c r="L220" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="221" spans="1:12">
@@ -15763,7 +15778,7 @@
         <v>2351</v>
       </c>
       <c r="L223" t="s">
-        <v>2494</v>
+        <v>2495</v>
       </c>
     </row>
     <row r="224" spans="1:12">
@@ -15973,7 +15988,7 @@
         <v>2344</v>
       </c>
       <c r="L229" t="s">
-        <v>2495</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="230" spans="1:12">
@@ -16008,7 +16023,7 @@
         <v>2339</v>
       </c>
       <c r="L230" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="231" spans="1:12">
@@ -16638,7 +16653,7 @@
         <v>2348</v>
       </c>
       <c r="L248" t="s">
-        <v>2496</v>
+        <v>2497</v>
       </c>
     </row>
     <row r="249" spans="1:12">
@@ -16673,7 +16688,7 @@
         <v>2351</v>
       </c>
       <c r="L249" t="s">
-        <v>2497</v>
+        <v>2498</v>
       </c>
     </row>
     <row r="250" spans="1:12">
@@ -16778,7 +16793,7 @@
         <v>2337</v>
       </c>
       <c r="L252" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="253" spans="1:12">
@@ -17023,7 +17038,7 @@
         <v>2398</v>
       </c>
       <c r="L259" t="s">
-        <v>2499</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="260" spans="1:12">
@@ -17443,7 +17458,7 @@
         <v>2380</v>
       </c>
       <c r="L271" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="272" spans="1:12">
@@ -17548,7 +17563,7 @@
         <v>2368</v>
       </c>
       <c r="L274" t="s">
-        <v>2501</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="275" spans="1:12">
@@ -17831,7 +17846,7 @@
         <v>2351</v>
       </c>
       <c r="L282" t="s">
-        <v>2497</v>
+        <v>2498</v>
       </c>
     </row>
     <row r="283" spans="1:12">
@@ -17901,7 +17916,7 @@
         <v>2406</v>
       </c>
       <c r="L284" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="285" spans="1:12">
@@ -18076,7 +18091,7 @@
         <v>2407</v>
       </c>
       <c r="L289" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="290" spans="1:12">
@@ -18954,7 +18969,7 @@
         <v>2374</v>
       </c>
       <c r="L314" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="315" spans="1:12">
@@ -18989,7 +19004,7 @@
         <v>2409</v>
       </c>
       <c r="L315" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="316" spans="1:12">
@@ -19024,7 +19039,7 @@
         <v>2409</v>
       </c>
       <c r="L316" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="317" spans="1:12">
@@ -19059,7 +19074,7 @@
         <v>2409</v>
       </c>
       <c r="L317" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="318" spans="1:12">
@@ -19094,7 +19109,7 @@
         <v>2409</v>
       </c>
       <c r="L318" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="319" spans="1:12">
@@ -19129,7 +19144,7 @@
         <v>2409</v>
       </c>
       <c r="L319" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="320" spans="1:12">
@@ -19164,7 +19179,7 @@
         <v>2409</v>
       </c>
       <c r="L320" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="321" spans="1:12">
@@ -19199,7 +19214,7 @@
         <v>2409</v>
       </c>
       <c r="L321" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="322" spans="1:12">
@@ -19234,7 +19249,7 @@
         <v>2409</v>
       </c>
       <c r="L322" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="323" spans="1:12">
@@ -19269,7 +19284,7 @@
         <v>2409</v>
       </c>
       <c r="L323" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="324" spans="1:12">
@@ -19304,7 +19319,7 @@
         <v>2409</v>
       </c>
       <c r="L324" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="325" spans="1:12">
@@ -19339,7 +19354,7 @@
         <v>2409</v>
       </c>
       <c r="L325" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="326" spans="1:12">
@@ -19374,7 +19389,7 @@
         <v>2409</v>
       </c>
       <c r="L326" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="327" spans="1:12">
@@ -19409,7 +19424,7 @@
         <v>2409</v>
       </c>
       <c r="L327" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="328" spans="1:12">
@@ -19444,7 +19459,7 @@
         <v>2409</v>
       </c>
       <c r="L328" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="329" spans="1:12">
@@ -19479,7 +19494,7 @@
         <v>2409</v>
       </c>
       <c r="L329" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="330" spans="1:12">
@@ -19514,7 +19529,7 @@
         <v>2409</v>
       </c>
       <c r="L330" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="331" spans="1:12">
@@ -19549,7 +19564,7 @@
         <v>2409</v>
       </c>
       <c r="L331" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="332" spans="1:12">
@@ -19584,7 +19599,7 @@
         <v>2409</v>
       </c>
       <c r="L332" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="333" spans="1:12">
@@ -19654,7 +19669,7 @@
         <v>2410</v>
       </c>
       <c r="L334" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="335" spans="1:12">
@@ -19759,7 +19774,7 @@
         <v>2399</v>
       </c>
       <c r="L337" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="338" spans="1:12">
@@ -20115,7 +20130,7 @@
         <v>2336</v>
       </c>
       <c r="L347" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="348" spans="1:12">
@@ -20150,7 +20165,7 @@
         <v>2374</v>
       </c>
       <c r="L348" t="s">
-        <v>2506</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="349" spans="1:12">
@@ -20185,7 +20200,7 @@
         <v>2413</v>
       </c>
       <c r="L349" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="350" spans="1:12">
@@ -20430,7 +20445,7 @@
         <v>2414</v>
       </c>
       <c r="L356" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="357" spans="1:12">
@@ -20640,7 +20655,7 @@
         <v>2393</v>
       </c>
       <c r="L362" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="363" spans="1:12">
@@ -20675,7 +20690,7 @@
         <v>2349</v>
       </c>
       <c r="L363" t="s">
-        <v>2489</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="364" spans="1:12">
@@ -20780,7 +20795,7 @@
         <v>2415</v>
       </c>
       <c r="L366" t="s">
-        <v>2507</v>
+        <v>2508</v>
       </c>
     </row>
     <row r="367" spans="1:12">
@@ -20815,7 +20830,7 @@
         <v>2331</v>
       </c>
       <c r="L367" t="s">
-        <v>2506</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="368" spans="1:12">
@@ -20885,7 +20900,7 @@
         <v>2416</v>
       </c>
       <c r="L369" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="370" spans="1:12">
@@ -21025,7 +21040,7 @@
         <v>2417</v>
       </c>
       <c r="L373" t="s">
-        <v>2508</v>
+        <v>2509</v>
       </c>
     </row>
     <row r="374" spans="1:12">
@@ -21340,7 +21355,7 @@
         <v>2347</v>
       </c>
       <c r="L382" t="s">
-        <v>2509</v>
+        <v>2510</v>
       </c>
     </row>
     <row r="383" spans="1:12">
@@ -21375,7 +21390,7 @@
         <v>2350</v>
       </c>
       <c r="L383" t="s">
-        <v>2510</v>
+        <v>2511</v>
       </c>
     </row>
     <row r="384" spans="1:12">
@@ -21690,7 +21705,7 @@
         <v>2360</v>
       </c>
       <c r="L392" t="s">
-        <v>2511</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="393" spans="1:12">
@@ -21868,7 +21883,7 @@
         <v>2383</v>
       </c>
       <c r="L397" t="s">
-        <v>2491</v>
+        <v>2492</v>
       </c>
     </row>
     <row r="398" spans="1:12">
@@ -21903,7 +21918,7 @@
         <v>2380</v>
       </c>
       <c r="L398" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="399" spans="1:12">
@@ -22148,7 +22163,7 @@
         <v>2349</v>
       </c>
       <c r="L405" t="s">
-        <v>2512</v>
+        <v>2513</v>
       </c>
     </row>
     <row r="406" spans="1:12">
@@ -22218,7 +22233,7 @@
         <v>2354</v>
       </c>
       <c r="L407" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="408" spans="1:12">
@@ -22393,7 +22408,7 @@
         <v>2366</v>
       </c>
       <c r="L412" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="413" spans="1:12">
@@ -22533,7 +22548,7 @@
         <v>2413</v>
       </c>
       <c r="L416" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="417" spans="1:12">
@@ -22708,7 +22723,7 @@
         <v>2370</v>
       </c>
       <c r="L421" t="s">
-        <v>2510</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="422" spans="1:12">
@@ -23023,7 +23038,7 @@
         <v>2356</v>
       </c>
       <c r="L430" t="s">
-        <v>2513</v>
+        <v>2515</v>
       </c>
     </row>
     <row r="431" spans="1:12">
@@ -23408,7 +23423,7 @@
         <v>2370</v>
       </c>
       <c r="L441" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="442" spans="1:12">
@@ -23723,7 +23738,7 @@
         <v>2425</v>
       </c>
       <c r="L450" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="451" spans="1:12">
@@ -23758,7 +23773,7 @@
         <v>2351</v>
       </c>
       <c r="L451" t="s">
-        <v>2512</v>
+        <v>2513</v>
       </c>
     </row>
     <row r="452" spans="1:12">
@@ -23828,7 +23843,7 @@
         <v>2426</v>
       </c>
       <c r="L453" t="s">
-        <v>2514</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="454" spans="1:12">
@@ -23863,7 +23878,7 @@
         <v>2362</v>
       </c>
       <c r="L454" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="455" spans="1:12">
@@ -24006,7 +24021,7 @@
         <v>2428</v>
       </c>
       <c r="L458" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="459" spans="1:12">
@@ -24995,7 +25010,7 @@
         <v>2364</v>
       </c>
       <c r="L486" t="s">
-        <v>2515</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="487" spans="1:12">
@@ -25205,7 +25220,7 @@
         <v>2430</v>
       </c>
       <c r="L492" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="493" spans="1:12">
@@ -25278,7 +25293,7 @@
         <v>2364</v>
       </c>
       <c r="L494" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="495" spans="1:12">
@@ -25418,7 +25433,7 @@
         <v>2376</v>
       </c>
       <c r="L498" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="499" spans="1:12">
@@ -25453,7 +25468,7 @@
         <v>2354</v>
       </c>
       <c r="L499" t="s">
-        <v>2516</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="500" spans="1:12">
@@ -25698,7 +25713,7 @@
         <v>2431</v>
       </c>
       <c r="L506" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="507" spans="1:12">
@@ -25841,7 +25856,7 @@
         <v>2369</v>
       </c>
       <c r="L510" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="511" spans="1:12">
@@ -25876,7 +25891,7 @@
         <v>2369</v>
       </c>
       <c r="L511" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="512" spans="1:12">
@@ -25911,7 +25926,7 @@
         <v>2362</v>
       </c>
       <c r="L512" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="513" spans="1:12">
@@ -26051,7 +26066,7 @@
         <v>2421</v>
       </c>
       <c r="L516" t="s">
-        <v>2510</v>
+        <v>2511</v>
       </c>
     </row>
     <row r="517" spans="1:12">
@@ -26366,7 +26381,7 @@
         <v>2353</v>
       </c>
       <c r="L525" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="526" spans="1:12">
@@ -26401,7 +26416,7 @@
         <v>2389</v>
       </c>
       <c r="L526" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="527" spans="1:12">
@@ -26436,7 +26451,7 @@
         <v>2355</v>
       </c>
       <c r="L527" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="528" spans="1:12">
@@ -26471,7 +26486,7 @@
         <v>2421</v>
       </c>
       <c r="L528" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="529" spans="1:12">
@@ -26541,7 +26556,7 @@
         <v>2371</v>
       </c>
       <c r="L530" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="531" spans="1:12">
@@ -26754,7 +26769,7 @@
         <v>2370</v>
       </c>
       <c r="L536" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="537" spans="1:12">
@@ -26827,7 +26842,7 @@
         <v>2379</v>
       </c>
       <c r="L538" t="s">
-        <v>2490</v>
+        <v>2491</v>
       </c>
     </row>
     <row r="539" spans="1:12">
@@ -26967,7 +26982,7 @@
         <v>2435</v>
       </c>
       <c r="L542" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="543" spans="1:12">
@@ -27037,7 +27052,7 @@
         <v>2335</v>
       </c>
       <c r="L544" t="s">
-        <v>2489</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="545" spans="1:12">
@@ -27072,7 +27087,7 @@
         <v>2431</v>
       </c>
       <c r="L545" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="546" spans="1:12">
@@ -27390,7 +27405,7 @@
         <v>2352</v>
       </c>
       <c r="L554" t="s">
-        <v>2517</v>
+        <v>2519</v>
       </c>
     </row>
     <row r="555" spans="1:12">
@@ -27743,7 +27758,7 @@
         <v>2348</v>
       </c>
       <c r="L564" t="s">
-        <v>2493</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="565" spans="1:12">
@@ -27778,7 +27793,7 @@
         <v>2351</v>
       </c>
       <c r="L565" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="566" spans="1:12">
@@ -27813,7 +27828,7 @@
         <v>2351</v>
       </c>
       <c r="L566" t="s">
-        <v>2497</v>
+        <v>2498</v>
       </c>
     </row>
     <row r="567" spans="1:12">
@@ -27848,7 +27863,7 @@
         <v>2351</v>
       </c>
       <c r="L567" t="s">
-        <v>2518</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="568" spans="1:12">
@@ -28169,7 +28184,7 @@
         <v>2346</v>
       </c>
       <c r="L576" t="s">
-        <v>2489</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="577" spans="1:12">
@@ -29085,7 +29100,7 @@
         <v>2343</v>
       </c>
       <c r="L602" t="s">
-        <v>2504</v>
+        <v>2521</v>
       </c>
     </row>
     <row r="603" spans="1:12">
@@ -29269,7 +29284,7 @@
         <v>2356</v>
       </c>
       <c r="L607" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="608" spans="1:12">
@@ -29380,7 +29395,7 @@
         <v>2332</v>
       </c>
       <c r="L610" t="s">
-        <v>2519</v>
+        <v>2522</v>
       </c>
     </row>
     <row r="611" spans="1:12">
@@ -29663,7 +29678,7 @@
         <v>2357</v>
       </c>
       <c r="L618" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="619" spans="1:12">
@@ -29698,7 +29713,7 @@
         <v>2380</v>
       </c>
       <c r="L619" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="620" spans="1:12">
@@ -29873,7 +29888,7 @@
         <v>2370</v>
       </c>
       <c r="L624" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="625" spans="1:12">
@@ -29908,7 +29923,7 @@
         <v>2370</v>
       </c>
       <c r="L625" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="626" spans="1:12">
@@ -29981,7 +29996,7 @@
         <v>2339</v>
       </c>
       <c r="L627" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="628" spans="1:12">
@@ -30019,7 +30034,7 @@
         <v>2339</v>
       </c>
       <c r="L628" t="s">
-        <v>2520</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="629" spans="1:12">
@@ -30089,7 +30104,7 @@
         <v>2370</v>
       </c>
       <c r="L630" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="631" spans="1:12">
@@ -30238,7 +30253,7 @@
         <v>2359</v>
       </c>
       <c r="L634" t="s">
-        <v>2521</v>
+        <v>2524</v>
       </c>
     </row>
     <row r="635" spans="1:12">
@@ -30314,7 +30329,7 @@
         <v>2359</v>
       </c>
       <c r="L636" t="s">
-        <v>2462</v>
+        <v>2525</v>
       </c>
     </row>
     <row r="637" spans="1:12">
@@ -30349,7 +30364,7 @@
         <v>2351</v>
       </c>
       <c r="L637" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="638" spans="1:12">
@@ -30492,7 +30507,7 @@
         <v>2440</v>
       </c>
       <c r="L641" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="642" spans="1:12">
@@ -30527,7 +30542,7 @@
         <v>2370</v>
       </c>
       <c r="L642" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="643" spans="1:12">
@@ -30562,7 +30577,7 @@
         <v>2339</v>
       </c>
       <c r="L643" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="644" spans="1:12">
@@ -30600,7 +30615,7 @@
         <v>2359</v>
       </c>
       <c r="L644" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="645" spans="1:12">
@@ -30635,7 +30650,7 @@
         <v>2375</v>
       </c>
       <c r="L645" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="646" spans="1:12">
@@ -30670,7 +30685,7 @@
         <v>2329</v>
       </c>
       <c r="L646" t="s">
-        <v>2503</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="647" spans="1:12">
@@ -30740,7 +30755,7 @@
         <v>2442</v>
       </c>
       <c r="L648" t="s">
-        <v>2522</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="649" spans="1:12">
@@ -30775,7 +30790,7 @@
         <v>2442</v>
       </c>
       <c r="L649" t="s">
-        <v>2516</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="650" spans="1:12">
@@ -30807,7 +30822,7 @@
         <v>2443</v>
       </c>
       <c r="L650" t="s">
-        <v>2487</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="651" spans="1:12">
@@ -30839,7 +30854,7 @@
         <v>2443</v>
       </c>
       <c r="L651" t="s">
-        <v>2523</v>
+        <v>2528</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-28 18:30:04
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -15744,7 +15744,7 @@
         <v>1576</v>
       </c>
       <c r="I218" t="s">
-        <v>1608</v>
+        <v>1605</v>
       </c>
       <c r="J218" t="s">
         <v>1946</v>
@@ -31246,7 +31246,7 @@
         <v>1576</v>
       </c>
       <c r="I658" t="s">
-        <v>1608</v>
+        <v>1722</v>
       </c>
       <c r="J658" t="s">
         <v>2364</v>
@@ -31284,7 +31284,7 @@
         <v>1602</v>
       </c>
       <c r="I659" t="s">
-        <v>1608</v>
+        <v>1729</v>
       </c>
       <c r="J659" t="s">
         <v>2365</v>
@@ -31322,7 +31322,7 @@
         <v>1603</v>
       </c>
       <c r="I660" t="s">
-        <v>1608</v>
+        <v>1713</v>
       </c>
       <c r="J660" t="s">
         <v>2366</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-29 08:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6660" uniqueCount="2569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6660" uniqueCount="2570">
   <si>
     <t>NUCLEO</t>
   </si>
@@ -7654,57 +7654,57 @@
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
+    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
+  </si>
+  <si>
+    <t>FARMÁCIA,SAÚDE</t>
+  </si>
+  <si>
+    <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
+  </si>
+  <si>
+    <t>URBANISMO,MOBILIDADE E TRANSPORTE,RECURSOS HÍDRICOS,BIOLOGIA</t>
+  </si>
+  <si>
+    <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
+  </si>
+  <si>
+    <t>ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE</t>
+  </si>
+  <si>
+    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
+    <t>ECONOMIA,ECONOMICIDADE CONTÁBIL</t>
+  </si>
+  <si>
+    <t>RECURSOS HÍDRICOS,ECONOMICIDADE OBRAS</t>
+  </si>
+  <si>
+    <t>ENGENHARIA AMBIENTAL,ENGENHARIA FLORESTAL</t>
+  </si>
+  <si>
     <t>ECONOMICIDADE OBRAS,ECONOMICIDADE CONTÁBIL</t>
   </si>
   <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,GEOLOGIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,ENGENHARIA QUÍMICA,FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
-  </si>
-  <si>
-    <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,PATRIMÔNIO HISTÓRICO E CULTURAL</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>ENGENHARIA FLORESTAL,URBANISMO</t>
-  </si>
-  <si>
-    <t>FARMÁCIA,SAÚDE</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,ENGENHARIA AMBIENTAL</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMICIDADE OBRAS</t>
-  </si>
-  <si>
-    <t>URBANISMO,ENGENHARIA FLORESTAL</t>
-  </si>
-  <si>
-    <t>MOBILIDADE E TRANSPORTE,BIOLOGIA,RECURSOS HÍDRICOS,URBANISMO</t>
-  </si>
-  <si>
-    <t>ENGENHARIA CIVIL,MOBILIDADE E TRANSPORTE</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL</t>
-  </si>
-  <si>
-    <t>ECONOMICIDADE CONTÁBIL,ECONOMIA</t>
-  </si>
-  <si>
-    <t>ENGENHARIA AMBIENTAL,ENGENHARIA FLORESTAL</t>
-  </si>
-  <si>
     <t>GEOLOGIA,VALORAÇÃO DANOS AMBIENTAIS</t>
   </si>
   <si>
@@ -7717,10 +7717,13 @@
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,EDIFICAÇÕES</t>
   </si>
   <si>
+    <t>ASSISTÊNCIA SOCIAL,SAÚDE</t>
+  </si>
+  <si>
     <t>GEOTECNIA,ENGENHARIA CIVIL</t>
   </si>
   <si>
-    <t>ECONOMIA,PSICOLOGIA,SAÚDE,AVALIAÇÃO DE IMÓVEIS,ECONOMICIDADE CONTÁBIL,MOBILIDADE E TRANSPORTE,URBANISMO,ASSISTÊNCIA SOCIAL,ORÇAMENTO,SAÚDE MENTAL</t>
+    <t>URBANISMO,ORÇAMENTO,ECONOMIA,PSICOLOGIA,SAÚDE,SAÚDE MENTAL,AVALIAÇÃO DE IMÓVEIS,MOBILIDADE E TRANSPORTE,ASSISTÊNCIA SOCIAL,ECONOMICIDADE CONTÁBIL</t>
   </si>
 </sst>
 </file>
@@ -22070,7 +22073,7 @@
         <v>2391</v>
       </c>
       <c r="L399" t="s">
-        <v>2555</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="400" spans="1:12">
@@ -22560,7 +22563,7 @@
         <v>2409</v>
       </c>
       <c r="L413" t="s">
-        <v>2556</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="414" spans="1:12">
@@ -22875,7 +22878,7 @@
         <v>2393</v>
       </c>
       <c r="L422" t="s">
-        <v>2557</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="423" spans="1:12">
@@ -23680,7 +23683,7 @@
         <v>2463</v>
       </c>
       <c r="L445" t="s">
-        <v>2558</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="446" spans="1:12">
@@ -24847,7 +24850,7 @@
         <v>2401</v>
       </c>
       <c r="L478" t="s">
-        <v>2559</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="479" spans="1:12">
@@ -25305,7 +25308,7 @@
         <v>2391</v>
       </c>
       <c r="L491" t="s">
-        <v>2560</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="492" spans="1:12">
@@ -27242,7 +27245,7 @@
         <v>2389</v>
       </c>
       <c r="L546" t="s">
-        <v>2561</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="547" spans="1:12">
@@ -27665,7 +27668,7 @@
         <v>2388</v>
       </c>
       <c r="L558" t="s">
-        <v>2539</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="559" spans="1:12">
@@ -27700,7 +27703,7 @@
         <v>2388</v>
       </c>
       <c r="L559" t="s">
-        <v>2562</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="560" spans="1:12">
@@ -28902,7 +28905,7 @@
         <v>2380</v>
       </c>
       <c r="L593" t="s">
-        <v>2546</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="594" spans="1:12">
@@ -29164,7 +29167,7 @@
     </row>
     <row r="601" spans="1:12">
       <c r="A601" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="B601" t="s">
         <v>644</v>
@@ -29188,7 +29191,7 @@
         <v>1583</v>
       </c>
       <c r="I601" t="s">
-        <v>1623</v>
+        <v>1601</v>
       </c>
       <c r="J601" t="s">
         <v>2303</v>
@@ -31158,7 +31161,7 @@
         <v>2406</v>
       </c>
       <c r="L656" t="s">
-        <v>2545</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="657" spans="1:12">
@@ -31333,7 +31336,7 @@
         <v>2485</v>
       </c>
       <c r="L661" t="s">
-        <v>2567</v>
+        <v>2568</v>
       </c>
     </row>
     <row r="662" spans="1:12">
@@ -31365,7 +31368,7 @@
         <v>2485</v>
       </c>
       <c r="L662" t="s">
-        <v>2568</v>
+        <v>2569</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-30 14:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -76,6 +76,9 @@
     <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS</t>
   </si>
   <si>
+    <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO, SECRETARIA GERAL DO GATE</t>
+  </si>
+  <si>
     <t>NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ENGENHARIA</t>
   </si>
   <si>
@@ -145,9 +148,6 @@
     <t>NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE ECONOMIA</t>
   </si>
   <si>
-    <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO, SECRETARIA GERAL DO GATE</t>
-  </si>
-  <si>
     <t>NÚCLEO TÉCNICO DE ARQUITETURA E URBANISMO,NÚCLEO TÉCNICO DE CIÊNCIA DE DADOS,NÚCLEO TÉCNICO DE CIÊNCIAS NATURAIS,NÚCLEO TÉCNICO DE ENGENHARIA,NÚCLEO TÉCNICO DE POLÍTICAS PÚBLICAS</t>
   </si>
   <si>
@@ -4831,7 +4831,7 @@
     <t>ELIANA MIRANDA ARAUJO DA SILVA SOARES,RODRIGO VENTURA MARRA</t>
   </si>
   <si>
-    <t>LILIAN ALVES DE ARAUJO,SIMONE MANNHEIMER DE ALVARENGA</t>
+    <t>LILIAN ALVES DE ARAUJO, _SEM USUARIO ATRIBUIDO</t>
   </si>
   <si>
     <t>CASSIA CRISTINA DA SILVA</t>
@@ -9990,7 +9990,7 @@
     </row>
     <row r="56" spans="1:12">
       <c r="A56" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B56" t="s">
         <v>100</v>
@@ -10095,7 +10095,7 @@
     </row>
     <row r="59" spans="1:12">
       <c r="A59" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B59" t="s">
         <v>103</v>
@@ -10305,7 +10305,7 @@
     </row>
     <row r="65" spans="1:12">
       <c r="A65" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B65" t="s">
         <v>109</v>
@@ -10445,7 +10445,7 @@
     </row>
     <row r="69" spans="1:12">
       <c r="A69" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B69" t="s">
         <v>113</v>
@@ -10620,7 +10620,7 @@
     </row>
     <row r="74" spans="1:12">
       <c r="A74" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B74" t="s">
         <v>118</v>
@@ -10655,7 +10655,7 @@
     </row>
     <row r="75" spans="1:12">
       <c r="A75" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B75" t="s">
         <v>119</v>
@@ -10725,7 +10725,7 @@
     </row>
     <row r="77" spans="1:12">
       <c r="A77" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B77" t="s">
         <v>120</v>
@@ -10795,7 +10795,7 @@
     </row>
     <row r="79" spans="1:12">
       <c r="A79" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B79" t="s">
         <v>122</v>
@@ -10830,7 +10830,7 @@
     </row>
     <row r="80" spans="1:12">
       <c r="A80" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B80" t="s">
         <v>123</v>
@@ -10865,7 +10865,7 @@
     </row>
     <row r="81" spans="1:12">
       <c r="A81" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B81" t="s">
         <v>124</v>
@@ -10900,7 +10900,7 @@
     </row>
     <row r="82" spans="1:12">
       <c r="A82" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B82" t="s">
         <v>125</v>
@@ -11145,7 +11145,7 @@
     </row>
     <row r="89" spans="1:12">
       <c r="A89" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B89" t="s">
         <v>132</v>
@@ -11285,7 +11285,7 @@
     </row>
     <row r="93" spans="1:12">
       <c r="A93" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B93" t="s">
         <v>136</v>
@@ -11390,7 +11390,7 @@
     </row>
     <row r="96" spans="1:12">
       <c r="A96" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B96" t="s">
         <v>139</v>
@@ -11495,7 +11495,7 @@
     </row>
     <row r="99" spans="1:12">
       <c r="A99" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B99" t="s">
         <v>142</v>
@@ -11635,7 +11635,7 @@
     </row>
     <row r="103" spans="1:12">
       <c r="A103" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B103" t="s">
         <v>146</v>
@@ -11775,7 +11775,7 @@
     </row>
     <row r="107" spans="1:12">
       <c r="A107" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B107" t="s">
         <v>150</v>
@@ -11845,7 +11845,7 @@
     </row>
     <row r="109" spans="1:12">
       <c r="A109" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B109" t="s">
         <v>152</v>
@@ -11880,7 +11880,7 @@
     </row>
     <row r="110" spans="1:12">
       <c r="A110" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B110" t="s">
         <v>153</v>
@@ -12160,7 +12160,7 @@
     </row>
     <row r="118" spans="1:12">
       <c r="A118" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B118" t="s">
         <v>161</v>
@@ -12265,7 +12265,7 @@
     </row>
     <row r="121" spans="1:12">
       <c r="A121" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B121" t="s">
         <v>164</v>
@@ -12335,7 +12335,7 @@
     </row>
     <row r="123" spans="1:12">
       <c r="A123" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B123" t="s">
         <v>166</v>
@@ -12370,7 +12370,7 @@
     </row>
     <row r="124" spans="1:12">
       <c r="A124" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B124" t="s">
         <v>167</v>
@@ -12405,7 +12405,7 @@
     </row>
     <row r="125" spans="1:12">
       <c r="A125" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B125" t="s">
         <v>168</v>
@@ -12510,7 +12510,7 @@
     </row>
     <row r="128" spans="1:12">
       <c r="A128" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B128" t="s">
         <v>171</v>
@@ -12720,7 +12720,7 @@
     </row>
     <row r="134" spans="1:12">
       <c r="A134" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B134" t="s">
         <v>177</v>
@@ -12790,7 +12790,7 @@
     </row>
     <row r="136" spans="1:12">
       <c r="A136" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B136" t="s">
         <v>179</v>
@@ -12825,7 +12825,7 @@
     </row>
     <row r="137" spans="1:12">
       <c r="A137" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B137" t="s">
         <v>180</v>
@@ -12860,7 +12860,7 @@
     </row>
     <row r="138" spans="1:12">
       <c r="A138" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B138" t="s">
         <v>181</v>
@@ -12933,7 +12933,7 @@
     </row>
     <row r="140" spans="1:12">
       <c r="A140" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B140" t="s">
         <v>183</v>
@@ -13003,7 +13003,7 @@
     </row>
     <row r="142" spans="1:12">
       <c r="A142" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B142" t="s">
         <v>185</v>
@@ -13038,7 +13038,7 @@
     </row>
     <row r="143" spans="1:12">
       <c r="A143" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B143" t="s">
         <v>186</v>
@@ -13073,7 +13073,7 @@
     </row>
     <row r="144" spans="1:12">
       <c r="A144" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B144" t="s">
         <v>187</v>
@@ -13213,7 +13213,7 @@
     </row>
     <row r="148" spans="1:12">
       <c r="A148" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B148" t="s">
         <v>191</v>
@@ -13248,7 +13248,7 @@
     </row>
     <row r="149" spans="1:12">
       <c r="A149" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B149" t="s">
         <v>192</v>
@@ -13493,7 +13493,7 @@
     </row>
     <row r="156" spans="1:12">
       <c r="A156" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B156" t="s">
         <v>199</v>
@@ -13528,7 +13528,7 @@
     </row>
     <row r="157" spans="1:12">
       <c r="A157" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B157" t="s">
         <v>200</v>
@@ -13633,7 +13633,7 @@
     </row>
     <row r="160" spans="1:12">
       <c r="A160" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B160" t="s">
         <v>203</v>
@@ -13668,7 +13668,7 @@
     </row>
     <row r="161" spans="1:12">
       <c r="A161" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B161" t="s">
         <v>204</v>
@@ -14158,7 +14158,7 @@
     </row>
     <row r="175" spans="1:12">
       <c r="A175" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B175" t="s">
         <v>218</v>
@@ -14263,7 +14263,7 @@
     </row>
     <row r="178" spans="1:12">
       <c r="A178" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B178" t="s">
         <v>221</v>
@@ -14368,7 +14368,7 @@
     </row>
     <row r="181" spans="1:12">
       <c r="A181" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B181" t="s">
         <v>224</v>
@@ -14438,7 +14438,7 @@
     </row>
     <row r="183" spans="1:12">
       <c r="A183" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B183" t="s">
         <v>226</v>
@@ -14473,7 +14473,7 @@
     </row>
     <row r="184" spans="1:12">
       <c r="A184" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B184" t="s">
         <v>227</v>
@@ -14508,7 +14508,7 @@
     </row>
     <row r="185" spans="1:12">
       <c r="A185" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B185" t="s">
         <v>228</v>
@@ -14543,7 +14543,7 @@
     </row>
     <row r="186" spans="1:12">
       <c r="A186" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B186" t="s">
         <v>229</v>
@@ -14578,7 +14578,7 @@
     </row>
     <row r="187" spans="1:12">
       <c r="A187" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B187" t="s">
         <v>230</v>
@@ -14753,7 +14753,7 @@
     </row>
     <row r="192" spans="1:12">
       <c r="A192" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B192" t="s">
         <v>235</v>
@@ -14858,7 +14858,7 @@
     </row>
     <row r="195" spans="1:12">
       <c r="A195" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B195" t="s">
         <v>238</v>
@@ -15068,7 +15068,7 @@
     </row>
     <row r="201" spans="1:12">
       <c r="A201" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B201" t="s">
         <v>244</v>
@@ -15103,7 +15103,7 @@
     </row>
     <row r="202" spans="1:12">
       <c r="A202" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B202" t="s">
         <v>245</v>
@@ -15386,7 +15386,7 @@
     </row>
     <row r="210" spans="1:12">
       <c r="A210" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B210" t="s">
         <v>253</v>
@@ -15561,7 +15561,7 @@
     </row>
     <row r="215" spans="1:12">
       <c r="A215" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B215" t="s">
         <v>258</v>
@@ -15806,7 +15806,7 @@
     </row>
     <row r="222" spans="1:12">
       <c r="A222" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B222" t="s">
         <v>265</v>
@@ -15841,7 +15841,7 @@
     </row>
     <row r="223" spans="1:12">
       <c r="A223" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B223" t="s">
         <v>266</v>
@@ -15911,7 +15911,7 @@
     </row>
     <row r="225" spans="1:12">
       <c r="A225" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B225" t="s">
         <v>268</v>
@@ -16016,7 +16016,7 @@
     </row>
     <row r="228" spans="1:12">
       <c r="A228" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B228" t="s">
         <v>271</v>
@@ -16086,7 +16086,7 @@
     </row>
     <row r="230" spans="1:12">
       <c r="A230" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B230" t="s">
         <v>273</v>
@@ -16191,7 +16191,7 @@
     </row>
     <row r="233" spans="1:12">
       <c r="A233" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B233" t="s">
         <v>276</v>
@@ -16681,7 +16681,7 @@
     </row>
     <row r="247" spans="1:12">
       <c r="A247" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B247" t="s">
         <v>290</v>
@@ -16751,7 +16751,7 @@
     </row>
     <row r="249" spans="1:12">
       <c r="A249" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B249" t="s">
         <v>292</v>
@@ -16891,7 +16891,7 @@
     </row>
     <row r="253" spans="1:12">
       <c r="A253" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B253" t="s">
         <v>296</v>
@@ -17031,7 +17031,7 @@
     </row>
     <row r="257" spans="1:12">
       <c r="A257" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B257" t="s">
         <v>300</v>
@@ -17066,7 +17066,7 @@
     </row>
     <row r="258" spans="1:12">
       <c r="A258" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B258" t="s">
         <v>301</v>
@@ -17171,7 +17171,7 @@
     </row>
     <row r="261" spans="1:12">
       <c r="A261" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B261" t="s">
         <v>304</v>
@@ -17206,7 +17206,7 @@
     </row>
     <row r="262" spans="1:12">
       <c r="A262" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B262" t="s">
         <v>305</v>
@@ -17314,7 +17314,7 @@
     </row>
     <row r="265" spans="1:12">
       <c r="A265" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B265" t="s">
         <v>308</v>
@@ -17384,7 +17384,7 @@
     </row>
     <row r="267" spans="1:12">
       <c r="A267" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B267" t="s">
         <v>310</v>
@@ -17454,7 +17454,7 @@
     </row>
     <row r="269" spans="1:12">
       <c r="A269" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B269" t="s">
         <v>312</v>
@@ -17559,7 +17559,7 @@
     </row>
     <row r="272" spans="1:12">
       <c r="A272" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B272" t="s">
         <v>315</v>
@@ -17629,7 +17629,7 @@
     </row>
     <row r="274" spans="1:12">
       <c r="A274" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B274" t="s">
         <v>317</v>
@@ -17664,7 +17664,7 @@
     </row>
     <row r="275" spans="1:12">
       <c r="A275" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B275" t="s">
         <v>318</v>
@@ -17734,7 +17734,7 @@
     </row>
     <row r="277" spans="1:12">
       <c r="A277" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B277" t="s">
         <v>320</v>
@@ -17769,7 +17769,7 @@
     </row>
     <row r="278" spans="1:12">
       <c r="A278" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B278" t="s">
         <v>321</v>
@@ -17804,7 +17804,7 @@
     </row>
     <row r="279" spans="1:12">
       <c r="A279" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B279" t="s">
         <v>322</v>
@@ -17839,7 +17839,7 @@
     </row>
     <row r="280" spans="1:12">
       <c r="A280" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B280" t="s">
         <v>323</v>
@@ -18017,7 +18017,7 @@
     </row>
     <row r="285" spans="1:12">
       <c r="A285" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B285" t="s">
         <v>328</v>
@@ -18052,7 +18052,7 @@
     </row>
     <row r="286" spans="1:12">
       <c r="A286" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B286" t="s">
         <v>329</v>
@@ -18087,7 +18087,7 @@
     </row>
     <row r="287" spans="1:12">
       <c r="A287" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B287" t="s">
         <v>330</v>
@@ -18227,7 +18227,7 @@
     </row>
     <row r="291" spans="1:12">
       <c r="A291" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B291" t="s">
         <v>334</v>
@@ -18262,7 +18262,7 @@
     </row>
     <row r="292" spans="1:12">
       <c r="A292" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B292" t="s">
         <v>335</v>
@@ -18297,7 +18297,7 @@
     </row>
     <row r="293" spans="1:12">
       <c r="A293" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B293" t="s">
         <v>336</v>
@@ -18367,7 +18367,7 @@
     </row>
     <row r="295" spans="1:12">
       <c r="A295" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B295" t="s">
         <v>338</v>
@@ -19207,7 +19207,7 @@
     </row>
     <row r="319" spans="1:12">
       <c r="A319" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B319" t="s">
         <v>362</v>
@@ -19242,7 +19242,7 @@
     </row>
     <row r="320" spans="1:12">
       <c r="A320" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B320" t="s">
         <v>363</v>
@@ -19347,7 +19347,7 @@
     </row>
     <row r="323" spans="1:12">
       <c r="A323" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B323" t="s">
         <v>366</v>
@@ -19382,7 +19382,7 @@
     </row>
     <row r="324" spans="1:12">
       <c r="A324" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B324" t="s">
         <v>367</v>
@@ -19417,7 +19417,7 @@
     </row>
     <row r="325" spans="1:12">
       <c r="A325" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B325" t="s">
         <v>367</v>
@@ -19452,7 +19452,7 @@
     </row>
     <row r="326" spans="1:12">
       <c r="A326" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B326" t="s">
         <v>368</v>
@@ -19522,7 +19522,7 @@
     </row>
     <row r="328" spans="1:12">
       <c r="A328" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B328" t="s">
         <v>370</v>
@@ -19630,7 +19630,7 @@
     </row>
     <row r="331" spans="1:12">
       <c r="A331" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B331" t="s">
         <v>373</v>
@@ -19665,7 +19665,7 @@
     </row>
     <row r="332" spans="1:12">
       <c r="A332" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B332" t="s">
         <v>374</v>
@@ -19700,7 +19700,7 @@
     </row>
     <row r="333" spans="1:12">
       <c r="A333" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B333" t="s">
         <v>375</v>
@@ -19773,7 +19773,7 @@
     </row>
     <row r="335" spans="1:12">
       <c r="A335" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B335" t="s">
         <v>377</v>
@@ -19808,7 +19808,7 @@
     </row>
     <row r="336" spans="1:12">
       <c r="A336" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B336" t="s">
         <v>378</v>
@@ -19983,7 +19983,7 @@
     </row>
     <row r="341" spans="1:12">
       <c r="A341" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B341" t="s">
         <v>383</v>
@@ -20018,7 +20018,7 @@
     </row>
     <row r="342" spans="1:12">
       <c r="A342" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B342" t="s">
         <v>384</v>
@@ -20158,7 +20158,7 @@
     </row>
     <row r="346" spans="1:12">
       <c r="A346" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B346" t="s">
         <v>388</v>
@@ -20193,7 +20193,7 @@
     </row>
     <row r="347" spans="1:12">
       <c r="A347" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B347" t="s">
         <v>389</v>
@@ -20438,7 +20438,7 @@
     </row>
     <row r="354" spans="1:12">
       <c r="A354" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B354" t="s">
         <v>395</v>
@@ -20473,7 +20473,7 @@
     </row>
     <row r="355" spans="1:12">
       <c r="A355" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B355" t="s">
         <v>396</v>
@@ -20508,7 +20508,7 @@
     </row>
     <row r="356" spans="1:12">
       <c r="A356" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B356" t="s">
         <v>397</v>
@@ -20543,7 +20543,7 @@
     </row>
     <row r="357" spans="1:12">
       <c r="A357" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B357" t="s">
         <v>398</v>
@@ -20578,7 +20578,7 @@
     </row>
     <row r="358" spans="1:12">
       <c r="A358" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B358" t="s">
         <v>399</v>
@@ -20613,7 +20613,7 @@
     </row>
     <row r="359" spans="1:12">
       <c r="A359" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B359" t="s">
         <v>400</v>
@@ -20683,7 +20683,7 @@
     </row>
     <row r="361" spans="1:12">
       <c r="A361" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B361" t="s">
         <v>402</v>
@@ -20753,7 +20753,7 @@
     </row>
     <row r="363" spans="1:12">
       <c r="A363" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B363" t="s">
         <v>404</v>
@@ -20788,7 +20788,7 @@
     </row>
     <row r="364" spans="1:12">
       <c r="A364" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B364" t="s">
         <v>405</v>
@@ -20823,7 +20823,7 @@
     </row>
     <row r="365" spans="1:12">
       <c r="A365" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B365" t="s">
         <v>406</v>
@@ -20858,7 +20858,7 @@
     </row>
     <row r="366" spans="1:12">
       <c r="A366" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B366" t="s">
         <v>407</v>
@@ -20963,7 +20963,7 @@
     </row>
     <row r="369" spans="1:12">
       <c r="A369" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B369" t="s">
         <v>410</v>
@@ -21068,7 +21068,7 @@
     </row>
     <row r="372" spans="1:12">
       <c r="A372" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B372" t="s">
         <v>413</v>
@@ -21103,7 +21103,7 @@
     </row>
     <row r="373" spans="1:12">
       <c r="A373" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B373" t="s">
         <v>414</v>
@@ -21138,7 +21138,7 @@
     </row>
     <row r="374" spans="1:12">
       <c r="A374" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B374" t="s">
         <v>415</v>
@@ -21173,7 +21173,7 @@
     </row>
     <row r="375" spans="1:12">
       <c r="A375" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B375" t="s">
         <v>416</v>
@@ -21208,7 +21208,7 @@
     </row>
     <row r="376" spans="1:12">
       <c r="A376" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B376" t="s">
         <v>417</v>
@@ -21278,7 +21278,7 @@
     </row>
     <row r="378" spans="1:12">
       <c r="A378" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B378" t="s">
         <v>419</v>
@@ -21313,7 +21313,7 @@
     </row>
     <row r="379" spans="1:12">
       <c r="A379" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B379" t="s">
         <v>420</v>
@@ -21386,7 +21386,7 @@
     </row>
     <row r="381" spans="1:12">
       <c r="A381" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B381" t="s">
         <v>422</v>
@@ -21456,7 +21456,7 @@
     </row>
     <row r="383" spans="1:12">
       <c r="A383" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B383" t="s">
         <v>424</v>
@@ -21491,7 +21491,7 @@
     </row>
     <row r="384" spans="1:12">
       <c r="A384" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B384" t="s">
         <v>425</v>
@@ -21526,7 +21526,7 @@
     </row>
     <row r="385" spans="1:12">
       <c r="A385" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B385" t="s">
         <v>426</v>
@@ -21631,7 +21631,7 @@
     </row>
     <row r="388" spans="1:12">
       <c r="A388" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B388" t="s">
         <v>429</v>
@@ -21736,7 +21736,7 @@
     </row>
     <row r="391" spans="1:12">
       <c r="A391" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B391" t="s">
         <v>432</v>
@@ -21771,7 +21771,7 @@
     </row>
     <row r="392" spans="1:12">
       <c r="A392" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B392" t="s">
         <v>433</v>
@@ -21946,7 +21946,7 @@
     </row>
     <row r="397" spans="1:12">
       <c r="A397" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B397" t="s">
         <v>438</v>
@@ -22086,7 +22086,7 @@
     </row>
     <row r="401" spans="1:12">
       <c r="A401" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B401" t="s">
         <v>442</v>
@@ -22156,7 +22156,7 @@
     </row>
     <row r="403" spans="1:12">
       <c r="A403" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B403" t="s">
         <v>444</v>
@@ -22226,7 +22226,7 @@
     </row>
     <row r="405" spans="1:12">
       <c r="A405" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B405" t="s">
         <v>446</v>
@@ -22261,7 +22261,7 @@
     </row>
     <row r="406" spans="1:12">
       <c r="A406" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B406" t="s">
         <v>447</v>
@@ -22506,7 +22506,7 @@
     </row>
     <row r="413" spans="1:12">
       <c r="A413" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B413" t="s">
         <v>454</v>
@@ -22576,7 +22576,7 @@
     </row>
     <row r="415" spans="1:12">
       <c r="A415" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B415" t="s">
         <v>456</v>
@@ -22611,7 +22611,7 @@
     </row>
     <row r="416" spans="1:12">
       <c r="A416" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B416" t="s">
         <v>457</v>
@@ -22681,7 +22681,7 @@
     </row>
     <row r="418" spans="1:12">
       <c r="A418" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B418" t="s">
         <v>459</v>
@@ -22751,7 +22751,7 @@
     </row>
     <row r="420" spans="1:12">
       <c r="A420" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B420" t="s">
         <v>461</v>
@@ -22891,7 +22891,7 @@
     </row>
     <row r="424" spans="1:12">
       <c r="A424" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B424" t="s">
         <v>465</v>
@@ -22961,7 +22961,7 @@
     </row>
     <row r="426" spans="1:12">
       <c r="A426" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B426" t="s">
         <v>467</v>
@@ -23031,7 +23031,7 @@
     </row>
     <row r="428" spans="1:12">
       <c r="A428" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B428" t="s">
         <v>469</v>
@@ -23066,7 +23066,7 @@
     </row>
     <row r="429" spans="1:12">
       <c r="A429" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B429" t="s">
         <v>470</v>
@@ -23101,7 +23101,7 @@
     </row>
     <row r="430" spans="1:12">
       <c r="A430" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B430" t="s">
         <v>471</v>
@@ -23171,7 +23171,7 @@
     </row>
     <row r="432" spans="1:12">
       <c r="A432" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B432" t="s">
         <v>473</v>
@@ -23206,7 +23206,7 @@
     </row>
     <row r="433" spans="1:12">
       <c r="A433" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B433" t="s">
         <v>474</v>
@@ -23241,7 +23241,7 @@
     </row>
     <row r="434" spans="1:12">
       <c r="A434" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B434" t="s">
         <v>475</v>
@@ -23276,7 +23276,7 @@
     </row>
     <row r="435" spans="1:12">
       <c r="A435" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B435" t="s">
         <v>476</v>
@@ -23311,7 +23311,7 @@
     </row>
     <row r="436" spans="1:12">
       <c r="A436" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B436" t="s">
         <v>477</v>
@@ -23381,7 +23381,7 @@
     </row>
     <row r="438" spans="1:12">
       <c r="A438" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B438" t="s">
         <v>479</v>
@@ -23486,7 +23486,7 @@
     </row>
     <row r="441" spans="1:12">
       <c r="A441" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B441" t="s">
         <v>482</v>
@@ -23556,7 +23556,7 @@
     </row>
     <row r="443" spans="1:12">
       <c r="A443" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B443" t="s">
         <v>484</v>
@@ -23629,7 +23629,7 @@
     </row>
     <row r="445" spans="1:12">
       <c r="A445" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B445" t="s">
         <v>486</v>
@@ -23667,7 +23667,7 @@
     </row>
     <row r="446" spans="1:12">
       <c r="A446" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B446" t="s">
         <v>487</v>
@@ -23702,7 +23702,7 @@
     </row>
     <row r="447" spans="1:12">
       <c r="A447" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B447" t="s">
         <v>488</v>
@@ -23880,7 +23880,7 @@
     </row>
     <row r="452" spans="1:12">
       <c r="A452" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B452" t="s">
         <v>493</v>
@@ -23915,7 +23915,7 @@
     </row>
     <row r="453" spans="1:12">
       <c r="A453" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B453" t="s">
         <v>494</v>
@@ -23950,7 +23950,7 @@
     </row>
     <row r="454" spans="1:12">
       <c r="A454" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B454" t="s">
         <v>495</v>
@@ -23985,7 +23985,7 @@
     </row>
     <row r="455" spans="1:12">
       <c r="A455" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B455" t="s">
         <v>496</v>
@@ -24023,7 +24023,7 @@
     </row>
     <row r="456" spans="1:12">
       <c r="A456" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B456" t="s">
         <v>497</v>
@@ -24128,7 +24128,7 @@
     </row>
     <row r="459" spans="1:12">
       <c r="A459" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B459" t="s">
         <v>499</v>
@@ -24163,7 +24163,7 @@
     </row>
     <row r="460" spans="1:12">
       <c r="A460" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B460" t="s">
         <v>500</v>
@@ -24233,7 +24233,7 @@
     </row>
     <row r="462" spans="1:12">
       <c r="A462" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B462" t="s">
         <v>502</v>
@@ -24268,7 +24268,7 @@
     </row>
     <row r="463" spans="1:12">
       <c r="A463" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B463" t="s">
         <v>503</v>
@@ -24303,7 +24303,7 @@
     </row>
     <row r="464" spans="1:12">
       <c r="A464" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B464" t="s">
         <v>504</v>
@@ -24338,7 +24338,7 @@
     </row>
     <row r="465" spans="1:12">
       <c r="A465" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B465" t="s">
         <v>505</v>
@@ -24373,7 +24373,7 @@
     </row>
     <row r="466" spans="1:12">
       <c r="A466" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B466" t="s">
         <v>506</v>
@@ -24408,7 +24408,7 @@
     </row>
     <row r="467" spans="1:12">
       <c r="A467" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B467" t="s">
         <v>507</v>
@@ -24478,7 +24478,7 @@
     </row>
     <row r="469" spans="1:12">
       <c r="A469" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B469" t="s">
         <v>509</v>
@@ -24548,7 +24548,7 @@
     </row>
     <row r="471" spans="1:12">
       <c r="A471" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B471" t="s">
         <v>511</v>
@@ -24618,7 +24618,7 @@
     </row>
     <row r="473" spans="1:12">
       <c r="A473" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B473" t="s">
         <v>513</v>
@@ -24688,7 +24688,7 @@
     </row>
     <row r="475" spans="1:12">
       <c r="A475" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B475" t="s">
         <v>515</v>
@@ -24723,7 +24723,7 @@
     </row>
     <row r="476" spans="1:12">
       <c r="A476" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B476" t="s">
         <v>516</v>
@@ -24796,7 +24796,7 @@
     </row>
     <row r="478" spans="1:12">
       <c r="A478" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B478" t="s">
         <v>518</v>
@@ -24866,7 +24866,7 @@
     </row>
     <row r="480" spans="1:12">
       <c r="A480" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B480" t="s">
         <v>520</v>
@@ -24936,7 +24936,7 @@
     </row>
     <row r="482" spans="1:12">
       <c r="A482" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B482" t="s">
         <v>522</v>
@@ -24971,7 +24971,7 @@
     </row>
     <row r="483" spans="1:12">
       <c r="A483" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B483" t="s">
         <v>523</v>
@@ -25006,7 +25006,7 @@
     </row>
     <row r="484" spans="1:12">
       <c r="A484" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B484" t="s">
         <v>524</v>
@@ -25076,7 +25076,7 @@
     </row>
     <row r="486" spans="1:12">
       <c r="A486" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B486" t="s">
         <v>526</v>
@@ -25111,7 +25111,7 @@
     </row>
     <row r="487" spans="1:12">
       <c r="A487" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B487" t="s">
         <v>527</v>
@@ -25146,7 +25146,7 @@
     </row>
     <row r="488" spans="1:12">
       <c r="A488" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B488" t="s">
         <v>528</v>
@@ -25181,7 +25181,7 @@
     </row>
     <row r="489" spans="1:12">
       <c r="A489" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B489" t="s">
         <v>529</v>
@@ -25216,7 +25216,7 @@
     </row>
     <row r="490" spans="1:12">
       <c r="A490" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B490" t="s">
         <v>530</v>
@@ -25359,7 +25359,7 @@
     </row>
     <row r="494" spans="1:12">
       <c r="A494" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B494" t="s">
         <v>534</v>
@@ -25464,7 +25464,7 @@
     </row>
     <row r="497" spans="1:12">
       <c r="A497" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B497" t="s">
         <v>537</v>
@@ -25499,7 +25499,7 @@
     </row>
     <row r="498" spans="1:12">
       <c r="A498" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B498" t="s">
         <v>538</v>
@@ -25534,7 +25534,7 @@
     </row>
     <row r="499" spans="1:12">
       <c r="A499" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B499" t="s">
         <v>539</v>
@@ -25569,7 +25569,7 @@
     </row>
     <row r="500" spans="1:12">
       <c r="A500" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B500" t="s">
         <v>540</v>
@@ -25779,7 +25779,7 @@
     </row>
     <row r="506" spans="1:12">
       <c r="A506" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B506" t="s">
         <v>546</v>
@@ -25814,7 +25814,7 @@
     </row>
     <row r="507" spans="1:12">
       <c r="A507" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B507" t="s">
         <v>547</v>
@@ -25849,7 +25849,7 @@
     </row>
     <row r="508" spans="1:12">
       <c r="A508" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B508" t="s">
         <v>548</v>
@@ -25884,7 +25884,7 @@
     </row>
     <row r="509" spans="1:12">
       <c r="A509" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B509" t="s">
         <v>549</v>
@@ -25919,7 +25919,7 @@
     </row>
     <row r="510" spans="1:12">
       <c r="A510" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B510" t="s">
         <v>550</v>
@@ -25954,7 +25954,7 @@
     </row>
     <row r="511" spans="1:12">
       <c r="A511" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B511" t="s">
         <v>551</v>
@@ -25989,7 +25989,7 @@
     </row>
     <row r="512" spans="1:12">
       <c r="A512" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B512" t="s">
         <v>552</v>
@@ -26024,7 +26024,7 @@
     </row>
     <row r="513" spans="1:12">
       <c r="A513" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B513" t="s">
         <v>553</v>
@@ -26097,7 +26097,7 @@
     </row>
     <row r="515" spans="1:12">
       <c r="A515" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B515" t="s">
         <v>555</v>
@@ -26132,7 +26132,7 @@
     </row>
     <row r="516" spans="1:12">
       <c r="A516" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B516" t="s">
         <v>556</v>
@@ -26202,7 +26202,7 @@
     </row>
     <row r="518" spans="1:12">
       <c r="A518" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B518" t="s">
         <v>558</v>
@@ -26237,7 +26237,7 @@
     </row>
     <row r="519" spans="1:12">
       <c r="A519" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B519" t="s">
         <v>559</v>
@@ -26272,7 +26272,7 @@
     </row>
     <row r="520" spans="1:12">
       <c r="A520" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B520" t="s">
         <v>560</v>
@@ -26342,7 +26342,7 @@
     </row>
     <row r="522" spans="1:12">
       <c r="A522" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B522" t="s">
         <v>562</v>
@@ -26377,7 +26377,7 @@
     </row>
     <row r="523" spans="1:12">
       <c r="A523" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B523" t="s">
         <v>563</v>
@@ -26412,7 +26412,7 @@
     </row>
     <row r="524" spans="1:12">
       <c r="A524" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B524" t="s">
         <v>564</v>
@@ -26447,7 +26447,7 @@
     </row>
     <row r="525" spans="1:12">
       <c r="A525" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B525" t="s">
         <v>565</v>
@@ -26552,7 +26552,7 @@
     </row>
     <row r="528" spans="1:12">
       <c r="A528" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B528" t="s">
         <v>568</v>
@@ -26587,7 +26587,7 @@
     </row>
     <row r="529" spans="1:12">
       <c r="A529" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B529" t="s">
         <v>569</v>
@@ -26657,7 +26657,7 @@
     </row>
     <row r="531" spans="1:12">
       <c r="A531" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B531" t="s">
         <v>571</v>
@@ -26730,7 +26730,7 @@
     </row>
     <row r="533" spans="1:12">
       <c r="A533" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B533" t="s">
         <v>573</v>
@@ -26800,7 +26800,7 @@
     </row>
     <row r="535" spans="1:12">
       <c r="A535" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B535" t="s">
         <v>575</v>
@@ -27188,7 +27188,7 @@
     </row>
     <row r="546" spans="1:12">
       <c r="A546" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B546" t="s">
         <v>586</v>
@@ -27258,7 +27258,7 @@
     </row>
     <row r="548" spans="1:12">
       <c r="A548" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B548" t="s">
         <v>588</v>
@@ -27296,7 +27296,7 @@
     </row>
     <row r="549" spans="1:12">
       <c r="A549" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B549" t="s">
         <v>589</v>
@@ -27331,7 +27331,7 @@
     </row>
     <row r="550" spans="1:12">
       <c r="A550" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B550" t="s">
         <v>590</v>
@@ -27366,7 +27366,7 @@
     </row>
     <row r="551" spans="1:12">
       <c r="A551" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B551" t="s">
         <v>591</v>
@@ -27436,7 +27436,7 @@
     </row>
     <row r="553" spans="1:12">
       <c r="A553" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B553" t="s">
         <v>593</v>
@@ -27541,7 +27541,7 @@
     </row>
     <row r="556" spans="1:12">
       <c r="A556" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B556" t="s">
         <v>596</v>
@@ -27576,7 +27576,7 @@
     </row>
     <row r="557" spans="1:12">
       <c r="A557" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B557" t="s">
         <v>597</v>
@@ -27611,7 +27611,7 @@
     </row>
     <row r="558" spans="1:12">
       <c r="A558" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B558" t="s">
         <v>598</v>
@@ -27646,7 +27646,7 @@
     </row>
     <row r="559" spans="1:12">
       <c r="A559" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B559" t="s">
         <v>599</v>
@@ -27751,7 +27751,7 @@
     </row>
     <row r="562" spans="1:12">
       <c r="A562" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B562" t="s">
         <v>602</v>
@@ -27824,7 +27824,7 @@
     </row>
     <row r="564" spans="1:12">
       <c r="A564" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B564" t="s">
         <v>604</v>
@@ -27929,7 +27929,7 @@
     </row>
     <row r="567" spans="1:12">
       <c r="A567" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B567" t="s">
         <v>607</v>
@@ -28072,7 +28072,7 @@
     </row>
     <row r="571" spans="1:12">
       <c r="A571" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B571" t="s">
         <v>611</v>
@@ -28142,7 +28142,7 @@
     </row>
     <row r="573" spans="1:12">
       <c r="A573" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B573" t="s">
         <v>613</v>
@@ -28212,7 +28212,7 @@
     </row>
     <row r="575" spans="1:12">
       <c r="A575" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B575" t="s">
         <v>615</v>
@@ -28317,7 +28317,7 @@
     </row>
     <row r="578" spans="1:12">
       <c r="A578" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B578" t="s">
         <v>618</v>
@@ -28387,7 +28387,7 @@
     </row>
     <row r="580" spans="1:12">
       <c r="A580" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B580" t="s">
         <v>620</v>
@@ -28422,7 +28422,7 @@
     </row>
     <row r="581" spans="1:12">
       <c r="A581" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B581" t="s">
         <v>621</v>
@@ -28527,7 +28527,7 @@
     </row>
     <row r="584" spans="1:12">
       <c r="A584" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B584" t="s">
         <v>624</v>
@@ -28565,7 +28565,7 @@
     </row>
     <row r="585" spans="1:12">
       <c r="A585" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B585" t="s">
         <v>625</v>
@@ -28600,7 +28600,7 @@
     </row>
     <row r="586" spans="1:12">
       <c r="A586" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B586" t="s">
         <v>626</v>
@@ -28740,7 +28740,7 @@
     </row>
     <row r="590" spans="1:12">
       <c r="A590" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="B590" t="s">
         <v>630</v>
@@ -28880,7 +28880,7 @@
     </row>
     <row r="594" spans="1:12">
       <c r="A594" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B594" t="s">
         <v>634</v>
@@ -29055,7 +29055,7 @@
     </row>
     <row r="599" spans="1:12">
       <c r="A599" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B599" t="s">
         <v>639</v>
@@ -29166,7 +29166,7 @@
     </row>
     <row r="602" spans="1:12">
       <c r="A602" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="B602" t="s">
         <v>641</v>
@@ -29347,7 +29347,7 @@
     </row>
     <row r="607" spans="1:12">
       <c r="A607" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B607" t="s">
         <v>646</v>
@@ -29528,7 +29528,7 @@
     </row>
     <row r="612" spans="1:12">
       <c r="A612" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B612" t="s">
         <v>651</v>
@@ -29709,7 +29709,7 @@
     </row>
     <row r="617" spans="1:12">
       <c r="A617" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B617" t="s">
         <v>656</v>
@@ -29779,7 +29779,7 @@
     </row>
     <row r="619" spans="1:12">
       <c r="A619" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B619" t="s">
         <v>658</v>
@@ -29849,7 +29849,7 @@
     </row>
     <row r="621" spans="1:12">
       <c r="A621" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B621" t="s">
         <v>660</v>
@@ -29884,7 +29884,7 @@
     </row>
     <row r="622" spans="1:12">
       <c r="A622" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B622" t="s">
         <v>661</v>
@@ -29957,7 +29957,7 @@
     </row>
     <row r="624" spans="1:12">
       <c r="A624" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B624" t="s">
         <v>663</v>
@@ -29992,7 +29992,7 @@
     </row>
     <row r="625" spans="1:12">
       <c r="A625" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B625" t="s">
         <v>664</v>
@@ -30027,7 +30027,7 @@
     </row>
     <row r="626" spans="1:12">
       <c r="A626" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B626" t="s">
         <v>665</v>
@@ -30062,7 +30062,7 @@
     </row>
     <row r="627" spans="1:12">
       <c r="A627" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B627" t="s">
         <v>666</v>
@@ -30132,7 +30132,7 @@
     </row>
     <row r="629" spans="1:12">
       <c r="A629" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B629" t="s">
         <v>668</v>
@@ -30202,7 +30202,7 @@
     </row>
     <row r="631" spans="1:12">
       <c r="A631" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="B631" t="s">
         <v>670</v>
@@ -30237,7 +30237,7 @@
     </row>
     <row r="632" spans="1:12">
       <c r="A632" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B632" t="s">
         <v>671</v>
@@ -30272,7 +30272,7 @@
     </row>
     <row r="633" spans="1:12">
       <c r="A633" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B633" t="s">
         <v>672</v>
@@ -30307,7 +30307,7 @@
     </row>
     <row r="634" spans="1:12">
       <c r="A634" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B634" t="s">
         <v>673</v>
@@ -30342,7 +30342,7 @@
     </row>
     <row r="635" spans="1:12">
       <c r="A635" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B635" t="s">
         <v>674</v>
@@ -30418,7 +30418,7 @@
     </row>
     <row r="637" spans="1:12">
       <c r="A637" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B637" t="s">
         <v>676</v>
@@ -30453,7 +30453,7 @@
     </row>
     <row r="638" spans="1:12">
       <c r="A638" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B638" t="s">
         <v>677</v>
@@ -30488,7 +30488,7 @@
     </row>
     <row r="639" spans="1:12">
       <c r="A639" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B639" t="s">
         <v>678</v>
@@ -30707,7 +30707,7 @@
     </row>
     <row r="645" spans="1:12">
       <c r="A645" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B645" t="s">
         <v>684</v>
@@ -30891,7 +30891,7 @@
     </row>
     <row r="650" spans="1:12">
       <c r="A650" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B650" t="s">
         <v>689</v>
@@ -30929,7 +30929,7 @@
     </row>
     <row r="651" spans="1:12">
       <c r="A651" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B651" t="s">
         <v>690</v>
@@ -30999,7 +30999,7 @@
     </row>
     <row r="653" spans="1:12">
       <c r="A653" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B653" t="s">
         <v>692</v>
@@ -31034,7 +31034,7 @@
     </row>
     <row r="654" spans="1:12">
       <c r="A654" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B654" t="s">
         <v>693</v>
@@ -31069,7 +31069,7 @@
     </row>
     <row r="655" spans="1:12">
       <c r="A655" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B655" t="s">
         <v>694</v>
@@ -31104,7 +31104,7 @@
     </row>
     <row r="656" spans="1:12">
       <c r="A656" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B656" t="s">
         <v>695</v>
@@ -31139,7 +31139,7 @@
     </row>
     <row r="657" spans="1:12">
       <c r="A657" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B657" t="s">
         <v>696</v>
@@ -31177,7 +31177,7 @@
     </row>
     <row r="658" spans="1:12">
       <c r="A658" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B658" t="s">
         <v>697</v>
@@ -31212,7 +31212,7 @@
     </row>
     <row r="659" spans="1:12">
       <c r="A659" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B659" t="s">
         <v>698</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-10-30 20:30:03
</commit_message>
<xml_diff>
--- a/BacklogGATEAutoCompleto.xlsx
+++ b/BacklogGATEAutoCompleto.xlsx
@@ -4843,19 +4843,19 @@
     <t>MOEMA BELLONI SCHMIDT,RENATA DE ARAUJO RIOS</t>
   </si>
   <si>
+    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
+  </si>
+  <si>
+    <t>EDIWAN SOUSA DA SILVA</t>
+  </si>
+  <si>
+    <t>CELSO BARBOSA MONTENEGRO,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
+  </si>
+  <si>
+    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
+  </si>
+  <si>
     <t>LUZIA LAMOSA ARANTES</t>
-  </si>
-  <si>
-    <t>HIAN GOMES DE OLIVEIRA DA COSTA</t>
-  </si>
-  <si>
-    <t>EDIWAN SOUSA DA SILVA</t>
-  </si>
-  <si>
-    <t>CELSO BARBOSA MONTENEGRO,VALÉRIA FERREIRA DA SILVA LÚCIO</t>
-  </si>
-  <si>
-    <t>IZABEL CHRISTINA DE ALCANTARA FIGUEIREDO PIMENTA</t>
   </si>
   <si>
     <t>CELSO BARBOSA MONTENEGRO,CLAUDIA DA SILVA LUNARDI</t>
@@ -10442,7 +10442,7 @@
     </row>
     <row r="69" spans="1:12">
       <c r="A69" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B69" t="s">
         <v>113</v>
@@ -10463,7 +10463,7 @@
         <v>1560</v>
       </c>
       <c r="I69" t="s">
-        <v>1609</v>
+        <v>1591</v>
       </c>
       <c r="J69" t="s">
         <v>1778</v>
@@ -10533,7 +10533,7 @@
         <v>1560</v>
       </c>
       <c r="I71" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="J71" t="s">
         <v>1780</v>
@@ -10603,7 +10603,7 @@
         <v>1560</v>
       </c>
       <c r="I73" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J73" t="s">
         <v>1782</v>
@@ -10638,7 +10638,7 @@
         <v>1560</v>
       </c>
       <c r="I74" t="s">
-        <v>1612</v>
+        <v>1611</v>
       </c>
       <c r="J74" t="s">
         <v>1783</v>
@@ -10673,7 +10673,7 @@
         <v>1560</v>
       </c>
       <c r="I75" t="s">
-        <v>1612</v>
+        <v>1611</v>
       </c>
       <c r="J75" t="s">
         <v>1784</v>
@@ -10743,7 +10743,7 @@
         <v>1560</v>
       </c>
       <c r="I77" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J77" t="s">
         <v>1785</v>
@@ -10813,7 +10813,7 @@
         <v>1560</v>
       </c>
       <c r="I79" t="s">
-        <v>1609</v>
+        <v>1613</v>
       </c>
       <c r="J79" t="s">
         <v>1787</v>
@@ -11443,7 +11443,7 @@
         <v>1560</v>
       </c>
       <c r="I97" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J97" t="s">
         <v>1805</v>
@@ -11583,7 +11583,7 @@
         <v>1560</v>
       </c>
       <c r="I101" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J101" t="s">
         <v>1809</v>
@@ -12108,7 +12108,7 @@
         <v>1560</v>
       </c>
       <c r="I116" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J116" t="s">
         <v>1824</v>
@@ -12423,7 +12423,7 @@
         <v>1560</v>
       </c>
       <c r="I125" t="s">
-        <v>1612</v>
+        <v>1611</v>
       </c>
       <c r="J125" t="s">
         <v>1833</v>
@@ -14736,7 +14736,7 @@
         <v>1560</v>
       </c>
       <c r="I191" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J191" t="s">
         <v>1899</v>
@@ -17930,7 +17930,7 @@
         <v>1566</v>
       </c>
       <c r="I282" t="s">
-        <v>1610</v>
+        <v>1609</v>
       </c>
       <c r="J282" t="s">
         <v>1990</v>
@@ -19365,7 +19365,7 @@
         <v>1560</v>
       </c>
       <c r="I323" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J323" t="s">
         <v>2029</v>
@@ -20771,7 +20771,7 @@
         <v>1560</v>
       </c>
       <c r="I363" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J363" t="s">
         <v>2067</v>
@@ -20841,7 +20841,7 @@
         <v>1560</v>
       </c>
       <c r="I365" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J365" t="s">
         <v>2069</v>
@@ -21226,7 +21226,7 @@
         <v>1560</v>
       </c>
       <c r="I376" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J376" t="s">
         <v>2080</v>
@@ -23084,7 +23084,7 @@
         <v>1560</v>
       </c>
       <c r="I429" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J429" t="s">
         <v>2131</v>
@@ -23650,7 +23650,7 @@
         <v>1566</v>
       </c>
       <c r="I445" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J445" t="s">
         <v>2146</v>
@@ -23933,7 +23933,7 @@
         <v>1560</v>
       </c>
       <c r="I453" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J453" t="s">
         <v>2154</v>
@@ -24181,7 +24181,7 @@
         <v>1560</v>
       </c>
       <c r="I460" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J460" t="s">
         <v>2160</v>
@@ -25164,7 +25164,7 @@
         <v>1560</v>
       </c>
       <c r="I488" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J488" t="s">
         <v>2187</v>
@@ -26150,7 +26150,7 @@
         <v>1560</v>
       </c>
       <c r="I516" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J516" t="s">
         <v>2214</v>
@@ -26220,7 +26220,7 @@
         <v>1560</v>
       </c>
       <c r="I518" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J518" t="s">
         <v>2216</v>
@@ -26290,7 +26290,7 @@
         <v>1560</v>
       </c>
       <c r="I520" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J520" t="s">
         <v>2218</v>
@@ -26748,7 +26748,7 @@
         <v>1560</v>
       </c>
       <c r="I533" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J533" t="s">
         <v>2231</v>
@@ -27664,7 +27664,7 @@
         <v>1560</v>
       </c>
       <c r="I559" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J559" t="s">
         <v>2251</v>
@@ -27842,7 +27842,7 @@
         <v>1560</v>
       </c>
       <c r="I564" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J564" t="s">
         <v>2256</v>
@@ -28265,7 +28265,7 @@
         <v>1560</v>
       </c>
       <c r="I576" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J576" t="s">
         <v>2268</v>
@@ -28898,7 +28898,7 @@
         <v>1560</v>
       </c>
       <c r="I594" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J594" t="s">
         <v>2286</v>
@@ -29073,7 +29073,7 @@
         <v>1560</v>
       </c>
       <c r="I599" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J599" t="s">
         <v>2290</v>
@@ -29254,7 +29254,7 @@
         <v>1560</v>
       </c>
       <c r="I604" t="s">
-        <v>1611</v>
+        <v>1610</v>
       </c>
       <c r="J604" t="s">
         <v>2294</v>
@@ -29867,7 +29867,7 @@
         <v>1560</v>
       </c>
       <c r="I621" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J621" t="s">
         <v>2311</v>
@@ -30471,7 +30471,7 @@
         <v>1560</v>
       </c>
       <c r="I638" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J638" t="s">
         <v>2328</v>
@@ -30912,7 +30912,7 @@
         <v>1567</v>
       </c>
       <c r="I650" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J650" t="s">
         <v>2340</v>
@@ -31017,7 +31017,7 @@
         <v>1560</v>
       </c>
       <c r="I653" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J653" t="s">
         <v>2343</v>
@@ -31230,7 +31230,7 @@
         <v>1560</v>
       </c>
       <c r="I659" t="s">
-        <v>1613</v>
+        <v>1612</v>
       </c>
       <c r="J659" t="s">
         <v>2349</v>

</xml_diff>